<commit_message>
Çarpanlar ve Katlar soru üretici eklendi; web şablonu ortak klasöre taşındı
- CarpanlarKatlar: 425 soruluk havuz (çarpanlar, katlar, asal sayılar,
  asal çarpanlara ayırma, ortak bölenler, ortak katlar)
- Şablona dikdörtgen modeli, sayı doğrusu, çarpan ağacı ve bölen
  merdiveni çizimleri eklendi
- Dosya doğrudan açıldığında boş puan çubuğunun görünmesi düzeltildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6qBE8e6Wkv628t1Q47HQM
</commit_message>
<xml_diff>
--- a/KupSorulari/KupSoruHavuzu.xlsx
+++ b/KupSorulari/KupSoruHavuzu.xlsx
@@ -2144,23 +2144,23 @@
       </c>
       <c r="B12" s="11" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J12))</f>
-        <v>(2 + 4)³ ifadesinin değeri kaçtır?</v>
+        <v>Aşağıdakilerden hangisinin değeri en küçüktür?</v>
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J12))</f>
-        <v>36</v>
+        <v>5³</v>
       </c>
       <c r="D12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J12))</f>
-        <v>18</v>
+        <v>4²</v>
       </c>
       <c r="E12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J12))</f>
-        <v>216</v>
+        <v>10²</v>
       </c>
       <c r="F12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J12))</f>
-        <v>72</v>
+        <v>2⁵</v>
       </c>
       <c r="G12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J12))</f>
@@ -2168,11 +2168,11 @@
       </c>
       <c r="H12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J12))</f>
-        <v>Zor</v>
+        <v>Orta</v>
       </c>
       <c r="J12" s="10" t="n">
         <f aca="false">IF(1&lt;=MIN($B$3,$B$6),MATCH(1,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>88</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2182,149 +2182,149 @@
       </c>
       <c r="B13" s="11" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J13))</f>
-        <v>3³ − 2 · 8 + 6 işleminin sonucu kaçtır?</v>
+        <v>Bir ayrıtı 12 cm olan küp şeklindeki bir kutunun içine, bir ayrıtı 4 cm olan küp şeklindeki kutulardan en fazla kaç tane yerleştirilebilir?</v>
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J13))</f>
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="D13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J13))</f>
-        <v>206</v>
+        <v>54</v>
       </c>
       <c r="E13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J13))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J13))</f>
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J13))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J13))</f>
-        <v>Zor</v>
+        <v>Orta</v>
       </c>
       <c r="J13" s="10" t="n">
         <f aca="false">IF(2&lt;=MIN($B$3,$B$6),MATCH(2,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="n">
         <f aca="false">IF($J14="","",3)</f>
         <v>3</v>
       </c>
       <c r="B14" s="11" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J14))</f>
-        <v>Bir doğal sayının küpünün 13 fazlası 40'dir. Bu sayı kaçtır?</v>
+        <v>Bir ayrıtı 6 cm olan küpün hacmi kaç cm³'tür?</v>
       </c>
       <c r="C14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J14))</f>
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="D14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J14))</f>
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J14))</f>
-        <v>13</v>
+        <v>216</v>
       </c>
       <c r="F14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J14))</f>
-        <v>2</v>
+        <v>72</v>
       </c>
       <c r="G14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J14))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J14))</f>
-        <v>Zor</v>
+        <v>Kolay</v>
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">IF(3&lt;=MIN($B$3,$B$6),MATCH(3,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="n">
         <f aca="false">IF($J15="","",4)</f>
         <v>4</v>
       </c>
       <c r="B15" s="11" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J15))</f>
-        <v>5³ − 3² işleminin sonucu kaçtır?</v>
+        <v>Küpün yüzleri hangi geometrik şekle sahiptir?</v>
       </c>
       <c r="C15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J15))</f>
-        <v>36</v>
+        <v>Üçgen</v>
       </c>
       <c r="D15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J15))</f>
-        <v>116</v>
+        <v>Dikdörtgen</v>
       </c>
       <c r="E15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J15))</f>
-        <v>22</v>
+        <v>Beşgen</v>
       </c>
       <c r="F15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J15))</f>
-        <v>119</v>
+        <v>Kare</v>
       </c>
       <c r="G15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J15))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Özellikleri</v>
       </c>
       <c r="H15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J15))</f>
-        <v>Orta</v>
+        <v>Kolay</v>
       </c>
       <c r="J15" s="10" t="n">
         <f aca="false">IF(4&lt;=MIN($B$3,$B$6),MATCH(4,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="n">
         <f aca="false">IF($J16="","",5)</f>
         <v>5</v>
       </c>
       <c r="B16" s="11" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J16))</f>
-        <v>Bir doğal sayının küpü 64'dir. Bu sayının 2 fazlasının karesi kaçtır?</v>
+        <v>Hacmi 1000 cm³ olan küpün bir ayrıtı kaç cm'dir?</v>
       </c>
       <c r="C16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J16))</f>
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J16))</f>
-        <v>12</v>
+        <v>333</v>
       </c>
       <c r="E16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J16))</f>
-        <v>66</v>
+        <v>9</v>
       </c>
       <c r="F16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J16))</f>
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="G16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J16))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J16))</f>
-        <v>Zor</v>
+        <v>Orta</v>
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">IF(5&lt;=MIN($B$3,$B$6),MATCH(5,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>100</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2334,23 +2334,23 @@
       </c>
       <c r="B17" s="11" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J17))</f>
-        <v>Küpün kaç köşesi vardır?</v>
+        <v>Bir ayrıtı 2 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
       </c>
       <c r="C17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J17))</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J17))</f>
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J17))</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J17))</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J17))</f>
@@ -2358,49 +2358,49 @@
       </c>
       <c r="H17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J17))</f>
-        <v>Kolay</v>
+        <v>Orta</v>
       </c>
       <c r="J17" s="10" t="n">
         <f aca="false">IF(6&lt;=MIN($B$3,$B$6),MATCH(6,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>171</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="n">
         <f aca="false">IF($J18="","",7)</f>
         <v>7</v>
       </c>
       <c r="B18" s="11" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J18))</f>
-        <v>Bir doğal sayının küpünün 6 fazlası 70'dir. Bu sayı kaçtır?</v>
+        <v>Bir ayrıtı 5 birim olan küp kaç birim küpten oluşur?</v>
       </c>
       <c r="C18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J18))</f>
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="D18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J18))</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J18))</f>
-        <v>23</v>
+        <v>125</v>
       </c>
       <c r="F18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J18))</f>
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J18))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J18))</f>
-        <v>Zor</v>
+        <v>Kolay</v>
       </c>
       <c r="J18" s="10" t="n">
         <f aca="false">IF(7&lt;=MIN($B$3,$B$6),MATCH(7,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>91</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2410,23 +2410,23 @@
       </c>
       <c r="B19" s="11" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J19))</f>
-        <v>Bir ayrıtı 10 cm olan küp şeklindeki bir kutunun içine, bir ayrıtı 2 cm olan küp şeklindeki kutulardan en fazla kaç tane yerleştirilebilir?</v>
+        <v>Bir ayrıtı 40 cm olan küp şeklindeki su deposu kaç litre su alır? (1 L = 1000 cm³)</v>
       </c>
       <c r="C19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J19))</f>
-        <v>125</v>
+        <v>16 L</v>
       </c>
       <c r="D19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J19))</f>
-        <v>15</v>
+        <v>64 L</v>
       </c>
       <c r="E19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J19))</f>
-        <v>25</v>
+        <v>12 L</v>
       </c>
       <c r="F19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J19))</f>
-        <v>5</v>
+        <v>640 L</v>
       </c>
       <c r="G19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J19))</f>
@@ -2434,67 +2434,67 @@
       </c>
       <c r="H19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J19))</f>
-        <v>Orta</v>
+        <v>Zor</v>
       </c>
       <c r="J19" s="10" t="n">
         <f aca="false">IF(8&lt;=MIN($B$3,$B$6),MATCH(8,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>137</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="n">
         <f aca="false">IF($J20="","",9)</f>
         <v>9</v>
       </c>
       <c r="B20" s="11" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J20))</f>
-        <v>Hacmi 343 cm³ olan küpün bir ayrıtı kaç cm'dir?</v>
+        <v>Bir doğal sayının küpünün 6 fazlası 70'dir. Bu sayı kaçtır?</v>
       </c>
       <c r="C20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J20))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J20))</f>
-        <v>114</v>
+        <v>5</v>
       </c>
       <c r="E20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J20))</f>
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J20))</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J20))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J20))</f>
-        <v>Orta</v>
+        <v>Zor</v>
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">IF(9&lt;=MIN($B$3,$B$6),MATCH(9,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>124</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="n">
         <f aca="false">IF($J21="","",10)</f>
         <v>10</v>
       </c>
       <c r="B21" s="11" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J21))</f>
-        <v>4³ ifadesinin değeri kaçtır?</v>
+        <v>Birim küplerden oluşan bir küpün dış yüzeyi boyanıyor. 3 yüzü boyalı kaç birim küp vardır?</v>
       </c>
       <c r="C21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J21))</f>
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="D21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J21))</f>
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J21))</f>
@@ -2502,19 +2502,19 @@
       </c>
       <c r="F21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J21))</f>
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J21))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Özellikleri</v>
       </c>
       <c r="H21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J21))</f>
-        <v>Kolay</v>
+        <v>Zor</v>
       </c>
       <c r="J21" s="10" t="n">
         <f aca="false">IF(10&lt;=MIN($B$3,$B$6),MATCH(10,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>4</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6063,11 +6063,11 @@
       </c>
       <c r="K2" s="10" t="n">
         <f aca="true">IF($J2=1,RAND(),-1)</f>
-        <v>0.321054743125979</v>
+        <v>0.904295007931261</v>
       </c>
       <c r="L2" s="10" t="n">
         <f aca="false">IF($J2=1,RANK($K2,$K$2:$K$1001),"")</f>
-        <v>160</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6104,11 +6104,11 @@
       </c>
       <c r="K3" s="10" t="n">
         <f aca="true">IF($J3=1,RAND(),-1)</f>
-        <v>0.384598888308546</v>
+        <v>0.347832027480229</v>
       </c>
       <c r="L3" s="10" t="n">
         <f aca="false">IF($J3=1,RANK($K3,$K$2:$K$1001),"")</f>
-        <v>143</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6145,11 +6145,11 @@
       </c>
       <c r="K4" s="10" t="n">
         <f aca="true">IF($J4=1,RAND(),-1)</f>
-        <v>0.0584539293938929</v>
+        <v>0.750082894605377</v>
       </c>
       <c r="L4" s="10" t="n">
         <f aca="false">IF($J4=1,RANK($K4,$K$2:$K$1001),"")</f>
-        <v>215</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6186,11 +6186,11 @@
       </c>
       <c r="K5" s="10" t="n">
         <f aca="true">IF($J5=1,RAND(),-1)</f>
-        <v>0.964264205427944</v>
+        <v>0.208943243672564</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">IF($J5=1,RANK($K5,$K$2:$K$1001),"")</f>
-        <v>10</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6227,11 +6227,11 @@
       </c>
       <c r="K6" s="10" t="n">
         <f aca="true">IF($J6=1,RAND(),-1)</f>
-        <v>0.878112697859801</v>
+        <v>0.918706047564604</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">IF($J6=1,RANK($K6,$K$2:$K$1001),"")</f>
-        <v>40</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6268,11 +6268,11 @@
       </c>
       <c r="K7" s="10" t="n">
         <f aca="true">IF($J7=1,RAND(),-1)</f>
-        <v>0.539691346544046</v>
+        <v>0.421819935215955</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">IF($J7=1,RANK($K7,$K$2:$K$1001),"")</f>
-        <v>112</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6309,11 +6309,11 @@
       </c>
       <c r="K8" s="10" t="n">
         <f aca="true">IF($J8=1,RAND(),-1)</f>
-        <v>0.377301601442696</v>
+        <v>0.47111732576979</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">IF($J8=1,RANK($K8,$K$2:$K$1001),"")</f>
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6350,11 +6350,11 @@
       </c>
       <c r="K9" s="10" t="n">
         <f aca="true">IF($J9=1,RAND(),-1)</f>
-        <v>0.901221280518825</v>
+        <v>0.607174716423806</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">IF($J9=1,RANK($K9,$K$2:$K$1001),"")</f>
-        <v>30</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6391,11 +6391,11 @@
       </c>
       <c r="K10" s="10" t="n">
         <f aca="true">IF($J10=1,RAND(),-1)</f>
-        <v>0.887589376721244</v>
+        <v>0.556146243639258</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">IF($J10=1,RANK($K10,$K$2:$K$1001),"")</f>
-        <v>36</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6432,11 +6432,11 @@
       </c>
       <c r="K11" s="10" t="n">
         <f aca="true">IF($J11=1,RAND(),-1)</f>
-        <v>0.238642843824526</v>
+        <v>0.893599285111705</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">IF($J11=1,RANK($K11,$K$2:$K$1001),"")</f>
-        <v>182</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6473,11 +6473,11 @@
       </c>
       <c r="K12" s="10" t="n">
         <f aca="true">IF($J12=1,RAND(),-1)</f>
-        <v>0.0848996340027945</v>
+        <v>0.563962333146206</v>
       </c>
       <c r="L12" s="10" t="n">
         <f aca="false">IF($J12=1,RANK($K12,$K$2:$K$1001),"")</f>
-        <v>208</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6514,11 +6514,11 @@
       </c>
       <c r="K13" s="10" t="n">
         <f aca="true">IF($J13=1,RAND(),-1)</f>
-        <v>0.40265740129931</v>
+        <v>0.779208103293628</v>
       </c>
       <c r="L13" s="10" t="n">
         <f aca="false">IF($J13=1,RANK($K13,$K$2:$K$1001),"")</f>
-        <v>139</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6555,11 +6555,11 @@
       </c>
       <c r="K14" s="10" t="n">
         <f aca="true">IF($J14=1,RAND(),-1)</f>
-        <v>0.392341153389639</v>
+        <v>0.334655143949095</v>
       </c>
       <c r="L14" s="10" t="n">
         <f aca="false">IF($J14=1,RANK($K14,$K$2:$K$1001),"")</f>
-        <v>141</v>
+        <v>169</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6596,11 +6596,11 @@
       </c>
       <c r="K15" s="10" t="n">
         <f aca="true">IF($J15=1,RAND(),-1)</f>
-        <v>0.786839504409143</v>
+        <v>0.644995654731458</v>
       </c>
       <c r="L15" s="10" t="n">
         <f aca="false">IF($J15=1,RANK($K15,$K$2:$K$1001),"")</f>
-        <v>61</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6637,11 +6637,11 @@
       </c>
       <c r="K16" s="10" t="n">
         <f aca="true">IF($J16=1,RAND(),-1)</f>
-        <v>0.942831377147614</v>
+        <v>0.619759625644779</v>
       </c>
       <c r="L16" s="10" t="n">
         <f aca="false">IF($J16=1,RANK($K16,$K$2:$K$1001),"")</f>
-        <v>16</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6678,11 +6678,11 @@
       </c>
       <c r="K17" s="10" t="n">
         <f aca="true">IF($J17=1,RAND(),-1)</f>
-        <v>0.522420653331653</v>
+        <v>0.698544711384879</v>
       </c>
       <c r="L17" s="10" t="n">
         <f aca="false">IF($J17=1,RANK($K17,$K$2:$K$1001),"")</f>
-        <v>115</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6719,11 +6719,11 @@
       </c>
       <c r="K18" s="10" t="n">
         <f aca="true">IF($J18=1,RAND(),-1)</f>
-        <v>0.957458184295798</v>
+        <v>0.0381110063181314</v>
       </c>
       <c r="L18" s="10" t="n">
         <f aca="false">IF($J18=1,RANK($K18,$K$2:$K$1001),"")</f>
-        <v>14</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="K19" s="10" t="n">
         <f aca="true">IF($J19=1,RAND(),-1)</f>
-        <v>0.676618859001941</v>
+        <v>0.687625955122907</v>
       </c>
       <c r="L19" s="10" t="n">
         <f aca="false">IF($J19=1,RANK($K19,$K$2:$K$1001),"")</f>
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6801,11 +6801,11 @@
       </c>
       <c r="K20" s="10" t="n">
         <f aca="true">IF($J20=1,RAND(),-1)</f>
-        <v>0.343285887777687</v>
+        <v>0.765734535717859</v>
       </c>
       <c r="L20" s="10" t="n">
         <f aca="false">IF($J20=1,RANK($K20,$K$2:$K$1001),"")</f>
-        <v>157</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6842,11 +6842,11 @@
       </c>
       <c r="K21" s="10" t="n">
         <f aca="true">IF($J21=1,RAND(),-1)</f>
-        <v>0.000724066322001364</v>
+        <v>0.452288454609707</v>
       </c>
       <c r="L21" s="10" t="n">
         <f aca="false">IF($J21=1,RANK($K21,$K$2:$K$1001),"")</f>
-        <v>224</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="K22" s="10" t="n">
         <f aca="true">IF($J22=1,RAND(),-1)</f>
-        <v>0.0457418539055362</v>
+        <v>0.129526145422593</v>
       </c>
       <c r="L22" s="10" t="n">
         <f aca="false">IF($J22=1,RANK($K22,$K$2:$K$1001),"")</f>
-        <v>218</v>
+        <v>194</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6924,11 +6924,11 @@
       </c>
       <c r="K23" s="10" t="n">
         <f aca="true">IF($J23=1,RAND(),-1)</f>
-        <v>0.921391476025998</v>
+        <v>0.758716552972226</v>
       </c>
       <c r="L23" s="10" t="n">
         <f aca="false">IF($J23=1,RANK($K23,$K$2:$K$1001),"")</f>
-        <v>22</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6965,11 +6965,11 @@
       </c>
       <c r="K24" s="10" t="n">
         <f aca="true">IF($J24=1,RAND(),-1)</f>
-        <v>0.517640079057633</v>
+        <v>0.122989473265731</v>
       </c>
       <c r="L24" s="10" t="n">
         <f aca="false">IF($J24=1,RANK($K24,$K$2:$K$1001),"")</f>
-        <v>117</v>
+        <v>196</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7006,11 +7006,11 @@
       </c>
       <c r="K25" s="10" t="n">
         <f aca="true">IF($J25=1,RAND(),-1)</f>
-        <v>0.83773920364386</v>
+        <v>0.08448286353226</v>
       </c>
       <c r="L25" s="10" t="n">
         <f aca="false">IF($J25=1,RANK($K25,$K$2:$K$1001),"")</f>
-        <v>50</v>
+        <v>205</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7047,11 +7047,11 @@
       </c>
       <c r="K26" s="10" t="n">
         <f aca="true">IF($J26=1,RAND(),-1)</f>
-        <v>0.890775600679341</v>
+        <v>0.275418033471049</v>
       </c>
       <c r="L26" s="10" t="n">
         <f aca="false">IF($J26=1,RANK($K26,$K$2:$K$1001),"")</f>
-        <v>35</v>
+        <v>174</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7088,11 +7088,11 @@
       </c>
       <c r="K27" s="10" t="n">
         <f aca="true">IF($J27=1,RAND(),-1)</f>
-        <v>0.865913314557069</v>
+        <v>0.954656548506431</v>
       </c>
       <c r="L27" s="10" t="n">
         <f aca="false">IF($J27=1,RANK($K27,$K$2:$K$1001),"")</f>
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7129,11 +7129,11 @@
       </c>
       <c r="K28" s="10" t="n">
         <f aca="true">IF($J28=1,RAND(),-1)</f>
-        <v>0.0857687784112365</v>
+        <v>0.422555556138029</v>
       </c>
       <c r="L28" s="10" t="n">
         <f aca="false">IF($J28=1,RANK($K28,$K$2:$K$1001),"")</f>
-        <v>207</v>
+        <v>142</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7170,11 +7170,11 @@
       </c>
       <c r="K29" s="10" t="n">
         <f aca="true">IF($J29=1,RAND(),-1)</f>
-        <v>0.314745757426291</v>
+        <v>0.22260363951565</v>
       </c>
       <c r="L29" s="10" t="n">
         <f aca="false">IF($J29=1,RANK($K29,$K$2:$K$1001),"")</f>
-        <v>162</v>
+        <v>180</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7211,11 +7211,11 @@
       </c>
       <c r="K30" s="10" t="n">
         <f aca="true">IF($J30=1,RAND(),-1)</f>
-        <v>0.506376367625587</v>
+        <v>0.892300576640369</v>
       </c>
       <c r="L30" s="10" t="n">
         <f aca="false">IF($J30=1,RANK($K30,$K$2:$K$1001),"")</f>
-        <v>121</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7252,11 +7252,11 @@
       </c>
       <c r="K31" s="10" t="n">
         <f aca="true">IF($J31=1,RAND(),-1)</f>
-        <v>0.880175985271621</v>
+        <v>0.066248128534441</v>
       </c>
       <c r="L31" s="10" t="n">
         <f aca="false">IF($J31=1,RANK($K31,$K$2:$K$1001),"")</f>
-        <v>39</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7293,11 +7293,11 @@
       </c>
       <c r="K32" s="10" t="n">
         <f aca="true">IF($J32=1,RAND(),-1)</f>
-        <v>0.7582180147776</v>
+        <v>0.844167020171817</v>
       </c>
       <c r="L32" s="10" t="n">
         <f aca="false">IF($J32=1,RANK($K32,$K$2:$K$1001),"")</f>
-        <v>66</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7334,11 +7334,11 @@
       </c>
       <c r="K33" s="10" t="n">
         <f aca="true">IF($J33=1,RAND(),-1)</f>
-        <v>0.701904527115478</v>
+        <v>0.726525481264205</v>
       </c>
       <c r="L33" s="10" t="n">
         <f aca="false">IF($J33=1,RANK($K33,$K$2:$K$1001),"")</f>
-        <v>79</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7375,11 +7375,11 @@
       </c>
       <c r="K34" s="10" t="n">
         <f aca="true">IF($J34=1,RAND(),-1)</f>
-        <v>0.501122557004555</v>
+        <v>0.808747741055165</v>
       </c>
       <c r="L34" s="10" t="n">
         <f aca="false">IF($J34=1,RANK($K34,$K$2:$K$1001),"")</f>
-        <v>123</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7416,11 +7416,11 @@
       </c>
       <c r="K35" s="10" t="n">
         <f aca="true">IF($J35=1,RAND(),-1)</f>
-        <v>0.186892210539637</v>
+        <v>0.680875338208257</v>
       </c>
       <c r="L35" s="10" t="n">
         <f aca="false">IF($J35=1,RANK($K35,$K$2:$K$1001),"")</f>
-        <v>192</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7457,11 +7457,11 @@
       </c>
       <c r="K36" s="10" t="n">
         <f aca="true">IF($J36=1,RAND(),-1)</f>
-        <v>0.450703786045933</v>
+        <v>0.536375961688599</v>
       </c>
       <c r="L36" s="10" t="n">
         <f aca="false">IF($J36=1,RANK($K36,$K$2:$K$1001),"")</f>
-        <v>131</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7498,11 +7498,11 @@
       </c>
       <c r="K37" s="10" t="n">
         <f aca="true">IF($J37=1,RAND(),-1)</f>
-        <v>0.899058941479296</v>
+        <v>0.361172896427552</v>
       </c>
       <c r="L37" s="10" t="n">
         <f aca="false">IF($J37=1,RANK($K37,$K$2:$K$1001),"")</f>
-        <v>31</v>
+        <v>160</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7539,11 +7539,11 @@
       </c>
       <c r="K38" s="10" t="n">
         <f aca="true">IF($J38=1,RAND(),-1)</f>
-        <v>0.893750505903681</v>
+        <v>0.471302650246549</v>
       </c>
       <c r="L38" s="10" t="n">
         <f aca="false">IF($J38=1,RANK($K38,$K$2:$K$1001),"")</f>
-        <v>33</v>
+        <v>133</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7580,11 +7580,11 @@
       </c>
       <c r="K39" s="10" t="n">
         <f aca="true">IF($J39=1,RAND(),-1)</f>
-        <v>0.699502659717926</v>
+        <v>0.782620755840389</v>
       </c>
       <c r="L39" s="10" t="n">
         <f aca="false">IF($J39=1,RANK($K39,$K$2:$K$1001),"")</f>
-        <v>80</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7621,11 +7621,11 @@
       </c>
       <c r="K40" s="10" t="n">
         <f aca="true">IF($J40=1,RAND(),-1)</f>
-        <v>0.926218829384034</v>
+        <v>0.756501435086049</v>
       </c>
       <c r="L40" s="10" t="n">
         <f aca="false">IF($J40=1,RANK($K40,$K$2:$K$1001),"")</f>
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7662,11 +7662,11 @@
       </c>
       <c r="K41" s="10" t="n">
         <f aca="true">IF($J41=1,RAND(),-1)</f>
-        <v>0.365871547366787</v>
+        <v>0.655292643470257</v>
       </c>
       <c r="L41" s="10" t="n">
         <f aca="false">IF($J41=1,RANK($K41,$K$2:$K$1001),"")</f>
-        <v>149</v>
+        <v>89</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7703,11 +7703,11 @@
       </c>
       <c r="K42" s="10" t="n">
         <f aca="true">IF($J42=1,RAND(),-1)</f>
-        <v>0.722900099692097</v>
+        <v>0.668420087896298</v>
       </c>
       <c r="L42" s="10" t="n">
         <f aca="false">IF($J42=1,RANK($K42,$K$2:$K$1001),"")</f>
-        <v>72</v>
+        <v>87</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7744,11 +7744,11 @@
       </c>
       <c r="K43" s="10" t="n">
         <f aca="true">IF($J43=1,RAND(),-1)</f>
-        <v>0.354702512490873</v>
+        <v>0.0476734288266797</v>
       </c>
       <c r="L43" s="10" t="n">
         <f aca="false">IF($J43=1,RANK($K43,$K$2:$K$1001),"")</f>
-        <v>152</v>
+        <v>214</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7785,11 +7785,11 @@
       </c>
       <c r="K44" s="10" t="n">
         <f aca="true">IF($J44=1,RAND(),-1)</f>
-        <v>0.361303861545298</v>
+        <v>0.747040795286031</v>
       </c>
       <c r="L44" s="10" t="n">
         <f aca="false">IF($J44=1,RANK($K44,$K$2:$K$1001),"")</f>
-        <v>151</v>
+        <v>62</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7826,11 +7826,11 @@
       </c>
       <c r="K45" s="10" t="n">
         <f aca="true">IF($J45=1,RAND(),-1)</f>
-        <v>0.460027294507204</v>
+        <v>0.340781259847172</v>
       </c>
       <c r="L45" s="10" t="n">
         <f aca="false">IF($J45=1,RANK($K45,$K$2:$K$1001),"")</f>
-        <v>129</v>
+        <v>167</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7867,11 +7867,11 @@
       </c>
       <c r="K46" s="10" t="n">
         <f aca="true">IF($J46=1,RAND(),-1)</f>
-        <v>0.868418682904993</v>
+        <v>0.325524596297083</v>
       </c>
       <c r="L46" s="10" t="n">
         <f aca="false">IF($J46=1,RANK($K46,$K$2:$K$1001),"")</f>
-        <v>42</v>
+        <v>171</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7908,11 +7908,11 @@
       </c>
       <c r="K47" s="10" t="n">
         <f aca="true">IF($J47=1,RAND(),-1)</f>
-        <v>0.256270084092139</v>
+        <v>0.933956665100782</v>
       </c>
       <c r="L47" s="10" t="n">
         <f aca="false">IF($J47=1,RANK($K47,$K$2:$K$1001),"")</f>
-        <v>181</v>
+        <v>19</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7949,11 +7949,11 @@
       </c>
       <c r="K48" s="10" t="n">
         <f aca="true">IF($J48=1,RAND(),-1)</f>
-        <v>0.852781338620763</v>
+        <v>0.763986664084633</v>
       </c>
       <c r="L48" s="10" t="n">
         <f aca="false">IF($J48=1,RANK($K48,$K$2:$K$1001),"")</f>
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7990,11 +7990,11 @@
       </c>
       <c r="K49" s="10" t="n">
         <f aca="true">IF($J49=1,RAND(),-1)</f>
-        <v>0.544231872300435</v>
+        <v>0.353676881976362</v>
       </c>
       <c r="L49" s="10" t="n">
         <f aca="false">IF($J49=1,RANK($K49,$K$2:$K$1001),"")</f>
-        <v>110</v>
+        <v>164</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8031,11 +8031,11 @@
       </c>
       <c r="K50" s="10" t="n">
         <f aca="true">IF($J50=1,RAND(),-1)</f>
-        <v>0.187341488260824</v>
+        <v>0.200278989353445</v>
       </c>
       <c r="L50" s="10" t="n">
         <f aca="false">IF($J50=1,RANK($K50,$K$2:$K$1001),"")</f>
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8072,11 +8072,11 @@
       </c>
       <c r="K51" s="10" t="n">
         <f aca="true">IF($J51=1,RAND(),-1)</f>
-        <v>0.987376308701382</v>
+        <v>0.724833098385281</v>
       </c>
       <c r="L51" s="10" t="n">
         <f aca="false">IF($J51=1,RANK($K51,$K$2:$K$1001),"")</f>
-        <v>4</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8113,11 +8113,11 @@
       </c>
       <c r="K52" s="10" t="n">
         <f aca="true">IF($J52=1,RAND(),-1)</f>
-        <v>0.672635435722617</v>
+        <v>0.402392725859177</v>
       </c>
       <c r="L52" s="10" t="n">
         <f aca="false">IF($J52=1,RANK($K52,$K$2:$K$1001),"")</f>
-        <v>88</v>
+        <v>148</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8154,11 +8154,11 @@
       </c>
       <c r="K53" s="10" t="n">
         <f aca="true">IF($J53=1,RAND(),-1)</f>
-        <v>0.912999142346874</v>
+        <v>0.266176952336694</v>
       </c>
       <c r="L53" s="10" t="n">
         <f aca="false">IF($J53=1,RANK($K53,$K$2:$K$1001),"")</f>
-        <v>27</v>
+        <v>176</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8195,11 +8195,11 @@
       </c>
       <c r="K54" s="10" t="n">
         <f aca="true">IF($J54=1,RAND(),-1)</f>
-        <v>0.791459022159191</v>
+        <v>0.78933696993077</v>
       </c>
       <c r="L54" s="10" t="n">
         <f aca="false">IF($J54=1,RANK($K54,$K$2:$K$1001),"")</f>
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8236,11 +8236,11 @@
       </c>
       <c r="K55" s="10" t="n">
         <f aca="true">IF($J55=1,RAND(),-1)</f>
-        <v>0.412007636541367</v>
+        <v>0.547697860727407</v>
       </c>
       <c r="L55" s="10" t="n">
         <f aca="false">IF($J55=1,RANK($K55,$K$2:$K$1001),"")</f>
-        <v>137</v>
+        <v>113</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8277,11 +8277,11 @@
       </c>
       <c r="K56" s="10" t="n">
         <f aca="true">IF($J56=1,RAND(),-1)</f>
-        <v>0.588766651369442</v>
+        <v>0.510707930871119</v>
       </c>
       <c r="L56" s="10" t="n">
         <f aca="false">IF($J56=1,RANK($K56,$K$2:$K$1001),"")</f>
-        <v>102</v>
+        <v>120</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8318,11 +8318,11 @@
       </c>
       <c r="K57" s="10" t="n">
         <f aca="true">IF($J57=1,RAND(),-1)</f>
-        <v>0.582070069754401</v>
+        <v>0.906484637982813</v>
       </c>
       <c r="L57" s="10" t="n">
         <f aca="false">IF($J57=1,RANK($K57,$K$2:$K$1001),"")</f>
-        <v>103</v>
+        <v>26</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8359,11 +8359,11 @@
       </c>
       <c r="K58" s="10" t="n">
         <f aca="true">IF($J58=1,RAND(),-1)</f>
-        <v>0.882069771769106</v>
+        <v>0.718851959362426</v>
       </c>
       <c r="L58" s="10" t="n">
         <f aca="false">IF($J58=1,RANK($K58,$K$2:$K$1001),"")</f>
-        <v>37</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8400,11 +8400,11 @@
       </c>
       <c r="K59" s="10" t="n">
         <f aca="true">IF($J59=1,RAND(),-1)</f>
-        <v>0.913187256043816</v>
+        <v>0.195184762927591</v>
       </c>
       <c r="L59" s="10" t="n">
         <f aca="false">IF($J59=1,RANK($K59,$K$2:$K$1001),"")</f>
-        <v>26</v>
+        <v>186</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8441,11 +8441,11 @@
       </c>
       <c r="K60" s="10" t="n">
         <f aca="true">IF($J60=1,RAND(),-1)</f>
-        <v>0.460745389743696</v>
+        <v>0.999551985157311</v>
       </c>
       <c r="L60" s="10" t="n">
         <f aca="false">IF($J60=1,RANK($K60,$K$2:$K$1001),"")</f>
-        <v>128</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8482,11 +8482,11 @@
       </c>
       <c r="K61" s="10" t="n">
         <f aca="true">IF($J61=1,RAND(),-1)</f>
-        <v>0.00298708153362025</v>
+        <v>0.510102461717866</v>
       </c>
       <c r="L61" s="10" t="n">
         <f aca="false">IF($J61=1,RANK($K61,$K$2:$K$1001),"")</f>
-        <v>223</v>
+        <v>121</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8523,11 +8523,11 @@
       </c>
       <c r="K62" s="10" t="n">
         <f aca="true">IF($J62=1,RAND(),-1)</f>
-        <v>0.344648717623054</v>
+        <v>0.717626235737797</v>
       </c>
       <c r="L62" s="10" t="n">
         <f aca="false">IF($J62=1,RANK($K62,$K$2:$K$1001),"")</f>
-        <v>155</v>
+        <v>72</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8564,11 +8564,11 @@
       </c>
       <c r="K63" s="10" t="n">
         <f aca="true">IF($J63=1,RAND(),-1)</f>
-        <v>0.86646519515439</v>
+        <v>0.113315961125073</v>
       </c>
       <c r="L63" s="10" t="n">
         <f aca="false">IF($J63=1,RANK($K63,$K$2:$K$1001),"")</f>
-        <v>43</v>
+        <v>198</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8605,11 +8605,11 @@
       </c>
       <c r="K64" s="10" t="n">
         <f aca="true">IF($J64=1,RAND(),-1)</f>
-        <v>0.699236504990158</v>
+        <v>0.6495412141826</v>
       </c>
       <c r="L64" s="10" t="n">
         <f aca="false">IF($J64=1,RANK($K64,$K$2:$K$1001),"")</f>
-        <v>81</v>
+        <v>92</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8646,11 +8646,11 @@
       </c>
       <c r="K65" s="10" t="n">
         <f aca="true">IF($J65=1,RAND(),-1)</f>
-        <v>0.292590538664918</v>
+        <v>0.800251729270813</v>
       </c>
       <c r="L65" s="10" t="n">
         <f aca="false">IF($J65=1,RANK($K65,$K$2:$K$1001),"")</f>
-        <v>167</v>
+        <v>49</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8687,11 +8687,11 @@
       </c>
       <c r="K66" s="10" t="n">
         <f aca="true">IF($J66=1,RAND(),-1)</f>
-        <v>0.398419145902015</v>
+        <v>0.0156827454217206</v>
       </c>
       <c r="L66" s="10" t="n">
         <f aca="false">IF($J66=1,RANK($K66,$K$2:$K$1001),"")</f>
-        <v>140</v>
+        <v>223</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8728,11 +8728,11 @@
       </c>
       <c r="K67" s="10" t="n">
         <f aca="true">IF($J67=1,RAND(),-1)</f>
-        <v>0.545871419506997</v>
+        <v>0.357769525282947</v>
       </c>
       <c r="L67" s="10" t="n">
         <f aca="false">IF($J67=1,RANK($K67,$K$2:$K$1001),"")</f>
-        <v>108</v>
+        <v>162</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8769,11 +8769,11 @@
       </c>
       <c r="K68" s="10" t="n">
         <f aca="true">IF($J68=1,RAND(),-1)</f>
-        <v>0.267855345571095</v>
+        <v>0.397190967643178</v>
       </c>
       <c r="L68" s="10" t="n">
         <f aca="false">IF($J68=1,RANK($K68,$K$2:$K$1001),"")</f>
-        <v>176</v>
+        <v>150</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8810,11 +8810,11 @@
       </c>
       <c r="K69" s="10" t="n">
         <f aca="true">IF($J69=1,RAND(),-1)</f>
-        <v>0.0821801429982869</v>
+        <v>0.390710393683268</v>
       </c>
       <c r="L69" s="10" t="n">
         <f aca="false">IF($J69=1,RANK($K69,$K$2:$K$1001),"")</f>
-        <v>209</v>
+        <v>153</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8851,11 +8851,11 @@
       </c>
       <c r="K70" s="10" t="n">
         <f aca="true">IF($J70=1,RAND(),-1)</f>
-        <v>0.304385614801334</v>
+        <v>0.421121987436668</v>
       </c>
       <c r="L70" s="10" t="n">
         <f aca="false">IF($J70=1,RANK($K70,$K$2:$K$1001),"")</f>
-        <v>165</v>
+        <v>146</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8892,11 +8892,11 @@
       </c>
       <c r="K71" s="10" t="n">
         <f aca="true">IF($J71=1,RAND(),-1)</f>
-        <v>0.0930600873597427</v>
+        <v>0.135218157428132</v>
       </c>
       <c r="L71" s="10" t="n">
         <f aca="false">IF($J71=1,RANK($K71,$K$2:$K$1001),"")</f>
-        <v>204</v>
+        <v>192</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="K72" s="10" t="n">
         <f aca="true">IF($J72=1,RAND(),-1)</f>
-        <v>0.783845477698188</v>
+        <v>0.499212467498197</v>
       </c>
       <c r="L72" s="10" t="n">
         <f aca="false">IF($J72=1,RANK($K72,$K$2:$K$1001),"")</f>
-        <v>62</v>
+        <v>125</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8974,11 +8974,11 @@
       </c>
       <c r="K73" s="10" t="n">
         <f aca="true">IF($J73=1,RAND(),-1)</f>
-        <v>0.551447586111324</v>
+        <v>0.437854155122886</v>
       </c>
       <c r="L73" s="10" t="n">
         <f aca="false">IF($J73=1,RANK($K73,$K$2:$K$1001),"")</f>
-        <v>106</v>
+        <v>140</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9015,11 +9015,11 @@
       </c>
       <c r="K74" s="10" t="n">
         <f aca="true">IF($J74=1,RAND(),-1)</f>
-        <v>0.957629302549045</v>
+        <v>0.69375450282616</v>
       </c>
       <c r="L74" s="10" t="n">
         <f aca="false">IF($J74=1,RANK($K74,$K$2:$K$1001),"")</f>
-        <v>13</v>
+        <v>75</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9056,11 +9056,11 @@
       </c>
       <c r="K75" s="10" t="n">
         <f aca="true">IF($J75=1,RAND(),-1)</f>
-        <v>0.702731174713981</v>
+        <v>0.67673852045873</v>
       </c>
       <c r="L75" s="10" t="n">
         <f aca="false">IF($J75=1,RANK($K75,$K$2:$K$1001),"")</f>
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9097,11 +9097,11 @@
       </c>
       <c r="K76" s="10" t="n">
         <f aca="true">IF($J76=1,RAND(),-1)</f>
-        <v>0.721176495709353</v>
+        <v>0.766690813614934</v>
       </c>
       <c r="L76" s="10" t="n">
         <f aca="false">IF($J76=1,RANK($K76,$K$2:$K$1001),"")</f>
-        <v>73</v>
+        <v>54</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9138,11 +9138,11 @@
       </c>
       <c r="K77" s="10" t="n">
         <f aca="true">IF($J77=1,RAND(),-1)</f>
-        <v>0.609349200640748</v>
+        <v>0.718404063346434</v>
       </c>
       <c r="L77" s="10" t="n">
         <f aca="false">IF($J77=1,RANK($K77,$K$2:$K$1001),"")</f>
-        <v>96</v>
+        <v>71</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9179,11 +9179,11 @@
       </c>
       <c r="K78" s="10" t="n">
         <f aca="true">IF($J78=1,RAND(),-1)</f>
-        <v>0.42359316996192</v>
+        <v>0.488931431906967</v>
       </c>
       <c r="L78" s="10" t="n">
         <f aca="false">IF($J78=1,RANK($K78,$K$2:$K$1001),"")</f>
-        <v>135</v>
+        <v>127</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9220,11 +9220,11 @@
       </c>
       <c r="K79" s="10" t="n">
         <f aca="true">IF($J79=1,RAND(),-1)</f>
-        <v>0.993072330924769</v>
+        <v>0.421980951200375</v>
       </c>
       <c r="L79" s="10" t="n">
         <f aca="false">IF($J79=1,RANK($K79,$K$2:$K$1001),"")</f>
-        <v>2</v>
+        <v>143</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9261,11 +9261,11 @@
       </c>
       <c r="K80" s="10" t="n">
         <f aca="true">IF($J80=1,RAND(),-1)</f>
-        <v>0.927402017909473</v>
+        <v>0.655296912166902</v>
       </c>
       <c r="L80" s="10" t="n">
         <f aca="false">IF($J80=1,RANK($K80,$K$2:$K$1001),"")</f>
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9302,11 +9302,11 @@
       </c>
       <c r="K81" s="10" t="n">
         <f aca="true">IF($J81=1,RAND(),-1)</f>
-        <v>0.790285622397383</v>
+        <v>0.529114095023939</v>
       </c>
       <c r="L81" s="10" t="n">
         <f aca="false">IF($J81=1,RANK($K81,$K$2:$K$1001),"")</f>
-        <v>60</v>
+        <v>117</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9343,11 +9343,11 @@
       </c>
       <c r="K82" s="10" t="n">
         <f aca="true">IF($J82=1,RAND(),-1)</f>
-        <v>0.775068113520462</v>
+        <v>0.146844773973692</v>
       </c>
       <c r="L82" s="10" t="n">
         <f aca="false">IF($J82=1,RANK($K82,$K$2:$K$1001),"")</f>
-        <v>63</v>
+        <v>190</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9384,11 +9384,11 @@
       </c>
       <c r="K83" s="10" t="n">
         <f aca="true">IF($J83=1,RAND(),-1)</f>
-        <v>0.155959637392738</v>
+        <v>0.942758279377395</v>
       </c>
       <c r="L83" s="10" t="n">
         <f aca="false">IF($J83=1,RANK($K83,$K$2:$K$1001),"")</f>
-        <v>193</v>
+        <v>18</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9425,11 +9425,11 @@
       </c>
       <c r="K84" s="10" t="n">
         <f aca="true">IF($J84=1,RAND(),-1)</f>
-        <v>0.567107312161331</v>
+        <v>0.0513854400229985</v>
       </c>
       <c r="L84" s="10" t="n">
         <f aca="false">IF($J84=1,RANK($K84,$K$2:$K$1001),"")</f>
-        <v>105</v>
+        <v>212</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9466,11 +9466,11 @@
       </c>
       <c r="K85" s="10" t="n">
         <f aca="true">IF($J85=1,RAND(),-1)</f>
-        <v>0.633946336283029</v>
+        <v>0.393108012747143</v>
       </c>
       <c r="L85" s="10" t="n">
         <f aca="false">IF($J85=1,RANK($K85,$K$2:$K$1001),"")</f>
-        <v>94</v>
+        <v>151</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9507,11 +9507,11 @@
       </c>
       <c r="K86" s="10" t="n">
         <f aca="true">IF($J86=1,RAND(),-1)</f>
-        <v>0.693560408139294</v>
+        <v>0.0192287357659517</v>
       </c>
       <c r="L86" s="10" t="n">
         <f aca="false">IF($J86=1,RANK($K86,$K$2:$K$1001),"")</f>
-        <v>82</v>
+        <v>221</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9548,11 +9548,11 @@
       </c>
       <c r="K87" s="10" t="n">
         <f aca="true">IF($J87=1,RAND(),-1)</f>
-        <v>0.602314290431705</v>
+        <v>0.760131741028468</v>
       </c>
       <c r="L87" s="10" t="n">
         <f aca="false">IF($J87=1,RANK($K87,$K$2:$K$1001),"")</f>
-        <v>98</v>
+        <v>58</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9589,11 +9589,11 @@
       </c>
       <c r="K88" s="10" t="n">
         <f aca="true">IF($J88=1,RAND(),-1)</f>
-        <v>0.100957506126352</v>
+        <v>0.586313235796245</v>
       </c>
       <c r="L88" s="10" t="n">
         <f aca="false">IF($J88=1,RANK($K88,$K$2:$K$1001),"")</f>
-        <v>202</v>
+        <v>106</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9630,11 +9630,11 @@
       </c>
       <c r="K89" s="10" t="n">
         <f aca="true">IF($J89=1,RAND(),-1)</f>
-        <v>0.993702379567221</v>
+        <v>0.0841933189336721</v>
       </c>
       <c r="L89" s="10" t="n">
         <f aca="false">IF($J89=1,RANK($K89,$K$2:$K$1001),"")</f>
-        <v>1</v>
+        <v>206</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9671,11 +9671,11 @@
       </c>
       <c r="K90" s="10" t="n">
         <f aca="true">IF($J90=1,RAND(),-1)</f>
-        <v>0.284221155148918</v>
+        <v>0.683792164618924</v>
       </c>
       <c r="L90" s="10" t="n">
         <f aca="false">IF($J90=1,RANK($K90,$K$2:$K$1001),"")</f>
-        <v>170</v>
+        <v>79</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9712,11 +9712,11 @@
       </c>
       <c r="K91" s="10" t="n">
         <f aca="true">IF($J91=1,RAND(),-1)</f>
-        <v>0.366305445771561</v>
+        <v>0.613431408599825</v>
       </c>
       <c r="L91" s="10" t="n">
         <f aca="false">IF($J91=1,RANK($K91,$K$2:$K$1001),"")</f>
-        <v>148</v>
+        <v>101</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9753,11 +9753,11 @@
       </c>
       <c r="K92" s="10" t="n">
         <f aca="true">IF($J92=1,RAND(),-1)</f>
-        <v>0.980319805787606</v>
+        <v>0.973164620038686</v>
       </c>
       <c r="L92" s="10" t="n">
         <f aca="false">IF($J92=1,RANK($K92,$K$2:$K$1001),"")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9794,11 +9794,11 @@
       </c>
       <c r="K93" s="10" t="n">
         <f aca="true">IF($J93=1,RAND(),-1)</f>
-        <v>0.71986683168781</v>
+        <v>0.0217147068657158</v>
       </c>
       <c r="L93" s="10" t="n">
         <f aca="false">IF($J93=1,RANK($K93,$K$2:$K$1001),"")</f>
-        <v>74</v>
+        <v>219</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9835,11 +9835,11 @@
       </c>
       <c r="K94" s="10" t="n">
         <f aca="true">IF($J94=1,RAND(),-1)</f>
-        <v>0.146979719307627</v>
+        <v>0.95053965787774</v>
       </c>
       <c r="L94" s="10" t="n">
         <f aca="false">IF($J94=1,RANK($K94,$K$2:$K$1001),"")</f>
-        <v>195</v>
+        <v>14</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9876,11 +9876,11 @@
       </c>
       <c r="K95" s="10" t="n">
         <f aca="true">IF($J95=1,RAND(),-1)</f>
-        <v>0.548783733055076</v>
+        <v>0.917363552628988</v>
       </c>
       <c r="L95" s="10" t="n">
         <f aca="false">IF($J95=1,RANK($K95,$K$2:$K$1001),"")</f>
-        <v>107</v>
+        <v>24</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9917,11 +9917,11 @@
       </c>
       <c r="K96" s="10" t="n">
         <f aca="true">IF($J96=1,RAND(),-1)</f>
-        <v>0.989609697837067</v>
+        <v>0.389912237009382</v>
       </c>
       <c r="L96" s="10" t="n">
         <f aca="false">IF($J96=1,RANK($K96,$K$2:$K$1001),"")</f>
-        <v>3</v>
+        <v>154</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9958,11 +9958,11 @@
       </c>
       <c r="K97" s="10" t="n">
         <f aca="true">IF($J97=1,RAND(),-1)</f>
-        <v>0.0556220188852542</v>
+        <v>0.689682134722515</v>
       </c>
       <c r="L97" s="10" t="n">
         <f aca="false">IF($J97=1,RANK($K97,$K$2:$K$1001),"")</f>
-        <v>216</v>
+        <v>76</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9999,11 +9999,11 @@
       </c>
       <c r="K98" s="10" t="n">
         <f aca="true">IF($J98=1,RAND(),-1)</f>
-        <v>0.603622836119142</v>
+        <v>0.831130677487203</v>
       </c>
       <c r="L98" s="10" t="n">
         <f aca="false">IF($J98=1,RANK($K98,$K$2:$K$1001),"")</f>
-        <v>97</v>
+        <v>43</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10040,11 +10040,11 @@
       </c>
       <c r="K99" s="10" t="n">
         <f aca="true">IF($J99=1,RAND(),-1)</f>
-        <v>0.072903260981467</v>
+        <v>0.0660374319659847</v>
       </c>
       <c r="L99" s="10" t="n">
         <f aca="false">IF($J99=1,RANK($K99,$K$2:$K$1001),"")</f>
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10081,11 +10081,11 @@
       </c>
       <c r="K100" s="10" t="n">
         <f aca="true">IF($J100=1,RAND(),-1)</f>
-        <v>0.114979864826773</v>
+        <v>0.0852646292386087</v>
       </c>
       <c r="L100" s="10" t="n">
         <f aca="false">IF($J100=1,RANK($K100,$K$2:$K$1001),"")</f>
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10122,11 +10122,11 @@
       </c>
       <c r="K101" s="10" t="n">
         <f aca="true">IF($J101=1,RAND(),-1)</f>
-        <v>0.982727974313833</v>
+        <v>0.487073852432185</v>
       </c>
       <c r="L101" s="10" t="n">
         <f aca="false">IF($J101=1,RANK($K101,$K$2:$K$1001),"")</f>
-        <v>5</v>
+        <v>128</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10163,11 +10163,11 @@
       </c>
       <c r="K102" s="10" t="n">
         <f aca="true">IF($J102=1,RAND(),-1)</f>
-        <v>0.301105658774713</v>
+        <v>0.523113156315361</v>
       </c>
       <c r="L102" s="10" t="n">
         <f aca="false">IF($J102=1,RANK($K102,$K$2:$K$1001),"")</f>
-        <v>166</v>
+        <v>119</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10204,11 +10204,11 @@
       </c>
       <c r="K103" s="10" t="n">
         <f aca="true">IF($J103=1,RAND(),-1)</f>
-        <v>0.071910992465681</v>
+        <v>0.398975668618823</v>
       </c>
       <c r="L103" s="10" t="n">
         <f aca="false">IF($J103=1,RANK($K103,$K$2:$K$1001),"")</f>
-        <v>211</v>
+        <v>149</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10245,11 +10245,11 @@
       </c>
       <c r="K104" s="10" t="n">
         <f aca="true">IF($J104=1,RAND(),-1)</f>
-        <v>0.456395882155106</v>
+        <v>0.865670454141115</v>
       </c>
       <c r="L104" s="10" t="n">
         <f aca="false">IF($J104=1,RANK($K104,$K$2:$K$1001),"")</f>
-        <v>130</v>
+        <v>35</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10286,11 +10286,11 @@
       </c>
       <c r="K105" s="10" t="n">
         <f aca="true">IF($J105=1,RAND(),-1)</f>
-        <v>0.936844110073475</v>
+        <v>0.441089734654638</v>
       </c>
       <c r="L105" s="10" t="n">
         <f aca="false">IF($J105=1,RANK($K105,$K$2:$K$1001),"")</f>
-        <v>17</v>
+        <v>139</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10327,11 +10327,11 @@
       </c>
       <c r="K106" s="10" t="n">
         <f aca="true">IF($J106=1,RAND(),-1)</f>
-        <v>0.38868217435086</v>
+        <v>0.339393269518721</v>
       </c>
       <c r="L106" s="10" t="n">
         <f aca="false">IF($J106=1,RANK($K106,$K$2:$K$1001),"")</f>
-        <v>142</v>
+        <v>168</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10368,11 +10368,11 @@
       </c>
       <c r="K107" s="10" t="n">
         <f aca="true">IF($J107=1,RAND(),-1)</f>
-        <v>0.529213377314827</v>
+        <v>0.872819371076916</v>
       </c>
       <c r="L107" s="10" t="n">
         <f aca="false">IF($J107=1,RANK($K107,$K$2:$K$1001),"")</f>
-        <v>113</v>
+        <v>34</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10409,11 +10409,11 @@
       </c>
       <c r="K108" s="10" t="n">
         <f aca="true">IF($J108=1,RAND(),-1)</f>
-        <v>0.280491721295199</v>
+        <v>0.207575512037134</v>
       </c>
       <c r="L108" s="10" t="n">
         <f aca="false">IF($J108=1,RANK($K108,$K$2:$K$1001),"")</f>
-        <v>172</v>
+        <v>184</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10450,11 +10450,11 @@
       </c>
       <c r="K109" s="10" t="n">
         <f aca="true">IF($J109=1,RAND(),-1)</f>
-        <v>0.596095953924459</v>
+        <v>0.991432036450121</v>
       </c>
       <c r="L109" s="10" t="n">
         <f aca="false">IF($J109=1,RANK($K109,$K$2:$K$1001),"")</f>
-        <v>100</v>
+        <v>3</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10491,11 +10491,11 @@
       </c>
       <c r="K110" s="10" t="n">
         <f aca="true">IF($J110=1,RAND(),-1)</f>
-        <v>0.818574280468979</v>
+        <v>0.524412915998203</v>
       </c>
       <c r="L110" s="10" t="n">
         <f aca="false">IF($J110=1,RANK($K110,$K$2:$K$1001),"")</f>
-        <v>55</v>
+        <v>118</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10532,11 +10532,11 @@
       </c>
       <c r="K111" s="10" t="n">
         <f aca="true">IF($J111=1,RAND(),-1)</f>
-        <v>0.513208330721213</v>
+        <v>0.0850888515376271</v>
       </c>
       <c r="L111" s="10" t="n">
         <f aca="false">IF($J111=1,RANK($K111,$K$2:$K$1001),"")</f>
-        <v>118</v>
+        <v>204</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10573,11 +10573,11 @@
       </c>
       <c r="K112" s="10" t="n">
         <f aca="true">IF($J112=1,RAND(),-1)</f>
-        <v>0.569222988115013</v>
+        <v>0.742410203039701</v>
       </c>
       <c r="L112" s="10" t="n">
         <f aca="false">IF($J112=1,RANK($K112,$K$2:$K$1001),"")</f>
-        <v>104</v>
+        <v>63</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10614,11 +10614,11 @@
       </c>
       <c r="K113" s="10" t="n">
         <f aca="true">IF($J113=1,RAND(),-1)</f>
-        <v>0.378670581895333</v>
+        <v>0.356513787659786</v>
       </c>
       <c r="L113" s="10" t="n">
         <f aca="false">IF($J113=1,RANK($K113,$K$2:$K$1001),"")</f>
-        <v>145</v>
+        <v>163</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10655,11 +10655,11 @@
       </c>
       <c r="K114" s="10" t="n">
         <f aca="true">IF($J114=1,RAND(),-1)</f>
-        <v>0.836825326399257</v>
+        <v>0.56460702458579</v>
       </c>
       <c r="L114" s="10" t="n">
         <f aca="false">IF($J114=1,RANK($K114,$K$2:$K$1001),"")</f>
-        <v>51</v>
+        <v>109</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10696,11 +10696,11 @@
       </c>
       <c r="K115" s="10" t="n">
         <f aca="true">IF($J115=1,RAND(),-1)</f>
-        <v>0.0908812607498628</v>
+        <v>0.25795498276222</v>
       </c>
       <c r="L115" s="10" t="n">
         <f aca="false">IF($J115=1,RANK($K115,$K$2:$K$1001),"")</f>
-        <v>205</v>
+        <v>177</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10737,11 +10737,11 @@
       </c>
       <c r="K116" s="10" t="n">
         <f aca="true">IF($J116=1,RAND(),-1)</f>
-        <v>0.0130923565010332</v>
+        <v>0.980871507716432</v>
       </c>
       <c r="L116" s="10" t="n">
         <f aca="false">IF($J116=1,RANK($K116,$K$2:$K$1001),"")</f>
-        <v>220</v>
+        <v>7</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10778,11 +10778,11 @@
       </c>
       <c r="K117" s="10" t="n">
         <f aca="true">IF($J117=1,RAND(),-1)</f>
-        <v>0.0907935908928488</v>
+        <v>0.649908140072581</v>
       </c>
       <c r="L117" s="10" t="n">
         <f aca="false">IF($J117=1,RANK($K117,$K$2:$K$1001),"")</f>
-        <v>206</v>
+        <v>91</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10819,11 +10819,11 @@
       </c>
       <c r="K118" s="10" t="n">
         <f aca="true">IF($J118=1,RAND(),-1)</f>
-        <v>0.506593395373589</v>
+        <v>0.273734783751288</v>
       </c>
       <c r="L118" s="10" t="n">
         <f aca="false">IF($J118=1,RANK($K118,$K$2:$K$1001),"")</f>
-        <v>120</v>
+        <v>175</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10860,11 +10860,11 @@
       </c>
       <c r="K119" s="10" t="n">
         <f aca="true">IF($J119=1,RAND(),-1)</f>
-        <v>0.292511580412807</v>
+        <v>0.44813547878738</v>
       </c>
       <c r="L119" s="10" t="n">
         <f aca="false">IF($J119=1,RANK($K119,$K$2:$K$1001),"")</f>
-        <v>168</v>
+        <v>138</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10901,11 +10901,11 @@
       </c>
       <c r="K120" s="10" t="n">
         <f aca="true">IF($J120=1,RAND(),-1)</f>
-        <v>0.891540623304423</v>
+        <v>0.807092468777348</v>
       </c>
       <c r="L120" s="10" t="n">
         <f aca="false">IF($J120=1,RANK($K120,$K$2:$K$1001),"")</f>
-        <v>34</v>
+        <v>48</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10942,11 +10942,11 @@
       </c>
       <c r="K121" s="10" t="n">
         <f aca="true">IF($J121=1,RAND(),-1)</f>
-        <v>0.95906889542164</v>
+        <v>0.961099946571037</v>
       </c>
       <c r="L121" s="10" t="n">
         <f aca="false">IF($J121=1,RANK($K121,$K$2:$K$1001),"")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10983,11 +10983,11 @@
       </c>
       <c r="K122" s="10" t="n">
         <f aca="true">IF($J122=1,RAND(),-1)</f>
-        <v>0.0148824225107697</v>
+        <v>0.890291763623129</v>
       </c>
       <c r="L122" s="10" t="n">
         <f aca="false">IF($J122=1,RANK($K122,$K$2:$K$1001),"")</f>
-        <v>219</v>
+        <v>32</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11024,11 +11024,11 @@
       </c>
       <c r="K123" s="10" t="n">
         <f aca="true">IF($J123=1,RAND(),-1)</f>
-        <v>0.233875160565133</v>
+        <v>0.502892914956412</v>
       </c>
       <c r="L123" s="10" t="n">
         <f aca="false">IF($J123=1,RANK($K123,$K$2:$K$1001),"")</f>
-        <v>183</v>
+        <v>124</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11065,11 +11065,11 @@
       </c>
       <c r="K124" s="10" t="n">
         <f aca="true">IF($J124=1,RAND(),-1)</f>
-        <v>0.857544680991472</v>
+        <v>0.473795604502162</v>
       </c>
       <c r="L124" s="10" t="n">
         <f aca="false">IF($J124=1,RANK($K124,$K$2:$K$1001),"")</f>
-        <v>46</v>
+        <v>132</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11106,11 +11106,11 @@
       </c>
       <c r="K125" s="10" t="n">
         <f aca="true">IF($J125=1,RAND(),-1)</f>
-        <v>0.965462993467076</v>
+        <v>0.614325490559818</v>
       </c>
       <c r="L125" s="10" t="n">
         <f aca="false">IF($J125=1,RANK($K125,$K$2:$K$1001),"")</f>
-        <v>9</v>
+        <v>100</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11147,11 +11147,11 @@
       </c>
       <c r="K126" s="10" t="n">
         <f aca="true">IF($J126=1,RAND(),-1)</f>
-        <v>0.957873267265074</v>
+        <v>0.132776566736654</v>
       </c>
       <c r="L126" s="10" t="n">
         <f aca="false">IF($J126=1,RANK($K126,$K$2:$K$1001),"")</f>
-        <v>12</v>
+        <v>193</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11188,11 +11188,11 @@
       </c>
       <c r="K127" s="10" t="n">
         <f aca="true">IF($J127=1,RAND(),-1)</f>
-        <v>0.466872395945857</v>
+        <v>0.189051813034249</v>
       </c>
       <c r="L127" s="10" t="n">
         <f aca="false">IF($J127=1,RANK($K127,$K$2:$K$1001),"")</f>
-        <v>126</v>
+        <v>187</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11229,11 +11229,11 @@
       </c>
       <c r="K128" s="10" t="n">
         <f aca="true">IF($J128=1,RAND(),-1)</f>
-        <v>0.0933244590928398</v>
+        <v>0.990516610950674</v>
       </c>
       <c r="L128" s="10" t="n">
         <f aca="false">IF($J128=1,RANK($K128,$K$2:$K$1001),"")</f>
-        <v>203</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11270,11 +11270,11 @@
       </c>
       <c r="K129" s="10" t="n">
         <f aca="true">IF($J129=1,RAND(),-1)</f>
-        <v>0.266999138897237</v>
+        <v>0.0417602720679885</v>
       </c>
       <c r="L129" s="10" t="n">
         <f aca="false">IF($J129=1,RANK($K129,$K$2:$K$1001),"")</f>
-        <v>177</v>
+        <v>215</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11311,11 +11311,11 @@
       </c>
       <c r="K130" s="10" t="n">
         <f aca="true">IF($J130=1,RAND(),-1)</f>
-        <v>0.91622563672929</v>
+        <v>0.944617560115091</v>
       </c>
       <c r="L130" s="10" t="n">
         <f aca="false">IF($J130=1,RANK($K130,$K$2:$K$1001),"")</f>
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11352,11 +11352,11 @@
       </c>
       <c r="K131" s="10" t="n">
         <f aca="true">IF($J131=1,RAND(),-1)</f>
-        <v>0.26888260370309</v>
+        <v>0.0934430859375336</v>
       </c>
       <c r="L131" s="10" t="n">
         <f aca="false">IF($J131=1,RANK($K131,$K$2:$K$1001),"")</f>
-        <v>175</v>
+        <v>202</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11393,11 +11393,11 @@
       </c>
       <c r="K132" s="10" t="n">
         <f aca="true">IF($J132=1,RAND(),-1)</f>
-        <v>0.281367421050038</v>
+        <v>0.36487123840181</v>
       </c>
       <c r="L132" s="10" t="n">
         <f aca="false">IF($J132=1,RANK($K132,$K$2:$K$1001),"")</f>
-        <v>171</v>
+        <v>158</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11434,11 +11434,11 @@
       </c>
       <c r="K133" s="10" t="n">
         <f aca="true">IF($J133=1,RAND(),-1)</f>
-        <v>0.830283143095011</v>
+        <v>0.422715133957519</v>
       </c>
       <c r="L133" s="10" t="n">
         <f aca="false">IF($J133=1,RANK($K133,$K$2:$K$1001),"")</f>
-        <v>53</v>
+        <v>141</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11475,11 +11475,11 @@
       </c>
       <c r="K134" s="10" t="n">
         <f aca="true">IF($J134=1,RAND(),-1)</f>
-        <v>0.376949188791565</v>
+        <v>0.920063759119961</v>
       </c>
       <c r="L134" s="10" t="n">
         <f aca="false">IF($J134=1,RANK($K134,$K$2:$K$1001),"")</f>
-        <v>147</v>
+        <v>22</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11516,11 +11516,11 @@
       </c>
       <c r="K135" s="10" t="n">
         <f aca="true">IF($J135=1,RAND(),-1)</f>
-        <v>0.226992386039777</v>
+        <v>0.722581957632156</v>
       </c>
       <c r="L135" s="10" t="n">
         <f aca="false">IF($J135=1,RANK($K135,$K$2:$K$1001),"")</f>
-        <v>186</v>
+        <v>69</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11557,11 +11557,11 @@
       </c>
       <c r="K136" s="10" t="n">
         <f aca="true">IF($J136=1,RAND(),-1)</f>
-        <v>0.0613315621995844</v>
+        <v>0.138586607432746</v>
       </c>
       <c r="L136" s="10" t="n">
         <f aca="false">IF($J136=1,RANK($K136,$K$2:$K$1001),"")</f>
-        <v>214</v>
+        <v>191</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11598,11 +11598,11 @@
       </c>
       <c r="K137" s="10" t="n">
         <f aca="true">IF($J137=1,RAND(),-1)</f>
-        <v>0.505318616615618</v>
+        <v>0.99534086835143</v>
       </c>
       <c r="L137" s="10" t="n">
         <f aca="false">IF($J137=1,RANK($K137,$K$2:$K$1001),"")</f>
-        <v>122</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11639,11 +11639,11 @@
       </c>
       <c r="K138" s="10" t="n">
         <f aca="true">IF($J138=1,RAND(),-1)</f>
-        <v>0.977992911399476</v>
+        <v>0.370303945897586</v>
       </c>
       <c r="L138" s="10" t="n">
         <f aca="false">IF($J138=1,RANK($K138,$K$2:$K$1001),"")</f>
-        <v>8</v>
+        <v>157</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11680,11 +11680,11 @@
       </c>
       <c r="K139" s="10" t="n">
         <f aca="true">IF($J139=1,RAND(),-1)</f>
-        <v>0.49206109379548</v>
+        <v>0.0984495131342001</v>
       </c>
       <c r="L139" s="10" t="n">
         <f aca="false">IF($J139=1,RANK($K139,$K$2:$K$1001),"")</f>
-        <v>124</v>
+        <v>200</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11721,11 +11721,11 @@
       </c>
       <c r="K140" s="10" t="n">
         <f aca="true">IF($J140=1,RAND(),-1)</f>
-        <v>0.353477023389495</v>
+        <v>0.0557956354136671</v>
       </c>
       <c r="L140" s="10" t="n">
         <f aca="false">IF($J140=1,RANK($K140,$K$2:$K$1001),"")</f>
-        <v>153</v>
+        <v>211</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11762,11 +11762,11 @@
       </c>
       <c r="K141" s="10" t="n">
         <f aca="true">IF($J141=1,RAND(),-1)</f>
-        <v>0.543259467720176</v>
+        <v>0.461354220535493</v>
       </c>
       <c r="L141" s="10" t="n">
         <f aca="false">IF($J141=1,RANK($K141,$K$2:$K$1001),"")</f>
-        <v>111</v>
+        <v>136</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11803,11 +11803,11 @@
       </c>
       <c r="K142" s="10" t="n">
         <f aca="true">IF($J142=1,RAND(),-1)</f>
-        <v>0.0615807055296683</v>
+        <v>0.484071403160236</v>
       </c>
       <c r="L142" s="10" t="n">
         <f aca="false">IF($J142=1,RANK($K142,$K$2:$K$1001),"")</f>
-        <v>213</v>
+        <v>129</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11844,11 +11844,11 @@
       </c>
       <c r="K143" s="10" t="n">
         <f aca="true">IF($J143=1,RAND(),-1)</f>
-        <v>0.689961331551237</v>
+        <v>0.633170212666792</v>
       </c>
       <c r="L143" s="10" t="n">
         <f aca="false">IF($J143=1,RANK($K143,$K$2:$K$1001),"")</f>
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11885,11 +11885,11 @@
       </c>
       <c r="K144" s="10" t="n">
         <f aca="true">IF($J144=1,RAND(),-1)</f>
-        <v>0.634732215600432</v>
+        <v>0.0607323225352403</v>
       </c>
       <c r="L144" s="10" t="n">
         <f aca="false">IF($J144=1,RANK($K144,$K$2:$K$1001),"")</f>
-        <v>93</v>
+        <v>210</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11926,11 +11926,11 @@
       </c>
       <c r="K145" s="10" t="n">
         <f aca="true">IF($J145=1,RAND(),-1)</f>
-        <v>0.919661054448333</v>
+        <v>0.331463265924977</v>
       </c>
       <c r="L145" s="10" t="n">
         <f aca="false">IF($J145=1,RANK($K145,$K$2:$K$1001),"")</f>
-        <v>23</v>
+        <v>170</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11967,11 +11967,11 @@
       </c>
       <c r="K146" s="10" t="n">
         <f aca="true">IF($J146=1,RAND(),-1)</f>
-        <v>0.757658188417032</v>
+        <v>0.766131708988458</v>
       </c>
       <c r="L146" s="10" t="n">
         <f aca="false">IF($J146=1,RANK($K146,$K$2:$K$1001),"")</f>
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12008,11 +12008,11 @@
       </c>
       <c r="K147" s="10" t="n">
         <f aca="true">IF($J147=1,RAND(),-1)</f>
-        <v>0.00799292459221343</v>
+        <v>0.923754656698638</v>
       </c>
       <c r="L147" s="10" t="n">
         <f aca="false">IF($J147=1,RANK($K147,$K$2:$K$1001),"")</f>
-        <v>221</v>
+        <v>20</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12049,11 +12049,11 @@
       </c>
       <c r="K148" s="10" t="n">
         <f aca="true">IF($J148=1,RAND(),-1)</f>
-        <v>0.311663668593694</v>
+        <v>0.117085753106017</v>
       </c>
       <c r="L148" s="10" t="n">
         <f aca="false">IF($J148=1,RANK($K148,$K$2:$K$1001),"")</f>
-        <v>164</v>
+        <v>197</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12090,11 +12090,11 @@
       </c>
       <c r="K149" s="10" t="n">
         <f aca="true">IF($J149=1,RAND(),-1)</f>
-        <v>0.480943156528259</v>
+        <v>0.0485224592751429</v>
       </c>
       <c r="L149" s="10" t="n">
         <f aca="false">IF($J149=1,RANK($K149,$K$2:$K$1001),"")</f>
-        <v>125</v>
+        <v>213</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12131,11 +12131,11 @@
       </c>
       <c r="K150" s="10" t="n">
         <f aca="true">IF($J150=1,RAND(),-1)</f>
-        <v>0.435952227060654</v>
+        <v>0.418194802597381</v>
       </c>
       <c r="L150" s="10" t="n">
         <f aca="false">IF($J150=1,RANK($K150,$K$2:$K$1001),"")</f>
-        <v>132</v>
+        <v>147</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12172,11 +12172,11 @@
       </c>
       <c r="K151" s="10" t="n">
         <f aca="true">IF($J151=1,RAND(),-1)</f>
-        <v>0.924858982945317</v>
+        <v>0.471259590968684</v>
       </c>
       <c r="L151" s="10" t="n">
         <f aca="false">IF($J151=1,RANK($K151,$K$2:$K$1001),"")</f>
-        <v>21</v>
+        <v>134</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12213,11 +12213,11 @@
       </c>
       <c r="K152" s="10" t="n">
         <f aca="true">IF($J152=1,RAND(),-1)</f>
-        <v>0.657476581441148</v>
+        <v>0.0185632209002587</v>
       </c>
       <c r="L152" s="10" t="n">
         <f aca="false">IF($J152=1,RANK($K152,$K$2:$K$1001),"")</f>
-        <v>91</v>
+        <v>222</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12254,11 +12254,11 @@
       </c>
       <c r="K153" s="10" t="n">
         <f aca="true">IF($J153=1,RAND(),-1)</f>
-        <v>0.861146289784898</v>
+        <v>0.626581178082474</v>
       </c>
       <c r="L153" s="10" t="n">
         <f aca="false">IF($J153=1,RANK($K153,$K$2:$K$1001),"")</f>
-        <v>45</v>
+        <v>97</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12295,11 +12295,11 @@
       </c>
       <c r="K154" s="10" t="n">
         <f aca="true">IF($J154=1,RAND(),-1)</f>
-        <v>0.846808107250374</v>
+        <v>0.421695775654918</v>
       </c>
       <c r="L154" s="10" t="n">
         <f aca="false">IF($J154=1,RANK($K154,$K$2:$K$1001),"")</f>
-        <v>48</v>
+        <v>145</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12336,11 +12336,11 @@
       </c>
       <c r="K155" s="10" t="n">
         <f aca="true">IF($J155=1,RAND(),-1)</f>
-        <v>0.796027435571524</v>
+        <v>0.61901900197766</v>
       </c>
       <c r="L155" s="10" t="n">
         <f aca="false">IF($J155=1,RANK($K155,$K$2:$K$1001),"")</f>
-        <v>56</v>
+        <v>99</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12377,11 +12377,11 @@
       </c>
       <c r="K156" s="10" t="n">
         <f aca="true">IF($J156=1,RAND(),-1)</f>
-        <v>0.314955778894573</v>
+        <v>0.905166244863152</v>
       </c>
       <c r="L156" s="10" t="n">
         <f aca="false">IF($J156=1,RANK($K156,$K$2:$K$1001),"")</f>
-        <v>161</v>
+        <v>27</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12418,11 +12418,11 @@
       </c>
       <c r="K157" s="10" t="n">
         <f aca="true">IF($J157=1,RAND(),-1)</f>
-        <v>0.361457152328532</v>
+        <v>0.923665488845327</v>
       </c>
       <c r="L157" s="10" t="n">
         <f aca="false">IF($J157=1,RANK($K157,$K$2:$K$1001),"")</f>
-        <v>150</v>
+        <v>21</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12459,11 +12459,11 @@
       </c>
       <c r="K158" s="10" t="n">
         <f aca="true">IF($J158=1,RAND(),-1)</f>
-        <v>0.675980123511877</v>
+        <v>0.391734454779476</v>
       </c>
       <c r="L158" s="10" t="n">
         <f aca="false">IF($J158=1,RANK($K158,$K$2:$K$1001),"")</f>
-        <v>87</v>
+        <v>152</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12500,11 +12500,11 @@
       </c>
       <c r="K159" s="10" t="n">
         <f aca="true">IF($J159=1,RAND(),-1)</f>
-        <v>0.258165665588401</v>
+        <v>0.710553943631941</v>
       </c>
       <c r="L159" s="10" t="n">
         <f aca="false">IF($J159=1,RANK($K159,$K$2:$K$1001),"")</f>
-        <v>180</v>
+        <v>73</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12541,11 +12541,11 @@
       </c>
       <c r="K160" s="10" t="n">
         <f aca="true">IF($J160=1,RAND(),-1)</f>
-        <v>0.339414249369609</v>
+        <v>0.671302428719376</v>
       </c>
       <c r="L160" s="10" t="n">
         <f aca="false">IF($J160=1,RANK($K160,$K$2:$K$1001),"")</f>
-        <v>159</v>
+        <v>86</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12582,11 +12582,11 @@
       </c>
       <c r="K161" s="10" t="n">
         <f aca="true">IF($J161=1,RAND(),-1)</f>
-        <v>0.914922142308868</v>
+        <v>0.736248072522536</v>
       </c>
       <c r="L161" s="10" t="n">
         <f aca="false">IF($J161=1,RANK($K161,$K$2:$K$1001),"")</f>
-        <v>25</v>
+        <v>64</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12623,11 +12623,11 @@
       </c>
       <c r="K162" s="10" t="n">
         <f aca="true">IF($J162=1,RAND(),-1)</f>
-        <v>0.829899674120361</v>
+        <v>0.21375892412478</v>
       </c>
       <c r="L162" s="10" t="n">
         <f aca="false">IF($J162=1,RANK($K162,$K$2:$K$1001),"")</f>
-        <v>54</v>
+        <v>182</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12664,11 +12664,11 @@
       </c>
       <c r="K163" s="10" t="n">
         <f aca="true">IF($J163=1,RAND(),-1)</f>
-        <v>0.731051467715913</v>
+        <v>0.25615981300488</v>
       </c>
       <c r="L163" s="10" t="n">
         <f aca="false">IF($J163=1,RANK($K163,$K$2:$K$1001),"")</f>
-        <v>71</v>
+        <v>178</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12705,11 +12705,11 @@
       </c>
       <c r="K164" s="10" t="n">
         <f aca="true">IF($J164=1,RAND(),-1)</f>
-        <v>0.912873250057545</v>
+        <v>0.974930759890085</v>
       </c>
       <c r="L164" s="10" t="n">
         <f aca="false">IF($J164=1,RANK($K164,$K$2:$K$1001),"")</f>
-        <v>28</v>
+        <v>8</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12746,11 +12746,11 @@
       </c>
       <c r="K165" s="10" t="n">
         <f aca="true">IF($J165=1,RAND(),-1)</f>
-        <v>0.26319638249825</v>
+        <v>0.887248627315951</v>
       </c>
       <c r="L165" s="10" t="n">
         <f aca="false">IF($J165=1,RANK($K165,$K$2:$K$1001),"")</f>
-        <v>178</v>
+        <v>33</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12787,11 +12787,11 @@
       </c>
       <c r="K166" s="10" t="n">
         <f aca="true">IF($J166=1,RAND(),-1)</f>
-        <v>0.113422465840784</v>
+        <v>0.961919360936854</v>
       </c>
       <c r="L166" s="10" t="n">
         <f aca="false">IF($J166=1,RANK($K166,$K$2:$K$1001),"")</f>
-        <v>200</v>
+        <v>11</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12828,11 +12828,11 @@
       </c>
       <c r="K167" s="10" t="n">
         <f aca="true">IF($J167=1,RAND(),-1)</f>
-        <v>0.689638223484279</v>
+        <v>0.945835506678381</v>
       </c>
       <c r="L167" s="10" t="n">
         <f aca="false">IF($J167=1,RANK($K167,$K$2:$K$1001),"")</f>
-        <v>84</v>
+        <v>15</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12869,11 +12869,11 @@
       </c>
       <c r="K168" s="10" t="n">
         <f aca="true">IF($J168=1,RAND(),-1)</f>
-        <v>0.271329925984123</v>
+        <v>0.161040133801992</v>
       </c>
       <c r="L168" s="10" t="n">
         <f aca="false">IF($J168=1,RANK($K168,$K$2:$K$1001),"")</f>
-        <v>174</v>
+        <v>188</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12910,11 +12910,11 @@
       </c>
       <c r="K169" s="10" t="n">
         <f aca="true">IF($J169=1,RAND(),-1)</f>
-        <v>0.510809976366593</v>
+        <v>0.567666663558743</v>
       </c>
       <c r="L169" s="10" t="n">
         <f aca="false">IF($J169=1,RANK($K169,$K$2:$K$1001),"")</f>
-        <v>119</v>
+        <v>108</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12951,11 +12951,11 @@
       </c>
       <c r="K170" s="10" t="n">
         <f aca="true">IF($J170=1,RAND(),-1)</f>
-        <v>0.519285422324598</v>
+        <v>0.125322292683928</v>
       </c>
       <c r="L170" s="10" t="n">
         <f aca="false">IF($J170=1,RANK($K170,$K$2:$K$1001),"")</f>
-        <v>116</v>
+        <v>195</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12992,11 +12992,11 @@
       </c>
       <c r="K171" s="10" t="n">
         <f aca="true">IF($J171=1,RAND(),-1)</f>
-        <v>0.403365762077151</v>
+        <v>0.216476261814549</v>
       </c>
       <c r="L171" s="10" t="n">
         <f aca="false">IF($J171=1,RANK($K171,$K$2:$K$1001),"")</f>
-        <v>138</v>
+        <v>181</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13033,11 +13033,11 @@
       </c>
       <c r="K172" s="10" t="n">
         <f aca="true">IF($J172=1,RAND(),-1)</f>
-        <v>0.982017285060737</v>
+        <v>0.724641729150762</v>
       </c>
       <c r="L172" s="10" t="n">
         <f aca="false">IF($J172=1,RANK($K172,$K$2:$K$1001),"")</f>
-        <v>6</v>
+        <v>68</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13074,11 +13074,11 @@
       </c>
       <c r="K173" s="10" t="n">
         <f aca="true">IF($J173=1,RAND(),-1)</f>
-        <v>0.902687338367649</v>
+        <v>0.990782422996433</v>
       </c>
       <c r="L173" s="10" t="n">
         <f aca="false">IF($J173=1,RANK($K173,$K$2:$K$1001),"")</f>
-        <v>29</v>
+        <v>4</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13115,11 +13115,11 @@
       </c>
       <c r="K174" s="10" t="n">
         <f aca="true">IF($J174=1,RAND(),-1)</f>
-        <v>0.288977063777027</v>
+        <v>0.892522075380948</v>
       </c>
       <c r="L174" s="10" t="n">
         <f aca="false">IF($J174=1,RANK($K174,$K$2:$K$1001),"")</f>
-        <v>169</v>
+        <v>30</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13156,11 +13156,11 @@
       </c>
       <c r="K175" s="10" t="n">
         <f aca="true">IF($J175=1,RAND(),-1)</f>
-        <v>0.350384365357117</v>
+        <v>0.593642430533568</v>
       </c>
       <c r="L175" s="10" t="n">
         <f aca="false">IF($J175=1,RANK($K175,$K$2:$K$1001),"")</f>
-        <v>154</v>
+        <v>104</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13197,11 +13197,11 @@
       </c>
       <c r="K176" s="10" t="n">
         <f aca="true">IF($J176=1,RAND(),-1)</f>
-        <v>0.839481836395349</v>
+        <v>0.020061912389495</v>
       </c>
       <c r="L176" s="10" t="n">
         <f aca="false">IF($J176=1,RANK($K176,$K$2:$K$1001),"")</f>
-        <v>49</v>
+        <v>220</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13238,11 +13238,11 @@
       </c>
       <c r="K177" s="10" t="n">
         <f aca="true">IF($J177=1,RAND(),-1)</f>
-        <v>0.678382465557549</v>
+        <v>0.358163586391755</v>
       </c>
       <c r="L177" s="10" t="n">
         <f aca="false">IF($J177=1,RANK($K177,$K$2:$K$1001),"")</f>
-        <v>85</v>
+        <v>161</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13279,11 +13279,11 @@
       </c>
       <c r="K178" s="10" t="n">
         <f aca="true">IF($J178=1,RAND(),-1)</f>
-        <v>0.944902926730304</v>
+        <v>0.986512682944112</v>
       </c>
       <c r="L178" s="10" t="n">
         <f aca="false">IF($J178=1,RANK($K178,$K$2:$K$1001),"")</f>
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13320,11 +13320,11 @@
       </c>
       <c r="K179" s="10" t="n">
         <f aca="true">IF($J179=1,RAND(),-1)</f>
-        <v>0.893843679290147</v>
+        <v>0.0953262143792325</v>
       </c>
       <c r="L179" s="10" t="n">
         <f aca="false">IF($J179=1,RANK($K179,$K$2:$K$1001),"")</f>
-        <v>32</v>
+        <v>201</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13361,11 +13361,11 @@
       </c>
       <c r="K180" s="10" t="n">
         <f aca="true">IF($J180=1,RAND(),-1)</f>
-        <v>0.064224808809516</v>
+        <v>0.672761349001386</v>
       </c>
       <c r="L180" s="10" t="n">
         <f aca="false">IF($J180=1,RANK($K180,$K$2:$K$1001),"")</f>
-        <v>212</v>
+        <v>84</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13402,11 +13402,11 @@
       </c>
       <c r="K181" s="10" t="n">
         <f aca="true">IF($J181=1,RAND(),-1)</f>
-        <v>0.121540353180408</v>
+        <v>0.671949756922808</v>
       </c>
       <c r="L181" s="10" t="n">
         <f aca="false">IF($J181=1,RANK($K181,$K$2:$K$1001),"")</f>
-        <v>198</v>
+        <v>85</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13443,11 +13443,11 @@
       </c>
       <c r="K182" s="10" t="n">
         <f aca="true">IF($J182=1,RAND(),-1)</f>
-        <v>0.2214971981101</v>
+        <v>0.558580494230847</v>
       </c>
       <c r="L182" s="10" t="n">
         <f aca="false">IF($J182=1,RANK($K182,$K$2:$K$1001),"")</f>
-        <v>188</v>
+        <v>111</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13484,11 +13484,11 @@
       </c>
       <c r="K183" s="10" t="n">
         <f aca="true">IF($J183=1,RAND(),-1)</f>
-        <v>0.413897988025109</v>
+        <v>0.687078293132016</v>
       </c>
       <c r="L183" s="10" t="n">
         <f aca="false">IF($J183=1,RANK($K183,$K$2:$K$1001),"")</f>
-        <v>136</v>
+        <v>78</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13525,11 +13525,11 @@
       </c>
       <c r="K184" s="10" t="n">
         <f aca="true">IF($J184=1,RAND(),-1)</f>
-        <v>0.00743865998821544</v>
+        <v>0.654338467742136</v>
       </c>
       <c r="L184" s="10" t="n">
         <f aca="false">IF($J184=1,RANK($K184,$K$2:$K$1001),"")</f>
-        <v>222</v>
+        <v>90</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13566,11 +13566,11 @@
       </c>
       <c r="K185" s="10" t="n">
         <f aca="true">IF($J185=1,RAND(),-1)</f>
-        <v>0.719635780243448</v>
+        <v>0.839344828047269</v>
       </c>
       <c r="L185" s="10" t="n">
         <f aca="false">IF($J185=1,RANK($K185,$K$2:$K$1001),"")</f>
-        <v>75</v>
+        <v>42</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13607,11 +13607,11 @@
       </c>
       <c r="K186" s="10" t="n">
         <f aca="true">IF($J186=1,RAND(),-1)</f>
-        <v>0.742199268297902</v>
+        <v>0.24285021774966</v>
       </c>
       <c r="L186" s="10" t="n">
         <f aca="false">IF($J186=1,RANK($K186,$K$2:$K$1001),"")</f>
-        <v>69</v>
+        <v>179</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13648,11 +13648,11 @@
       </c>
       <c r="K187" s="10" t="n">
         <f aca="true">IF($J187=1,RAND(),-1)</f>
-        <v>0.424288785107608</v>
+        <v>0.475878564922878</v>
       </c>
       <c r="L187" s="10" t="n">
         <f aca="false">IF($J187=1,RANK($K187,$K$2:$K$1001),"")</f>
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13689,11 +13689,11 @@
       </c>
       <c r="K188" s="10" t="n">
         <f aca="true">IF($J188=1,RAND(),-1)</f>
-        <v>0.71890055191772</v>
+        <v>0.498869318639051</v>
       </c>
       <c r="L188" s="10" t="n">
         <f aca="false">IF($J188=1,RANK($K188,$K$2:$K$1001),"")</f>
-        <v>76</v>
+        <v>126</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13730,11 +13730,11 @@
       </c>
       <c r="K189" s="10" t="n">
         <f aca="true">IF($J189=1,RAND(),-1)</f>
-        <v>0.748486174196644</v>
+        <v>0.479707014776962</v>
       </c>
       <c r="L189" s="10" t="n">
         <f aca="false">IF($J189=1,RANK($K189,$K$2:$K$1001),"")</f>
-        <v>68</v>
+        <v>130</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13771,11 +13771,11 @@
       </c>
       <c r="K190" s="10" t="n">
         <f aca="true">IF($J190=1,RAND(),-1)</f>
-        <v>0.652335492425806</v>
+        <v>0.857959418803281</v>
       </c>
       <c r="L190" s="10" t="n">
         <f aca="false">IF($J190=1,RANK($K190,$K$2:$K$1001),"")</f>
-        <v>92</v>
+        <v>37</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13812,11 +13812,11 @@
       </c>
       <c r="K191" s="10" t="n">
         <f aca="true">IF($J191=1,RAND(),-1)</f>
-        <v>0.314255865459243</v>
+        <v>0.38523856562845</v>
       </c>
       <c r="L191" s="10" t="n">
         <f aca="false">IF($J191=1,RANK($K191,$K$2:$K$1001),"")</f>
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13853,11 +13853,11 @@
       </c>
       <c r="K192" s="10" t="n">
         <f aca="true">IF($J192=1,RAND(),-1)</f>
-        <v>0.770418987103472</v>
+        <v>0.673762015603208</v>
       </c>
       <c r="L192" s="10" t="n">
         <f aca="false">IF($J192=1,RANK($K192,$K$2:$K$1001),"")</f>
-        <v>64</v>
+        <v>83</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13894,11 +13894,11 @@
       </c>
       <c r="K193" s="10" t="n">
         <f aca="true">IF($J193=1,RAND(),-1)</f>
-        <v>0.464190314759186</v>
+        <v>0.825903854310135</v>
       </c>
       <c r="L193" s="10" t="n">
         <f aca="false">IF($J193=1,RANK($K193,$K$2:$K$1001),"")</f>
-        <v>127</v>
+        <v>45</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13935,11 +13935,11 @@
       </c>
       <c r="K194" s="10" t="n">
         <f aca="true">IF($J194=1,RAND(),-1)</f>
-        <v>0.19322836220356</v>
+        <v>0.380553393054452</v>
       </c>
       <c r="L194" s="10" t="n">
         <f aca="false">IF($J194=1,RANK($K194,$K$2:$K$1001),"")</f>
-        <v>189</v>
+        <v>156</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13976,11 +13976,11 @@
       </c>
       <c r="K195" s="10" t="n">
         <f aca="true">IF($J195=1,RAND(),-1)</f>
-        <v>0.599018936255446</v>
+        <v>0.915238532828926</v>
       </c>
       <c r="L195" s="10" t="n">
         <f aca="false">IF($J195=1,RANK($K195,$K$2:$K$1001),"")</f>
-        <v>99</v>
+        <v>25</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14017,11 +14017,11 @@
       </c>
       <c r="K196" s="10" t="n">
         <f aca="true">IF($J196=1,RAND(),-1)</f>
-        <v>0.714945932997077</v>
+        <v>0.841164801275629</v>
       </c>
       <c r="L196" s="10" t="n">
         <f aca="false">IF($J196=1,RANK($K196,$K$2:$K$1001),"")</f>
-        <v>77</v>
+        <v>41</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14058,11 +14058,11 @@
       </c>
       <c r="K197" s="10" t="n">
         <f aca="true">IF($J197=1,RAND(),-1)</f>
-        <v>0.231551661506118</v>
+        <v>0.679413891468517</v>
       </c>
       <c r="L197" s="10" t="n">
         <f aca="false">IF($J197=1,RANK($K197,$K$2:$K$1001),"")</f>
-        <v>184</v>
+        <v>81</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14099,11 +14099,11 @@
       </c>
       <c r="K198" s="10" t="n">
         <f aca="true">IF($J198=1,RAND(),-1)</f>
-        <v>0.834589919153058</v>
+        <v>0.5041037040628</v>
       </c>
       <c r="L198" s="10" t="n">
         <f aca="false">IF($J198=1,RANK($K198,$K$2:$K$1001),"")</f>
-        <v>52</v>
+        <v>123</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14140,11 +14140,11 @@
       </c>
       <c r="K199" s="10" t="n">
         <f aca="true">IF($J199=1,RAND(),-1)</f>
-        <v>0.664829848155658</v>
+        <v>0.538075995148389</v>
       </c>
       <c r="L199" s="10" t="n">
         <f aca="false">IF($J199=1,RANK($K199,$K$2:$K$1001),"")</f>
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14181,11 +14181,11 @@
       </c>
       <c r="K200" s="10" t="n">
         <f aca="true">IF($J200=1,RAND(),-1)</f>
-        <v>0.79509622805324</v>
+        <v>0.631791190958596</v>
       </c>
       <c r="L200" s="10" t="n">
         <f aca="false">IF($J200=1,RANK($K200,$K$2:$K$1001),"")</f>
-        <v>57</v>
+        <v>95</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14222,11 +14222,11 @@
       </c>
       <c r="K201" s="10" t="n">
         <f aca="true">IF($J201=1,RAND(),-1)</f>
-        <v>0.769197918845963</v>
+        <v>0.810385985148248</v>
       </c>
       <c r="L201" s="10" t="n">
         <f aca="false">IF($J201=1,RANK($K201,$K$2:$K$1001),"")</f>
-        <v>65</v>
+        <v>46</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14263,11 +14263,11 @@
       </c>
       <c r="K202" s="10" t="n">
         <f aca="true">IF($J202=1,RAND(),-1)</f>
-        <v>0.668707315252484</v>
+        <v>0.729731798924547</v>
       </c>
       <c r="L202" s="10" t="n">
         <f aca="false">IF($J202=1,RANK($K202,$K$2:$K$1001),"")</f>
-        <v>89</v>
+        <v>65</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14304,11 +14304,11 @@
       </c>
       <c r="K203" s="10" t="n">
         <f aca="true">IF($J203=1,RAND(),-1)</f>
-        <v>0.881933104786761</v>
+        <v>0.586393070460748</v>
       </c>
       <c r="L203" s="10" t="n">
         <f aca="false">IF($J203=1,RANK($K203,$K$2:$K$1001),"")</f>
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14345,11 +14345,11 @@
       </c>
       <c r="K204" s="10" t="n">
         <f aca="true">IF($J204=1,RAND(),-1)</f>
-        <v>0.142324415777136</v>
+        <v>0.847150784444591</v>
       </c>
       <c r="L204" s="10" t="n">
         <f aca="false">IF($J204=1,RANK($K204,$K$2:$K$1001),"")</f>
-        <v>196</v>
+        <v>38</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14386,11 +14386,11 @@
       </c>
       <c r="K205" s="10" t="n">
         <f aca="true">IF($J205=1,RAND(),-1)</f>
-        <v>0.594826887009376</v>
+        <v>0.583895041192</v>
       </c>
       <c r="L205" s="10" t="n">
         <f aca="false">IF($J205=1,RANK($K205,$K$2:$K$1001),"")</f>
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14427,11 +14427,11 @@
       </c>
       <c r="K206" s="10" t="n">
         <f aca="true">IF($J206=1,RAND(),-1)</f>
-        <v>0.225514509895087</v>
+        <v>0.159803779011923</v>
       </c>
       <c r="L206" s="10" t="n">
         <f aca="false">IF($J206=1,RANK($K206,$K$2:$K$1001),"")</f>
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14468,11 +14468,11 @@
       </c>
       <c r="K207" s="10" t="n">
         <f aca="true">IF($J207=1,RAND(),-1)</f>
-        <v>0.735594112861668</v>
+        <v>0.0304406665378357</v>
       </c>
       <c r="L207" s="10" t="n">
         <f aca="false">IF($J207=1,RANK($K207,$K$2:$K$1001),"")</f>
-        <v>70</v>
+        <v>217</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14509,11 +14509,11 @@
       </c>
       <c r="K208" s="10" t="n">
         <f aca="true">IF($J208=1,RAND(),-1)</f>
-        <v>0.262295479326717</v>
+        <v>0.798107771656446</v>
       </c>
       <c r="L208" s="10" t="n">
         <f aca="false">IF($J208=1,RANK($K208,$K$2:$K$1001),"")</f>
-        <v>179</v>
+        <v>50</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14550,11 +14550,11 @@
       </c>
       <c r="K209" s="10" t="n">
         <f aca="true">IF($J209=1,RAND(),-1)</f>
-        <v>0.382208266431876</v>
+        <v>0.510088145884903</v>
       </c>
       <c r="L209" s="10" t="n">
         <f aca="false">IF($J209=1,RANK($K209,$K$2:$K$1001),"")</f>
-        <v>144</v>
+        <v>122</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14591,11 +14591,11 @@
       </c>
       <c r="K210" s="10" t="n">
         <f aca="true">IF($J210=1,RAND(),-1)</f>
-        <v>0.140141032559434</v>
+        <v>0.0817505043322784</v>
       </c>
       <c r="L210" s="10" t="n">
         <f aca="false">IF($J210=1,RANK($K210,$K$2:$K$1001),"")</f>
-        <v>197</v>
+        <v>207</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14632,11 +14632,11 @@
       </c>
       <c r="K211" s="10" t="n">
         <f aca="true">IF($J211=1,RAND(),-1)</f>
-        <v>0.0500674270602088</v>
+        <v>0.628437552457917</v>
       </c>
       <c r="L211" s="10" t="n">
         <f aca="false">IF($J211=1,RANK($K211,$K$2:$K$1001),"")</f>
-        <v>217</v>
+        <v>96</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14673,11 +14673,11 @@
       </c>
       <c r="K212" s="10" t="n">
         <f aca="true">IF($J212=1,RAND(),-1)</f>
-        <v>0.544734448306043</v>
+        <v>0.00780384973492043</v>
       </c>
       <c r="L212" s="10" t="n">
         <f aca="false">IF($J212=1,RANK($K212,$K$2:$K$1001),"")</f>
-        <v>109</v>
+        <v>224</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14714,11 +14714,11 @@
       </c>
       <c r="K213" s="10" t="n">
         <f aca="true">IF($J213=1,RAND(),-1)</f>
-        <v>0.152786062032745</v>
+        <v>0.600274458994674</v>
       </c>
       <c r="L213" s="10" t="n">
         <f aca="false">IF($J213=1,RANK($K213,$K$2:$K$1001),"")</f>
-        <v>194</v>
+        <v>103</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14755,11 +14755,11 @@
       </c>
       <c r="K214" s="10" t="n">
         <f aca="true">IF($J214=1,RAND(),-1)</f>
-        <v>0.342096959626996</v>
+        <v>0.286918280990554</v>
       </c>
       <c r="L214" s="10" t="n">
         <f aca="false">IF($J214=1,RANK($K214,$K$2:$K$1001),"")</f>
-        <v>158</v>
+        <v>172</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14796,11 +14796,11 @@
       </c>
       <c r="K215" s="10" t="n">
         <f aca="true">IF($J215=1,RAND(),-1)</f>
-        <v>0.102911265832333</v>
+        <v>0.341295666633272</v>
       </c>
       <c r="L215" s="10" t="n">
         <f aca="false">IF($J215=1,RANK($K215,$K$2:$K$1001),"")</f>
-        <v>201</v>
+        <v>166</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14837,11 +14837,11 @@
       </c>
       <c r="K216" s="10" t="n">
         <f aca="true">IF($J216=1,RAND(),-1)</f>
-        <v>0.794455153546793</v>
+        <v>0.826126084088441</v>
       </c>
       <c r="L216" s="10" t="n">
         <f aca="false">IF($J216=1,RANK($K216,$K$2:$K$1001),"")</f>
-        <v>58</v>
+        <v>44</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14878,11 +14878,11 @@
       </c>
       <c r="K217" s="10" t="n">
         <f aca="true">IF($J217=1,RAND(),-1)</f>
-        <v>0.427825377394522</v>
+        <v>0.029975714800847</v>
       </c>
       <c r="L217" s="10" t="n">
         <f aca="false">IF($J217=1,RANK($K217,$K$2:$K$1001),"")</f>
-        <v>133</v>
+        <v>218</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14919,11 +14919,11 @@
       </c>
       <c r="K218" s="10" t="n">
         <f aca="true">IF($J218=1,RAND(),-1)</f>
-        <v>0.343663117449316</v>
+        <v>0.362536756039723</v>
       </c>
       <c r="L218" s="10" t="n">
         <f aca="false">IF($J218=1,RANK($K218,$K$2:$K$1001),"")</f>
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14960,11 +14960,11 @@
       </c>
       <c r="K219" s="10" t="n">
         <f aca="true">IF($J219=1,RAND(),-1)</f>
-        <v>0.933882770058957</v>
+        <v>0.858819405198279</v>
       </c>
       <c r="L219" s="10" t="n">
         <f aca="false">IF($J219=1,RANK($K219,$K$2:$K$1001),"")</f>
-        <v>18</v>
+        <v>36</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15001,11 +15001,11 @@
       </c>
       <c r="K220" s="10" t="n">
         <f aca="true">IF($J220=1,RAND(),-1)</f>
-        <v>0.227196625107299</v>
+        <v>0.280384066838397</v>
       </c>
       <c r="L220" s="10" t="n">
         <f aca="false">IF($J220=1,RANK($K220,$K$2:$K$1001),"")</f>
-        <v>185</v>
+        <v>173</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15042,11 +15042,11 @@
       </c>
       <c r="K221" s="10" t="n">
         <f aca="true">IF($J221=1,RAND(),-1)</f>
-        <v>0.623467817802674</v>
+        <v>0.942793976686422</v>
       </c>
       <c r="L221" s="10" t="n">
         <f aca="false">IF($J221=1,RANK($K221,$K$2:$K$1001),"")</f>
-        <v>95</v>
+        <v>17</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15083,11 +15083,11 @@
       </c>
       <c r="K222" s="10" t="n">
         <f aca="true">IF($J222=1,RAND(),-1)</f>
-        <v>0.279503854357236</v>
+        <v>0.534422073182594</v>
       </c>
       <c r="L222" s="10" t="n">
         <f aca="false">IF($J222=1,RANK($K222,$K$2:$K$1001),"")</f>
-        <v>173</v>
+        <v>116</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15124,11 +15124,11 @@
       </c>
       <c r="K223" s="10" t="n">
         <f aca="true">IF($J223=1,RAND(),-1)</f>
-        <v>0.524044878801365</v>
+        <v>0.100801664025524</v>
       </c>
       <c r="L223" s="10" t="n">
         <f aca="false">IF($J223=1,RANK($K223,$K$2:$K$1001),"")</f>
-        <v>114</v>
+        <v>199</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15165,11 +15165,11 @@
       </c>
       <c r="K224" s="10" t="n">
         <f aca="true">IF($J224=1,RAND(),-1)</f>
-        <v>0.19204468607196</v>
+        <v>0.844421590999132</v>
       </c>
       <c r="L224" s="10" t="n">
         <f aca="false">IF($J224=1,RANK($K224,$K$2:$K$1001),"")</f>
-        <v>190</v>
+        <v>39</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15206,11 +15206,11 @@
       </c>
       <c r="K225" s="10" t="n">
         <f aca="true">IF($J225=1,RAND(),-1)</f>
-        <v>0.869077690582068</v>
+        <v>0.973023993318143</v>
       </c>
       <c r="L225" s="10" t="n">
         <f aca="false">IF($J225=1,RANK($K225,$K$2:$K$1001),"")</f>
-        <v>41</v>
+        <v>10</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26125,11 +26125,11 @@
       </c>
       <c r="B4" s="5" t="str">
         <f aca="false">IF(Test!$J12="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J12))</f>
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="C4" s="12" t="str">
         <f aca="false">IF(B4="","",INDEX(Test!$C12:$F12,MATCH(B4,{"A","B","C","D"},0)))</f>
-        <v>216</v>
+        <v>4²</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26139,11 +26139,11 @@
       </c>
       <c r="B5" s="5" t="str">
         <f aca="false">IF(Test!$J13="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J13))</f>
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="C5" s="12" t="str">
         <f aca="false">IF(B5="","",INDEX(Test!$C13:$F13,MATCH(B5,{"A","B","C","D"},0)))</f>
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26153,11 +26153,11 @@
       </c>
       <c r="B6" s="5" t="str">
         <f aca="false">IF(Test!$J14="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J14))</f>
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="C6" s="12" t="str">
         <f aca="false">IF(B6="","",INDEX(Test!$C14:$F14,MATCH(B6,{"A","B","C","D"},0)))</f>
-        <v>3</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26167,11 +26167,11 @@
       </c>
       <c r="B7" s="5" t="str">
         <f aca="false">IF(Test!$J15="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J15))</f>
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="C7" s="12" t="str">
         <f aca="false">IF(B7="","",INDEX(Test!$C15:$F15,MATCH(B7,{"A","B","C","D"},0)))</f>
-        <v>116</v>
+        <v>Kare</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26181,11 +26181,11 @@
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">IF(Test!$J16="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J16))</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="C8" s="12" t="str">
         <f aca="false">IF(B8="","",INDEX(Test!$C16:$F16,MATCH(B8,{"A","B","C","D"},0)))</f>
-        <v>36</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26195,11 +26195,11 @@
       </c>
       <c r="B9" s="5" t="str">
         <f aca="false">IF(Test!$J17="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J17))</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="C9" s="12" t="str">
         <f aca="false">IF(B9="","",INDEX(Test!$C17:$F17,MATCH(B9,{"A","B","C","D"},0)))</f>
-        <v>8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26209,11 +26209,11 @@
       </c>
       <c r="B10" s="5" t="str">
         <f aca="false">IF(Test!$J18="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J18))</f>
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="C10" s="12" t="str">
         <f aca="false">IF(B10="","",INDEX(Test!$C18:$F18,MATCH(B10,{"A","B","C","D"},0)))</f>
-        <v>4</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26223,11 +26223,11 @@
       </c>
       <c r="B11" s="5" t="str">
         <f aca="false">IF(Test!$J19="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J19))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="C11" s="12" t="str">
         <f aca="false">IF(B11="","",INDEX(Test!$C19:$F19,MATCH(B11,{"A","B","C","D"},0)))</f>
-        <v>125</v>
+        <v>64 L</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26237,11 +26237,11 @@
       </c>
       <c r="B12" s="5" t="str">
         <f aca="false">IF(Test!$J20="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J20))</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF(B12="","",INDEX(Test!$C20:$F20,MATCH(B12,{"A","B","C","D"},0)))</f>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26255,7 +26255,7 @@
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF(B13="","",INDEX(Test!$C21:$F21,MATCH(B13,{"A","B","C","D"},0)))</f>
-        <v>64</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Türkçe Söz Varlığı soru üretici eklendi
- 577 soruluk havuz: sözcükte anlam, sözcükler arası anlam ilişkileri,
  söz grupları (deyim, atasözü, ikileme, pekiştirme, yansıma)
- Ortak şablon: uzun cümleli şıklar tek sütunda gösteriliyor

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6qBE8e6Wkv628t1Q47HQM
</commit_message>
<xml_diff>
--- a/KupSorulari/KupSoruHavuzu.xlsx
+++ b/KupSorulari/KupSoruHavuzu.xlsx
@@ -2144,27 +2144,27 @@
       </c>
       <c r="B12" s="11" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J12))</f>
-        <v>Aşağıdakilerden hangisinin değeri en küçüktür?</v>
+        <v>Bir ayrıtı 2 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J12))</f>
-        <v>5³</v>
+        <v>16</v>
       </c>
       <c r="D12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J12))</f>
-        <v>4²</v>
+        <v>24</v>
       </c>
       <c r="E12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J12))</f>
-        <v>10²</v>
+        <v>8</v>
       </c>
       <c r="F12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J12))</f>
-        <v>2⁵</v>
+        <v>12</v>
       </c>
       <c r="G12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J12))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Özellikleri</v>
       </c>
       <c r="H12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J12))</f>
@@ -2172,45 +2172,45 @@
       </c>
       <c r="J12" s="10" t="n">
         <f aca="false">IF(1&lt;=MIN($B$3,$B$6),MATCH(1,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
         <f aca="false">IF($J13="","",2)</f>
         <v>2</v>
       </c>
       <c r="B13" s="11" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J13))</f>
-        <v>Bir ayrıtı 12 cm olan küp şeklindeki bir kutunun içine, bir ayrıtı 4 cm olan küp şeklindeki kutulardan en fazla kaç tane yerleştirilebilir?</v>
+        <v>7³ ifadesinin değeri kaçtır?</v>
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J13))</f>
-        <v>3</v>
+        <v>343</v>
       </c>
       <c r="D13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J13))</f>
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J13))</f>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J13))</f>
-        <v>27</v>
+        <v>350</v>
       </c>
       <c r="G13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J13))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J13))</f>
-        <v>Orta</v>
+        <v>Kolay</v>
       </c>
       <c r="J13" s="10" t="n">
         <f aca="false">IF(2&lt;=MIN($B$3,$B$6),MATCH(2,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>136</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2220,35 +2220,35 @@
       </c>
       <c r="B14" s="11" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J14))</f>
-        <v>Bir ayrıtı 6 cm olan küpün hacmi kaç cm³'tür?</v>
+        <v>Bir ayrıtı 7 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
       </c>
       <c r="C14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J14))</f>
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J14))</f>
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="E14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J14))</f>
-        <v>216</v>
+        <v>84</v>
       </c>
       <c r="F14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J14))</f>
-        <v>72</v>
+        <v>343</v>
       </c>
       <c r="G14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J14))</f>
-        <v>Küpün Hacmi</v>
+        <v>Küpün Özellikleri</v>
       </c>
       <c r="H14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J14))</f>
-        <v>Kolay</v>
+        <v>Orta</v>
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">IF(3&lt;=MIN($B$3,$B$6),MATCH(3,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>108</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2258,35 +2258,35 @@
       </c>
       <c r="B15" s="11" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J15))</f>
-        <v>Küpün yüzleri hangi geometrik şekle sahiptir?</v>
+        <v>Hacmi 8 cm³ olan küpün bir ayrıtı kaç cm'dir?</v>
       </c>
       <c r="C15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J15))</f>
-        <v>Üçgen</v>
+        <v>2</v>
       </c>
       <c r="D15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J15))</f>
-        <v>Dikdörtgen</v>
+        <v>3</v>
       </c>
       <c r="E15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J15))</f>
-        <v>Beşgen</v>
+        <v>4</v>
       </c>
       <c r="F15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J15))</f>
-        <v>Kare</v>
+        <v>1</v>
       </c>
       <c r="G15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J15))</f>
-        <v>Küpün Özellikleri</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J15))</f>
-        <v>Kolay</v>
+        <v>Orta</v>
       </c>
       <c r="J15" s="10" t="n">
         <f aca="false">IF(4&lt;=MIN($B$3,$B$6),MATCH(4,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>172</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B16" s="11" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J16))</f>
-        <v>Hacmi 1000 cm³ olan küpün bir ayrıtı kaç cm'dir?</v>
+        <v>(2 + 2)³ ifadesinin değeri kaçtır?</v>
       </c>
       <c r="C16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J16))</f>
@@ -2304,27 +2304,27 @@
       </c>
       <c r="D16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J16))</f>
-        <v>333</v>
+        <v>12</v>
       </c>
       <c r="E16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J16))</f>
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J16))</f>
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="G16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J16))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J16))</f>
-        <v>Orta</v>
+        <v>Zor</v>
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">IF(5&lt;=MIN($B$3,$B$6),MATCH(5,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>127</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2334,27 +2334,27 @@
       </c>
       <c r="B17" s="11" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J17))</f>
-        <v>Bir ayrıtı 2 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
+        <v>Aşağıdakilerden hangisinin değeri en büyüktür?</v>
       </c>
       <c r="C17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J17))</f>
-        <v>16</v>
+        <v>6²</v>
       </c>
       <c r="D17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J17))</f>
-        <v>24</v>
+        <v>7²</v>
       </c>
       <c r="E17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J17))</f>
-        <v>8</v>
+        <v>3²</v>
       </c>
       <c r="F17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J17))</f>
-        <v>12</v>
+        <v>10²</v>
       </c>
       <c r="G17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J17))</f>
-        <v>Küpün Özellikleri</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J17))</f>
@@ -2362,37 +2362,37 @@
       </c>
       <c r="J17" s="10" t="n">
         <f aca="false">IF(6&lt;=MIN($B$3,$B$6),MATCH(6,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>177</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="n">
         <f aca="false">IF($J18="","",7)</f>
         <v>7</v>
       </c>
       <c r="B18" s="11" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J18))</f>
-        <v>Bir ayrıtı 5 birim olan küp kaç birim küpten oluşur?</v>
+        <v>6³ ifadesinin anlamı aşağıdakilerden hangisidir?</v>
       </c>
       <c r="C18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J18))</f>
-        <v>150</v>
+        <v>6 · 3</v>
       </c>
       <c r="D18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J18))</f>
-        <v>15</v>
+        <v>6 + 6 + 6</v>
       </c>
       <c r="E18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J18))</f>
-        <v>125</v>
+        <v>6 · 6 · 6</v>
       </c>
       <c r="F18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J18))</f>
-        <v>25</v>
+        <v>3 · 3 · 3 · 3 · 3 · 3</v>
       </c>
       <c r="G18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J18))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J18))</f>
@@ -2400,45 +2400,45 @@
       </c>
       <c r="J18" s="10" t="n">
         <f aca="false">IF(7&lt;=MIN($B$3,$B$6),MATCH(7,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>115</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="n">
         <f aca="false">IF($J19="","",8)</f>
         <v>8</v>
       </c>
       <c r="B19" s="11" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J19))</f>
-        <v>Bir ayrıtı 40 cm olan küp şeklindeki su deposu kaç litre su alır? (1 L = 1000 cm³)</v>
+        <v>Aşağıdakilerden hangisinin değeri en büyüktür?</v>
       </c>
       <c r="C19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J19))</f>
-        <v>16 L</v>
+        <v>5²</v>
       </c>
       <c r="D19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J19))</f>
-        <v>64 L</v>
+        <v>3²</v>
       </c>
       <c r="E19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J19))</f>
-        <v>12 L</v>
+        <v>7²</v>
       </c>
       <c r="F19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J19))</f>
-        <v>640 L</v>
+        <v>9²</v>
       </c>
       <c r="G19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J19))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J19))</f>
-        <v>Zor</v>
+        <v>Orta</v>
       </c>
       <c r="J19" s="10" t="n">
         <f aca="false">IF(8&lt;=MIN($B$3,$B$6),MATCH(8,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>163</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2448,23 +2448,23 @@
       </c>
       <c r="B20" s="11" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J20))</f>
-        <v>Bir doğal sayının küpünün 6 fazlası 70'dir. Bu sayı kaçtır?</v>
+        <v>Aşağıdakilerden hangisi bir doğal sayının küpü değildir?</v>
       </c>
       <c r="C20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J20))</f>
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="D20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J20))</f>
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="E20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J20))</f>
-        <v>23</v>
+        <v>512</v>
       </c>
       <c r="F20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J20))</f>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J20))</f>
@@ -2472,49 +2472,49 @@
       </c>
       <c r="H20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J20))</f>
-        <v>Zor</v>
+        <v>Orta</v>
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">IF(9&lt;=MIN($B$3,$B$6),MATCH(9,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>91</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="n">
         <f aca="false">IF($J21="","",10)</f>
         <v>10</v>
       </c>
       <c r="B21" s="11" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J21))</f>
-        <v>Birim küplerden oluşan bir küpün dış yüzeyi boyanıyor. 3 yüzü boyalı kaç birim küp vardır?</v>
+        <v>Bir ayrıtı 9 cm olan küpün hacmi kaç cm³'tür?</v>
       </c>
       <c r="C21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J21))</f>
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J21))</f>
-        <v>4</v>
+        <v>486</v>
       </c>
       <c r="E21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J21))</f>
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="F21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J21))</f>
-        <v>6</v>
+        <v>729</v>
       </c>
       <c r="G21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J21))</f>
-        <v>Küpün Özellikleri</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J21))</f>
-        <v>Zor</v>
+        <v>Kolay</v>
       </c>
       <c r="J21" s="10" t="n">
         <f aca="false">IF(10&lt;=MIN($B$3,$B$6),MATCH(10,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>224</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6063,11 +6063,11 @@
       </c>
       <c r="K2" s="10" t="n">
         <f aca="true">IF($J2=1,RAND(),-1)</f>
-        <v>0.904295007931261</v>
+        <v>0.0411754098130525</v>
       </c>
       <c r="L2" s="10" t="n">
         <f aca="false">IF($J2=1,RANK($K2,$K$2:$K$1001),"")</f>
-        <v>28</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6104,11 +6104,11 @@
       </c>
       <c r="K3" s="10" t="n">
         <f aca="true">IF($J3=1,RAND(),-1)</f>
-        <v>0.347832027480229</v>
+        <v>0.449411186215152</v>
       </c>
       <c r="L3" s="10" t="n">
         <f aca="false">IF($J3=1,RANK($K3,$K$2:$K$1001),"")</f>
-        <v>165</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6145,11 +6145,11 @@
       </c>
       <c r="K4" s="10" t="n">
         <f aca="true">IF($J4=1,RAND(),-1)</f>
-        <v>0.750082894605377</v>
+        <v>0.601096491243837</v>
       </c>
       <c r="L4" s="10" t="n">
         <f aca="false">IF($J4=1,RANK($K4,$K$2:$K$1001),"")</f>
-        <v>61</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6186,11 +6186,11 @@
       </c>
       <c r="K5" s="10" t="n">
         <f aca="true">IF($J5=1,RAND(),-1)</f>
-        <v>0.208943243672564</v>
+        <v>0.830308326299626</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">IF($J5=1,RANK($K5,$K$2:$K$1001),"")</f>
-        <v>183</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6227,11 +6227,11 @@
       </c>
       <c r="K6" s="10" t="n">
         <f aca="true">IF($J6=1,RAND(),-1)</f>
-        <v>0.918706047564604</v>
+        <v>0.868923679808951</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">IF($J6=1,RANK($K6,$K$2:$K$1001),"")</f>
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6268,11 +6268,11 @@
       </c>
       <c r="K7" s="10" t="n">
         <f aca="true">IF($J7=1,RAND(),-1)</f>
-        <v>0.421819935215955</v>
+        <v>0.0283675435125936</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">IF($J7=1,RANK($K7,$K$2:$K$1001),"")</f>
-        <v>144</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6309,11 +6309,11 @@
       </c>
       <c r="K8" s="10" t="n">
         <f aca="true">IF($J8=1,RAND(),-1)</f>
-        <v>0.47111732576979</v>
+        <v>0.999634046901793</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">IF($J8=1,RANK($K8,$K$2:$K$1001),"")</f>
-        <v>135</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6350,11 +6350,11 @@
       </c>
       <c r="K9" s="10" t="n">
         <f aca="true">IF($J9=1,RAND(),-1)</f>
-        <v>0.607174716423806</v>
+        <v>0.353863187978133</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">IF($J9=1,RANK($K9,$K$2:$K$1001),"")</f>
-        <v>102</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6391,11 +6391,11 @@
       </c>
       <c r="K10" s="10" t="n">
         <f aca="true">IF($J10=1,RAND(),-1)</f>
-        <v>0.556146243639258</v>
+        <v>0.941179663664032</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">IF($J10=1,RANK($K10,$K$2:$K$1001),"")</f>
-        <v>112</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6432,11 +6432,11 @@
       </c>
       <c r="K11" s="10" t="n">
         <f aca="true">IF($J11=1,RAND(),-1)</f>
-        <v>0.893599285111705</v>
+        <v>0.316302629889705</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">IF($J11=1,RANK($K11,$K$2:$K$1001),"")</f>
-        <v>29</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6473,11 +6473,11 @@
       </c>
       <c r="K12" s="10" t="n">
         <f aca="true">IF($J12=1,RAND(),-1)</f>
-        <v>0.563962333146206</v>
+        <v>0.146854722041688</v>
       </c>
       <c r="L12" s="10" t="n">
         <f aca="false">IF($J12=1,RANK($K12,$K$2:$K$1001),"")</f>
-        <v>110</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6514,11 +6514,11 @@
       </c>
       <c r="K13" s="10" t="n">
         <f aca="true">IF($J13=1,RAND(),-1)</f>
-        <v>0.779208103293628</v>
+        <v>0.31813579023357</v>
       </c>
       <c r="L13" s="10" t="n">
         <f aca="false">IF($J13=1,RANK($K13,$K$2:$K$1001),"")</f>
-        <v>53</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6555,11 +6555,11 @@
       </c>
       <c r="K14" s="10" t="n">
         <f aca="true">IF($J14=1,RAND(),-1)</f>
-        <v>0.334655143949095</v>
+        <v>0.396125657932773</v>
       </c>
       <c r="L14" s="10" t="n">
         <f aca="false">IF($J14=1,RANK($K14,$K$2:$K$1001),"")</f>
-        <v>169</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6596,11 +6596,11 @@
       </c>
       <c r="K15" s="10" t="n">
         <f aca="true">IF($J15=1,RAND(),-1)</f>
-        <v>0.644995654731458</v>
+        <v>0.35035549198795</v>
       </c>
       <c r="L15" s="10" t="n">
         <f aca="false">IF($J15=1,RANK($K15,$K$2:$K$1001),"")</f>
-        <v>93</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6637,11 +6637,11 @@
       </c>
       <c r="K16" s="10" t="n">
         <f aca="true">IF($J16=1,RAND(),-1)</f>
-        <v>0.619759625644779</v>
+        <v>0.220307498844939</v>
       </c>
       <c r="L16" s="10" t="n">
         <f aca="false">IF($J16=1,RANK($K16,$K$2:$K$1001),"")</f>
-        <v>98</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6678,11 +6678,11 @@
       </c>
       <c r="K17" s="10" t="n">
         <f aca="true">IF($J17=1,RAND(),-1)</f>
-        <v>0.698544711384879</v>
+        <v>0.792532760650073</v>
       </c>
       <c r="L17" s="10" t="n">
         <f aca="false">IF($J17=1,RANK($K17,$K$2:$K$1001),"")</f>
-        <v>74</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6719,11 +6719,11 @@
       </c>
       <c r="K18" s="10" t="n">
         <f aca="true">IF($J18=1,RAND(),-1)</f>
-        <v>0.0381110063181314</v>
+        <v>0.742026833599792</v>
       </c>
       <c r="L18" s="10" t="n">
         <f aca="false">IF($J18=1,RANK($K18,$K$2:$K$1001),"")</f>
-        <v>216</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="K19" s="10" t="n">
         <f aca="true">IF($J19=1,RAND(),-1)</f>
-        <v>0.687625955122907</v>
+        <v>0.0545691977933067</v>
       </c>
       <c r="L19" s="10" t="n">
         <f aca="false">IF($J19=1,RANK($K19,$K$2:$K$1001),"")</f>
-        <v>77</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6801,11 +6801,11 @@
       </c>
       <c r="K20" s="10" t="n">
         <f aca="true">IF($J20=1,RAND(),-1)</f>
-        <v>0.765734535717859</v>
+        <v>0.606779866493235</v>
       </c>
       <c r="L20" s="10" t="n">
         <f aca="false">IF($J20=1,RANK($K20,$K$2:$K$1001),"")</f>
-        <v>56</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6842,11 +6842,11 @@
       </c>
       <c r="K21" s="10" t="n">
         <f aca="true">IF($J21=1,RAND(),-1)</f>
-        <v>0.452288454609707</v>
+        <v>0.758069521944036</v>
       </c>
       <c r="L21" s="10" t="n">
         <f aca="false">IF($J21=1,RANK($K21,$K$2:$K$1001),"")</f>
-        <v>137</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="K22" s="10" t="n">
         <f aca="true">IF($J22=1,RAND(),-1)</f>
-        <v>0.129526145422593</v>
+        <v>0.097479103659455</v>
       </c>
       <c r="L22" s="10" t="n">
         <f aca="false">IF($J22=1,RANK($K22,$K$2:$K$1001),"")</f>
-        <v>194</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6924,11 +6924,11 @@
       </c>
       <c r="K23" s="10" t="n">
         <f aca="true">IF($J23=1,RAND(),-1)</f>
-        <v>0.758716552972226</v>
+        <v>0.621714421198653</v>
       </c>
       <c r="L23" s="10" t="n">
         <f aca="false">IF($J23=1,RANK($K23,$K$2:$K$1001),"")</f>
-        <v>59</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6965,11 +6965,11 @@
       </c>
       <c r="K24" s="10" t="n">
         <f aca="true">IF($J24=1,RAND(),-1)</f>
-        <v>0.122989473265731</v>
+        <v>0.981790367842763</v>
       </c>
       <c r="L24" s="10" t="n">
         <f aca="false">IF($J24=1,RANK($K24,$K$2:$K$1001),"")</f>
-        <v>196</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7006,11 +7006,11 @@
       </c>
       <c r="K25" s="10" t="n">
         <f aca="true">IF($J25=1,RAND(),-1)</f>
-        <v>0.08448286353226</v>
+        <v>0.902143084310058</v>
       </c>
       <c r="L25" s="10" t="n">
         <f aca="false">IF($J25=1,RANK($K25,$K$2:$K$1001),"")</f>
-        <v>205</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7047,11 +7047,11 @@
       </c>
       <c r="K26" s="10" t="n">
         <f aca="true">IF($J26=1,RAND(),-1)</f>
-        <v>0.275418033471049</v>
+        <v>0.226134123656925</v>
       </c>
       <c r="L26" s="10" t="n">
         <f aca="false">IF($J26=1,RANK($K26,$K$2:$K$1001),"")</f>
-        <v>174</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7088,11 +7088,11 @@
       </c>
       <c r="K27" s="10" t="n">
         <f aca="true">IF($J27=1,RAND(),-1)</f>
-        <v>0.954656548506431</v>
+        <v>0.722689264659609</v>
       </c>
       <c r="L27" s="10" t="n">
         <f aca="false">IF($J27=1,RANK($K27,$K$2:$K$1001),"")</f>
-        <v>13</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7129,11 +7129,11 @@
       </c>
       <c r="K28" s="10" t="n">
         <f aca="true">IF($J28=1,RAND(),-1)</f>
-        <v>0.422555556138029</v>
+        <v>0.344365759983099</v>
       </c>
       <c r="L28" s="10" t="n">
         <f aca="false">IF($J28=1,RANK($K28,$K$2:$K$1001),"")</f>
-        <v>142</v>
+        <v>157</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7170,11 +7170,11 @@
       </c>
       <c r="K29" s="10" t="n">
         <f aca="true">IF($J29=1,RAND(),-1)</f>
-        <v>0.22260363951565</v>
+        <v>0.909128990003166</v>
       </c>
       <c r="L29" s="10" t="n">
         <f aca="false">IF($J29=1,RANK($K29,$K$2:$K$1001),"")</f>
-        <v>180</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7211,11 +7211,11 @@
       </c>
       <c r="K30" s="10" t="n">
         <f aca="true">IF($J30=1,RAND(),-1)</f>
-        <v>0.892300576640369</v>
+        <v>0.900243355202201</v>
       </c>
       <c r="L30" s="10" t="n">
         <f aca="false">IF($J30=1,RANK($K30,$K$2:$K$1001),"")</f>
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7252,11 +7252,11 @@
       </c>
       <c r="K31" s="10" t="n">
         <f aca="true">IF($J31=1,RAND(),-1)</f>
-        <v>0.066248128534441</v>
+        <v>0.640763855247545</v>
       </c>
       <c r="L31" s="10" t="n">
         <f aca="false">IF($J31=1,RANK($K31,$K$2:$K$1001),"")</f>
-        <v>208</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7293,11 +7293,11 @@
       </c>
       <c r="K32" s="10" t="n">
         <f aca="true">IF($J32=1,RAND(),-1)</f>
-        <v>0.844167020171817</v>
+        <v>0.257453052017052</v>
       </c>
       <c r="L32" s="10" t="n">
         <f aca="false">IF($J32=1,RANK($K32,$K$2:$K$1001),"")</f>
-        <v>40</v>
+        <v>174</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7334,11 +7334,11 @@
       </c>
       <c r="K33" s="10" t="n">
         <f aca="true">IF($J33=1,RAND(),-1)</f>
-        <v>0.726525481264205</v>
+        <v>0.481484915811606</v>
       </c>
       <c r="L33" s="10" t="n">
         <f aca="false">IF($J33=1,RANK($K33,$K$2:$K$1001),"")</f>
-        <v>66</v>
+        <v>122</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7375,11 +7375,11 @@
       </c>
       <c r="K34" s="10" t="n">
         <f aca="true">IF($J34=1,RAND(),-1)</f>
-        <v>0.808747741055165</v>
+        <v>0.416940668017262</v>
       </c>
       <c r="L34" s="10" t="n">
         <f aca="false">IF($J34=1,RANK($K34,$K$2:$K$1001),"")</f>
-        <v>47</v>
+        <v>139</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7416,11 +7416,11 @@
       </c>
       <c r="K35" s="10" t="n">
         <f aca="true">IF($J35=1,RAND(),-1)</f>
-        <v>0.680875338208257</v>
+        <v>0.820388828856205</v>
       </c>
       <c r="L35" s="10" t="n">
         <f aca="false">IF($J35=1,RANK($K35,$K$2:$K$1001),"")</f>
-        <v>80</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7457,11 +7457,11 @@
       </c>
       <c r="K36" s="10" t="n">
         <f aca="true">IF($J36=1,RAND(),-1)</f>
-        <v>0.536375961688599</v>
+        <v>0.553381749169604</v>
       </c>
       <c r="L36" s="10" t="n">
         <f aca="false">IF($J36=1,RANK($K36,$K$2:$K$1001),"")</f>
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7498,11 +7498,11 @@
       </c>
       <c r="K37" s="10" t="n">
         <f aca="true">IF($J37=1,RAND(),-1)</f>
-        <v>0.361172896427552</v>
+        <v>0.655876820002614</v>
       </c>
       <c r="L37" s="10" t="n">
         <f aca="false">IF($J37=1,RANK($K37,$K$2:$K$1001),"")</f>
-        <v>160</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7539,11 +7539,11 @@
       </c>
       <c r="K38" s="10" t="n">
         <f aca="true">IF($J38=1,RAND(),-1)</f>
-        <v>0.471302650246549</v>
+        <v>0.727839815520398</v>
       </c>
       <c r="L38" s="10" t="n">
         <f aca="false">IF($J38=1,RANK($K38,$K$2:$K$1001),"")</f>
-        <v>133</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7580,11 +7580,11 @@
       </c>
       <c r="K39" s="10" t="n">
         <f aca="true">IF($J39=1,RAND(),-1)</f>
-        <v>0.782620755840389</v>
+        <v>0.477193157601631</v>
       </c>
       <c r="L39" s="10" t="n">
         <f aca="false">IF($J39=1,RANK($K39,$K$2:$K$1001),"")</f>
-        <v>52</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7621,11 +7621,11 @@
       </c>
       <c r="K40" s="10" t="n">
         <f aca="true">IF($J40=1,RAND(),-1)</f>
-        <v>0.756501435086049</v>
+        <v>0.458217693305363</v>
       </c>
       <c r="L40" s="10" t="n">
         <f aca="false">IF($J40=1,RANK($K40,$K$2:$K$1001),"")</f>
-        <v>60</v>
+        <v>129</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7662,11 +7662,11 @@
       </c>
       <c r="K41" s="10" t="n">
         <f aca="true">IF($J41=1,RAND(),-1)</f>
-        <v>0.655292643470257</v>
+        <v>0.270579327250338</v>
       </c>
       <c r="L41" s="10" t="n">
         <f aca="false">IF($J41=1,RANK($K41,$K$2:$K$1001),"")</f>
-        <v>89</v>
+        <v>173</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7703,11 +7703,11 @@
       </c>
       <c r="K42" s="10" t="n">
         <f aca="true">IF($J42=1,RAND(),-1)</f>
-        <v>0.668420087896298</v>
+        <v>0.257142699906581</v>
       </c>
       <c r="L42" s="10" t="n">
         <f aca="false">IF($J42=1,RANK($K42,$K$2:$K$1001),"")</f>
-        <v>87</v>
+        <v>175</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7744,11 +7744,11 @@
       </c>
       <c r="K43" s="10" t="n">
         <f aca="true">IF($J43=1,RAND(),-1)</f>
-        <v>0.0476734288266797</v>
+        <v>0.747941383616858</v>
       </c>
       <c r="L43" s="10" t="n">
         <f aca="false">IF($J43=1,RANK($K43,$K$2:$K$1001),"")</f>
-        <v>214</v>
+        <v>66</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7785,11 +7785,11 @@
       </c>
       <c r="K44" s="10" t="n">
         <f aca="true">IF($J44=1,RAND(),-1)</f>
-        <v>0.747040795286031</v>
+        <v>0.682350550397438</v>
       </c>
       <c r="L44" s="10" t="n">
         <f aca="false">IF($J44=1,RANK($K44,$K$2:$K$1001),"")</f>
-        <v>62</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7826,11 +7826,11 @@
       </c>
       <c r="K45" s="10" t="n">
         <f aca="true">IF($J45=1,RAND(),-1)</f>
-        <v>0.340781259847172</v>
+        <v>0.957242143566014</v>
       </c>
       <c r="L45" s="10" t="n">
         <f aca="false">IF($J45=1,RANK($K45,$K$2:$K$1001),"")</f>
-        <v>167</v>
+        <v>13</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7867,11 +7867,11 @@
       </c>
       <c r="K46" s="10" t="n">
         <f aca="true">IF($J46=1,RAND(),-1)</f>
-        <v>0.325524596297083</v>
+        <v>0.564191503182607</v>
       </c>
       <c r="L46" s="10" t="n">
         <f aca="false">IF($J46=1,RANK($K46,$K$2:$K$1001),"")</f>
-        <v>171</v>
+        <v>106</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7908,11 +7908,11 @@
       </c>
       <c r="K47" s="10" t="n">
         <f aca="true">IF($J47=1,RAND(),-1)</f>
-        <v>0.933956665100782</v>
+        <v>0.718936128430385</v>
       </c>
       <c r="L47" s="10" t="n">
         <f aca="false">IF($J47=1,RANK($K47,$K$2:$K$1001),"")</f>
-        <v>19</v>
+        <v>73</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7949,11 +7949,11 @@
       </c>
       <c r="K48" s="10" t="n">
         <f aca="true">IF($J48=1,RAND(),-1)</f>
-        <v>0.763986664084633</v>
+        <v>0.830303633578037</v>
       </c>
       <c r="L48" s="10" t="n">
         <f aca="false">IF($J48=1,RANK($K48,$K$2:$K$1001),"")</f>
-        <v>57</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7990,11 +7990,11 @@
       </c>
       <c r="K49" s="10" t="n">
         <f aca="true">IF($J49=1,RAND(),-1)</f>
-        <v>0.353676881976362</v>
+        <v>0.105797343930896</v>
       </c>
       <c r="L49" s="10" t="n">
         <f aca="false">IF($J49=1,RANK($K49,$K$2:$K$1001),"")</f>
-        <v>164</v>
+        <v>203</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8031,11 +8031,11 @@
       </c>
       <c r="K50" s="10" t="n">
         <f aca="true">IF($J50=1,RAND(),-1)</f>
-        <v>0.200278989353445</v>
+        <v>0.461674405168116</v>
       </c>
       <c r="L50" s="10" t="n">
         <f aca="false">IF($J50=1,RANK($K50,$K$2:$K$1001),"")</f>
-        <v>185</v>
+        <v>128</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8072,11 +8072,11 @@
       </c>
       <c r="K51" s="10" t="n">
         <f aca="true">IF($J51=1,RAND(),-1)</f>
-        <v>0.724833098385281</v>
+        <v>0.471491576486297</v>
       </c>
       <c r="L51" s="10" t="n">
         <f aca="false">IF($J51=1,RANK($K51,$K$2:$K$1001),"")</f>
-        <v>67</v>
+        <v>127</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8113,11 +8113,11 @@
       </c>
       <c r="K52" s="10" t="n">
         <f aca="true">IF($J52=1,RAND(),-1)</f>
-        <v>0.402392725859177</v>
+        <v>0.335547521413743</v>
       </c>
       <c r="L52" s="10" t="n">
         <f aca="false">IF($J52=1,RANK($K52,$K$2:$K$1001),"")</f>
-        <v>148</v>
+        <v>161</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8154,11 +8154,11 @@
       </c>
       <c r="K53" s="10" t="n">
         <f aca="true">IF($J53=1,RAND(),-1)</f>
-        <v>0.266176952336694</v>
+        <v>0.399194913705203</v>
       </c>
       <c r="L53" s="10" t="n">
         <f aca="false">IF($J53=1,RANK($K53,$K$2:$K$1001),"")</f>
-        <v>176</v>
+        <v>148</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8195,11 +8195,11 @@
       </c>
       <c r="K54" s="10" t="n">
         <f aca="true">IF($J54=1,RAND(),-1)</f>
-        <v>0.78933696993077</v>
+        <v>0.287927786335275</v>
       </c>
       <c r="L54" s="10" t="n">
         <f aca="false">IF($J54=1,RANK($K54,$K$2:$K$1001),"")</f>
-        <v>51</v>
+        <v>169</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8236,11 +8236,11 @@
       </c>
       <c r="K55" s="10" t="n">
         <f aca="true">IF($J55=1,RAND(),-1)</f>
-        <v>0.547697860727407</v>
+        <v>0.982083403409526</v>
       </c>
       <c r="L55" s="10" t="n">
         <f aca="false">IF($J55=1,RANK($K55,$K$2:$K$1001),"")</f>
-        <v>113</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8277,11 +8277,11 @@
       </c>
       <c r="K56" s="10" t="n">
         <f aca="true">IF($J56=1,RAND(),-1)</f>
-        <v>0.510707930871119</v>
+        <v>0.887989054334326</v>
       </c>
       <c r="L56" s="10" t="n">
         <f aca="false">IF($J56=1,RANK($K56,$K$2:$K$1001),"")</f>
-        <v>120</v>
+        <v>33</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8318,11 +8318,11 @@
       </c>
       <c r="K57" s="10" t="n">
         <f aca="true">IF($J57=1,RAND(),-1)</f>
-        <v>0.906484637982813</v>
+        <v>0.977716180093909</v>
       </c>
       <c r="L57" s="10" t="n">
         <f aca="false">IF($J57=1,RANK($K57,$K$2:$K$1001),"")</f>
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8359,11 +8359,11 @@
       </c>
       <c r="K58" s="10" t="n">
         <f aca="true">IF($J58=1,RAND(),-1)</f>
-        <v>0.718851959362426</v>
+        <v>0.308030767623289</v>
       </c>
       <c r="L58" s="10" t="n">
         <f aca="false">IF($J58=1,RANK($K58,$K$2:$K$1001),"")</f>
-        <v>70</v>
+        <v>165</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8400,11 +8400,11 @@
       </c>
       <c r="K59" s="10" t="n">
         <f aca="true">IF($J59=1,RAND(),-1)</f>
-        <v>0.195184762927591</v>
+        <v>0.495895388504701</v>
       </c>
       <c r="L59" s="10" t="n">
         <f aca="false">IF($J59=1,RANK($K59,$K$2:$K$1001),"")</f>
-        <v>186</v>
+        <v>120</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8441,11 +8441,11 @@
       </c>
       <c r="K60" s="10" t="n">
         <f aca="true">IF($J60=1,RAND(),-1)</f>
-        <v>0.999551985157311</v>
+        <v>0.596637310922611</v>
       </c>
       <c r="L60" s="10" t="n">
         <f aca="false">IF($J60=1,RANK($K60,$K$2:$K$1001),"")</f>
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8482,11 +8482,11 @@
       </c>
       <c r="K61" s="10" t="n">
         <f aca="true">IF($J61=1,RAND(),-1)</f>
-        <v>0.510102461717866</v>
+        <v>0.21185582582072</v>
       </c>
       <c r="L61" s="10" t="n">
         <f aca="false">IF($J61=1,RANK($K61,$K$2:$K$1001),"")</f>
-        <v>121</v>
+        <v>186</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8523,11 +8523,11 @@
       </c>
       <c r="K62" s="10" t="n">
         <f aca="true">IF($J62=1,RAND(),-1)</f>
-        <v>0.717626235737797</v>
+        <v>0.188242001890644</v>
       </c>
       <c r="L62" s="10" t="n">
         <f aca="false">IF($J62=1,RANK($K62,$K$2:$K$1001),"")</f>
-        <v>72</v>
+        <v>190</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8564,11 +8564,11 @@
       </c>
       <c r="K63" s="10" t="n">
         <f aca="true">IF($J63=1,RAND(),-1)</f>
-        <v>0.113315961125073</v>
+        <v>0.812339756334825</v>
       </c>
       <c r="L63" s="10" t="n">
         <f aca="false">IF($J63=1,RANK($K63,$K$2:$K$1001),"")</f>
-        <v>198</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8605,11 +8605,11 @@
       </c>
       <c r="K64" s="10" t="n">
         <f aca="true">IF($J64=1,RAND(),-1)</f>
-        <v>0.6495412141826</v>
+        <v>0.800928435580494</v>
       </c>
       <c r="L64" s="10" t="n">
         <f aca="false">IF($J64=1,RANK($K64,$K$2:$K$1001),"")</f>
-        <v>92</v>
+        <v>53</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8646,11 +8646,11 @@
       </c>
       <c r="K65" s="10" t="n">
         <f aca="true">IF($J65=1,RAND(),-1)</f>
-        <v>0.800251729270813</v>
+        <v>0.40415861166416</v>
       </c>
       <c r="L65" s="10" t="n">
         <f aca="false">IF($J65=1,RANK($K65,$K$2:$K$1001),"")</f>
-        <v>49</v>
+        <v>147</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8687,11 +8687,11 @@
       </c>
       <c r="K66" s="10" t="n">
         <f aca="true">IF($J66=1,RAND(),-1)</f>
-        <v>0.0156827454217206</v>
+        <v>0.140235757977395</v>
       </c>
       <c r="L66" s="10" t="n">
         <f aca="false">IF($J66=1,RANK($K66,$K$2:$K$1001),"")</f>
-        <v>223</v>
+        <v>197</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8728,11 +8728,11 @@
       </c>
       <c r="K67" s="10" t="n">
         <f aca="true">IF($J67=1,RAND(),-1)</f>
-        <v>0.357769525282947</v>
+        <v>0.753613265232359</v>
       </c>
       <c r="L67" s="10" t="n">
         <f aca="false">IF($J67=1,RANK($K67,$K$2:$K$1001),"")</f>
-        <v>162</v>
+        <v>65</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8769,11 +8769,11 @@
       </c>
       <c r="K68" s="10" t="n">
         <f aca="true">IF($J68=1,RAND(),-1)</f>
-        <v>0.397190967643178</v>
+        <v>0.976040052293349</v>
       </c>
       <c r="L68" s="10" t="n">
         <f aca="false">IF($J68=1,RANK($K68,$K$2:$K$1001),"")</f>
-        <v>150</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8810,11 +8810,11 @@
       </c>
       <c r="K69" s="10" t="n">
         <f aca="true">IF($J69=1,RAND(),-1)</f>
-        <v>0.390710393683268</v>
+        <v>0.132659301939662</v>
       </c>
       <c r="L69" s="10" t="n">
         <f aca="false">IF($J69=1,RANK($K69,$K$2:$K$1001),"")</f>
-        <v>153</v>
+        <v>199</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8851,11 +8851,11 @@
       </c>
       <c r="K70" s="10" t="n">
         <f aca="true">IF($J70=1,RAND(),-1)</f>
-        <v>0.421121987436668</v>
+        <v>0.871058164385805</v>
       </c>
       <c r="L70" s="10" t="n">
         <f aca="false">IF($J70=1,RANK($K70,$K$2:$K$1001),"")</f>
-        <v>146</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8892,11 +8892,11 @@
       </c>
       <c r="K71" s="10" t="n">
         <f aca="true">IF($J71=1,RAND(),-1)</f>
-        <v>0.135218157428132</v>
+        <v>0.841723396132882</v>
       </c>
       <c r="L71" s="10" t="n">
         <f aca="false">IF($J71=1,RANK($K71,$K$2:$K$1001),"")</f>
-        <v>192</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="K72" s="10" t="n">
         <f aca="true">IF($J72=1,RAND(),-1)</f>
-        <v>0.499212467498197</v>
+        <v>0.664741586310112</v>
       </c>
       <c r="L72" s="10" t="n">
         <f aca="false">IF($J72=1,RANK($K72,$K$2:$K$1001),"")</f>
-        <v>125</v>
+        <v>85</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8974,11 +8974,11 @@
       </c>
       <c r="K73" s="10" t="n">
         <f aca="true">IF($J73=1,RAND(),-1)</f>
-        <v>0.437854155122886</v>
+        <v>0.126455421028607</v>
       </c>
       <c r="L73" s="10" t="n">
         <f aca="false">IF($J73=1,RANK($K73,$K$2:$K$1001),"")</f>
-        <v>140</v>
+        <v>201</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9015,11 +9015,11 @@
       </c>
       <c r="K74" s="10" t="n">
         <f aca="true">IF($J74=1,RAND(),-1)</f>
-        <v>0.69375450282616</v>
+        <v>0.238762401024499</v>
       </c>
       <c r="L74" s="10" t="n">
         <f aca="false">IF($J74=1,RANK($K74,$K$2:$K$1001),"")</f>
-        <v>75</v>
+        <v>179</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9056,11 +9056,11 @@
       </c>
       <c r="K75" s="10" t="n">
         <f aca="true">IF($J75=1,RAND(),-1)</f>
-        <v>0.67673852045873</v>
+        <v>0.21784742330843</v>
       </c>
       <c r="L75" s="10" t="n">
         <f aca="false">IF($J75=1,RANK($K75,$K$2:$K$1001),"")</f>
-        <v>82</v>
+        <v>185</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9097,11 +9097,11 @@
       </c>
       <c r="K76" s="10" t="n">
         <f aca="true">IF($J76=1,RAND(),-1)</f>
-        <v>0.766690813614934</v>
+        <v>0.440900603171454</v>
       </c>
       <c r="L76" s="10" t="n">
         <f aca="false">IF($J76=1,RANK($K76,$K$2:$K$1001),"")</f>
-        <v>54</v>
+        <v>133</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9138,11 +9138,11 @@
       </c>
       <c r="K77" s="10" t="n">
         <f aca="true">IF($J77=1,RAND(),-1)</f>
-        <v>0.718404063346434</v>
+        <v>0.241320669304064</v>
       </c>
       <c r="L77" s="10" t="n">
         <f aca="false">IF($J77=1,RANK($K77,$K$2:$K$1001),"")</f>
-        <v>71</v>
+        <v>178</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9179,11 +9179,11 @@
       </c>
       <c r="K78" s="10" t="n">
         <f aca="true">IF($J78=1,RAND(),-1)</f>
-        <v>0.488931431906967</v>
+        <v>0.340763078945877</v>
       </c>
       <c r="L78" s="10" t="n">
         <f aca="false">IF($J78=1,RANK($K78,$K$2:$K$1001),"")</f>
-        <v>127</v>
+        <v>159</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9220,11 +9220,11 @@
       </c>
       <c r="K79" s="10" t="n">
         <f aca="true">IF($J79=1,RAND(),-1)</f>
-        <v>0.421980951200375</v>
+        <v>0.632485875980518</v>
       </c>
       <c r="L79" s="10" t="n">
         <f aca="false">IF($J79=1,RANK($K79,$K$2:$K$1001),"")</f>
-        <v>143</v>
+        <v>91</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9261,11 +9261,11 @@
       </c>
       <c r="K80" s="10" t="n">
         <f aca="true">IF($J80=1,RAND(),-1)</f>
-        <v>0.655296912166902</v>
+        <v>0.43491216022024</v>
       </c>
       <c r="L80" s="10" t="n">
         <f aca="false">IF($J80=1,RANK($K80,$K$2:$K$1001),"")</f>
-        <v>88</v>
+        <v>136</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9302,11 +9302,11 @@
       </c>
       <c r="K81" s="10" t="n">
         <f aca="true">IF($J81=1,RAND(),-1)</f>
-        <v>0.529114095023939</v>
+        <v>0.289808184631809</v>
       </c>
       <c r="L81" s="10" t="n">
         <f aca="false">IF($J81=1,RANK($K81,$K$2:$K$1001),"")</f>
-        <v>117</v>
+        <v>167</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9343,11 +9343,11 @@
       </c>
       <c r="K82" s="10" t="n">
         <f aca="true">IF($J82=1,RAND(),-1)</f>
-        <v>0.146844773973692</v>
+        <v>0.517393647041842</v>
       </c>
       <c r="L82" s="10" t="n">
         <f aca="false">IF($J82=1,RANK($K82,$K$2:$K$1001),"")</f>
-        <v>190</v>
+        <v>117</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9384,11 +9384,11 @@
       </c>
       <c r="K83" s="10" t="n">
         <f aca="true">IF($J83=1,RAND(),-1)</f>
-        <v>0.942758279377395</v>
+        <v>0.0485859722977174</v>
       </c>
       <c r="L83" s="10" t="n">
         <f aca="false">IF($J83=1,RANK($K83,$K$2:$K$1001),"")</f>
-        <v>18</v>
+        <v>215</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9425,11 +9425,11 @@
       </c>
       <c r="K84" s="10" t="n">
         <f aca="true">IF($J84=1,RAND(),-1)</f>
-        <v>0.0513854400229985</v>
+        <v>0.687398153556858</v>
       </c>
       <c r="L84" s="10" t="n">
         <f aca="false">IF($J84=1,RANK($K84,$K$2:$K$1001),"")</f>
-        <v>212</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9466,11 +9466,11 @@
       </c>
       <c r="K85" s="10" t="n">
         <f aca="true">IF($J85=1,RAND(),-1)</f>
-        <v>0.393108012747143</v>
+        <v>0.985274015158048</v>
       </c>
       <c r="L85" s="10" t="n">
         <f aca="false">IF($J85=1,RANK($K85,$K$2:$K$1001),"")</f>
-        <v>151</v>
+        <v>5</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9507,11 +9507,11 @@
       </c>
       <c r="K86" s="10" t="n">
         <f aca="true">IF($J86=1,RAND(),-1)</f>
-        <v>0.0192287357659517</v>
+        <v>0.184848672188111</v>
       </c>
       <c r="L86" s="10" t="n">
         <f aca="false">IF($J86=1,RANK($K86,$K$2:$K$1001),"")</f>
-        <v>221</v>
+        <v>191</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9548,11 +9548,11 @@
       </c>
       <c r="K87" s="10" t="n">
         <f aca="true">IF($J87=1,RAND(),-1)</f>
-        <v>0.760131741028468</v>
+        <v>0.0538107612208909</v>
       </c>
       <c r="L87" s="10" t="n">
         <f aca="false">IF($J87=1,RANK($K87,$K$2:$K$1001),"")</f>
-        <v>58</v>
+        <v>214</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9589,11 +9589,11 @@
       </c>
       <c r="K88" s="10" t="n">
         <f aca="true">IF($J88=1,RAND(),-1)</f>
-        <v>0.586313235796245</v>
+        <v>0.0658790644957822</v>
       </c>
       <c r="L88" s="10" t="n">
         <f aca="false">IF($J88=1,RANK($K88,$K$2:$K$1001),"")</f>
-        <v>106</v>
+        <v>211</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9630,11 +9630,11 @@
       </c>
       <c r="K89" s="10" t="n">
         <f aca="true">IF($J89=1,RAND(),-1)</f>
-        <v>0.0841933189336721</v>
+        <v>0.482451385017774</v>
       </c>
       <c r="L89" s="10" t="n">
         <f aca="false">IF($J89=1,RANK($K89,$K$2:$K$1001),"")</f>
-        <v>206</v>
+        <v>121</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9671,11 +9671,11 @@
       </c>
       <c r="K90" s="10" t="n">
         <f aca="true">IF($J90=1,RAND(),-1)</f>
-        <v>0.683792164618924</v>
+        <v>0.862579276901756</v>
       </c>
       <c r="L90" s="10" t="n">
         <f aca="false">IF($J90=1,RANK($K90,$K$2:$K$1001),"")</f>
-        <v>79</v>
+        <v>36</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9712,11 +9712,11 @@
       </c>
       <c r="K91" s="10" t="n">
         <f aca="true">IF($J91=1,RAND(),-1)</f>
-        <v>0.613431408599825</v>
+        <v>0.861398017883458</v>
       </c>
       <c r="L91" s="10" t="n">
         <f aca="false">IF($J91=1,RANK($K91,$K$2:$K$1001),"")</f>
-        <v>101</v>
+        <v>37</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9753,11 +9753,11 @@
       </c>
       <c r="K92" s="10" t="n">
         <f aca="true">IF($J92=1,RAND(),-1)</f>
-        <v>0.973164620038686</v>
+        <v>0.801706944009685</v>
       </c>
       <c r="L92" s="10" t="n">
         <f aca="false">IF($J92=1,RANK($K92,$K$2:$K$1001),"")</f>
-        <v>9</v>
+        <v>52</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9794,11 +9794,11 @@
       </c>
       <c r="K93" s="10" t="n">
         <f aca="true">IF($J93=1,RAND(),-1)</f>
-        <v>0.0217147068657158</v>
+        <v>0.905759625927511</v>
       </c>
       <c r="L93" s="10" t="n">
         <f aca="false">IF($J93=1,RANK($K93,$K$2:$K$1001),"")</f>
-        <v>219</v>
+        <v>26</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9835,11 +9835,11 @@
       </c>
       <c r="K94" s="10" t="n">
         <f aca="true">IF($J94=1,RAND(),-1)</f>
-        <v>0.95053965787774</v>
+        <v>0.358497303402479</v>
       </c>
       <c r="L94" s="10" t="n">
         <f aca="false">IF($J94=1,RANK($K94,$K$2:$K$1001),"")</f>
-        <v>14</v>
+        <v>154</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9876,11 +9876,11 @@
       </c>
       <c r="K95" s="10" t="n">
         <f aca="true">IF($J95=1,RAND(),-1)</f>
-        <v>0.917363552628988</v>
+        <v>0.934320432102909</v>
       </c>
       <c r="L95" s="10" t="n">
         <f aca="false">IF($J95=1,RANK($K95,$K$2:$K$1001),"")</f>
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9917,11 +9917,11 @@
       </c>
       <c r="K96" s="10" t="n">
         <f aca="true">IF($J96=1,RAND(),-1)</f>
-        <v>0.389912237009382</v>
+        <v>0.888631598846162</v>
       </c>
       <c r="L96" s="10" t="n">
         <f aca="false">IF($J96=1,RANK($K96,$K$2:$K$1001),"")</f>
-        <v>154</v>
+        <v>32</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9958,11 +9958,11 @@
       </c>
       <c r="K97" s="10" t="n">
         <f aca="true">IF($J97=1,RAND(),-1)</f>
-        <v>0.689682134722515</v>
+        <v>0.0317133351585759</v>
       </c>
       <c r="L97" s="10" t="n">
         <f aca="false">IF($J97=1,RANK($K97,$K$2:$K$1001),"")</f>
-        <v>76</v>
+        <v>220</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9999,11 +9999,11 @@
       </c>
       <c r="K98" s="10" t="n">
         <f aca="true">IF($J98=1,RAND(),-1)</f>
-        <v>0.831130677487203</v>
+        <v>0.28760844865551</v>
       </c>
       <c r="L98" s="10" t="n">
         <f aca="false">IF($J98=1,RANK($K98,$K$2:$K$1001),"")</f>
-        <v>43</v>
+        <v>170</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10040,11 +10040,11 @@
       </c>
       <c r="K99" s="10" t="n">
         <f aca="true">IF($J99=1,RAND(),-1)</f>
-        <v>0.0660374319659847</v>
+        <v>0.472075482254373</v>
       </c>
       <c r="L99" s="10" t="n">
         <f aca="false">IF($J99=1,RANK($K99,$K$2:$K$1001),"")</f>
-        <v>209</v>
+        <v>126</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10081,11 +10081,11 @@
       </c>
       <c r="K100" s="10" t="n">
         <f aca="true">IF($J100=1,RAND(),-1)</f>
-        <v>0.0852646292386087</v>
+        <v>0.338319001652816</v>
       </c>
       <c r="L100" s="10" t="n">
         <f aca="false">IF($J100=1,RANK($K100,$K$2:$K$1001),"")</f>
-        <v>203</v>
+        <v>160</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10122,11 +10122,11 @@
       </c>
       <c r="K101" s="10" t="n">
         <f aca="true">IF($J101=1,RAND(),-1)</f>
-        <v>0.487073852432185</v>
+        <v>0.762020224112932</v>
       </c>
       <c r="L101" s="10" t="n">
         <f aca="false">IF($J101=1,RANK($K101,$K$2:$K$1001),"")</f>
-        <v>128</v>
+        <v>61</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10163,11 +10163,11 @@
       </c>
       <c r="K102" s="10" t="n">
         <f aca="true">IF($J102=1,RAND(),-1)</f>
-        <v>0.523113156315361</v>
+        <v>0.288705400487277</v>
       </c>
       <c r="L102" s="10" t="n">
         <f aca="false">IF($J102=1,RANK($K102,$K$2:$K$1001),"")</f>
-        <v>119</v>
+        <v>168</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10204,11 +10204,11 @@
       </c>
       <c r="K103" s="10" t="n">
         <f aca="true">IF($J103=1,RAND(),-1)</f>
-        <v>0.398975668618823</v>
+        <v>0.0822147750307033</v>
       </c>
       <c r="L103" s="10" t="n">
         <f aca="false">IF($J103=1,RANK($K103,$K$2:$K$1001),"")</f>
-        <v>149</v>
+        <v>208</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10245,11 +10245,11 @@
       </c>
       <c r="K104" s="10" t="n">
         <f aca="true">IF($J104=1,RAND(),-1)</f>
-        <v>0.865670454141115</v>
+        <v>0.79739944687822</v>
       </c>
       <c r="L104" s="10" t="n">
         <f aca="false">IF($J104=1,RANK($K104,$K$2:$K$1001),"")</f>
-        <v>35</v>
+        <v>55</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10286,11 +10286,11 @@
       </c>
       <c r="K105" s="10" t="n">
         <f aca="true">IF($J105=1,RAND(),-1)</f>
-        <v>0.441089734654638</v>
+        <v>0.627628393023457</v>
       </c>
       <c r="L105" s="10" t="n">
         <f aca="false">IF($J105=1,RANK($K105,$K$2:$K$1001),"")</f>
-        <v>139</v>
+        <v>93</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10327,11 +10327,11 @@
       </c>
       <c r="K106" s="10" t="n">
         <f aca="true">IF($J106=1,RAND(),-1)</f>
-        <v>0.339393269518721</v>
+        <v>0.546193229951315</v>
       </c>
       <c r="L106" s="10" t="n">
         <f aca="false">IF($J106=1,RANK($K106,$K$2:$K$1001),"")</f>
-        <v>168</v>
+        <v>111</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10368,11 +10368,11 @@
       </c>
       <c r="K107" s="10" t="n">
         <f aca="true">IF($J107=1,RAND(),-1)</f>
-        <v>0.872819371076916</v>
+        <v>0.945795679582426</v>
       </c>
       <c r="L107" s="10" t="n">
         <f aca="false">IF($J107=1,RANK($K107,$K$2:$K$1001),"")</f>
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10409,11 +10409,11 @@
       </c>
       <c r="K108" s="10" t="n">
         <f aca="true">IF($J108=1,RAND(),-1)</f>
-        <v>0.207575512037134</v>
+        <v>0.837144964138006</v>
       </c>
       <c r="L108" s="10" t="n">
         <f aca="false">IF($J108=1,RANK($K108,$K$2:$K$1001),"")</f>
-        <v>184</v>
+        <v>43</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10450,11 +10450,11 @@
       </c>
       <c r="K109" s="10" t="n">
         <f aca="true">IF($J109=1,RAND(),-1)</f>
-        <v>0.991432036450121</v>
+        <v>0.715031320928351</v>
       </c>
       <c r="L109" s="10" t="n">
         <f aca="false">IF($J109=1,RANK($K109,$K$2:$K$1001),"")</f>
-        <v>3</v>
+        <v>74</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10491,11 +10491,11 @@
       </c>
       <c r="K110" s="10" t="n">
         <f aca="true">IF($J110=1,RAND(),-1)</f>
-        <v>0.524412915998203</v>
+        <v>0.252958954479738</v>
       </c>
       <c r="L110" s="10" t="n">
         <f aca="false">IF($J110=1,RANK($K110,$K$2:$K$1001),"")</f>
-        <v>118</v>
+        <v>177</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10532,11 +10532,11 @@
       </c>
       <c r="K111" s="10" t="n">
         <f aca="true">IF($J111=1,RAND(),-1)</f>
-        <v>0.0850888515376271</v>
+        <v>0.702308129490228</v>
       </c>
       <c r="L111" s="10" t="n">
         <f aca="false">IF($J111=1,RANK($K111,$K$2:$K$1001),"")</f>
-        <v>204</v>
+        <v>78</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10573,11 +10573,11 @@
       </c>
       <c r="K112" s="10" t="n">
         <f aca="true">IF($J112=1,RAND(),-1)</f>
-        <v>0.742410203039701</v>
+        <v>0.972773529451049</v>
       </c>
       <c r="L112" s="10" t="n">
         <f aca="false">IF($J112=1,RANK($K112,$K$2:$K$1001),"")</f>
-        <v>63</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10614,11 +10614,11 @@
       </c>
       <c r="K113" s="10" t="n">
         <f aca="true">IF($J113=1,RAND(),-1)</f>
-        <v>0.356513787659786</v>
+        <v>0.0219550478897127</v>
       </c>
       <c r="L113" s="10" t="n">
         <f aca="false">IF($J113=1,RANK($K113,$K$2:$K$1001),"")</f>
-        <v>163</v>
+        <v>222</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10655,11 +10655,11 @@
       </c>
       <c r="K114" s="10" t="n">
         <f aca="true">IF($J114=1,RAND(),-1)</f>
-        <v>0.56460702458579</v>
+        <v>0.769520820393269</v>
       </c>
       <c r="L114" s="10" t="n">
         <f aca="false">IF($J114=1,RANK($K114,$K$2:$K$1001),"")</f>
-        <v>109</v>
+        <v>60</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10696,11 +10696,11 @@
       </c>
       <c r="K115" s="10" t="n">
         <f aca="true">IF($J115=1,RAND(),-1)</f>
-        <v>0.25795498276222</v>
+        <v>0.531254748973906</v>
       </c>
       <c r="L115" s="10" t="n">
         <f aca="false">IF($J115=1,RANK($K115,$K$2:$K$1001),"")</f>
-        <v>177</v>
+        <v>115</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10737,11 +10737,11 @@
       </c>
       <c r="K116" s="10" t="n">
         <f aca="true">IF($J116=1,RAND(),-1)</f>
-        <v>0.980871507716432</v>
+        <v>0.033196114783662</v>
       </c>
       <c r="L116" s="10" t="n">
         <f aca="false">IF($J116=1,RANK($K116,$K$2:$K$1001),"")</f>
-        <v>7</v>
+        <v>219</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10778,11 +10778,11 @@
       </c>
       <c r="K117" s="10" t="n">
         <f aca="true">IF($J117=1,RAND(),-1)</f>
-        <v>0.649908140072581</v>
+        <v>0.676507200931158</v>
       </c>
       <c r="L117" s="10" t="n">
         <f aca="false">IF($J117=1,RANK($K117,$K$2:$K$1001),"")</f>
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10819,11 +10819,11 @@
       </c>
       <c r="K118" s="10" t="n">
         <f aca="true">IF($J118=1,RAND(),-1)</f>
-        <v>0.273734783751288</v>
+        <v>0.644483604385032</v>
       </c>
       <c r="L118" s="10" t="n">
         <f aca="false">IF($J118=1,RANK($K118,$K$2:$K$1001),"")</f>
-        <v>175</v>
+        <v>89</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10860,11 +10860,11 @@
       </c>
       <c r="K119" s="10" t="n">
         <f aca="true">IF($J119=1,RAND(),-1)</f>
-        <v>0.44813547878738</v>
+        <v>0.06795855857783</v>
       </c>
       <c r="L119" s="10" t="n">
         <f aca="false">IF($J119=1,RANK($K119,$K$2:$K$1001),"")</f>
-        <v>138</v>
+        <v>210</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10901,11 +10901,11 @@
       </c>
       <c r="K120" s="10" t="n">
         <f aca="true">IF($J120=1,RAND(),-1)</f>
-        <v>0.807092468777348</v>
+        <v>0.989397896281922</v>
       </c>
       <c r="L120" s="10" t="n">
         <f aca="false">IF($J120=1,RANK($K120,$K$2:$K$1001),"")</f>
-        <v>48</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10942,11 +10942,11 @@
       </c>
       <c r="K121" s="10" t="n">
         <f aca="true">IF($J121=1,RAND(),-1)</f>
-        <v>0.961099946571037</v>
+        <v>0.362057665929153</v>
       </c>
       <c r="L121" s="10" t="n">
         <f aca="false">IF($J121=1,RANK($K121,$K$2:$K$1001),"")</f>
-        <v>12</v>
+        <v>153</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10983,11 +10983,11 @@
       </c>
       <c r="K122" s="10" t="n">
         <f aca="true">IF($J122=1,RAND(),-1)</f>
-        <v>0.890291763623129</v>
+        <v>0.946830533187004</v>
       </c>
       <c r="L122" s="10" t="n">
         <f aca="false">IF($J122=1,RANK($K122,$K$2:$K$1001),"")</f>
-        <v>32</v>
+        <v>18</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11024,11 +11024,11 @@
       </c>
       <c r="K123" s="10" t="n">
         <f aca="true">IF($J123=1,RAND(),-1)</f>
-        <v>0.502892914956412</v>
+        <v>0.342227412206893</v>
       </c>
       <c r="L123" s="10" t="n">
         <f aca="false">IF($J123=1,RANK($K123,$K$2:$K$1001),"")</f>
-        <v>124</v>
+        <v>158</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11065,11 +11065,11 @@
       </c>
       <c r="K124" s="10" t="n">
         <f aca="true">IF($J124=1,RAND(),-1)</f>
-        <v>0.473795604502162</v>
+        <v>0.225860930875128</v>
       </c>
       <c r="L124" s="10" t="n">
         <f aca="false">IF($J124=1,RANK($K124,$K$2:$K$1001),"")</f>
-        <v>132</v>
+        <v>182</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11106,11 +11106,11 @@
       </c>
       <c r="K125" s="10" t="n">
         <f aca="true">IF($J125=1,RAND(),-1)</f>
-        <v>0.614325490559818</v>
+        <v>0.513383257943733</v>
       </c>
       <c r="L125" s="10" t="n">
         <f aca="false">IF($J125=1,RANK($K125,$K$2:$K$1001),"")</f>
-        <v>100</v>
+        <v>118</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11147,11 +11147,11 @@
       </c>
       <c r="K126" s="10" t="n">
         <f aca="true">IF($J126=1,RAND(),-1)</f>
-        <v>0.132776566736654</v>
+        <v>0.453193652870636</v>
       </c>
       <c r="L126" s="10" t="n">
         <f aca="false">IF($J126=1,RANK($K126,$K$2:$K$1001),"")</f>
-        <v>193</v>
+        <v>130</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11188,11 +11188,11 @@
       </c>
       <c r="K127" s="10" t="n">
         <f aca="true">IF($J127=1,RAND(),-1)</f>
-        <v>0.189051813034249</v>
+        <v>0.409946950232981</v>
       </c>
       <c r="L127" s="10" t="n">
         <f aca="false">IF($J127=1,RANK($K127,$K$2:$K$1001),"")</f>
-        <v>187</v>
+        <v>143</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11229,11 +11229,11 @@
       </c>
       <c r="K128" s="10" t="n">
         <f aca="true">IF($J128=1,RAND(),-1)</f>
-        <v>0.990516610950674</v>
+        <v>0.364862574556525</v>
       </c>
       <c r="L128" s="10" t="n">
         <f aca="false">IF($J128=1,RANK($K128,$K$2:$K$1001),"")</f>
-        <v>5</v>
+        <v>152</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11270,11 +11270,11 @@
       </c>
       <c r="K129" s="10" t="n">
         <f aca="true">IF($J129=1,RAND(),-1)</f>
-        <v>0.0417602720679885</v>
+        <v>0.681277636107591</v>
       </c>
       <c r="L129" s="10" t="n">
         <f aca="false">IF($J129=1,RANK($K129,$K$2:$K$1001),"")</f>
-        <v>215</v>
+        <v>82</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11311,11 +11311,11 @@
       </c>
       <c r="K130" s="10" t="n">
         <f aca="true">IF($J130=1,RAND(),-1)</f>
-        <v>0.944617560115091</v>
+        <v>0.0619886456919915</v>
       </c>
       <c r="L130" s="10" t="n">
         <f aca="false">IF($J130=1,RANK($K130,$K$2:$K$1001),"")</f>
-        <v>16</v>
+        <v>212</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11352,11 +11352,11 @@
       </c>
       <c r="K131" s="10" t="n">
         <f aca="true">IF($J131=1,RAND(),-1)</f>
-        <v>0.0934430859375336</v>
+        <v>0.594247697900076</v>
       </c>
       <c r="L131" s="10" t="n">
         <f aca="false">IF($J131=1,RANK($K131,$K$2:$K$1001),"")</f>
-        <v>202</v>
+        <v>102</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11393,11 +11393,11 @@
       </c>
       <c r="K132" s="10" t="n">
         <f aca="true">IF($J132=1,RAND(),-1)</f>
-        <v>0.36487123840181</v>
+        <v>0.195225623084306</v>
       </c>
       <c r="L132" s="10" t="n">
         <f aca="false">IF($J132=1,RANK($K132,$K$2:$K$1001),"")</f>
-        <v>158</v>
+        <v>188</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11434,11 +11434,11 @@
       </c>
       <c r="K133" s="10" t="n">
         <f aca="true">IF($J133=1,RAND(),-1)</f>
-        <v>0.422715133957519</v>
+        <v>0.704987817861447</v>
       </c>
       <c r="L133" s="10" t="n">
         <f aca="false">IF($J133=1,RANK($K133,$K$2:$K$1001),"")</f>
-        <v>141</v>
+        <v>77</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11475,11 +11475,11 @@
       </c>
       <c r="K134" s="10" t="n">
         <f aca="true">IF($J134=1,RAND(),-1)</f>
-        <v>0.920063759119961</v>
+        <v>0.305714296660201</v>
       </c>
       <c r="L134" s="10" t="n">
         <f aca="false">IF($J134=1,RANK($K134,$K$2:$K$1001),"")</f>
-        <v>22</v>
+        <v>166</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11516,11 +11516,11 @@
       </c>
       <c r="K135" s="10" t="n">
         <f aca="true">IF($J135=1,RAND(),-1)</f>
-        <v>0.722581957632156</v>
+        <v>0.42815538465626</v>
       </c>
       <c r="L135" s="10" t="n">
         <f aca="false">IF($J135=1,RANK($K135,$K$2:$K$1001),"")</f>
-        <v>69</v>
+        <v>137</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11557,11 +11557,11 @@
       </c>
       <c r="K136" s="10" t="n">
         <f aca="true">IF($J136=1,RAND(),-1)</f>
-        <v>0.138586607432746</v>
+        <v>0.709082790030487</v>
       </c>
       <c r="L136" s="10" t="n">
         <f aca="false">IF($J136=1,RANK($K136,$K$2:$K$1001),"")</f>
-        <v>191</v>
+        <v>76</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11598,11 +11598,11 @@
       </c>
       <c r="K137" s="10" t="n">
         <f aca="true">IF($J137=1,RAND(),-1)</f>
-        <v>0.99534086835143</v>
+        <v>0.414550121258611</v>
       </c>
       <c r="L137" s="10" t="n">
         <f aca="false">IF($J137=1,RANK($K137,$K$2:$K$1001),"")</f>
-        <v>2</v>
+        <v>141</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11639,11 +11639,11 @@
       </c>
       <c r="K138" s="10" t="n">
         <f aca="true">IF($J138=1,RAND(),-1)</f>
-        <v>0.370303945897586</v>
+        <v>0.173858022146357</v>
       </c>
       <c r="L138" s="10" t="n">
         <f aca="false">IF($J138=1,RANK($K138,$K$2:$K$1001),"")</f>
-        <v>157</v>
+        <v>192</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11680,11 +11680,11 @@
       </c>
       <c r="K139" s="10" t="n">
         <f aca="true">IF($J139=1,RAND(),-1)</f>
-        <v>0.0984495131342001</v>
+        <v>0.599760520611638</v>
       </c>
       <c r="L139" s="10" t="n">
         <f aca="false">IF($J139=1,RANK($K139,$K$2:$K$1001),"")</f>
-        <v>200</v>
+        <v>99</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11721,11 +11721,11 @@
       </c>
       <c r="K140" s="10" t="n">
         <f aca="true">IF($J140=1,RAND(),-1)</f>
-        <v>0.0557956354136671</v>
+        <v>0.413377285277045</v>
       </c>
       <c r="L140" s="10" t="n">
         <f aca="false">IF($J140=1,RANK($K140,$K$2:$K$1001),"")</f>
-        <v>211</v>
+        <v>142</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11762,11 +11762,11 @@
       </c>
       <c r="K141" s="10" t="n">
         <f aca="true">IF($J141=1,RAND(),-1)</f>
-        <v>0.461354220535493</v>
+        <v>0.139133874352596</v>
       </c>
       <c r="L141" s="10" t="n">
         <f aca="false">IF($J141=1,RANK($K141,$K$2:$K$1001),"")</f>
-        <v>136</v>
+        <v>198</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11803,11 +11803,11 @@
       </c>
       <c r="K142" s="10" t="n">
         <f aca="true">IF($J142=1,RAND(),-1)</f>
-        <v>0.484071403160236</v>
+        <v>0.608086185590007</v>
       </c>
       <c r="L142" s="10" t="n">
         <f aca="false">IF($J142=1,RANK($K142,$K$2:$K$1001),"")</f>
-        <v>129</v>
+        <v>96</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11844,11 +11844,11 @@
       </c>
       <c r="K143" s="10" t="n">
         <f aca="true">IF($J143=1,RAND(),-1)</f>
-        <v>0.633170212666792</v>
+        <v>0.160115914510948</v>
       </c>
       <c r="L143" s="10" t="n">
         <f aca="false">IF($J143=1,RANK($K143,$K$2:$K$1001),"")</f>
-        <v>94</v>
+        <v>193</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11885,11 +11885,11 @@
       </c>
       <c r="K144" s="10" t="n">
         <f aca="true">IF($J144=1,RAND(),-1)</f>
-        <v>0.0607323225352403</v>
+        <v>0.946953679266957</v>
       </c>
       <c r="L144" s="10" t="n">
         <f aca="false">IF($J144=1,RANK($K144,$K$2:$K$1001),"")</f>
-        <v>210</v>
+        <v>17</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11926,11 +11926,11 @@
       </c>
       <c r="K145" s="10" t="n">
         <f aca="true">IF($J145=1,RAND(),-1)</f>
-        <v>0.331463265924977</v>
+        <v>0.854942386004297</v>
       </c>
       <c r="L145" s="10" t="n">
         <f aca="false">IF($J145=1,RANK($K145,$K$2:$K$1001),"")</f>
-        <v>170</v>
+        <v>40</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11967,11 +11967,11 @@
       </c>
       <c r="K146" s="10" t="n">
         <f aca="true">IF($J146=1,RAND(),-1)</f>
-        <v>0.766131708988458</v>
+        <v>0.507205127115467</v>
       </c>
       <c r="L146" s="10" t="n">
         <f aca="false">IF($J146=1,RANK($K146,$K$2:$K$1001),"")</f>
-        <v>55</v>
+        <v>119</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12008,11 +12008,11 @@
       </c>
       <c r="K147" s="10" t="n">
         <f aca="true">IF($J147=1,RAND(),-1)</f>
-        <v>0.923754656698638</v>
+        <v>0.795670140648793</v>
       </c>
       <c r="L147" s="10" t="n">
         <f aca="false">IF($J147=1,RANK($K147,$K$2:$K$1001),"")</f>
-        <v>20</v>
+        <v>56</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12049,11 +12049,11 @@
       </c>
       <c r="K148" s="10" t="n">
         <f aca="true">IF($J148=1,RAND(),-1)</f>
-        <v>0.117085753106017</v>
+        <v>0.0149257459333267</v>
       </c>
       <c r="L148" s="10" t="n">
         <f aca="false">IF($J148=1,RANK($K148,$K$2:$K$1001),"")</f>
-        <v>197</v>
+        <v>224</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12090,11 +12090,11 @@
       </c>
       <c r="K149" s="10" t="n">
         <f aca="true">IF($J149=1,RAND(),-1)</f>
-        <v>0.0485224592751429</v>
+        <v>0.556788747325838</v>
       </c>
       <c r="L149" s="10" t="n">
         <f aca="false">IF($J149=1,RANK($K149,$K$2:$K$1001),"")</f>
-        <v>213</v>
+        <v>107</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12131,11 +12131,11 @@
       </c>
       <c r="K150" s="10" t="n">
         <f aca="true">IF($J150=1,RAND(),-1)</f>
-        <v>0.418194802597381</v>
+        <v>0.584127369565144</v>
       </c>
       <c r="L150" s="10" t="n">
         <f aca="false">IF($J150=1,RANK($K150,$K$2:$K$1001),"")</f>
-        <v>147</v>
+        <v>104</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12172,11 +12172,11 @@
       </c>
       <c r="K151" s="10" t="n">
         <f aca="true">IF($J151=1,RAND(),-1)</f>
-        <v>0.471259590968684</v>
+        <v>0.207853958156584</v>
       </c>
       <c r="L151" s="10" t="n">
         <f aca="false">IF($J151=1,RANK($K151,$K$2:$K$1001),"")</f>
-        <v>134</v>
+        <v>187</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12213,11 +12213,11 @@
       </c>
       <c r="K152" s="10" t="n">
         <f aca="true">IF($J152=1,RAND(),-1)</f>
-        <v>0.0185632209002587</v>
+        <v>0.725881988500393</v>
       </c>
       <c r="L152" s="10" t="n">
         <f aca="false">IF($J152=1,RANK($K152,$K$2:$K$1001),"")</f>
-        <v>222</v>
+        <v>69</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12254,11 +12254,11 @@
       </c>
       <c r="K153" s="10" t="n">
         <f aca="true">IF($J153=1,RAND(),-1)</f>
-        <v>0.626581178082474</v>
+        <v>0.531139959506004</v>
       </c>
       <c r="L153" s="10" t="n">
         <f aca="false">IF($J153=1,RANK($K153,$K$2:$K$1001),"")</f>
-        <v>97</v>
+        <v>116</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12295,11 +12295,11 @@
       </c>
       <c r="K154" s="10" t="n">
         <f aca="true">IF($J154=1,RAND(),-1)</f>
-        <v>0.421695775654918</v>
+        <v>0.827471955594048</v>
       </c>
       <c r="L154" s="10" t="n">
         <f aca="false">IF($J154=1,RANK($K154,$K$2:$K$1001),"")</f>
-        <v>145</v>
+        <v>46</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12336,11 +12336,11 @@
       </c>
       <c r="K155" s="10" t="n">
         <f aca="true">IF($J155=1,RAND(),-1)</f>
-        <v>0.61901900197766</v>
+        <v>0.0334957027072327</v>
       </c>
       <c r="L155" s="10" t="n">
         <f aca="false">IF($J155=1,RANK($K155,$K$2:$K$1001),"")</f>
-        <v>99</v>
+        <v>218</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12377,11 +12377,11 @@
       </c>
       <c r="K156" s="10" t="n">
         <f aca="true">IF($J156=1,RAND(),-1)</f>
-        <v>0.905166244863152</v>
+        <v>0.370516905554842</v>
       </c>
       <c r="L156" s="10" t="n">
         <f aca="false">IF($J156=1,RANK($K156,$K$2:$K$1001),"")</f>
-        <v>27</v>
+        <v>151</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12418,11 +12418,11 @@
       </c>
       <c r="K157" s="10" t="n">
         <f aca="true">IF($J157=1,RAND(),-1)</f>
-        <v>0.923665488845327</v>
+        <v>0.284768112790164</v>
       </c>
       <c r="L157" s="10" t="n">
         <f aca="false">IF($J157=1,RANK($K157,$K$2:$K$1001),"")</f>
-        <v>21</v>
+        <v>172</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12459,11 +12459,11 @@
       </c>
       <c r="K158" s="10" t="n">
         <f aca="true">IF($J158=1,RAND(),-1)</f>
-        <v>0.391734454779476</v>
+        <v>0.955810481614674</v>
       </c>
       <c r="L158" s="10" t="n">
         <f aca="false">IF($J158=1,RANK($K158,$K$2:$K$1001),"")</f>
-        <v>152</v>
+        <v>15</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12500,11 +12500,11 @@
       </c>
       <c r="K159" s="10" t="n">
         <f aca="true">IF($J159=1,RAND(),-1)</f>
-        <v>0.710553943631941</v>
+        <v>0.0456701680033478</v>
       </c>
       <c r="L159" s="10" t="n">
         <f aca="false">IF($J159=1,RANK($K159,$K$2:$K$1001),"")</f>
-        <v>73</v>
+        <v>216</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12541,11 +12541,11 @@
       </c>
       <c r="K160" s="10" t="n">
         <f aca="true">IF($J160=1,RAND(),-1)</f>
-        <v>0.671302428719376</v>
+        <v>0.629204407540554</v>
       </c>
       <c r="L160" s="10" t="n">
         <f aca="false">IF($J160=1,RANK($K160,$K$2:$K$1001),"")</f>
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12582,11 +12582,11 @@
       </c>
       <c r="K161" s="10" t="n">
         <f aca="true">IF($J161=1,RAND(),-1)</f>
-        <v>0.736248072522536</v>
+        <v>0.856450828399992</v>
       </c>
       <c r="L161" s="10" t="n">
         <f aca="false">IF($J161=1,RANK($K161,$K$2:$K$1001),"")</f>
-        <v>64</v>
+        <v>39</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12623,11 +12623,11 @@
       </c>
       <c r="K162" s="10" t="n">
         <f aca="true">IF($J162=1,RAND(),-1)</f>
-        <v>0.21375892412478</v>
+        <v>0.438693442436811</v>
       </c>
       <c r="L162" s="10" t="n">
         <f aca="false">IF($J162=1,RANK($K162,$K$2:$K$1001),"")</f>
-        <v>182</v>
+        <v>134</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12664,11 +12664,11 @@
       </c>
       <c r="K163" s="10" t="n">
         <f aca="true">IF($J163=1,RAND(),-1)</f>
-        <v>0.25615981300488</v>
+        <v>0.308617186434505</v>
       </c>
       <c r="L163" s="10" t="n">
         <f aca="false">IF($J163=1,RANK($K163,$K$2:$K$1001),"")</f>
-        <v>178</v>
+        <v>164</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12705,11 +12705,11 @@
       </c>
       <c r="K164" s="10" t="n">
         <f aca="true">IF($J164=1,RAND(),-1)</f>
-        <v>0.974930759890085</v>
+        <v>0.409173372759522</v>
       </c>
       <c r="L164" s="10" t="n">
         <f aca="false">IF($J164=1,RANK($K164,$K$2:$K$1001),"")</f>
-        <v>8</v>
+        <v>145</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12746,11 +12746,11 @@
       </c>
       <c r="K165" s="10" t="n">
         <f aca="true">IF($J165=1,RAND(),-1)</f>
-        <v>0.887248627315951</v>
+        <v>0.425076059490222</v>
       </c>
       <c r="L165" s="10" t="n">
         <f aca="false">IF($J165=1,RANK($K165,$K$2:$K$1001),"")</f>
-        <v>33</v>
+        <v>138</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12787,11 +12787,11 @@
       </c>
       <c r="K166" s="10" t="n">
         <f aca="true">IF($J166=1,RAND(),-1)</f>
-        <v>0.961919360936854</v>
+        <v>0.142481993413371</v>
       </c>
       <c r="L166" s="10" t="n">
         <f aca="false">IF($J166=1,RANK($K166,$K$2:$K$1001),"")</f>
-        <v>11</v>
+        <v>196</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12828,11 +12828,11 @@
       </c>
       <c r="K167" s="10" t="n">
         <f aca="true">IF($J167=1,RAND(),-1)</f>
-        <v>0.945835506678381</v>
+        <v>0.809073900619529</v>
       </c>
       <c r="L167" s="10" t="n">
         <f aca="false">IF($J167=1,RANK($K167,$K$2:$K$1001),"")</f>
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12869,11 +12869,11 @@
       </c>
       <c r="K168" s="10" t="n">
         <f aca="true">IF($J168=1,RAND(),-1)</f>
-        <v>0.161040133801992</v>
+        <v>0.889345502662645</v>
       </c>
       <c r="L168" s="10" t="n">
         <f aca="false">IF($J168=1,RANK($K168,$K$2:$K$1001),"")</f>
-        <v>188</v>
+        <v>31</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12910,11 +12910,11 @@
       </c>
       <c r="K169" s="10" t="n">
         <f aca="true">IF($J169=1,RAND(),-1)</f>
-        <v>0.567666663558743</v>
+        <v>0.711015826434592</v>
       </c>
       <c r="L169" s="10" t="n">
         <f aca="false">IF($J169=1,RANK($K169,$K$2:$K$1001),"")</f>
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12951,11 +12951,11 @@
       </c>
       <c r="K170" s="10" t="n">
         <f aca="true">IF($J170=1,RAND(),-1)</f>
-        <v>0.125322292683928</v>
+        <v>0.156995526430745</v>
       </c>
       <c r="L170" s="10" t="n">
         <f aca="false">IF($J170=1,RANK($K170,$K$2:$K$1001),"")</f>
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12992,11 +12992,11 @@
       </c>
       <c r="K171" s="10" t="n">
         <f aca="true">IF($J171=1,RAND(),-1)</f>
-        <v>0.216476261814549</v>
+        <v>0.253815659011041</v>
       </c>
       <c r="L171" s="10" t="n">
         <f aca="false">IF($J171=1,RANK($K171,$K$2:$K$1001),"")</f>
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13033,11 +13033,11 @@
       </c>
       <c r="K172" s="10" t="n">
         <f aca="true">IF($J172=1,RAND(),-1)</f>
-        <v>0.724641729150762</v>
+        <v>0.815473324896565</v>
       </c>
       <c r="L172" s="10" t="n">
         <f aca="false">IF($J172=1,RANK($K172,$K$2:$K$1001),"")</f>
-        <v>68</v>
+        <v>48</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13074,11 +13074,11 @@
       </c>
       <c r="K173" s="10" t="n">
         <f aca="true">IF($J173=1,RAND(),-1)</f>
-        <v>0.990782422996433</v>
+        <v>0.583366151364514</v>
       </c>
       <c r="L173" s="10" t="n">
         <f aca="false">IF($J173=1,RANK($K173,$K$2:$K$1001),"")</f>
-        <v>4</v>
+        <v>105</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13115,11 +13115,11 @@
       </c>
       <c r="K174" s="10" t="n">
         <f aca="true">IF($J174=1,RAND(),-1)</f>
-        <v>0.892522075380948</v>
+        <v>0.1912413735177</v>
       </c>
       <c r="L174" s="10" t="n">
         <f aca="false">IF($J174=1,RANK($K174,$K$2:$K$1001),"")</f>
-        <v>30</v>
+        <v>189</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13156,11 +13156,11 @@
       </c>
       <c r="K175" s="10" t="n">
         <f aca="true">IF($J175=1,RAND(),-1)</f>
-        <v>0.593642430533568</v>
+        <v>0.684954170374515</v>
       </c>
       <c r="L175" s="10" t="n">
         <f aca="false">IF($J175=1,RANK($K175,$K$2:$K$1001),"")</f>
-        <v>104</v>
+        <v>80</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13197,11 +13197,11 @@
       </c>
       <c r="K176" s="10" t="n">
         <f aca="true">IF($J176=1,RAND(),-1)</f>
-        <v>0.020061912389495</v>
+        <v>0.0746246862775301</v>
       </c>
       <c r="L176" s="10" t="n">
         <f aca="false">IF($J176=1,RANK($K176,$K$2:$K$1001),"")</f>
-        <v>220</v>
+        <v>209</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13238,11 +13238,11 @@
       </c>
       <c r="K177" s="10" t="n">
         <f aca="true">IF($J177=1,RAND(),-1)</f>
-        <v>0.358163586391755</v>
+        <v>0.480235755811466</v>
       </c>
       <c r="L177" s="10" t="n">
         <f aca="false">IF($J177=1,RANK($K177,$K$2:$K$1001),"")</f>
-        <v>161</v>
+        <v>123</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13279,11 +13279,11 @@
       </c>
       <c r="K178" s="10" t="n">
         <f aca="true">IF($J178=1,RAND(),-1)</f>
-        <v>0.986512682944112</v>
+        <v>0.999843865010908</v>
       </c>
       <c r="L178" s="10" t="n">
         <f aca="false">IF($J178=1,RANK($K178,$K$2:$K$1001),"")</f>
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13320,11 +13320,11 @@
       </c>
       <c r="K179" s="10" t="n">
         <f aca="true">IF($J179=1,RAND(),-1)</f>
-        <v>0.0953262143792325</v>
+        <v>0.850536387731825</v>
       </c>
       <c r="L179" s="10" t="n">
         <f aca="false">IF($J179=1,RANK($K179,$K$2:$K$1001),"")</f>
-        <v>201</v>
+        <v>41</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13361,11 +13361,11 @@
       </c>
       <c r="K180" s="10" t="n">
         <f aca="true">IF($J180=1,RAND(),-1)</f>
-        <v>0.672761349001386</v>
+        <v>0.955951225254102</v>
       </c>
       <c r="L180" s="10" t="n">
         <f aca="false">IF($J180=1,RANK($K180,$K$2:$K$1001),"")</f>
-        <v>84</v>
+        <v>14</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13402,11 +13402,11 @@
       </c>
       <c r="K181" s="10" t="n">
         <f aca="true">IF($J181=1,RAND(),-1)</f>
-        <v>0.671949756922808</v>
+        <v>0.543536864397052</v>
       </c>
       <c r="L181" s="10" t="n">
         <f aca="false">IF($J181=1,RANK($K181,$K$2:$K$1001),"")</f>
-        <v>85</v>
+        <v>113</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13443,11 +13443,11 @@
       </c>
       <c r="K182" s="10" t="n">
         <f aca="true">IF($J182=1,RAND(),-1)</f>
-        <v>0.558580494230847</v>
+        <v>0.107647081945333</v>
       </c>
       <c r="L182" s="10" t="n">
         <f aca="false">IF($J182=1,RANK($K182,$K$2:$K$1001),"")</f>
-        <v>111</v>
+        <v>202</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13484,11 +13484,11 @@
       </c>
       <c r="K183" s="10" t="n">
         <f aca="true">IF($J183=1,RAND(),-1)</f>
-        <v>0.687078293132016</v>
+        <v>0.990240404062735</v>
       </c>
       <c r="L183" s="10" t="n">
         <f aca="false">IF($J183=1,RANK($K183,$K$2:$K$1001),"")</f>
-        <v>78</v>
+        <v>3</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13525,11 +13525,11 @@
       </c>
       <c r="K184" s="10" t="n">
         <f aca="true">IF($J184=1,RAND(),-1)</f>
-        <v>0.654338467742136</v>
+        <v>0.540205458014351</v>
       </c>
       <c r="L184" s="10" t="n">
         <f aca="false">IF($J184=1,RANK($K184,$K$2:$K$1001),"")</f>
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13566,11 +13566,11 @@
       </c>
       <c r="K185" s="10" t="n">
         <f aca="true">IF($J185=1,RAND(),-1)</f>
-        <v>0.839344828047269</v>
+        <v>0.478333104792128</v>
       </c>
       <c r="L185" s="10" t="n">
         <f aca="false">IF($J185=1,RANK($K185,$K$2:$K$1001),"")</f>
-        <v>42</v>
+        <v>124</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13607,11 +13607,11 @@
       </c>
       <c r="K186" s="10" t="n">
         <f aca="true">IF($J186=1,RAND(),-1)</f>
-        <v>0.24285021774966</v>
+        <v>0.772540808789482</v>
       </c>
       <c r="L186" s="10" t="n">
         <f aca="false">IF($J186=1,RANK($K186,$K$2:$K$1001),"")</f>
-        <v>179</v>
+        <v>58</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13648,11 +13648,11 @@
       </c>
       <c r="K187" s="10" t="n">
         <f aca="true">IF($J187=1,RAND(),-1)</f>
-        <v>0.475878564922878</v>
+        <v>0.754624017696931</v>
       </c>
       <c r="L187" s="10" t="n">
         <f aca="false">IF($J187=1,RANK($K187,$K$2:$K$1001),"")</f>
-        <v>131</v>
+        <v>64</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13689,11 +13689,11 @@
       </c>
       <c r="K188" s="10" t="n">
         <f aca="true">IF($J188=1,RAND(),-1)</f>
-        <v>0.498869318639051</v>
+        <v>0.0971843450490324</v>
       </c>
       <c r="L188" s="10" t="n">
         <f aca="false">IF($J188=1,RANK($K188,$K$2:$K$1001),"")</f>
-        <v>126</v>
+        <v>205</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13730,11 +13730,11 @@
       </c>
       <c r="K189" s="10" t="n">
         <f aca="true">IF($J189=1,RAND(),-1)</f>
-        <v>0.479707014776962</v>
+        <v>0.668059191596061</v>
       </c>
       <c r="L189" s="10" t="n">
         <f aca="false">IF($J189=1,RANK($K189,$K$2:$K$1001),"")</f>
-        <v>130</v>
+        <v>84</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13771,11 +13771,11 @@
       </c>
       <c r="K190" s="10" t="n">
         <f aca="true">IF($J190=1,RAND(),-1)</f>
-        <v>0.857959418803281</v>
+        <v>0.0846206108643594</v>
       </c>
       <c r="L190" s="10" t="n">
         <f aca="false">IF($J190=1,RANK($K190,$K$2:$K$1001),"")</f>
-        <v>37</v>
+        <v>207</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13812,11 +13812,11 @@
       </c>
       <c r="K191" s="10" t="n">
         <f aca="true">IF($J191=1,RAND(),-1)</f>
-        <v>0.38523856562845</v>
+        <v>0.799602364550998</v>
       </c>
       <c r="L191" s="10" t="n">
         <f aca="false">IF($J191=1,RANK($K191,$K$2:$K$1001),"")</f>
-        <v>155</v>
+        <v>54</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13853,11 +13853,11 @@
       </c>
       <c r="K192" s="10" t="n">
         <f aca="true">IF($J192=1,RAND(),-1)</f>
-        <v>0.673762015603208</v>
+        <v>0.661569024291627</v>
       </c>
       <c r="L192" s="10" t="n">
         <f aca="false">IF($J192=1,RANK($K192,$K$2:$K$1001),"")</f>
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13894,11 +13894,11 @@
       </c>
       <c r="K193" s="10" t="n">
         <f aca="true">IF($J193=1,RAND(),-1)</f>
-        <v>0.825903854310135</v>
+        <v>0.545462984596294</v>
       </c>
       <c r="L193" s="10" t="n">
         <f aca="false">IF($J193=1,RANK($K193,$K$2:$K$1001),"")</f>
-        <v>45</v>
+        <v>112</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13935,11 +13935,11 @@
       </c>
       <c r="K194" s="10" t="n">
         <f aca="true">IF($J194=1,RAND(),-1)</f>
-        <v>0.380553393054452</v>
+        <v>0.859551219003739</v>
       </c>
       <c r="L194" s="10" t="n">
         <f aca="false">IF($J194=1,RANK($K194,$K$2:$K$1001),"")</f>
-        <v>156</v>
+        <v>38</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13976,11 +13976,11 @@
       </c>
       <c r="K195" s="10" t="n">
         <f aca="true">IF($J195=1,RAND(),-1)</f>
-        <v>0.915238532828926</v>
+        <v>0.451819318746158</v>
       </c>
       <c r="L195" s="10" t="n">
         <f aca="false">IF($J195=1,RANK($K195,$K$2:$K$1001),"")</f>
-        <v>25</v>
+        <v>131</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14017,11 +14017,11 @@
       </c>
       <c r="K196" s="10" t="n">
         <f aca="true">IF($J196=1,RAND(),-1)</f>
-        <v>0.841164801275629</v>
+        <v>0.723253180773055</v>
       </c>
       <c r="L196" s="10" t="n">
         <f aca="false">IF($J196=1,RANK($K196,$K$2:$K$1001),"")</f>
-        <v>41</v>
+        <v>70</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14058,11 +14058,11 @@
       </c>
       <c r="K197" s="10" t="n">
         <f aca="true">IF($J197=1,RAND(),-1)</f>
-        <v>0.679413891468517</v>
+        <v>0.759554048212421</v>
       </c>
       <c r="L197" s="10" t="n">
         <f aca="false">IF($J197=1,RANK($K197,$K$2:$K$1001),"")</f>
-        <v>81</v>
+        <v>62</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14099,11 +14099,11 @@
       </c>
       <c r="K198" s="10" t="n">
         <f aca="true">IF($J198=1,RAND(),-1)</f>
-        <v>0.5041037040628</v>
+        <v>0.771394662682491</v>
       </c>
       <c r="L198" s="10" t="n">
         <f aca="false">IF($J198=1,RANK($K198,$K$2:$K$1001),"")</f>
-        <v>123</v>
+        <v>59</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14140,11 +14140,11 @@
       </c>
       <c r="K199" s="10" t="n">
         <f aca="true">IF($J199=1,RAND(),-1)</f>
-        <v>0.538075995148389</v>
+        <v>0.594321518862726</v>
       </c>
       <c r="L199" s="10" t="n">
         <f aca="false">IF($J199=1,RANK($K199,$K$2:$K$1001),"")</f>
-        <v>114</v>
+        <v>101</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14181,11 +14181,11 @@
       </c>
       <c r="K200" s="10" t="n">
         <f aca="true">IF($J200=1,RAND(),-1)</f>
-        <v>0.631791190958596</v>
+        <v>0.969284391314685</v>
       </c>
       <c r="L200" s="10" t="n">
         <f aca="false">IF($J200=1,RANK($K200,$K$2:$K$1001),"")</f>
-        <v>95</v>
+        <v>12</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14222,11 +14222,11 @@
       </c>
       <c r="K201" s="10" t="n">
         <f aca="true">IF($J201=1,RAND(),-1)</f>
-        <v>0.810385985148248</v>
+        <v>0.392009302430543</v>
       </c>
       <c r="L201" s="10" t="n">
         <f aca="false">IF($J201=1,RANK($K201,$K$2:$K$1001),"")</f>
-        <v>46</v>
+        <v>150</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14263,11 +14263,11 @@
       </c>
       <c r="K202" s="10" t="n">
         <f aca="true">IF($J202=1,RAND(),-1)</f>
-        <v>0.729731798924547</v>
+        <v>0.230599097116318</v>
       </c>
       <c r="L202" s="10" t="n">
         <f aca="false">IF($J202=1,RANK($K202,$K$2:$K$1001),"")</f>
-        <v>65</v>
+        <v>180</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14304,11 +14304,11 @@
       </c>
       <c r="K203" s="10" t="n">
         <f aca="true">IF($J203=1,RAND(),-1)</f>
-        <v>0.586393070460748</v>
+        <v>0.551817468651813</v>
       </c>
       <c r="L203" s="10" t="n">
         <f aca="false">IF($J203=1,RANK($K203,$K$2:$K$1001),"")</f>
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14345,11 +14345,11 @@
       </c>
       <c r="K204" s="10" t="n">
         <f aca="true">IF($J204=1,RAND(),-1)</f>
-        <v>0.847150784444591</v>
+        <v>0.616636833816476</v>
       </c>
       <c r="L204" s="10" t="n">
         <f aca="false">IF($J204=1,RANK($K204,$K$2:$K$1001),"")</f>
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14386,11 +14386,11 @@
       </c>
       <c r="K205" s="10" t="n">
         <f aca="true">IF($J205=1,RAND(),-1)</f>
-        <v>0.583895041192</v>
+        <v>0.221645169077529</v>
       </c>
       <c r="L205" s="10" t="n">
         <f aca="false">IF($J205=1,RANK($K205,$K$2:$K$1001),"")</f>
-        <v>107</v>
+        <v>183</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14427,11 +14427,11 @@
       </c>
       <c r="K206" s="10" t="n">
         <f aca="true">IF($J206=1,RAND(),-1)</f>
-        <v>0.159803779011923</v>
+        <v>0.436602555837475</v>
       </c>
       <c r="L206" s="10" t="n">
         <f aca="false">IF($J206=1,RANK($K206,$K$2:$K$1001),"")</f>
-        <v>189</v>
+        <v>135</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14468,11 +14468,11 @@
       </c>
       <c r="K207" s="10" t="n">
         <f aca="true">IF($J207=1,RAND(),-1)</f>
-        <v>0.0304406665378357</v>
+        <v>0.409404439578388</v>
       </c>
       <c r="L207" s="10" t="n">
         <f aca="false">IF($J207=1,RANK($K207,$K$2:$K$1001),"")</f>
-        <v>217</v>
+        <v>144</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14509,11 +14509,11 @@
       </c>
       <c r="K208" s="10" t="n">
         <f aca="true">IF($J208=1,RAND(),-1)</f>
-        <v>0.798107771656446</v>
+        <v>0.553372963074263</v>
       </c>
       <c r="L208" s="10" t="n">
         <f aca="false">IF($J208=1,RANK($K208,$K$2:$K$1001),"")</f>
-        <v>50</v>
+        <v>109</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14550,11 +14550,11 @@
       </c>
       <c r="K209" s="10" t="n">
         <f aca="true">IF($J209=1,RAND(),-1)</f>
-        <v>0.510088145884903</v>
+        <v>0.0938525582405713</v>
       </c>
       <c r="L209" s="10" t="n">
         <f aca="false">IF($J209=1,RANK($K209,$K$2:$K$1001),"")</f>
-        <v>122</v>
+        <v>206</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14591,11 +14591,11 @@
       </c>
       <c r="K210" s="10" t="n">
         <f aca="true">IF($J210=1,RAND(),-1)</f>
-        <v>0.0817505043322784</v>
+        <v>0.0188874080283083</v>
       </c>
       <c r="L210" s="10" t="n">
         <f aca="false">IF($J210=1,RANK($K210,$K$2:$K$1001),"")</f>
-        <v>207</v>
+        <v>223</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14632,11 +14632,11 @@
       </c>
       <c r="K211" s="10" t="n">
         <f aca="true">IF($J211=1,RAND(),-1)</f>
-        <v>0.628437552457917</v>
+        <v>0.287458515572727</v>
       </c>
       <c r="L211" s="10" t="n">
         <f aca="false">IF($J211=1,RANK($K211,$K$2:$K$1001),"")</f>
-        <v>96</v>
+        <v>171</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14673,11 +14673,11 @@
       </c>
       <c r="K212" s="10" t="n">
         <f aca="true">IF($J212=1,RAND(),-1)</f>
-        <v>0.00780384973492043</v>
+        <v>0.648622441677736</v>
       </c>
       <c r="L212" s="10" t="n">
         <f aca="false">IF($J212=1,RANK($K212,$K$2:$K$1001),"")</f>
-        <v>224</v>
+        <v>88</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14714,11 +14714,11 @@
       </c>
       <c r="K213" s="10" t="n">
         <f aca="true">IF($J213=1,RAND(),-1)</f>
-        <v>0.600274458994674</v>
+        <v>0.911125238480754</v>
       </c>
       <c r="L213" s="10" t="n">
         <f aca="false">IF($J213=1,RANK($K213,$K$2:$K$1001),"")</f>
-        <v>103</v>
+        <v>24</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14755,11 +14755,11 @@
       </c>
       <c r="K214" s="10" t="n">
         <f aca="true">IF($J214=1,RAND(),-1)</f>
-        <v>0.286918280990554</v>
+        <v>0.585189525589817</v>
       </c>
       <c r="L214" s="10" t="n">
         <f aca="false">IF($J214=1,RANK($K214,$K$2:$K$1001),"")</f>
-        <v>172</v>
+        <v>103</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14796,11 +14796,11 @@
       </c>
       <c r="K215" s="10" t="n">
         <f aca="true">IF($J215=1,RAND(),-1)</f>
-        <v>0.341295666633272</v>
+        <v>0.897442643385108</v>
       </c>
       <c r="L215" s="10" t="n">
         <f aca="false">IF($J215=1,RANK($K215,$K$2:$K$1001),"")</f>
-        <v>166</v>
+        <v>29</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14837,11 +14837,11 @@
       </c>
       <c r="K216" s="10" t="n">
         <f aca="true">IF($J216=1,RAND(),-1)</f>
-        <v>0.826126084088441</v>
+        <v>0.953672062320115</v>
       </c>
       <c r="L216" s="10" t="n">
         <f aca="false">IF($J216=1,RANK($K216,$K$2:$K$1001),"")</f>
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14878,11 +14878,11 @@
       </c>
       <c r="K217" s="10" t="n">
         <f aca="true">IF($J217=1,RAND(),-1)</f>
-        <v>0.029975714800847</v>
+        <v>0.808199142711801</v>
       </c>
       <c r="L217" s="10" t="n">
         <f aca="false">IF($J217=1,RANK($K217,$K$2:$K$1001),"")</f>
-        <v>218</v>
+        <v>51</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14919,11 +14919,11 @@
       </c>
       <c r="K218" s="10" t="n">
         <f aca="true">IF($J218=1,RAND(),-1)</f>
-        <v>0.362536756039723</v>
+        <v>0.97243505976961</v>
       </c>
       <c r="L218" s="10" t="n">
         <f aca="false">IF($J218=1,RANK($K218,$K$2:$K$1001),"")</f>
-        <v>159</v>
+        <v>11</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14960,11 +14960,11 @@
       </c>
       <c r="K219" s="10" t="n">
         <f aca="true">IF($J219=1,RAND(),-1)</f>
-        <v>0.858819405198279</v>
+        <v>0.940287769370756</v>
       </c>
       <c r="L219" s="10" t="n">
         <f aca="false">IF($J219=1,RANK($K219,$K$2:$K$1001),"")</f>
-        <v>36</v>
+        <v>22</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15001,11 +15001,11 @@
       </c>
       <c r="K220" s="10" t="n">
         <f aca="true">IF($J220=1,RAND(),-1)</f>
-        <v>0.280384066838397</v>
+        <v>0.722589008446227</v>
       </c>
       <c r="L220" s="10" t="n">
         <f aca="false">IF($J220=1,RANK($K220,$K$2:$K$1001),"")</f>
-        <v>173</v>
+        <v>72</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15042,11 +15042,11 @@
       </c>
       <c r="K221" s="10" t="n">
         <f aca="true">IF($J221=1,RAND(),-1)</f>
-        <v>0.942793976686422</v>
+        <v>0.415910863311862</v>
       </c>
       <c r="L221" s="10" t="n">
         <f aca="false">IF($J221=1,RANK($K221,$K$2:$K$1001),"")</f>
-        <v>17</v>
+        <v>140</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15083,11 +15083,11 @@
       </c>
       <c r="K222" s="10" t="n">
         <f aca="true">IF($J222=1,RAND(),-1)</f>
-        <v>0.534422073182594</v>
+        <v>0.407499094885848</v>
       </c>
       <c r="L222" s="10" t="n">
         <f aca="false">IF($J222=1,RANK($K222,$K$2:$K$1001),"")</f>
-        <v>116</v>
+        <v>146</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15124,11 +15124,11 @@
       </c>
       <c r="K223" s="10" t="n">
         <f aca="true">IF($J223=1,RAND(),-1)</f>
-        <v>0.100801664025524</v>
+        <v>0.128567689401755</v>
       </c>
       <c r="L223" s="10" t="n">
         <f aca="false">IF($J223=1,RANK($K223,$K$2:$K$1001),"")</f>
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15165,11 +15165,11 @@
       </c>
       <c r="K224" s="10" t="n">
         <f aca="true">IF($J224=1,RAND(),-1)</f>
-        <v>0.844421590999132</v>
+        <v>0.942269419807299</v>
       </c>
       <c r="L224" s="10" t="n">
         <f aca="false">IF($J224=1,RANK($K224,$K$2:$K$1001),"")</f>
-        <v>39</v>
+        <v>20</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15206,11 +15206,11 @@
       </c>
       <c r="K225" s="10" t="n">
         <f aca="true">IF($J225=1,RAND(),-1)</f>
-        <v>0.973023993318143</v>
+        <v>0.894257278763792</v>
       </c>
       <c r="L225" s="10" t="n">
         <f aca="false">IF($J225=1,RANK($K225,$K$2:$K$1001),"")</f>
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26129,7 +26129,7 @@
       </c>
       <c r="C4" s="12" t="str">
         <f aca="false">IF(B4="","",INDEX(Test!$C12:$F12,MATCH(B4,{"A","B","C","D"},0)))</f>
-        <v>4²</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26139,11 +26139,11 @@
       </c>
       <c r="B5" s="5" t="str">
         <f aca="false">IF(Test!$J13="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J13))</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="C5" s="12" t="str">
         <f aca="false">IF(B5="","",INDEX(Test!$C13:$F13,MATCH(B5,{"A","B","C","D"},0)))</f>
-        <v>27</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26157,7 +26157,7 @@
       </c>
       <c r="C6" s="12" t="str">
         <f aca="false">IF(B6="","",INDEX(Test!$C14:$F14,MATCH(B6,{"A","B","C","D"},0)))</f>
-        <v>216</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26167,11 +26167,11 @@
       </c>
       <c r="B7" s="5" t="str">
         <f aca="false">IF(Test!$J15="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J15))</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="C7" s="12" t="str">
         <f aca="false">IF(B7="","",INDEX(Test!$C15:$F15,MATCH(B7,{"A","B","C","D"},0)))</f>
-        <v>Kare</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26181,11 +26181,11 @@
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">IF(Test!$J16="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J16))</f>
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="C8" s="12" t="str">
         <f aca="false">IF(B8="","",INDEX(Test!$C16:$F16,MATCH(B8,{"A","B","C","D"},0)))</f>
-        <v>10</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26195,11 +26195,11 @@
       </c>
       <c r="B9" s="5" t="str">
         <f aca="false">IF(Test!$J17="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J17))</f>
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="C9" s="12" t="str">
         <f aca="false">IF(B9="","",INDEX(Test!$C17:$F17,MATCH(B9,{"A","B","C","D"},0)))</f>
-        <v>24</v>
+        <v>10²</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26213,7 +26213,7 @@
       </c>
       <c r="C10" s="12" t="str">
         <f aca="false">IF(B10="","",INDEX(Test!$C18:$F18,MATCH(B10,{"A","B","C","D"},0)))</f>
-        <v>125</v>
+        <v>6 · 6 · 6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26223,11 +26223,11 @@
       </c>
       <c r="B11" s="5" t="str">
         <f aca="false">IF(Test!$J19="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J19))</f>
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="C11" s="12" t="str">
         <f aca="false">IF(B11="","",INDEX(Test!$C19:$F19,MATCH(B11,{"A","B","C","D"},0)))</f>
-        <v>64 L</v>
+        <v>9²</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26241,7 +26241,7 @@
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF(B12="","",INDEX(Test!$C20:$F20,MATCH(B12,{"A","B","C","D"},0)))</f>
-        <v>4</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26251,11 +26251,11 @@
       </c>
       <c r="B13" s="5" t="str">
         <f aca="false">IF(Test!$J21="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J21))</f>
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF(B13="","",INDEX(Test!$C21:$F21,MATCH(B13,{"A","B","C","D"},0)))</f>
-        <v>8</v>
+        <v>729</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
6. sınıf eğitim seti: İngilizce, Matematik, Fen, Sosyal, Din Kültürü
- İngilizce: 10 ünitelik 631 soruluk havuz (kelime, dilbilgisi, diyalog,
  okuma, sesli dinleme) ve aralıklı tekrarlı Kelime Kartları uygulaması
- Matematik (296), Fen (136), Sosyal (84), Din Kültürü (63) soru havuzları
- Ana sayfa (Sinif6/index.html): tüm dersler ve İngilizce çalışma programı
- Ortak şablon: soru türü filtresi, sesli dinleme düğmesi, kontrol sonrası
  açıklama; ortak havuz yardımcıları ve tümünü yeniden üretme betiği

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6qBE8e6Wkv628t1Q47HQM
</commit_message>
<xml_diff>
--- a/KupSorulari/KupSoruHavuzu.xlsx
+++ b/KupSorulari/KupSoruHavuzu.xlsx
@@ -2144,23 +2144,23 @@
       </c>
       <c r="B12" s="11" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J12))</f>
-        <v>Bir ayrıtı 2 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
+        <v>Bir ayrıtı 8 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J12))</f>
-        <v>16</v>
+        <v>96</v>
       </c>
       <c r="D12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J12))</f>
-        <v>24</v>
+        <v>512</v>
       </c>
       <c r="E12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J12))</f>
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="F12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J12))</f>
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="G12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J12))</f>
@@ -2172,45 +2172,45 @@
       </c>
       <c r="J12" s="10" t="n">
         <f aca="false">IF(1&lt;=MIN($B$3,$B$6),MATCH(1,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>177</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
         <f aca="false">IF($J13="","",2)</f>
         <v>2</v>
       </c>
       <c r="B13" s="11" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J13))</f>
-        <v>7³ ifadesinin değeri kaçtır?</v>
+        <v>Bir ayrıtı 3 birim olan küp, birim küplerden oluşturuluyor ve dış yüzeyinin tamamı boyanıyor. Hiç boyanmamış kaç birim küp vardır?</v>
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J13))</f>
-        <v>343</v>
+        <v>6</v>
       </c>
       <c r="D13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J13))</f>
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J13))</f>
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J13))</f>
-        <v>350</v>
+        <v>1</v>
       </c>
       <c r="G13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J13))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Özellikleri</v>
       </c>
       <c r="H13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J13))</f>
-        <v>Kolay</v>
+        <v>Zor</v>
       </c>
       <c r="J13" s="10" t="n">
         <f aca="false">IF(2&lt;=MIN($B$3,$B$6),MATCH(2,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>7</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2220,23 +2220,23 @@
       </c>
       <c r="B14" s="11" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J14))</f>
-        <v>Bir ayrıtı 7 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
+        <v>Bir yüzünün alanı 49 cm² olan küpün bir ayrıtı kaç cm'dir?</v>
       </c>
       <c r="C14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J14))</f>
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="D14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J14))</f>
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="E14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J14))</f>
-        <v>84</v>
+        <v>8</v>
       </c>
       <c r="F14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J14))</f>
-        <v>343</v>
+        <v>24</v>
       </c>
       <c r="G14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J14))</f>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">IF(3&lt;=MIN($B$3,$B$6),MATCH(3,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>182</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2258,73 +2258,73 @@
       </c>
       <c r="B15" s="11" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J15))</f>
-        <v>Hacmi 8 cm³ olan küpün bir ayrıtı kaç cm'dir?</v>
+        <v>5³ ifadesinin değeri kaçtır?</v>
       </c>
       <c r="C15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J15))</f>
-        <v>2</v>
+        <v>130</v>
       </c>
       <c r="D15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J15))</f>
-        <v>3</v>
+        <v>125</v>
       </c>
       <c r="E15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J15))</f>
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="F15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J15))</f>
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J15))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J15))</f>
-        <v>Orta</v>
+        <v>Kolay</v>
       </c>
       <c r="J15" s="10" t="n">
         <f aca="false">IF(4&lt;=MIN($B$3,$B$6),MATCH(4,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>119</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="n">
         <f aca="false">IF($J16="","",5)</f>
         <v>5</v>
       </c>
       <c r="B16" s="11" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J16))</f>
-        <v>(2 + 2)³ ifadesinin değeri kaçtır?</v>
+        <v>Küpün bir köşesinde kaç ayrıt birleşir?</v>
       </c>
       <c r="C16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J16))</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J16))</f>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J16))</f>
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J16))</f>
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="G16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J16))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Özellikleri</v>
       </c>
       <c r="H16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J16))</f>
-        <v>Zor</v>
+        <v>Kolay</v>
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">IF(5&lt;=MIN($B$3,$B$6),MATCH(5,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>84</v>
+        <v>173</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2334,61 +2334,61 @@
       </c>
       <c r="B17" s="11" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J17))</f>
-        <v>Aşağıdakilerden hangisinin değeri en büyüktür?</v>
+        <v>Bir ayrıtı 3 dm olan küp şeklindeki boş akvaryum tamamen doldurulursa kaç litre su alır? (1 dm³ = 1 L)</v>
       </c>
       <c r="C17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J17))</f>
-        <v>6²</v>
+        <v>9 L</v>
       </c>
       <c r="D17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J17))</f>
-        <v>7²</v>
+        <v>28 L</v>
       </c>
       <c r="E17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J17))</f>
-        <v>3²</v>
+        <v>27 L</v>
       </c>
       <c r="F17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J17))</f>
-        <v>10²</v>
+        <v>54 L</v>
       </c>
       <c r="G17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J17))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J17))</f>
-        <v>Orta</v>
+        <v>Zor</v>
       </c>
       <c r="J17" s="10" t="n">
         <f aca="false">IF(6&lt;=MIN($B$3,$B$6),MATCH(6,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="n">
         <f aca="false">IF($J18="","",7)</f>
         <v>7</v>
       </c>
       <c r="B18" s="11" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J18))</f>
-        <v>6³ ifadesinin anlamı aşağıdakilerden hangisidir?</v>
+        <v>2³ + 5² işleminin sonucu kaçtır?</v>
       </c>
       <c r="C18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J18))</f>
-        <v>6 · 3</v>
+        <v>16</v>
       </c>
       <c r="D18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J18))</f>
-        <v>6 + 6 + 6</v>
+        <v>33</v>
       </c>
       <c r="E18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J18))</f>
-        <v>6 · 6 · 6</v>
+        <v>29</v>
       </c>
       <c r="F18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J18))</f>
-        <v>3 · 3 · 3 · 3 · 3 · 3</v>
+        <v>18</v>
       </c>
       <c r="G18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J18))</f>
@@ -2396,11 +2396,11 @@
       </c>
       <c r="H18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J18))</f>
-        <v>Kolay</v>
+        <v>Orta</v>
       </c>
       <c r="J18" s="10" t="n">
         <f aca="false">IF(7&lt;=MIN($B$3,$B$6),MATCH(7,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2410,23 +2410,23 @@
       </c>
       <c r="B19" s="11" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J19))</f>
-        <v>Aşağıdakilerden hangisinin değeri en büyüktür?</v>
+        <v>3³ ifadesinin değeri kaçtır?</v>
       </c>
       <c r="C19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J19))</f>
-        <v>5²</v>
+        <v>9</v>
       </c>
       <c r="D19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J19))</f>
-        <v>3²</v>
+        <v>30</v>
       </c>
       <c r="E19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J19))</f>
-        <v>7²</v>
+        <v>6</v>
       </c>
       <c r="F19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J19))</f>
-        <v>9²</v>
+        <v>27</v>
       </c>
       <c r="G19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J19))</f>
@@ -2434,41 +2434,41 @@
       </c>
       <c r="H19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J19))</f>
-        <v>Orta</v>
+        <v>Kolay</v>
       </c>
       <c r="J19" s="10" t="n">
         <f aca="false">IF(8&lt;=MIN($B$3,$B$6),MATCH(8,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="n">
         <f aca="false">IF($J20="","",9)</f>
         <v>9</v>
       </c>
       <c r="B20" s="11" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J20))</f>
-        <v>Aşağıdakilerden hangisi bir doğal sayının küpü değildir?</v>
+        <v>Bir ayrıtı 7 cm olan küpün yüzey alanı kaç cm²'dir?</v>
       </c>
       <c r="C20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J20))</f>
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J20))</f>
-        <v>27</v>
+        <v>294</v>
       </c>
       <c r="E20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J20))</f>
-        <v>512</v>
+        <v>343</v>
       </c>
       <c r="F20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J20))</f>
-        <v>8</v>
+        <v>196</v>
       </c>
       <c r="G20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J20))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Özellikleri</v>
       </c>
       <c r="H20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J20))</f>
@@ -2476,37 +2476,37 @@
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">IF(9&lt;=MIN($B$3,$B$6),MATCH(9,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="n">
         <f aca="false">IF($J21="","",10)</f>
         <v>10</v>
       </c>
       <c r="B21" s="11" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J21))</f>
-        <v>Bir ayrıtı 9 cm olan küpün hacmi kaç cm³'tür?</v>
+        <v>10³ ifadesinin değeri kaçtır?</v>
       </c>
       <c r="C21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J21))</f>
-        <v>27</v>
+        <v>1000</v>
       </c>
       <c r="D21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J21))</f>
-        <v>486</v>
+        <v>100</v>
       </c>
       <c r="E21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J21))</f>
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="F21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J21))</f>
-        <v>729</v>
+        <v>1010</v>
       </c>
       <c r="G21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J21))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J21))</f>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="J21" s="10" t="n">
         <f aca="false">IF(10&lt;=MIN($B$3,$B$6),MATCH(10,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>111</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6063,11 +6063,11 @@
       </c>
       <c r="K2" s="10" t="n">
         <f aca="true">IF($J2=1,RAND(),-1)</f>
-        <v>0.0411754098130525</v>
+        <v>0.401790495328625</v>
       </c>
       <c r="L2" s="10" t="n">
         <f aca="false">IF($J2=1,RANK($K2,$K$2:$K$1001),"")</f>
-        <v>217</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6104,11 +6104,11 @@
       </c>
       <c r="K3" s="10" t="n">
         <f aca="true">IF($J3=1,RAND(),-1)</f>
-        <v>0.449411186215152</v>
+        <v>0.270641339505107</v>
       </c>
       <c r="L3" s="10" t="n">
         <f aca="false">IF($J3=1,RANK($K3,$K$2:$K$1001),"")</f>
-        <v>132</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6145,11 +6145,11 @@
       </c>
       <c r="K4" s="10" t="n">
         <f aca="true">IF($J4=1,RAND(),-1)</f>
-        <v>0.601096491243837</v>
+        <v>0.965586382232213</v>
       </c>
       <c r="L4" s="10" t="n">
         <f aca="false">IF($J4=1,RANK($K4,$K$2:$K$1001),"")</f>
-        <v>98</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6186,11 +6186,11 @@
       </c>
       <c r="K5" s="10" t="n">
         <f aca="true">IF($J5=1,RAND(),-1)</f>
-        <v>0.830308326299626</v>
+        <v>0.195813075787506</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">IF($J5=1,RANK($K5,$K$2:$K$1001),"")</f>
-        <v>44</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6227,11 +6227,11 @@
       </c>
       <c r="K6" s="10" t="n">
         <f aca="true">IF($J6=1,RAND(),-1)</f>
-        <v>0.868923679808951</v>
+        <v>0.982684786987049</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">IF($J6=1,RANK($K6,$K$2:$K$1001),"")</f>
-        <v>35</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6268,11 +6268,11 @@
       </c>
       <c r="K7" s="10" t="n">
         <f aca="true">IF($J7=1,RAND(),-1)</f>
-        <v>0.0283675435125936</v>
+        <v>0.17632037147737</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">IF($J7=1,RANK($K7,$K$2:$K$1001),"")</f>
-        <v>221</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6309,11 +6309,11 @@
       </c>
       <c r="K8" s="10" t="n">
         <f aca="true">IF($J8=1,RAND(),-1)</f>
-        <v>0.999634046901793</v>
+        <v>0.452620305531729</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">IF($J8=1,RANK($K8,$K$2:$K$1001),"")</f>
-        <v>2</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6350,11 +6350,11 @@
       </c>
       <c r="K9" s="10" t="n">
         <f aca="true">IF($J9=1,RAND(),-1)</f>
-        <v>0.353863187978133</v>
+        <v>0.12334482841132</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">IF($J9=1,RANK($K9,$K$2:$K$1001),"")</f>
-        <v>155</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6391,11 +6391,11 @@
       </c>
       <c r="K10" s="10" t="n">
         <f aca="true">IF($J10=1,RAND(),-1)</f>
-        <v>0.941179663664032</v>
+        <v>0.76662941253123</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">IF($J10=1,RANK($K10,$K$2:$K$1001),"")</f>
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6432,11 +6432,11 @@
       </c>
       <c r="K11" s="10" t="n">
         <f aca="true">IF($J11=1,RAND(),-1)</f>
-        <v>0.316302629889705</v>
+        <v>0.948054806682241</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">IF($J11=1,RANK($K11,$K$2:$K$1001),"")</f>
-        <v>163</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6473,11 +6473,11 @@
       </c>
       <c r="K12" s="10" t="n">
         <f aca="true">IF($J12=1,RAND(),-1)</f>
-        <v>0.146854722041688</v>
+        <v>0.621598539142692</v>
       </c>
       <c r="L12" s="10" t="n">
         <f aca="false">IF($J12=1,RANK($K12,$K$2:$K$1001),"")</f>
-        <v>195</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6514,11 +6514,11 @@
       </c>
       <c r="K13" s="10" t="n">
         <f aca="true">IF($J13=1,RAND(),-1)</f>
-        <v>0.31813579023357</v>
+        <v>0.458327904043481</v>
       </c>
       <c r="L13" s="10" t="n">
         <f aca="false">IF($J13=1,RANK($K13,$K$2:$K$1001),"")</f>
-        <v>162</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6555,11 +6555,11 @@
       </c>
       <c r="K14" s="10" t="n">
         <f aca="true">IF($J14=1,RAND(),-1)</f>
-        <v>0.396125657932773</v>
+        <v>0.44691130729089</v>
       </c>
       <c r="L14" s="10" t="n">
         <f aca="false">IF($J14=1,RANK($K14,$K$2:$K$1001),"")</f>
-        <v>149</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6596,11 +6596,11 @@
       </c>
       <c r="K15" s="10" t="n">
         <f aca="true">IF($J15=1,RAND(),-1)</f>
-        <v>0.35035549198795</v>
+        <v>0.648730499163885</v>
       </c>
       <c r="L15" s="10" t="n">
         <f aca="false">IF($J15=1,RANK($K15,$K$2:$K$1001),"")</f>
-        <v>156</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6637,11 +6637,11 @@
       </c>
       <c r="K16" s="10" t="n">
         <f aca="true">IF($J16=1,RAND(),-1)</f>
-        <v>0.220307498844939</v>
+        <v>0.338123648188616</v>
       </c>
       <c r="L16" s="10" t="n">
         <f aca="false">IF($J16=1,RANK($K16,$K$2:$K$1001),"")</f>
-        <v>184</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6678,11 +6678,11 @@
       </c>
       <c r="K17" s="10" t="n">
         <f aca="true">IF($J17=1,RAND(),-1)</f>
-        <v>0.792532760650073</v>
+        <v>0.573864548316189</v>
       </c>
       <c r="L17" s="10" t="n">
         <f aca="false">IF($J17=1,RANK($K17,$K$2:$K$1001),"")</f>
-        <v>57</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6719,11 +6719,11 @@
       </c>
       <c r="K18" s="10" t="n">
         <f aca="true">IF($J18=1,RAND(),-1)</f>
-        <v>0.742026833599792</v>
+        <v>0.0601356146533304</v>
       </c>
       <c r="L18" s="10" t="n">
         <f aca="false">IF($J18=1,RANK($K18,$K$2:$K$1001),"")</f>
-        <v>67</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="K19" s="10" t="n">
         <f aca="true">IF($J19=1,RAND(),-1)</f>
-        <v>0.0545691977933067</v>
+        <v>0.904336703453878</v>
       </c>
       <c r="L19" s="10" t="n">
         <f aca="false">IF($J19=1,RANK($K19,$K$2:$K$1001),"")</f>
-        <v>213</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6801,11 +6801,11 @@
       </c>
       <c r="K20" s="10" t="n">
         <f aca="true">IF($J20=1,RAND(),-1)</f>
-        <v>0.606779866493235</v>
+        <v>0.216423731909305</v>
       </c>
       <c r="L20" s="10" t="n">
         <f aca="false">IF($J20=1,RANK($K20,$K$2:$K$1001),"")</f>
-        <v>97</v>
+        <v>180</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6842,11 +6842,11 @@
       </c>
       <c r="K21" s="10" t="n">
         <f aca="true">IF($J21=1,RAND(),-1)</f>
-        <v>0.758069521944036</v>
+        <v>0.734845784900409</v>
       </c>
       <c r="L21" s="10" t="n">
         <f aca="false">IF($J21=1,RANK($K21,$K$2:$K$1001),"")</f>
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="K22" s="10" t="n">
         <f aca="true">IF($J22=1,RAND(),-1)</f>
-        <v>0.097479103659455</v>
+        <v>0.466798374005103</v>
       </c>
       <c r="L22" s="10" t="n">
         <f aca="false">IF($J22=1,RANK($K22,$K$2:$K$1001),"")</f>
-        <v>204</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6924,11 +6924,11 @@
       </c>
       <c r="K23" s="10" t="n">
         <f aca="true">IF($J23=1,RAND(),-1)</f>
-        <v>0.621714421198653</v>
+        <v>0.8615541962897</v>
       </c>
       <c r="L23" s="10" t="n">
         <f aca="false">IF($J23=1,RANK($K23,$K$2:$K$1001),"")</f>
-        <v>94</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6965,11 +6965,11 @@
       </c>
       <c r="K24" s="10" t="n">
         <f aca="true">IF($J24=1,RAND(),-1)</f>
-        <v>0.981790367842763</v>
+        <v>0.791390689534383</v>
       </c>
       <c r="L24" s="10" t="n">
         <f aca="false">IF($J24=1,RANK($K24,$K$2:$K$1001),"")</f>
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7006,11 +7006,11 @@
       </c>
       <c r="K25" s="10" t="n">
         <f aca="true">IF($J25=1,RAND(),-1)</f>
-        <v>0.902143084310058</v>
+        <v>0.244657422641741</v>
       </c>
       <c r="L25" s="10" t="n">
         <f aca="false">IF($J25=1,RANK($K25,$K$2:$K$1001),"")</f>
-        <v>27</v>
+        <v>169</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7047,11 +7047,11 @@
       </c>
       <c r="K26" s="10" t="n">
         <f aca="true">IF($J26=1,RAND(),-1)</f>
-        <v>0.226134123656925</v>
+        <v>0.350708021994324</v>
       </c>
       <c r="L26" s="10" t="n">
         <f aca="false">IF($J26=1,RANK($K26,$K$2:$K$1001),"")</f>
-        <v>181</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7088,11 +7088,11 @@
       </c>
       <c r="K27" s="10" t="n">
         <f aca="true">IF($J27=1,RAND(),-1)</f>
-        <v>0.722689264659609</v>
+        <v>0.840393098282053</v>
       </c>
       <c r="L27" s="10" t="n">
         <f aca="false">IF($J27=1,RANK($K27,$K$2:$K$1001),"")</f>
-        <v>71</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7129,11 +7129,11 @@
       </c>
       <c r="K28" s="10" t="n">
         <f aca="true">IF($J28=1,RAND(),-1)</f>
-        <v>0.344365759983099</v>
+        <v>0.843615942388549</v>
       </c>
       <c r="L28" s="10" t="n">
         <f aca="false">IF($J28=1,RANK($K28,$K$2:$K$1001),"")</f>
-        <v>157</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7170,11 +7170,11 @@
       </c>
       <c r="K29" s="10" t="n">
         <f aca="true">IF($J29=1,RAND(),-1)</f>
-        <v>0.909128990003166</v>
+        <v>0.751863785052589</v>
       </c>
       <c r="L29" s="10" t="n">
         <f aca="false">IF($J29=1,RANK($K29,$K$2:$K$1001),"")</f>
-        <v>25</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7211,11 +7211,11 @@
       </c>
       <c r="K30" s="10" t="n">
         <f aca="true">IF($J30=1,RAND(),-1)</f>
-        <v>0.900243355202201</v>
+        <v>0.68817368126261</v>
       </c>
       <c r="L30" s="10" t="n">
         <f aca="false">IF($J30=1,RANK($K30,$K$2:$K$1001),"")</f>
-        <v>28</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7252,11 +7252,11 @@
       </c>
       <c r="K31" s="10" t="n">
         <f aca="true">IF($J31=1,RAND(),-1)</f>
-        <v>0.640763855247545</v>
+        <v>0.0227915968839275</v>
       </c>
       <c r="L31" s="10" t="n">
         <f aca="false">IF($J31=1,RANK($K31,$K$2:$K$1001),"")</f>
-        <v>90</v>
+        <v>221</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7293,11 +7293,11 @@
       </c>
       <c r="K32" s="10" t="n">
         <f aca="true">IF($J32=1,RAND(),-1)</f>
-        <v>0.257453052017052</v>
+        <v>0.427730869241869</v>
       </c>
       <c r="L32" s="10" t="n">
         <f aca="false">IF($J32=1,RANK($K32,$K$2:$K$1001),"")</f>
-        <v>174</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7334,11 +7334,11 @@
       </c>
       <c r="K33" s="10" t="n">
         <f aca="true">IF($J33=1,RAND(),-1)</f>
-        <v>0.481484915811606</v>
+        <v>0.445745721322508</v>
       </c>
       <c r="L33" s="10" t="n">
         <f aca="false">IF($J33=1,RANK($K33,$K$2:$K$1001),"")</f>
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7375,11 +7375,11 @@
       </c>
       <c r="K34" s="10" t="n">
         <f aca="true">IF($J34=1,RAND(),-1)</f>
-        <v>0.416940668017262</v>
+        <v>0.220301691470674</v>
       </c>
       <c r="L34" s="10" t="n">
         <f aca="false">IF($J34=1,RANK($K34,$K$2:$K$1001),"")</f>
-        <v>139</v>
+        <v>179</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7416,11 +7416,11 @@
       </c>
       <c r="K35" s="10" t="n">
         <f aca="true">IF($J35=1,RAND(),-1)</f>
-        <v>0.820388828856205</v>
+        <v>0.682209797115888</v>
       </c>
       <c r="L35" s="10" t="n">
         <f aca="false">IF($J35=1,RANK($K35,$K$2:$K$1001),"")</f>
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7457,11 +7457,11 @@
       </c>
       <c r="K36" s="10" t="n">
         <f aca="true">IF($J36=1,RAND(),-1)</f>
-        <v>0.553381749169604</v>
+        <v>0.0960798977981393</v>
       </c>
       <c r="L36" s="10" t="n">
         <f aca="false">IF($J36=1,RANK($K36,$K$2:$K$1001),"")</f>
-        <v>108</v>
+        <v>205</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7498,11 +7498,11 @@
       </c>
       <c r="K37" s="10" t="n">
         <f aca="true">IF($J37=1,RAND(),-1)</f>
-        <v>0.655876820002614</v>
+        <v>0.692902124286699</v>
       </c>
       <c r="L37" s="10" t="n">
         <f aca="false">IF($J37=1,RANK($K37,$K$2:$K$1001),"")</f>
-        <v>87</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7539,11 +7539,11 @@
       </c>
       <c r="K38" s="10" t="n">
         <f aca="true">IF($J38=1,RAND(),-1)</f>
-        <v>0.727839815520398</v>
+        <v>0.977111994593651</v>
       </c>
       <c r="L38" s="10" t="n">
         <f aca="false">IF($J38=1,RANK($K38,$K$2:$K$1001),"")</f>
-        <v>68</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7580,11 +7580,11 @@
       </c>
       <c r="K39" s="10" t="n">
         <f aca="true">IF($J39=1,RAND(),-1)</f>
-        <v>0.477193157601631</v>
+        <v>0.400035082626107</v>
       </c>
       <c r="L39" s="10" t="n">
         <f aca="false">IF($J39=1,RANK($K39,$K$2:$K$1001),"")</f>
-        <v>125</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7621,11 +7621,11 @@
       </c>
       <c r="K40" s="10" t="n">
         <f aca="true">IF($J40=1,RAND(),-1)</f>
-        <v>0.458217693305363</v>
+        <v>0.678477002933716</v>
       </c>
       <c r="L40" s="10" t="n">
         <f aca="false">IF($J40=1,RANK($K40,$K$2:$K$1001),"")</f>
-        <v>129</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7662,11 +7662,11 @@
       </c>
       <c r="K41" s="10" t="n">
         <f aca="true">IF($J41=1,RAND(),-1)</f>
-        <v>0.270579327250338</v>
+        <v>0.221261983730159</v>
       </c>
       <c r="L41" s="10" t="n">
         <f aca="false">IF($J41=1,RANK($K41,$K$2:$K$1001),"")</f>
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7703,11 +7703,11 @@
       </c>
       <c r="K42" s="10" t="n">
         <f aca="true">IF($J42=1,RAND(),-1)</f>
-        <v>0.257142699906581</v>
+        <v>0.762313580187798</v>
       </c>
       <c r="L42" s="10" t="n">
         <f aca="false">IF($J42=1,RANK($K42,$K$2:$K$1001),"")</f>
-        <v>175</v>
+        <v>46</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7744,11 +7744,11 @@
       </c>
       <c r="K43" s="10" t="n">
         <f aca="true">IF($J43=1,RAND(),-1)</f>
-        <v>0.747941383616858</v>
+        <v>0.880723488905978</v>
       </c>
       <c r="L43" s="10" t="n">
         <f aca="false">IF($J43=1,RANK($K43,$K$2:$K$1001),"")</f>
-        <v>66</v>
+        <v>24</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7785,11 +7785,11 @@
       </c>
       <c r="K44" s="10" t="n">
         <f aca="true">IF($J44=1,RAND(),-1)</f>
-        <v>0.682350550397438</v>
+        <v>0.573442898183365</v>
       </c>
       <c r="L44" s="10" t="n">
         <f aca="false">IF($J44=1,RANK($K44,$K$2:$K$1001),"")</f>
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7826,11 +7826,11 @@
       </c>
       <c r="K45" s="10" t="n">
         <f aca="true">IF($J45=1,RAND(),-1)</f>
-        <v>0.957242143566014</v>
+        <v>0.215244272613178</v>
       </c>
       <c r="L45" s="10" t="n">
         <f aca="false">IF($J45=1,RANK($K45,$K$2:$K$1001),"")</f>
-        <v>13</v>
+        <v>181</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7867,11 +7867,11 @@
       </c>
       <c r="K46" s="10" t="n">
         <f aca="true">IF($J46=1,RAND(),-1)</f>
-        <v>0.564191503182607</v>
+        <v>0.362908321866177</v>
       </c>
       <c r="L46" s="10" t="n">
         <f aca="false">IF($J46=1,RANK($K46,$K$2:$K$1001),"")</f>
-        <v>106</v>
+        <v>142</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7908,11 +7908,11 @@
       </c>
       <c r="K47" s="10" t="n">
         <f aca="true">IF($J47=1,RAND(),-1)</f>
-        <v>0.718936128430385</v>
+        <v>0.0135532480757304</v>
       </c>
       <c r="L47" s="10" t="n">
         <f aca="false">IF($J47=1,RANK($K47,$K$2:$K$1001),"")</f>
-        <v>73</v>
+        <v>222</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7949,11 +7949,11 @@
       </c>
       <c r="K48" s="10" t="n">
         <f aca="true">IF($J48=1,RAND(),-1)</f>
-        <v>0.830303633578037</v>
+        <v>0.0743131790430523</v>
       </c>
       <c r="L48" s="10" t="n">
         <f aca="false">IF($J48=1,RANK($K48,$K$2:$K$1001),"")</f>
-        <v>45</v>
+        <v>211</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7990,11 +7990,11 @@
       </c>
       <c r="K49" s="10" t="n">
         <f aca="true">IF($J49=1,RAND(),-1)</f>
-        <v>0.105797343930896</v>
+        <v>0.738615163116261</v>
       </c>
       <c r="L49" s="10" t="n">
         <f aca="false">IF($J49=1,RANK($K49,$K$2:$K$1001),"")</f>
-        <v>203</v>
+        <v>57</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8031,11 +8031,11 @@
       </c>
       <c r="K50" s="10" t="n">
         <f aca="true">IF($J50=1,RAND(),-1)</f>
-        <v>0.461674405168116</v>
+        <v>0.784024237119484</v>
       </c>
       <c r="L50" s="10" t="n">
         <f aca="false">IF($J50=1,RANK($K50,$K$2:$K$1001),"")</f>
-        <v>128</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8072,11 +8072,11 @@
       </c>
       <c r="K51" s="10" t="n">
         <f aca="true">IF($J51=1,RAND(),-1)</f>
-        <v>0.471491576486297</v>
+        <v>0.747539022888891</v>
       </c>
       <c r="L51" s="10" t="n">
         <f aca="false">IF($J51=1,RANK($K51,$K$2:$K$1001),"")</f>
-        <v>127</v>
+        <v>54</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8113,11 +8113,11 @@
       </c>
       <c r="K52" s="10" t="n">
         <f aca="true">IF($J52=1,RAND(),-1)</f>
-        <v>0.335547521413743</v>
+        <v>0.209782545801478</v>
       </c>
       <c r="L52" s="10" t="n">
         <f aca="false">IF($J52=1,RANK($K52,$K$2:$K$1001),"")</f>
-        <v>161</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8154,11 +8154,11 @@
       </c>
       <c r="K53" s="10" t="n">
         <f aca="true">IF($J53=1,RAND(),-1)</f>
-        <v>0.399194913705203</v>
+        <v>0.696554397787546</v>
       </c>
       <c r="L53" s="10" t="n">
         <f aca="false">IF($J53=1,RANK($K53,$K$2:$K$1001),"")</f>
-        <v>148</v>
+        <v>65</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8195,11 +8195,11 @@
       </c>
       <c r="K54" s="10" t="n">
         <f aca="true">IF($J54=1,RAND(),-1)</f>
-        <v>0.287927786335275</v>
+        <v>0.221279521917633</v>
       </c>
       <c r="L54" s="10" t="n">
         <f aca="false">IF($J54=1,RANK($K54,$K$2:$K$1001),"")</f>
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8236,11 +8236,11 @@
       </c>
       <c r="K55" s="10" t="n">
         <f aca="true">IF($J55=1,RAND(),-1)</f>
-        <v>0.982083403409526</v>
+        <v>0.871889297198561</v>
       </c>
       <c r="L55" s="10" t="n">
         <f aca="false">IF($J55=1,RANK($K55,$K$2:$K$1001),"")</f>
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8277,11 +8277,11 @@
       </c>
       <c r="K56" s="10" t="n">
         <f aca="true">IF($J56=1,RAND(),-1)</f>
-        <v>0.887989054334326</v>
+        <v>0.4465025555367</v>
       </c>
       <c r="L56" s="10" t="n">
         <f aca="false">IF($J56=1,RANK($K56,$K$2:$K$1001),"")</f>
-        <v>33</v>
+        <v>127</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8318,11 +8318,11 @@
       </c>
       <c r="K57" s="10" t="n">
         <f aca="true">IF($J57=1,RAND(),-1)</f>
-        <v>0.977716180093909</v>
+        <v>0.372086751790402</v>
       </c>
       <c r="L57" s="10" t="n">
         <f aca="false">IF($J57=1,RANK($K57,$K$2:$K$1001),"")</f>
-        <v>8</v>
+        <v>141</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8359,11 +8359,11 @@
       </c>
       <c r="K58" s="10" t="n">
         <f aca="true">IF($J58=1,RAND(),-1)</f>
-        <v>0.308030767623289</v>
+        <v>0.425043563848971</v>
       </c>
       <c r="L58" s="10" t="n">
         <f aca="false">IF($J58=1,RANK($K58,$K$2:$K$1001),"")</f>
-        <v>165</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8400,11 +8400,11 @@
       </c>
       <c r="K59" s="10" t="n">
         <f aca="true">IF($J59=1,RAND(),-1)</f>
-        <v>0.495895388504701</v>
+        <v>0.314997672579082</v>
       </c>
       <c r="L59" s="10" t="n">
         <f aca="false">IF($J59=1,RANK($K59,$K$2:$K$1001),"")</f>
-        <v>120</v>
+        <v>155</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8441,11 +8441,11 @@
       </c>
       <c r="K60" s="10" t="n">
         <f aca="true">IF($J60=1,RAND(),-1)</f>
-        <v>0.596637310922611</v>
+        <v>0.522303866033181</v>
       </c>
       <c r="L60" s="10" t="n">
         <f aca="false">IF($J60=1,RANK($K60,$K$2:$K$1001),"")</f>
-        <v>100</v>
+        <v>108</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8482,11 +8482,11 @@
       </c>
       <c r="K61" s="10" t="n">
         <f aca="true">IF($J61=1,RAND(),-1)</f>
-        <v>0.21185582582072</v>
+        <v>0.292853094160772</v>
       </c>
       <c r="L61" s="10" t="n">
         <f aca="false">IF($J61=1,RANK($K61,$K$2:$K$1001),"")</f>
-        <v>186</v>
+        <v>160</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8523,11 +8523,11 @@
       </c>
       <c r="K62" s="10" t="n">
         <f aca="true">IF($J62=1,RAND(),-1)</f>
-        <v>0.188242001890644</v>
+        <v>0.058016183756116</v>
       </c>
       <c r="L62" s="10" t="n">
         <f aca="false">IF($J62=1,RANK($K62,$K$2:$K$1001),"")</f>
-        <v>190</v>
+        <v>215</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8564,11 +8564,11 @@
       </c>
       <c r="K63" s="10" t="n">
         <f aca="true">IF($J63=1,RAND(),-1)</f>
-        <v>0.812339756334825</v>
+        <v>0.329955147193178</v>
       </c>
       <c r="L63" s="10" t="n">
         <f aca="false">IF($J63=1,RANK($K63,$K$2:$K$1001),"")</f>
-        <v>49</v>
+        <v>152</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8605,11 +8605,11 @@
       </c>
       <c r="K64" s="10" t="n">
         <f aca="true">IF($J64=1,RAND(),-1)</f>
-        <v>0.800928435580494</v>
+        <v>0.643412776415664</v>
       </c>
       <c r="L64" s="10" t="n">
         <f aca="false">IF($J64=1,RANK($K64,$K$2:$K$1001),"")</f>
-        <v>53</v>
+        <v>85</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8646,11 +8646,11 @@
       </c>
       <c r="K65" s="10" t="n">
         <f aca="true">IF($J65=1,RAND(),-1)</f>
-        <v>0.40415861166416</v>
+        <v>0.922554499432087</v>
       </c>
       <c r="L65" s="10" t="n">
         <f aca="false">IF($J65=1,RANK($K65,$K$2:$K$1001),"")</f>
-        <v>147</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8687,11 +8687,11 @@
       </c>
       <c r="K66" s="10" t="n">
         <f aca="true">IF($J66=1,RAND(),-1)</f>
-        <v>0.140235757977395</v>
+        <v>0.751870292434175</v>
       </c>
       <c r="L66" s="10" t="n">
         <f aca="false">IF($J66=1,RANK($K66,$K$2:$K$1001),"")</f>
-        <v>197</v>
+        <v>51</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8728,11 +8728,11 @@
       </c>
       <c r="K67" s="10" t="n">
         <f aca="true">IF($J67=1,RAND(),-1)</f>
-        <v>0.753613265232359</v>
+        <v>0.561625313716552</v>
       </c>
       <c r="L67" s="10" t="n">
         <f aca="false">IF($J67=1,RANK($K67,$K$2:$K$1001),"")</f>
-        <v>65</v>
+        <v>99</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8769,11 +8769,11 @@
       </c>
       <c r="K68" s="10" t="n">
         <f aca="true">IF($J68=1,RAND(),-1)</f>
-        <v>0.976040052293349</v>
+        <v>0.591914204363883</v>
       </c>
       <c r="L68" s="10" t="n">
         <f aca="false">IF($J68=1,RANK($K68,$K$2:$K$1001),"")</f>
-        <v>9</v>
+        <v>94</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8810,11 +8810,11 @@
       </c>
       <c r="K69" s="10" t="n">
         <f aca="true">IF($J69=1,RAND(),-1)</f>
-        <v>0.132659301939662</v>
+        <v>0.884451037768383</v>
       </c>
       <c r="L69" s="10" t="n">
         <f aca="false">IF($J69=1,RANK($K69,$K$2:$K$1001),"")</f>
-        <v>199</v>
+        <v>22</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8851,11 +8851,11 @@
       </c>
       <c r="K70" s="10" t="n">
         <f aca="true">IF($J70=1,RAND(),-1)</f>
-        <v>0.871058164385805</v>
+        <v>0.77351631504857</v>
       </c>
       <c r="L70" s="10" t="n">
         <f aca="false">IF($J70=1,RANK($K70,$K$2:$K$1001),"")</f>
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8892,11 +8892,11 @@
       </c>
       <c r="K71" s="10" t="n">
         <f aca="true">IF($J71=1,RAND(),-1)</f>
-        <v>0.841723396132882</v>
+        <v>0.822324980362926</v>
       </c>
       <c r="L71" s="10" t="n">
         <f aca="false">IF($J71=1,RANK($K71,$K$2:$K$1001),"")</f>
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="K72" s="10" t="n">
         <f aca="true">IF($J72=1,RAND(),-1)</f>
-        <v>0.664741586310112</v>
+        <v>0.321872213271924</v>
       </c>
       <c r="L72" s="10" t="n">
         <f aca="false">IF($J72=1,RANK($K72,$K$2:$K$1001),"")</f>
-        <v>85</v>
+        <v>153</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8974,11 +8974,11 @@
       </c>
       <c r="K73" s="10" t="n">
         <f aca="true">IF($J73=1,RAND(),-1)</f>
-        <v>0.126455421028607</v>
+        <v>0.667784451134759</v>
       </c>
       <c r="L73" s="10" t="n">
         <f aca="false">IF($J73=1,RANK($K73,$K$2:$K$1001),"")</f>
-        <v>201</v>
+        <v>77</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9015,11 +9015,11 @@
       </c>
       <c r="K74" s="10" t="n">
         <f aca="true">IF($J74=1,RAND(),-1)</f>
-        <v>0.238762401024499</v>
+        <v>0.133797529275187</v>
       </c>
       <c r="L74" s="10" t="n">
         <f aca="false">IF($J74=1,RANK($K74,$K$2:$K$1001),"")</f>
-        <v>179</v>
+        <v>199</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9056,11 +9056,11 @@
       </c>
       <c r="K75" s="10" t="n">
         <f aca="true">IF($J75=1,RAND(),-1)</f>
-        <v>0.21784742330843</v>
+        <v>0.254413503080995</v>
       </c>
       <c r="L75" s="10" t="n">
         <f aca="false">IF($J75=1,RANK($K75,$K$2:$K$1001),"")</f>
-        <v>185</v>
+        <v>167</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9097,11 +9097,11 @@
       </c>
       <c r="K76" s="10" t="n">
         <f aca="true">IF($J76=1,RAND(),-1)</f>
-        <v>0.440900603171454</v>
+        <v>0.944840121334961</v>
       </c>
       <c r="L76" s="10" t="n">
         <f aca="false">IF($J76=1,RANK($K76,$K$2:$K$1001),"")</f>
-        <v>133</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9138,11 +9138,11 @@
       </c>
       <c r="K77" s="10" t="n">
         <f aca="true">IF($J77=1,RAND(),-1)</f>
-        <v>0.241320669304064</v>
+        <v>0.869479177874123</v>
       </c>
       <c r="L77" s="10" t="n">
         <f aca="false">IF($J77=1,RANK($K77,$K$2:$K$1001),"")</f>
-        <v>178</v>
+        <v>28</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9179,11 +9179,11 @@
       </c>
       <c r="K78" s="10" t="n">
         <f aca="true">IF($J78=1,RAND(),-1)</f>
-        <v>0.340763078945877</v>
+        <v>0.657307714572043</v>
       </c>
       <c r="L78" s="10" t="n">
         <f aca="false">IF($J78=1,RANK($K78,$K$2:$K$1001),"")</f>
-        <v>159</v>
+        <v>80</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9220,11 +9220,11 @@
       </c>
       <c r="K79" s="10" t="n">
         <f aca="true">IF($J79=1,RAND(),-1)</f>
-        <v>0.632485875980518</v>
+        <v>0.921501881533406</v>
       </c>
       <c r="L79" s="10" t="n">
         <f aca="false">IF($J79=1,RANK($K79,$K$2:$K$1001),"")</f>
-        <v>91</v>
+        <v>16</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9261,11 +9261,11 @@
       </c>
       <c r="K80" s="10" t="n">
         <f aca="true">IF($J80=1,RAND(),-1)</f>
-        <v>0.43491216022024</v>
+        <v>0.265009583159018</v>
       </c>
       <c r="L80" s="10" t="n">
         <f aca="false">IF($J80=1,RANK($K80,$K$2:$K$1001),"")</f>
-        <v>136</v>
+        <v>165</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9302,11 +9302,11 @@
       </c>
       <c r="K81" s="10" t="n">
         <f aca="true">IF($J81=1,RAND(),-1)</f>
-        <v>0.289808184631809</v>
+        <v>0.0952195569671441</v>
       </c>
       <c r="L81" s="10" t="n">
         <f aca="false">IF($J81=1,RANK($K81,$K$2:$K$1001),"")</f>
-        <v>167</v>
+        <v>206</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9343,11 +9343,11 @@
       </c>
       <c r="K82" s="10" t="n">
         <f aca="true">IF($J82=1,RAND(),-1)</f>
-        <v>0.517393647041842</v>
+        <v>0.921345169608819</v>
       </c>
       <c r="L82" s="10" t="n">
         <f aca="false">IF($J82=1,RANK($K82,$K$2:$K$1001),"")</f>
-        <v>117</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9384,11 +9384,11 @@
       </c>
       <c r="K83" s="10" t="n">
         <f aca="true">IF($J83=1,RAND(),-1)</f>
-        <v>0.0485859722977174</v>
+        <v>0.720437804925562</v>
       </c>
       <c r="L83" s="10" t="n">
         <f aca="false">IF($J83=1,RANK($K83,$K$2:$K$1001),"")</f>
-        <v>215</v>
+        <v>61</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9425,11 +9425,11 @@
       </c>
       <c r="K84" s="10" t="n">
         <f aca="true">IF($J84=1,RAND(),-1)</f>
-        <v>0.687398153556858</v>
+        <v>0.882019226393073</v>
       </c>
       <c r="L84" s="10" t="n">
         <f aca="false">IF($J84=1,RANK($K84,$K$2:$K$1001),"")</f>
-        <v>79</v>
+        <v>23</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9466,11 +9466,11 @@
       </c>
       <c r="K85" s="10" t="n">
         <f aca="true">IF($J85=1,RAND(),-1)</f>
-        <v>0.985274015158048</v>
+        <v>0.599840158003984</v>
       </c>
       <c r="L85" s="10" t="n">
         <f aca="false">IF($J85=1,RANK($K85,$K$2:$K$1001),"")</f>
-        <v>5</v>
+        <v>93</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9507,11 +9507,11 @@
       </c>
       <c r="K86" s="10" t="n">
         <f aca="true">IF($J86=1,RAND(),-1)</f>
-        <v>0.184848672188111</v>
+        <v>0.309414765566614</v>
       </c>
       <c r="L86" s="10" t="n">
         <f aca="false">IF($J86=1,RANK($K86,$K$2:$K$1001),"")</f>
-        <v>191</v>
+        <v>157</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9548,11 +9548,11 @@
       </c>
       <c r="K87" s="10" t="n">
         <f aca="true">IF($J87=1,RAND(),-1)</f>
-        <v>0.0538107612208909</v>
+        <v>0.770276488238241</v>
       </c>
       <c r="L87" s="10" t="n">
         <f aca="false">IF($J87=1,RANK($K87,$K$2:$K$1001),"")</f>
-        <v>214</v>
+        <v>43</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9589,11 +9589,11 @@
       </c>
       <c r="K88" s="10" t="n">
         <f aca="true">IF($J88=1,RAND(),-1)</f>
-        <v>0.0658790644957822</v>
+        <v>0.613643854318183</v>
       </c>
       <c r="L88" s="10" t="n">
         <f aca="false">IF($J88=1,RANK($K88,$K$2:$K$1001),"")</f>
-        <v>211</v>
+        <v>91</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9630,11 +9630,11 @@
       </c>
       <c r="K89" s="10" t="n">
         <f aca="true">IF($J89=1,RAND(),-1)</f>
-        <v>0.482451385017774</v>
+        <v>0.319035162616265</v>
       </c>
       <c r="L89" s="10" t="n">
         <f aca="false">IF($J89=1,RANK($K89,$K$2:$K$1001),"")</f>
-        <v>121</v>
+        <v>154</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9671,11 +9671,11 @@
       </c>
       <c r="K90" s="10" t="n">
         <f aca="true">IF($J90=1,RAND(),-1)</f>
-        <v>0.862579276901756</v>
+        <v>0.542459441864758</v>
       </c>
       <c r="L90" s="10" t="n">
         <f aca="false">IF($J90=1,RANK($K90,$K$2:$K$1001),"")</f>
-        <v>36</v>
+        <v>106</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9712,11 +9712,11 @@
       </c>
       <c r="K91" s="10" t="n">
         <f aca="true">IF($J91=1,RAND(),-1)</f>
-        <v>0.861398017883458</v>
+        <v>0.759094058455269</v>
       </c>
       <c r="L91" s="10" t="n">
         <f aca="false">IF($J91=1,RANK($K91,$K$2:$K$1001),"")</f>
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9753,11 +9753,11 @@
       </c>
       <c r="K92" s="10" t="n">
         <f aca="true">IF($J92=1,RAND(),-1)</f>
-        <v>0.801706944009685</v>
+        <v>0.479620124590537</v>
       </c>
       <c r="L92" s="10" t="n">
         <f aca="false">IF($J92=1,RANK($K92,$K$2:$K$1001),"")</f>
-        <v>52</v>
+        <v>118</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9794,11 +9794,11 @@
       </c>
       <c r="K93" s="10" t="n">
         <f aca="true">IF($J93=1,RAND(),-1)</f>
-        <v>0.905759625927511</v>
+        <v>0.548137814837727</v>
       </c>
       <c r="L93" s="10" t="n">
         <f aca="false">IF($J93=1,RANK($K93,$K$2:$K$1001),"")</f>
-        <v>26</v>
+        <v>104</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9835,11 +9835,11 @@
       </c>
       <c r="K94" s="10" t="n">
         <f aca="true">IF($J94=1,RAND(),-1)</f>
-        <v>0.358497303402479</v>
+        <v>0.80848002134682</v>
       </c>
       <c r="L94" s="10" t="n">
         <f aca="false">IF($J94=1,RANK($K94,$K$2:$K$1001),"")</f>
-        <v>154</v>
+        <v>38</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9876,11 +9876,11 @@
       </c>
       <c r="K95" s="10" t="n">
         <f aca="true">IF($J95=1,RAND(),-1)</f>
-        <v>0.934320432102909</v>
+        <v>0.635082793882476</v>
       </c>
       <c r="L95" s="10" t="n">
         <f aca="false">IF($J95=1,RANK($K95,$K$2:$K$1001),"")</f>
-        <v>23</v>
+        <v>87</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9917,11 +9917,11 @@
       </c>
       <c r="K96" s="10" t="n">
         <f aca="true">IF($J96=1,RAND(),-1)</f>
-        <v>0.888631598846162</v>
+        <v>0.0423926407650656</v>
       </c>
       <c r="L96" s="10" t="n">
         <f aca="false">IF($J96=1,RANK($K96,$K$2:$K$1001),"")</f>
-        <v>32</v>
+        <v>218</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9958,11 +9958,11 @@
       </c>
       <c r="K97" s="10" t="n">
         <f aca="true">IF($J97=1,RAND(),-1)</f>
-        <v>0.0317133351585759</v>
+        <v>0.637608409198012</v>
       </c>
       <c r="L97" s="10" t="n">
         <f aca="false">IF($J97=1,RANK($K97,$K$2:$K$1001),"")</f>
-        <v>220</v>
+        <v>86</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9999,11 +9999,11 @@
       </c>
       <c r="K98" s="10" t="n">
         <f aca="true">IF($J98=1,RAND(),-1)</f>
-        <v>0.28760844865551</v>
+        <v>0.779207849745604</v>
       </c>
       <c r="L98" s="10" t="n">
         <f aca="false">IF($J98=1,RANK($K98,$K$2:$K$1001),"")</f>
-        <v>170</v>
+        <v>41</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10040,11 +10040,11 @@
       </c>
       <c r="K99" s="10" t="n">
         <f aca="true">IF($J99=1,RAND(),-1)</f>
-        <v>0.472075482254373</v>
+        <v>0.50668120328547</v>
       </c>
       <c r="L99" s="10" t="n">
         <f aca="false">IF($J99=1,RANK($K99,$K$2:$K$1001),"")</f>
-        <v>126</v>
+        <v>113</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10081,11 +10081,11 @@
       </c>
       <c r="K100" s="10" t="n">
         <f aca="true">IF($J100=1,RAND(),-1)</f>
-        <v>0.338319001652816</v>
+        <v>0.738550358783783</v>
       </c>
       <c r="L100" s="10" t="n">
         <f aca="false">IF($J100=1,RANK($K100,$K$2:$K$1001),"")</f>
-        <v>160</v>
+        <v>58</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10122,11 +10122,11 @@
       </c>
       <c r="K101" s="10" t="n">
         <f aca="true">IF($J101=1,RAND(),-1)</f>
-        <v>0.762020224112932</v>
+        <v>0.340154285135085</v>
       </c>
       <c r="L101" s="10" t="n">
         <f aca="false">IF($J101=1,RANK($K101,$K$2:$K$1001),"")</f>
-        <v>61</v>
+        <v>147</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10163,11 +10163,11 @@
       </c>
       <c r="K102" s="10" t="n">
         <f aca="true">IF($J102=1,RAND(),-1)</f>
-        <v>0.288705400487277</v>
+        <v>0.746174210407143</v>
       </c>
       <c r="L102" s="10" t="n">
         <f aca="false">IF($J102=1,RANK($K102,$K$2:$K$1001),"")</f>
-        <v>168</v>
+        <v>55</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10204,11 +10204,11 @@
       </c>
       <c r="K103" s="10" t="n">
         <f aca="true">IF($J103=1,RAND(),-1)</f>
-        <v>0.0822147750307033</v>
+        <v>0.341315955454172</v>
       </c>
       <c r="L103" s="10" t="n">
         <f aca="false">IF($J103=1,RANK($K103,$K$2:$K$1001),"")</f>
-        <v>208</v>
+        <v>146</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10245,11 +10245,11 @@
       </c>
       <c r="K104" s="10" t="n">
         <f aca="true">IF($J104=1,RAND(),-1)</f>
-        <v>0.79739944687822</v>
+        <v>0.00215534206579871</v>
       </c>
       <c r="L104" s="10" t="n">
         <f aca="false">IF($J104=1,RANK($K104,$K$2:$K$1001),"")</f>
-        <v>55</v>
+        <v>224</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10286,11 +10286,11 @@
       </c>
       <c r="K105" s="10" t="n">
         <f aca="true">IF($J105=1,RAND(),-1)</f>
-        <v>0.627628393023457</v>
+        <v>0.755592147915079</v>
       </c>
       <c r="L105" s="10" t="n">
         <f aca="false">IF($J105=1,RANK($K105,$K$2:$K$1001),"")</f>
-        <v>93</v>
+        <v>48</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10327,11 +10327,11 @@
       </c>
       <c r="K106" s="10" t="n">
         <f aca="true">IF($J106=1,RAND(),-1)</f>
-        <v>0.546193229951315</v>
+        <v>0.516989573728296</v>
       </c>
       <c r="L106" s="10" t="n">
         <f aca="false">IF($J106=1,RANK($K106,$K$2:$K$1001),"")</f>
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10368,11 +10368,11 @@
       </c>
       <c r="K107" s="10" t="n">
         <f aca="true">IF($J107=1,RAND(),-1)</f>
-        <v>0.945795679582426</v>
+        <v>0.630285688359229</v>
       </c>
       <c r="L107" s="10" t="n">
         <f aca="false">IF($J107=1,RANK($K107,$K$2:$K$1001),"")</f>
-        <v>19</v>
+        <v>88</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10409,11 +10409,11 @@
       </c>
       <c r="K108" s="10" t="n">
         <f aca="true">IF($J108=1,RAND(),-1)</f>
-        <v>0.837144964138006</v>
+        <v>0.417717872928716</v>
       </c>
       <c r="L108" s="10" t="n">
         <f aca="false">IF($J108=1,RANK($K108,$K$2:$K$1001),"")</f>
-        <v>43</v>
+        <v>133</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10450,11 +10450,11 @@
       </c>
       <c r="K109" s="10" t="n">
         <f aca="true">IF($J109=1,RAND(),-1)</f>
-        <v>0.715031320928351</v>
+        <v>0.927616239372093</v>
       </c>
       <c r="L109" s="10" t="n">
         <f aca="false">IF($J109=1,RANK($K109,$K$2:$K$1001),"")</f>
-        <v>74</v>
+        <v>14</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10491,11 +10491,11 @@
       </c>
       <c r="K110" s="10" t="n">
         <f aca="true">IF($J110=1,RAND(),-1)</f>
-        <v>0.252958954479738</v>
+        <v>0.247443042950957</v>
       </c>
       <c r="L110" s="10" t="n">
         <f aca="false">IF($J110=1,RANK($K110,$K$2:$K$1001),"")</f>
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10532,11 +10532,11 @@
       </c>
       <c r="K111" s="10" t="n">
         <f aca="true">IF($J111=1,RAND(),-1)</f>
-        <v>0.702308129490228</v>
+        <v>0.300470771786984</v>
       </c>
       <c r="L111" s="10" t="n">
         <f aca="false">IF($J111=1,RANK($K111,$K$2:$K$1001),"")</f>
-        <v>78</v>
+        <v>159</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10573,11 +10573,11 @@
       </c>
       <c r="K112" s="10" t="n">
         <f aca="true">IF($J112=1,RAND(),-1)</f>
-        <v>0.972773529451049</v>
+        <v>0.655680982953881</v>
       </c>
       <c r="L112" s="10" t="n">
         <f aca="false">IF($J112=1,RANK($K112,$K$2:$K$1001),"")</f>
-        <v>10</v>
+        <v>82</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10614,11 +10614,11 @@
       </c>
       <c r="K113" s="10" t="n">
         <f aca="true">IF($J113=1,RAND(),-1)</f>
-        <v>0.0219550478897127</v>
+        <v>0.121861610677491</v>
       </c>
       <c r="L113" s="10" t="n">
         <f aca="false">IF($J113=1,RANK($K113,$K$2:$K$1001),"")</f>
-        <v>222</v>
+        <v>203</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10655,11 +10655,11 @@
       </c>
       <c r="K114" s="10" t="n">
         <f aca="true">IF($J114=1,RAND(),-1)</f>
-        <v>0.769520820393269</v>
+        <v>0.196099628974739</v>
       </c>
       <c r="L114" s="10" t="n">
         <f aca="false">IF($J114=1,RANK($K114,$K$2:$K$1001),"")</f>
-        <v>60</v>
+        <v>190</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10696,11 +10696,11 @@
       </c>
       <c r="K115" s="10" t="n">
         <f aca="true">IF($J115=1,RAND(),-1)</f>
-        <v>0.531254748973906</v>
+        <v>0.443359526167945</v>
       </c>
       <c r="L115" s="10" t="n">
         <f aca="false">IF($J115=1,RANK($K115,$K$2:$K$1001),"")</f>
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10737,11 +10737,11 @@
       </c>
       <c r="K116" s="10" t="n">
         <f aca="true">IF($J116=1,RAND(),-1)</f>
-        <v>0.033196114783662</v>
+        <v>0.850541606578792</v>
       </c>
       <c r="L116" s="10" t="n">
         <f aca="false">IF($J116=1,RANK($K116,$K$2:$K$1001),"")</f>
-        <v>219</v>
+        <v>30</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10778,11 +10778,11 @@
       </c>
       <c r="K117" s="10" t="n">
         <f aca="true">IF($J117=1,RAND(),-1)</f>
-        <v>0.676507200931158</v>
+        <v>0.48969266027149</v>
       </c>
       <c r="L117" s="10" t="n">
         <f aca="false">IF($J117=1,RANK($K117,$K$2:$K$1001),"")</f>
-        <v>83</v>
+        <v>116</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10819,11 +10819,11 @@
       </c>
       <c r="K118" s="10" t="n">
         <f aca="true">IF($J118=1,RAND(),-1)</f>
-        <v>0.644483604385032</v>
+        <v>0.447273376993088</v>
       </c>
       <c r="L118" s="10" t="n">
         <f aca="false">IF($J118=1,RANK($K118,$K$2:$K$1001),"")</f>
-        <v>89</v>
+        <v>125</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10860,11 +10860,11 @@
       </c>
       <c r="K119" s="10" t="n">
         <f aca="true">IF($J119=1,RAND(),-1)</f>
-        <v>0.06795855857783</v>
+        <v>0.521175176280773</v>
       </c>
       <c r="L119" s="10" t="n">
         <f aca="false">IF($J119=1,RANK($K119,$K$2:$K$1001),"")</f>
-        <v>210</v>
+        <v>109</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10901,11 +10901,11 @@
       </c>
       <c r="K120" s="10" t="n">
         <f aca="true">IF($J120=1,RAND(),-1)</f>
-        <v>0.989397896281922</v>
+        <v>0.085699202164786</v>
       </c>
       <c r="L120" s="10" t="n">
         <f aca="false">IF($J120=1,RANK($K120,$K$2:$K$1001),"")</f>
-        <v>4</v>
+        <v>209</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10942,11 +10942,11 @@
       </c>
       <c r="K121" s="10" t="n">
         <f aca="true">IF($J121=1,RAND(),-1)</f>
-        <v>0.362057665929153</v>
+        <v>0.682203228816003</v>
       </c>
       <c r="L121" s="10" t="n">
         <f aca="false">IF($J121=1,RANK($K121,$K$2:$K$1001),"")</f>
-        <v>153</v>
+        <v>73</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10983,11 +10983,11 @@
       </c>
       <c r="K122" s="10" t="n">
         <f aca="true">IF($J122=1,RAND(),-1)</f>
-        <v>0.946830533187004</v>
+        <v>0.557647613963379</v>
       </c>
       <c r="L122" s="10" t="n">
         <f aca="false">IF($J122=1,RANK($K122,$K$2:$K$1001),"")</f>
-        <v>18</v>
+        <v>100</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11024,11 +11024,11 @@
       </c>
       <c r="K123" s="10" t="n">
         <f aca="true">IF($J123=1,RAND(),-1)</f>
-        <v>0.342227412206893</v>
+        <v>0.828808031928115</v>
       </c>
       <c r="L123" s="10" t="n">
         <f aca="false">IF($J123=1,RANK($K123,$K$2:$K$1001),"")</f>
-        <v>158</v>
+        <v>34</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11065,11 +11065,11 @@
       </c>
       <c r="K124" s="10" t="n">
         <f aca="true">IF($J124=1,RAND(),-1)</f>
-        <v>0.225860930875128</v>
+        <v>0.87233867851634</v>
       </c>
       <c r="L124" s="10" t="n">
         <f aca="false">IF($J124=1,RANK($K124,$K$2:$K$1001),"")</f>
-        <v>182</v>
+        <v>25</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11106,11 +11106,11 @@
       </c>
       <c r="K125" s="10" t="n">
         <f aca="true">IF($J125=1,RAND(),-1)</f>
-        <v>0.513383257943733</v>
+        <v>0.55539836076465</v>
       </c>
       <c r="L125" s="10" t="n">
         <f aca="false">IF($J125=1,RANK($K125,$K$2:$K$1001),"")</f>
-        <v>118</v>
+        <v>101</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11147,11 +11147,11 @@
       </c>
       <c r="K126" s="10" t="n">
         <f aca="true">IF($J126=1,RAND(),-1)</f>
-        <v>0.453193652870636</v>
+        <v>0.717474308952177</v>
       </c>
       <c r="L126" s="10" t="n">
         <f aca="false">IF($J126=1,RANK($K126,$K$2:$K$1001),"")</f>
-        <v>130</v>
+        <v>62</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11188,11 +11188,11 @@
       </c>
       <c r="K127" s="10" t="n">
         <f aca="true">IF($J127=1,RAND(),-1)</f>
-        <v>0.409946950232981</v>
+        <v>0.770005274964834</v>
       </c>
       <c r="L127" s="10" t="n">
         <f aca="false">IF($J127=1,RANK($K127,$K$2:$K$1001),"")</f>
-        <v>143</v>
+        <v>44</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11229,11 +11229,11 @@
       </c>
       <c r="K128" s="10" t="n">
         <f aca="true">IF($J128=1,RAND(),-1)</f>
-        <v>0.364862574556525</v>
+        <v>0.693337847553307</v>
       </c>
       <c r="L128" s="10" t="n">
         <f aca="false">IF($J128=1,RANK($K128,$K$2:$K$1001),"")</f>
-        <v>152</v>
+        <v>66</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11270,11 +11270,11 @@
       </c>
       <c r="K129" s="10" t="n">
         <f aca="true">IF($J129=1,RAND(),-1)</f>
-        <v>0.681277636107591</v>
+        <v>0.339734730289051</v>
       </c>
       <c r="L129" s="10" t="n">
         <f aca="false">IF($J129=1,RANK($K129,$K$2:$K$1001),"")</f>
-        <v>82</v>
+        <v>148</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11311,11 +11311,11 @@
       </c>
       <c r="K130" s="10" t="n">
         <f aca="true">IF($J130=1,RAND(),-1)</f>
-        <v>0.0619886456919915</v>
+        <v>0.462676854451784</v>
       </c>
       <c r="L130" s="10" t="n">
         <f aca="false">IF($J130=1,RANK($K130,$K$2:$K$1001),"")</f>
-        <v>212</v>
+        <v>121</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11352,11 +11352,11 @@
       </c>
       <c r="K131" s="10" t="n">
         <f aca="true">IF($J131=1,RAND(),-1)</f>
-        <v>0.594247697900076</v>
+        <v>0.0117478145349655</v>
       </c>
       <c r="L131" s="10" t="n">
         <f aca="false">IF($J131=1,RANK($K131,$K$2:$K$1001),"")</f>
-        <v>102</v>
+        <v>223</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11393,11 +11393,11 @@
       </c>
       <c r="K132" s="10" t="n">
         <f aca="true">IF($J132=1,RAND(),-1)</f>
-        <v>0.195225623084306</v>
+        <v>0.104452886900925</v>
       </c>
       <c r="L132" s="10" t="n">
         <f aca="false">IF($J132=1,RANK($K132,$K$2:$K$1001),"")</f>
-        <v>188</v>
+        <v>204</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11434,11 +11434,11 @@
       </c>
       <c r="K133" s="10" t="n">
         <f aca="true">IF($J133=1,RAND(),-1)</f>
-        <v>0.704987817861447</v>
+        <v>0.566823975446791</v>
       </c>
       <c r="L133" s="10" t="n">
         <f aca="false">IF($J133=1,RANK($K133,$K$2:$K$1001),"")</f>
-        <v>77</v>
+        <v>98</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11475,11 +11475,11 @@
       </c>
       <c r="K134" s="10" t="n">
         <f aca="true">IF($J134=1,RAND(),-1)</f>
-        <v>0.305714296660201</v>
+        <v>0.899664568396896</v>
       </c>
       <c r="L134" s="10" t="n">
         <f aca="false">IF($J134=1,RANK($K134,$K$2:$K$1001),"")</f>
-        <v>166</v>
+        <v>21</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11516,11 +11516,11 @@
       </c>
       <c r="K135" s="10" t="n">
         <f aca="true">IF($J135=1,RAND(),-1)</f>
-        <v>0.42815538465626</v>
+        <v>0.703217580624776</v>
       </c>
       <c r="L135" s="10" t="n">
         <f aca="false">IF($J135=1,RANK($K135,$K$2:$K$1001),"")</f>
-        <v>137</v>
+        <v>64</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11557,11 +11557,11 @@
       </c>
       <c r="K136" s="10" t="n">
         <f aca="true">IF($J136=1,RAND(),-1)</f>
-        <v>0.709082790030487</v>
+        <v>0.689125552468828</v>
       </c>
       <c r="L136" s="10" t="n">
         <f aca="false">IF($J136=1,RANK($K136,$K$2:$K$1001),"")</f>
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11598,11 +11598,11 @@
       </c>
       <c r="K137" s="10" t="n">
         <f aca="true">IF($J137=1,RAND(),-1)</f>
-        <v>0.414550121258611</v>
+        <v>0.750403063118331</v>
       </c>
       <c r="L137" s="10" t="n">
         <f aca="false">IF($J137=1,RANK($K137,$K$2:$K$1001),"")</f>
-        <v>141</v>
+        <v>53</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11639,11 +11639,11 @@
       </c>
       <c r="K138" s="10" t="n">
         <f aca="true">IF($J138=1,RAND(),-1)</f>
-        <v>0.173858022146357</v>
+        <v>0.395861700449384</v>
       </c>
       <c r="L138" s="10" t="n">
         <f aca="false">IF($J138=1,RANK($K138,$K$2:$K$1001),"")</f>
-        <v>192</v>
+        <v>138</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11680,11 +11680,11 @@
       </c>
       <c r="K139" s="10" t="n">
         <f aca="true">IF($J139=1,RAND(),-1)</f>
-        <v>0.599760520611638</v>
+        <v>0.266617483398485</v>
       </c>
       <c r="L139" s="10" t="n">
         <f aca="false">IF($J139=1,RANK($K139,$K$2:$K$1001),"")</f>
-        <v>99</v>
+        <v>164</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11721,11 +11721,11 @@
       </c>
       <c r="K140" s="10" t="n">
         <f aca="true">IF($J140=1,RAND(),-1)</f>
-        <v>0.413377285277045</v>
+        <v>0.301583796925558</v>
       </c>
       <c r="L140" s="10" t="n">
         <f aca="false">IF($J140=1,RANK($K140,$K$2:$K$1001),"")</f>
-        <v>142</v>
+        <v>158</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11762,11 +11762,11 @@
       </c>
       <c r="K141" s="10" t="n">
         <f aca="true">IF($J141=1,RAND(),-1)</f>
-        <v>0.139133874352596</v>
+        <v>0.0626956173311706</v>
       </c>
       <c r="L141" s="10" t="n">
         <f aca="false">IF($J141=1,RANK($K141,$K$2:$K$1001),"")</f>
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11803,11 +11803,11 @@
       </c>
       <c r="K142" s="10" t="n">
         <f aca="true">IF($J142=1,RAND(),-1)</f>
-        <v>0.608086185590007</v>
+        <v>0.231202680749116</v>
       </c>
       <c r="L142" s="10" t="n">
         <f aca="false">IF($J142=1,RANK($K142,$K$2:$K$1001),"")</f>
-        <v>96</v>
+        <v>174</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11844,11 +11844,11 @@
       </c>
       <c r="K143" s="10" t="n">
         <f aca="true">IF($J143=1,RAND(),-1)</f>
-        <v>0.160115914510948</v>
+        <v>0.820728171842168</v>
       </c>
       <c r="L143" s="10" t="n">
         <f aca="false">IF($J143=1,RANK($K143,$K$2:$K$1001),"")</f>
-        <v>193</v>
+        <v>36</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11885,11 +11885,11 @@
       </c>
       <c r="K144" s="10" t="n">
         <f aca="true">IF($J144=1,RAND(),-1)</f>
-        <v>0.946953679266957</v>
+        <v>0.161695879619471</v>
       </c>
       <c r="L144" s="10" t="n">
         <f aca="false">IF($J144=1,RANK($K144,$K$2:$K$1001),"")</f>
-        <v>17</v>
+        <v>195</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11926,11 +11926,11 @@
       </c>
       <c r="K145" s="10" t="n">
         <f aca="true">IF($J145=1,RAND(),-1)</f>
-        <v>0.854942386004297</v>
+        <v>0.23728613606772</v>
       </c>
       <c r="L145" s="10" t="n">
         <f aca="false">IF($J145=1,RANK($K145,$K$2:$K$1001),"")</f>
-        <v>40</v>
+        <v>172</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11967,11 +11967,11 @@
       </c>
       <c r="K146" s="10" t="n">
         <f aca="true">IF($J146=1,RAND(),-1)</f>
-        <v>0.507205127115467</v>
+        <v>0.255834361872587</v>
       </c>
       <c r="L146" s="10" t="n">
         <f aca="false">IF($J146=1,RANK($K146,$K$2:$K$1001),"")</f>
-        <v>119</v>
+        <v>166</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12008,11 +12008,11 @@
       </c>
       <c r="K147" s="10" t="n">
         <f aca="true">IF($J147=1,RAND(),-1)</f>
-        <v>0.795670140648793</v>
+        <v>0.655585730608817</v>
       </c>
       <c r="L147" s="10" t="n">
         <f aca="false">IF($J147=1,RANK($K147,$K$2:$K$1001),"")</f>
-        <v>56</v>
+        <v>83</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12049,11 +12049,11 @@
       </c>
       <c r="K148" s="10" t="n">
         <f aca="true">IF($J148=1,RAND(),-1)</f>
-        <v>0.0149257459333267</v>
+        <v>0.382063407839916</v>
       </c>
       <c r="L148" s="10" t="n">
         <f aca="false">IF($J148=1,RANK($K148,$K$2:$K$1001),"")</f>
-        <v>224</v>
+        <v>140</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12090,11 +12090,11 @@
       </c>
       <c r="K149" s="10" t="n">
         <f aca="true">IF($J149=1,RAND(),-1)</f>
-        <v>0.556788747325838</v>
+        <v>0.603051310496443</v>
       </c>
       <c r="L149" s="10" t="n">
         <f aca="false">IF($J149=1,RANK($K149,$K$2:$K$1001),"")</f>
-        <v>107</v>
+        <v>92</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12131,11 +12131,11 @@
       </c>
       <c r="K150" s="10" t="n">
         <f aca="true">IF($J150=1,RAND(),-1)</f>
-        <v>0.584127369565144</v>
+        <v>0.0338854736977528</v>
       </c>
       <c r="L150" s="10" t="n">
         <f aca="false">IF($J150=1,RANK($K150,$K$2:$K$1001),"")</f>
-        <v>104</v>
+        <v>220</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12172,11 +12172,11 @@
       </c>
       <c r="K151" s="10" t="n">
         <f aca="true">IF($J151=1,RAND(),-1)</f>
-        <v>0.207853958156584</v>
+        <v>0.487151604139895</v>
       </c>
       <c r="L151" s="10" t="n">
         <f aca="false">IF($J151=1,RANK($K151,$K$2:$K$1001),"")</f>
-        <v>187</v>
+        <v>117</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12213,11 +12213,11 @@
       </c>
       <c r="K152" s="10" t="n">
         <f aca="true">IF($J152=1,RAND(),-1)</f>
-        <v>0.725881988500393</v>
+        <v>0.209748709944224</v>
       </c>
       <c r="L152" s="10" t="n">
         <f aca="false">IF($J152=1,RANK($K152,$K$2:$K$1001),"")</f>
-        <v>69</v>
+        <v>184</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12254,11 +12254,11 @@
       </c>
       <c r="K153" s="10" t="n">
         <f aca="true">IF($J153=1,RAND(),-1)</f>
-        <v>0.531139959506004</v>
+        <v>0.549125921689886</v>
       </c>
       <c r="L153" s="10" t="n">
         <f aca="false">IF($J153=1,RANK($K153,$K$2:$K$1001),"")</f>
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12295,11 +12295,11 @@
       </c>
       <c r="K154" s="10" t="n">
         <f aca="true">IF($J154=1,RAND(),-1)</f>
-        <v>0.827471955594048</v>
+        <v>0.977769072890851</v>
       </c>
       <c r="L154" s="10" t="n">
         <f aca="false">IF($J154=1,RANK($K154,$K$2:$K$1001),"")</f>
-        <v>46</v>
+        <v>6</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12336,11 +12336,11 @@
       </c>
       <c r="K155" s="10" t="n">
         <f aca="true">IF($J155=1,RAND(),-1)</f>
-        <v>0.0334957027072327</v>
+        <v>0.721899558721715</v>
       </c>
       <c r="L155" s="10" t="n">
         <f aca="false">IF($J155=1,RANK($K155,$K$2:$K$1001),"")</f>
-        <v>218</v>
+        <v>60</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12377,11 +12377,11 @@
       </c>
       <c r="K156" s="10" t="n">
         <f aca="true">IF($J156=1,RAND(),-1)</f>
-        <v>0.370516905554842</v>
+        <v>0.508496316922985</v>
       </c>
       <c r="L156" s="10" t="n">
         <f aca="false">IF($J156=1,RANK($K156,$K$2:$K$1001),"")</f>
-        <v>151</v>
+        <v>112</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12418,11 +12418,11 @@
       </c>
       <c r="K157" s="10" t="n">
         <f aca="true">IF($J157=1,RAND(),-1)</f>
-        <v>0.284768112790164</v>
+        <v>0.337179863372609</v>
       </c>
       <c r="L157" s="10" t="n">
         <f aca="false">IF($J157=1,RANK($K157,$K$2:$K$1001),"")</f>
-        <v>172</v>
+        <v>150</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12459,11 +12459,11 @@
       </c>
       <c r="K158" s="10" t="n">
         <f aca="true">IF($J158=1,RAND(),-1)</f>
-        <v>0.955810481614674</v>
+        <v>0.753861264017616</v>
       </c>
       <c r="L158" s="10" t="n">
         <f aca="false">IF($J158=1,RANK($K158,$K$2:$K$1001),"")</f>
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12500,11 +12500,11 @@
       </c>
       <c r="K159" s="10" t="n">
         <f aca="true">IF($J159=1,RAND(),-1)</f>
-        <v>0.0456701680033478</v>
+        <v>0.685657388755455</v>
       </c>
       <c r="L159" s="10" t="n">
         <f aca="false">IF($J159=1,RANK($K159,$K$2:$K$1001),"")</f>
-        <v>216</v>
+        <v>71</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12541,11 +12541,11 @@
       </c>
       <c r="K160" s="10" t="n">
         <f aca="true">IF($J160=1,RAND(),-1)</f>
-        <v>0.629204407540554</v>
+        <v>0.163918923809161</v>
       </c>
       <c r="L160" s="10" t="n">
         <f aca="false">IF($J160=1,RANK($K160,$K$2:$K$1001),"")</f>
-        <v>92</v>
+        <v>194</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12582,11 +12582,11 @@
       </c>
       <c r="K161" s="10" t="n">
         <f aca="true">IF($J161=1,RAND(),-1)</f>
-        <v>0.856450828399992</v>
+        <v>0.815767602998773</v>
       </c>
       <c r="L161" s="10" t="n">
         <f aca="false">IF($J161=1,RANK($K161,$K$2:$K$1001),"")</f>
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12623,11 +12623,11 @@
       </c>
       <c r="K162" s="10" t="n">
         <f aca="true">IF($J162=1,RAND(),-1)</f>
-        <v>0.438693442436811</v>
+        <v>0.334341538662202</v>
       </c>
       <c r="L162" s="10" t="n">
         <f aca="false">IF($J162=1,RANK($K162,$K$2:$K$1001),"")</f>
-        <v>134</v>
+        <v>151</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12664,11 +12664,11 @@
       </c>
       <c r="K163" s="10" t="n">
         <f aca="true">IF($J163=1,RAND(),-1)</f>
-        <v>0.308617186434505</v>
+        <v>0.134071274788761</v>
       </c>
       <c r="L163" s="10" t="n">
         <f aca="false">IF($J163=1,RANK($K163,$K$2:$K$1001),"")</f>
-        <v>164</v>
+        <v>198</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12705,11 +12705,11 @@
       </c>
       <c r="K164" s="10" t="n">
         <f aca="true">IF($J164=1,RAND(),-1)</f>
-        <v>0.409173372759522</v>
+        <v>0.205390393028098</v>
       </c>
       <c r="L164" s="10" t="n">
         <f aca="false">IF($J164=1,RANK($K164,$K$2:$K$1001),"")</f>
-        <v>145</v>
+        <v>186</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12746,11 +12746,11 @@
       </c>
       <c r="K165" s="10" t="n">
         <f aca="true">IF($J165=1,RAND(),-1)</f>
-        <v>0.425076059490222</v>
+        <v>0.19985362622563</v>
       </c>
       <c r="L165" s="10" t="n">
         <f aca="false">IF($J165=1,RANK($K165,$K$2:$K$1001),"")</f>
-        <v>138</v>
+        <v>189</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12787,11 +12787,11 @@
       </c>
       <c r="K166" s="10" t="n">
         <f aca="true">IF($J166=1,RAND(),-1)</f>
-        <v>0.142481993413371</v>
+        <v>0.353863805768526</v>
       </c>
       <c r="L166" s="10" t="n">
         <f aca="false">IF($J166=1,RANK($K166,$K$2:$K$1001),"")</f>
-        <v>196</v>
+        <v>143</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12828,11 +12828,11 @@
       </c>
       <c r="K167" s="10" t="n">
         <f aca="true">IF($J167=1,RAND(),-1)</f>
-        <v>0.809073900619529</v>
+        <v>0.224897974806035</v>
       </c>
       <c r="L167" s="10" t="n">
         <f aca="false">IF($J167=1,RANK($K167,$K$2:$K$1001),"")</f>
-        <v>50</v>
+        <v>175</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12869,11 +12869,11 @@
       </c>
       <c r="K168" s="10" t="n">
         <f aca="true">IF($J168=1,RAND(),-1)</f>
-        <v>0.889345502662645</v>
+        <v>0.671675376000405</v>
       </c>
       <c r="L168" s="10" t="n">
         <f aca="false">IF($J168=1,RANK($K168,$K$2:$K$1001),"")</f>
-        <v>31</v>
+        <v>76</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12910,11 +12910,11 @@
       </c>
       <c r="K169" s="10" t="n">
         <f aca="true">IF($J169=1,RAND(),-1)</f>
-        <v>0.711015826434592</v>
+        <v>0.242528180185341</v>
       </c>
       <c r="L169" s="10" t="n">
         <f aca="false">IF($J169=1,RANK($K169,$K$2:$K$1001),"")</f>
-        <v>75</v>
+        <v>170</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12951,11 +12951,11 @@
       </c>
       <c r="K170" s="10" t="n">
         <f aca="true">IF($J170=1,RAND(),-1)</f>
-        <v>0.156995526430745</v>
+        <v>0.902060037908911</v>
       </c>
       <c r="L170" s="10" t="n">
         <f aca="false">IF($J170=1,RANK($K170,$K$2:$K$1001),"")</f>
-        <v>194</v>
+        <v>19</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12992,11 +12992,11 @@
       </c>
       <c r="K171" s="10" t="n">
         <f aca="true">IF($J171=1,RAND(),-1)</f>
-        <v>0.253815659011041</v>
+        <v>0.685965510224414</v>
       </c>
       <c r="L171" s="10" t="n">
         <f aca="false">IF($J171=1,RANK($K171,$K$2:$K$1001),"")</f>
-        <v>176</v>
+        <v>70</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13033,11 +13033,11 @@
       </c>
       <c r="K172" s="10" t="n">
         <f aca="true">IF($J172=1,RAND(),-1)</f>
-        <v>0.815473324896565</v>
+        <v>0.947827068218964</v>
       </c>
       <c r="L172" s="10" t="n">
         <f aca="false">IF($J172=1,RANK($K172,$K$2:$K$1001),"")</f>
-        <v>48</v>
+        <v>11</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13074,11 +13074,11 @@
       </c>
       <c r="K173" s="10" t="n">
         <f aca="true">IF($J173=1,RAND(),-1)</f>
-        <v>0.583366151364514</v>
+        <v>0.0512148855371338</v>
       </c>
       <c r="L173" s="10" t="n">
         <f aca="false">IF($J173=1,RANK($K173,$K$2:$K$1001),"")</f>
-        <v>105</v>
+        <v>216</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13115,11 +13115,11 @@
       </c>
       <c r="K174" s="10" t="n">
         <f aca="true">IF($J174=1,RAND(),-1)</f>
-        <v>0.1912413735177</v>
+        <v>0.98124004370203</v>
       </c>
       <c r="L174" s="10" t="n">
         <f aca="false">IF($J174=1,RANK($K174,$K$2:$K$1001),"")</f>
-        <v>189</v>
+        <v>5</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13156,11 +13156,11 @@
       </c>
       <c r="K175" s="10" t="n">
         <f aca="true">IF($J175=1,RAND(),-1)</f>
-        <v>0.684954170374515</v>
+        <v>0.205374799370152</v>
       </c>
       <c r="L175" s="10" t="n">
         <f aca="false">IF($J175=1,RANK($K175,$K$2:$K$1001),"")</f>
-        <v>80</v>
+        <v>187</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13197,11 +13197,11 @@
       </c>
       <c r="K176" s="10" t="n">
         <f aca="true">IF($J176=1,RAND(),-1)</f>
-        <v>0.0746246862775301</v>
+        <v>0.660739065571654</v>
       </c>
       <c r="L176" s="10" t="n">
         <f aca="false">IF($J176=1,RANK($K176,$K$2:$K$1001),"")</f>
-        <v>209</v>
+        <v>78</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13238,11 +13238,11 @@
       </c>
       <c r="K177" s="10" t="n">
         <f aca="true">IF($J177=1,RAND(),-1)</f>
-        <v>0.480235755811466</v>
+        <v>0.22372964825133</v>
       </c>
       <c r="L177" s="10" t="n">
         <f aca="false">IF($J177=1,RANK($K177,$K$2:$K$1001),"")</f>
-        <v>123</v>
+        <v>176</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13279,11 +13279,11 @@
       </c>
       <c r="K178" s="10" t="n">
         <f aca="true">IF($J178=1,RAND(),-1)</f>
-        <v>0.999843865010908</v>
+        <v>0.205407181625224</v>
       </c>
       <c r="L178" s="10" t="n">
         <f aca="false">IF($J178=1,RANK($K178,$K$2:$K$1001),"")</f>
-        <v>1</v>
+        <v>185</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13320,11 +13320,11 @@
       </c>
       <c r="K179" s="10" t="n">
         <f aca="true">IF($J179=1,RAND(),-1)</f>
-        <v>0.850536387731825</v>
+        <v>0.619824893006421</v>
       </c>
       <c r="L179" s="10" t="n">
         <f aca="false">IF($J179=1,RANK($K179,$K$2:$K$1001),"")</f>
-        <v>41</v>
+        <v>90</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13361,11 +13361,11 @@
       </c>
       <c r="K180" s="10" t="n">
         <f aca="true">IF($J180=1,RAND(),-1)</f>
-        <v>0.955951225254102</v>
+        <v>0.234540691598122</v>
       </c>
       <c r="L180" s="10" t="n">
         <f aca="false">IF($J180=1,RANK($K180,$K$2:$K$1001),"")</f>
-        <v>14</v>
+        <v>173</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13402,11 +13402,11 @@
       </c>
       <c r="K181" s="10" t="n">
         <f aca="true">IF($J181=1,RAND(),-1)</f>
-        <v>0.543536864397052</v>
+        <v>0.12417332513389</v>
       </c>
       <c r="L181" s="10" t="n">
         <f aca="false">IF($J181=1,RANK($K181,$K$2:$K$1001),"")</f>
-        <v>113</v>
+        <v>200</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13443,11 +13443,11 @@
       </c>
       <c r="K182" s="10" t="n">
         <f aca="true">IF($J182=1,RAND(),-1)</f>
-        <v>0.107647081945333</v>
+        <v>0.755333735876371</v>
       </c>
       <c r="L182" s="10" t="n">
         <f aca="false">IF($J182=1,RANK($K182,$K$2:$K$1001),"")</f>
-        <v>202</v>
+        <v>49</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13484,11 +13484,11 @@
       </c>
       <c r="K183" s="10" t="n">
         <f aca="true">IF($J183=1,RAND(),-1)</f>
-        <v>0.990240404062735</v>
+        <v>0.400898885594811</v>
       </c>
       <c r="L183" s="10" t="n">
         <f aca="false">IF($J183=1,RANK($K183,$K$2:$K$1001),"")</f>
-        <v>3</v>
+        <v>135</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13525,11 +13525,11 @@
       </c>
       <c r="K184" s="10" t="n">
         <f aca="true">IF($J184=1,RAND(),-1)</f>
-        <v>0.540205458014351</v>
+        <v>0.991426560939617</v>
       </c>
       <c r="L184" s="10" t="n">
         <f aca="false">IF($J184=1,RANK($K184,$K$2:$K$1001),"")</f>
-        <v>114</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13566,11 +13566,11 @@
       </c>
       <c r="K185" s="10" t="n">
         <f aca="true">IF($J185=1,RAND(),-1)</f>
-        <v>0.478333104792128</v>
+        <v>0.937456787432041</v>
       </c>
       <c r="L185" s="10" t="n">
         <f aca="false">IF($J185=1,RANK($K185,$K$2:$K$1001),"")</f>
-        <v>124</v>
+        <v>13</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13607,11 +13607,11 @@
       </c>
       <c r="K186" s="10" t="n">
         <f aca="true">IF($J186=1,RAND(),-1)</f>
-        <v>0.772540808789482</v>
+        <v>0.0918633295716413</v>
       </c>
       <c r="L186" s="10" t="n">
         <f aca="false">IF($J186=1,RANK($K186,$K$2:$K$1001),"")</f>
-        <v>58</v>
+        <v>208</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13648,11 +13648,11 @@
       </c>
       <c r="K187" s="10" t="n">
         <f aca="true">IF($J187=1,RAND(),-1)</f>
-        <v>0.754624017696931</v>
+        <v>0.0928951235954888</v>
       </c>
       <c r="L187" s="10" t="n">
         <f aca="false">IF($J187=1,RANK($K187,$K$2:$K$1001),"")</f>
-        <v>64</v>
+        <v>207</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13689,11 +13689,11 @@
       </c>
       <c r="K188" s="10" t="n">
         <f aca="true">IF($J188=1,RAND(),-1)</f>
-        <v>0.0971843450490324</v>
+        <v>0.287845533092415</v>
       </c>
       <c r="L188" s="10" t="n">
         <f aca="false">IF($J188=1,RANK($K188,$K$2:$K$1001),"")</f>
-        <v>205</v>
+        <v>161</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13730,11 +13730,11 @@
       </c>
       <c r="K189" s="10" t="n">
         <f aca="true">IF($J189=1,RAND(),-1)</f>
-        <v>0.668059191596061</v>
+        <v>0.513632256887471</v>
       </c>
       <c r="L189" s="10" t="n">
         <f aca="false">IF($J189=1,RANK($K189,$K$2:$K$1001),"")</f>
-        <v>84</v>
+        <v>111</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13771,11 +13771,11 @@
       </c>
       <c r="K190" s="10" t="n">
         <f aca="true">IF($J190=1,RAND(),-1)</f>
-        <v>0.0846206108643594</v>
+        <v>0.213734625138024</v>
       </c>
       <c r="L190" s="10" t="n">
         <f aca="false">IF($J190=1,RANK($K190,$K$2:$K$1001),"")</f>
-        <v>207</v>
+        <v>182</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13812,11 +13812,11 @@
       </c>
       <c r="K191" s="10" t="n">
         <f aca="true">IF($J191=1,RAND(),-1)</f>
-        <v>0.799602364550998</v>
+        <v>0.549772543356447</v>
       </c>
       <c r="L191" s="10" t="n">
         <f aca="false">IF($J191=1,RANK($K191,$K$2:$K$1001),"")</f>
-        <v>54</v>
+        <v>102</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13853,11 +13853,11 @@
       </c>
       <c r="K192" s="10" t="n">
         <f aca="true">IF($J192=1,RAND(),-1)</f>
-        <v>0.661569024291627</v>
+        <v>0.964740477711216</v>
       </c>
       <c r="L192" s="10" t="n">
         <f aca="false">IF($J192=1,RANK($K192,$K$2:$K$1001),"")</f>
-        <v>86</v>
+        <v>9</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13894,11 +13894,11 @@
       </c>
       <c r="K193" s="10" t="n">
         <f aca="true">IF($J193=1,RAND(),-1)</f>
-        <v>0.545462984596294</v>
+        <v>0.52863231421442</v>
       </c>
       <c r="L193" s="10" t="n">
         <f aca="false">IF($J193=1,RANK($K193,$K$2:$K$1001),"")</f>
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13935,11 +13935,11 @@
       </c>
       <c r="K194" s="10" t="n">
         <f aca="true">IF($J194=1,RAND(),-1)</f>
-        <v>0.859551219003739</v>
+        <v>0.746030674148794</v>
       </c>
       <c r="L194" s="10" t="n">
         <f aca="false">IF($J194=1,RANK($K194,$K$2:$K$1001),"")</f>
-        <v>38</v>
+        <v>56</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13976,11 +13976,11 @@
       </c>
       <c r="K195" s="10" t="n">
         <f aca="true">IF($J195=1,RAND(),-1)</f>
-        <v>0.451819318746158</v>
+        <v>0.461391732218371</v>
       </c>
       <c r="L195" s="10" t="n">
         <f aca="false">IF($J195=1,RANK($K195,$K$2:$K$1001),"")</f>
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14017,11 +14017,11 @@
       </c>
       <c r="K196" s="10" t="n">
         <f aca="true">IF($J196=1,RAND(),-1)</f>
-        <v>0.723253180773055</v>
+        <v>0.200154936373282</v>
       </c>
       <c r="L196" s="10" t="n">
         <f aca="false">IF($J196=1,RANK($K196,$K$2:$K$1001),"")</f>
-        <v>70</v>
+        <v>188</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14058,11 +14058,11 @@
       </c>
       <c r="K197" s="10" t="n">
         <f aca="true">IF($J197=1,RAND(),-1)</f>
-        <v>0.759554048212421</v>
+        <v>0.65645997674559</v>
       </c>
       <c r="L197" s="10" t="n">
         <f aca="false">IF($J197=1,RANK($K197,$K$2:$K$1001),"")</f>
-        <v>62</v>
+        <v>81</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14099,11 +14099,11 @@
       </c>
       <c r="K198" s="10" t="n">
         <f aca="true">IF($J198=1,RAND(),-1)</f>
-        <v>0.771394662682491</v>
+        <v>0.70804585461972</v>
       </c>
       <c r="L198" s="10" t="n">
         <f aca="false">IF($J198=1,RANK($K198,$K$2:$K$1001),"")</f>
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14140,11 +14140,11 @@
       </c>
       <c r="K199" s="10" t="n">
         <f aca="true">IF($J199=1,RAND(),-1)</f>
-        <v>0.594321518862726</v>
+        <v>0.39657515641171</v>
       </c>
       <c r="L199" s="10" t="n">
         <f aca="false">IF($J199=1,RANK($K199,$K$2:$K$1001),"")</f>
-        <v>101</v>
+        <v>137</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14181,11 +14181,11 @@
       </c>
       <c r="K200" s="10" t="n">
         <f aca="true">IF($J200=1,RAND(),-1)</f>
-        <v>0.969284391314685</v>
+        <v>0.314898988797767</v>
       </c>
       <c r="L200" s="10" t="n">
         <f aca="false">IF($J200=1,RANK($K200,$K$2:$K$1001),"")</f>
-        <v>12</v>
+        <v>156</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14222,11 +14222,11 @@
       </c>
       <c r="K201" s="10" t="n">
         <f aca="true">IF($J201=1,RAND(),-1)</f>
-        <v>0.392009302430543</v>
+        <v>0.987948584105874</v>
       </c>
       <c r="L201" s="10" t="n">
         <f aca="false">IF($J201=1,RANK($K201,$K$2:$K$1001),"")</f>
-        <v>150</v>
+        <v>3</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14263,11 +14263,11 @@
       </c>
       <c r="K202" s="10" t="n">
         <f aca="true">IF($J202=1,RAND(),-1)</f>
-        <v>0.230599097116318</v>
+        <v>0.492777007837669</v>
       </c>
       <c r="L202" s="10" t="n">
         <f aca="false">IF($J202=1,RANK($K202,$K$2:$K$1001),"")</f>
-        <v>180</v>
+        <v>115</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14304,11 +14304,11 @@
       </c>
       <c r="K203" s="10" t="n">
         <f aca="true">IF($J203=1,RAND(),-1)</f>
-        <v>0.551817468651813</v>
+        <v>0.158827215751489</v>
       </c>
       <c r="L203" s="10" t="n">
         <f aca="false">IF($J203=1,RANK($K203,$K$2:$K$1001),"")</f>
-        <v>110</v>
+        <v>196</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14345,11 +14345,11 @@
       </c>
       <c r="K204" s="10" t="n">
         <f aca="true">IF($J204=1,RAND(),-1)</f>
-        <v>0.616636833816476</v>
+        <v>0.431955979198979</v>
       </c>
       <c r="L204" s="10" t="n">
         <f aca="false">IF($J204=1,RANK($K204,$K$2:$K$1001),"")</f>
-        <v>95</v>
+        <v>130</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14386,11 +14386,11 @@
       </c>
       <c r="K205" s="10" t="n">
         <f aca="true">IF($J205=1,RAND(),-1)</f>
-        <v>0.221645169077529</v>
+        <v>0.0355310865587619</v>
       </c>
       <c r="L205" s="10" t="n">
         <f aca="false">IF($J205=1,RANK($K205,$K$2:$K$1001),"")</f>
-        <v>183</v>
+        <v>219</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14427,11 +14427,11 @@
       </c>
       <c r="K206" s="10" t="n">
         <f aca="true">IF($J206=1,RAND(),-1)</f>
-        <v>0.436602555837475</v>
+        <v>0.165315859747264</v>
       </c>
       <c r="L206" s="10" t="n">
         <f aca="false">IF($J206=1,RANK($K206,$K$2:$K$1001),"")</f>
-        <v>135</v>
+        <v>193</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14468,11 +14468,11 @@
       </c>
       <c r="K207" s="10" t="n">
         <f aca="true">IF($J207=1,RAND(),-1)</f>
-        <v>0.409404439578388</v>
+        <v>0.845115465557651</v>
       </c>
       <c r="L207" s="10" t="n">
         <f aca="false">IF($J207=1,RANK($K207,$K$2:$K$1001),"")</f>
-        <v>144</v>
+        <v>31</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14509,11 +14509,11 @@
       </c>
       <c r="K208" s="10" t="n">
         <f aca="true">IF($J208=1,RAND(),-1)</f>
-        <v>0.553372963074263</v>
+        <v>0.676140089274124</v>
       </c>
       <c r="L208" s="10" t="n">
         <f aca="false">IF($J208=1,RANK($K208,$K$2:$K$1001),"")</f>
-        <v>109</v>
+        <v>75</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14550,11 +14550,11 @@
       </c>
       <c r="K209" s="10" t="n">
         <f aca="true">IF($J209=1,RAND(),-1)</f>
-        <v>0.0938525582405713</v>
+        <v>0.241782721484014</v>
       </c>
       <c r="L209" s="10" t="n">
         <f aca="false">IF($J209=1,RANK($K209,$K$2:$K$1001),"")</f>
-        <v>206</v>
+        <v>171</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14591,11 +14591,11 @@
       </c>
       <c r="K210" s="10" t="n">
         <f aca="true">IF($J210=1,RAND(),-1)</f>
-        <v>0.0188874080283083</v>
+        <v>0.122971558332874</v>
       </c>
       <c r="L210" s="10" t="n">
         <f aca="false">IF($J210=1,RANK($K210,$K$2:$K$1001),"")</f>
-        <v>223</v>
+        <v>202</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14632,11 +14632,11 @@
       </c>
       <c r="K211" s="10" t="n">
         <f aca="true">IF($J211=1,RAND(),-1)</f>
-        <v>0.287458515572727</v>
+        <v>0.871383154827596</v>
       </c>
       <c r="L211" s="10" t="n">
         <f aca="false">IF($J211=1,RANK($K211,$K$2:$K$1001),"")</f>
-        <v>171</v>
+        <v>27</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14673,11 +14673,11 @@
       </c>
       <c r="K212" s="10" t="n">
         <f aca="true">IF($J212=1,RAND(),-1)</f>
-        <v>0.648622441677736</v>
+        <v>0.0737808739862672</v>
       </c>
       <c r="L212" s="10" t="n">
         <f aca="false">IF($J212=1,RANK($K212,$K$2:$K$1001),"")</f>
-        <v>88</v>
+        <v>212</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14714,11 +14714,11 @@
       </c>
       <c r="K213" s="10" t="n">
         <f aca="true">IF($J213=1,RAND(),-1)</f>
-        <v>0.911125238480754</v>
+        <v>0.501618801911886</v>
       </c>
       <c r="L213" s="10" t="n">
         <f aca="false">IF($J213=1,RANK($K213,$K$2:$K$1001),"")</f>
-        <v>24</v>
+        <v>114</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14755,11 +14755,11 @@
       </c>
       <c r="K214" s="10" t="n">
         <f aca="true">IF($J214=1,RAND(),-1)</f>
-        <v>0.585189525589817</v>
+        <v>0.6604906671634</v>
       </c>
       <c r="L214" s="10" t="n">
         <f aca="false">IF($J214=1,RANK($K214,$K$2:$K$1001),"")</f>
-        <v>103</v>
+        <v>79</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14796,11 +14796,11 @@
       </c>
       <c r="K215" s="10" t="n">
         <f aca="true">IF($J215=1,RAND(),-1)</f>
-        <v>0.897442643385108</v>
+        <v>0.15704667248935</v>
       </c>
       <c r="L215" s="10" t="n">
         <f aca="false">IF($J215=1,RANK($K215,$K$2:$K$1001),"")</f>
-        <v>29</v>
+        <v>197</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14837,11 +14837,11 @@
       </c>
       <c r="K216" s="10" t="n">
         <f aca="true">IF($J216=1,RAND(),-1)</f>
-        <v>0.953672062320115</v>
+        <v>0.990671621044228</v>
       </c>
       <c r="L216" s="10" t="n">
         <f aca="false">IF($J216=1,RANK($K216,$K$2:$K$1001),"")</f>
-        <v>16</v>
+        <v>2</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14878,11 +14878,11 @@
       </c>
       <c r="K217" s="10" t="n">
         <f aca="true">IF($J217=1,RAND(),-1)</f>
-        <v>0.808199142711801</v>
+        <v>0.353482771407603</v>
       </c>
       <c r="L217" s="10" t="n">
         <f aca="false">IF($J217=1,RANK($K217,$K$2:$K$1001),"")</f>
-        <v>51</v>
+        <v>144</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14919,11 +14919,11 @@
       </c>
       <c r="K218" s="10" t="n">
         <f aca="true">IF($J218=1,RAND(),-1)</f>
-        <v>0.97243505976961</v>
+        <v>0.578435704353801</v>
       </c>
       <c r="L218" s="10" t="n">
         <f aca="false">IF($J218=1,RANK($K218,$K$2:$K$1001),"")</f>
-        <v>11</v>
+        <v>95</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14960,11 +14960,11 @@
       </c>
       <c r="K219" s="10" t="n">
         <f aca="true">IF($J219=1,RAND(),-1)</f>
-        <v>0.940287769370756</v>
+        <v>0.544945531046399</v>
       </c>
       <c r="L219" s="10" t="n">
         <f aca="false">IF($J219=1,RANK($K219,$K$2:$K$1001),"")</f>
-        <v>22</v>
+        <v>105</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15001,11 +15001,11 @@
       </c>
       <c r="K220" s="10" t="n">
         <f aca="true">IF($J220=1,RAND(),-1)</f>
-        <v>0.722589008446227</v>
+        <v>0.049779700825681</v>
       </c>
       <c r="L220" s="10" t="n">
         <f aca="false">IF($J220=1,RANK($K220,$K$2:$K$1001),"")</f>
-        <v>72</v>
+        <v>217</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15042,11 +15042,11 @@
       </c>
       <c r="K221" s="10" t="n">
         <f aca="true">IF($J221=1,RAND(),-1)</f>
-        <v>0.415910863311862</v>
+        <v>0.464718922771775</v>
       </c>
       <c r="L221" s="10" t="n">
         <f aca="false">IF($J221=1,RANK($K221,$K$2:$K$1001),"")</f>
-        <v>140</v>
+        <v>120</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15083,11 +15083,11 @@
       </c>
       <c r="K222" s="10" t="n">
         <f aca="true">IF($J222=1,RAND(),-1)</f>
-        <v>0.407499094885848</v>
+        <v>0.0745229973619508</v>
       </c>
       <c r="L222" s="10" t="n">
         <f aca="false">IF($J222=1,RANK($K222,$K$2:$K$1001),"")</f>
-        <v>146</v>
+        <v>210</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15124,11 +15124,11 @@
       </c>
       <c r="K223" s="10" t="n">
         <f aca="true">IF($J223=1,RAND(),-1)</f>
-        <v>0.128567689401755</v>
+        <v>0.285300327261778</v>
       </c>
       <c r="L223" s="10" t="n">
         <f aca="false">IF($J223=1,RANK($K223,$K$2:$K$1001),"")</f>
-        <v>200</v>
+        <v>162</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15165,7 +15165,7 @@
       </c>
       <c r="K224" s="10" t="n">
         <f aca="true">IF($J224=1,RAND(),-1)</f>
-        <v>0.942269419807299</v>
+        <v>0.900710370681835</v>
       </c>
       <c r="L224" s="10" t="n">
         <f aca="false">IF($J224=1,RANK($K224,$K$2:$K$1001),"")</f>
@@ -15206,11 +15206,11 @@
       </c>
       <c r="K225" s="10" t="n">
         <f aca="true">IF($J225=1,RAND(),-1)</f>
-        <v>0.894257278763792</v>
+        <v>0.394796933386587</v>
       </c>
       <c r="L225" s="10" t="n">
         <f aca="false">IF($J225=1,RANK($K225,$K$2:$K$1001),"")</f>
-        <v>30</v>
+        <v>139</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26125,11 +26125,11 @@
       </c>
       <c r="B4" s="5" t="str">
         <f aca="false">IF(Test!$J12="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J12))</f>
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="C4" s="12" t="str">
         <f aca="false">IF(B4="","",INDEX(Test!$C12:$F12,MATCH(B4,{"A","B","C","D"},0)))</f>
-        <v>24</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26139,11 +26139,11 @@
       </c>
       <c r="B5" s="5" t="str">
         <f aca="false">IF(Test!$J13="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J13))</f>
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="C5" s="12" t="str">
         <f aca="false">IF(B5="","",INDEX(Test!$C13:$F13,MATCH(B5,{"A","B","C","D"},0)))</f>
-        <v>343</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26153,11 +26153,11 @@
       </c>
       <c r="B6" s="5" t="str">
         <f aca="false">IF(Test!$J14="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J14))</f>
-        <v>C</v>
+        <v>A</v>
       </c>
       <c r="C6" s="12" t="str">
         <f aca="false">IF(B6="","",INDEX(Test!$C14:$F14,MATCH(B6,{"A","B","C","D"},0)))</f>
-        <v>84</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26167,11 +26167,11 @@
       </c>
       <c r="B7" s="5" t="str">
         <f aca="false">IF(Test!$J15="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J15))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="C7" s="12" t="str">
         <f aca="false">IF(B7="","",INDEX(Test!$C15:$F15,MATCH(B7,{"A","B","C","D"},0)))</f>
-        <v>2</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26181,11 +26181,11 @@
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">IF(Test!$J16="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J16))</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="C8" s="12" t="str">
         <f aca="false">IF(B8="","",INDEX(Test!$C16:$F16,MATCH(B8,{"A","B","C","D"},0)))</f>
-        <v>64</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26195,11 +26195,11 @@
       </c>
       <c r="B9" s="5" t="str">
         <f aca="false">IF(Test!$J17="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J17))</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="C9" s="12" t="str">
         <f aca="false">IF(B9="","",INDEX(Test!$C17:$F17,MATCH(B9,{"A","B","C","D"},0)))</f>
-        <v>10²</v>
+        <v>27 L</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26209,11 +26209,11 @@
       </c>
       <c r="B10" s="5" t="str">
         <f aca="false">IF(Test!$J18="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J18))</f>
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="C10" s="12" t="str">
         <f aca="false">IF(B10="","",INDEX(Test!$C18:$F18,MATCH(B10,{"A","B","C","D"},0)))</f>
-        <v>6 · 6 · 6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26227,7 +26227,7 @@
       </c>
       <c r="C11" s="12" t="str">
         <f aca="false">IF(B11="","",INDEX(Test!$C19:$F19,MATCH(B11,{"A","B","C","D"},0)))</f>
-        <v>9²</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26237,11 +26237,11 @@
       </c>
       <c r="B12" s="5" t="str">
         <f aca="false">IF(Test!$J20="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J20))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF(B12="","",INDEX(Test!$C20:$F20,MATCH(B12,{"A","B","C","D"},0)))</f>
-        <v>49</v>
+        <v>294</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26251,11 +26251,11 @@
       </c>
       <c r="B13" s="5" t="str">
         <f aca="false">IF(Test!$J21="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J21))</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF(B13="","",INDEX(Test!$C21:$F21,MATCH(B13,{"A","B","C","D"},0)))</f>
-        <v>729</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Tablet paketi, Türkçe Macerası ve genişletilmiş Fen/Sosyal/Din havuzları
- 6Sinif_EgitimSeti_Tablet.html: tüm sayfalar tek dosyada, internetsiz çalışır
- Türkçe Macerası: sesli slaytlarla konu anlatımı, deneme soruları,
  açıklamalı pratik, hata defteri, yıldız ve rozetler
- Söz Varlığı: her şık için 'neden doğru / neden yanlış' açıklaması
  (mevcut sorular değişmedi)
- Fen 136→248, Sosyal 84→186, Din Kültürü 63→149 soru
- Ortak şablon: yanlış seçilen şıkkın açıklaması; tek dosya paketinde yazdırma

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6qBE8e6Wkv628t1Q47HQM
</commit_message>
<xml_diff>
--- a/KupSorulari/KupSoruHavuzu.xlsx
+++ b/KupSorulari/KupSoruHavuzu.xlsx
@@ -2144,27 +2144,27 @@
       </c>
       <c r="B12" s="11" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J12))</f>
-        <v>Bir ayrıtı 8 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
+        <v>2³ + 9² işleminin sonucu kaçtır?</v>
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J12))</f>
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="D12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J12))</f>
-        <v>512</v>
+        <v>24</v>
       </c>
       <c r="E12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J12))</f>
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="F12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J12))</f>
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="G12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J12))</f>
-        <v>Küpün Özellikleri</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H12" s="12" t="str">
         <f aca="false">IF($J12="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J12))</f>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="J12" s="10" t="n">
         <f aca="false">IF(1&lt;=MIN($B$3,$B$6),MATCH(1,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>183</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2182,23 +2182,23 @@
       </c>
       <c r="B13" s="11" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J13))</f>
-        <v>Bir ayrıtı 3 birim olan küp, birim küplerden oluşturuluyor ve dış yüzeyinin tamamı boyanıyor. Hiç boyanmamış kaç birim küp vardır?</v>
+        <v>Bir ayrıtı 5 birim olan küp, birim küplerden oluşturuluyor ve dış yüzeyinin tamamı boyanıyor. Yalnızca 2 yüzü boyalı kaç birim küp vardır?</v>
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J13))</f>
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="D13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J13))</f>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J13))</f>
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="F13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J13))</f>
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="G13" s="12" t="str">
         <f aca="false">IF($J13="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J13))</f>
@@ -2210,71 +2210,71 @@
       </c>
       <c r="J13" s="10" t="n">
         <f aca="false">IF(2&lt;=MIN($B$3,$B$6),MATCH(2,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>215</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="n">
         <f aca="false">IF($J14="","",3)</f>
         <v>3</v>
       </c>
       <c r="B14" s="11" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J14))</f>
-        <v>Bir yüzünün alanı 49 cm² olan küpün bir ayrıtı kaç cm'dir?</v>
+        <v>(1 + 2)³ ifadesinin değeri kaçtır?</v>
       </c>
       <c r="C14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J14))</f>
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J14))</f>
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J14))</f>
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J14))</f>
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J14))</f>
-        <v>Küpün Özellikleri</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H14" s="12" t="str">
         <f aca="false">IF($J14="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J14))</f>
-        <v>Orta</v>
+        <v>Zor</v>
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">IF(3&lt;=MIN($B$3,$B$6),MATCH(3,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="n">
         <f aca="false">IF($J15="","",4)</f>
         <v>4</v>
       </c>
       <c r="B15" s="11" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J15))</f>
-        <v>5³ ifadesinin değeri kaçtır?</v>
+        <v>(3 + 3)³ ifadesinin değeri kaçtır?</v>
       </c>
       <c r="C15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J15))</f>
-        <v>130</v>
+        <v>18</v>
       </c>
       <c r="D15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J15))</f>
-        <v>125</v>
+        <v>216</v>
       </c>
       <c r="E15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J15))</f>
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="F15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J15))</f>
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="G15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J15))</f>
@@ -2282,37 +2282,37 @@
       </c>
       <c r="H15" s="12" t="str">
         <f aca="false">IF($J15="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J15))</f>
-        <v>Kolay</v>
+        <v>Zor</v>
       </c>
       <c r="J15" s="10" t="n">
         <f aca="false">IF(4&lt;=MIN($B$3,$B$6),MATCH(4,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="n">
         <f aca="false">IF($J16="","",5)</f>
         <v>5</v>
       </c>
       <c r="B16" s="11" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J16))</f>
-        <v>Küpün bir köşesinde kaç ayrıt birleşir?</v>
+        <v>Bir ayrıtı 7 cm olan küpün tüm ayrıtlarının uzunlukları toplamı kaç cm'dir?</v>
       </c>
       <c r="C16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J16))</f>
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="D16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J16))</f>
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="E16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J16))</f>
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J16))</f>
-        <v>6</v>
+        <v>343</v>
       </c>
       <c r="G16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J16))</f>
@@ -2320,49 +2320,49 @@
       </c>
       <c r="H16" s="12" t="str">
         <f aca="false">IF($J16="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J16))</f>
-        <v>Kolay</v>
+        <v>Orta</v>
       </c>
       <c r="J16" s="10" t="n">
         <f aca="false">IF(5&lt;=MIN($B$3,$B$6),MATCH(5,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>173</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="n">
         <f aca="false">IF($J17="","",6)</f>
         <v>6</v>
       </c>
       <c r="B17" s="11" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J17))</f>
-        <v>Bir ayrıtı 3 dm olan küp şeklindeki boş akvaryum tamamen doldurulursa kaç litre su alır? (1 dm³ = 1 L)</v>
+        <v>Küpü 512 olan doğal sayı kaçtır?</v>
       </c>
       <c r="C17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J17))</f>
-        <v>9 L</v>
+        <v>8</v>
       </c>
       <c r="D17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J17))</f>
-        <v>28 L</v>
+        <v>10</v>
       </c>
       <c r="E17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J17))</f>
-        <v>27 L</v>
+        <v>7</v>
       </c>
       <c r="F17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J17))</f>
-        <v>54 L</v>
+        <v>9</v>
       </c>
       <c r="G17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J17))</f>
-        <v>Küpün Hacmi</v>
+        <v>Sayının Küpü</v>
       </c>
       <c r="H17" s="12" t="str">
         <f aca="false">IF($J17="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J17))</f>
-        <v>Zor</v>
+        <v>Orta</v>
       </c>
       <c r="J17" s="10" t="n">
         <f aca="false">IF(6&lt;=MIN($B$3,$B$6),MATCH(6,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>153</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2372,23 +2372,23 @@
       </c>
       <c r="B18" s="11" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J18))</f>
-        <v>2³ + 5² işleminin sonucu kaçtır?</v>
+        <v>Aşağıdakilerden hangisi bir doğal sayının küpü değildir?</v>
       </c>
       <c r="C18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J18))</f>
-        <v>16</v>
+        <v>343</v>
       </c>
       <c r="D18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J18))</f>
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="E18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J18))</f>
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J18))</f>
-        <v>18</v>
+        <v>512</v>
       </c>
       <c r="G18" s="12" t="str">
         <f aca="false">IF($J18="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J18))</f>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J18" s="10" t="n">
         <f aca="false">IF(7&lt;=MIN($B$3,$B$6),MATCH(7,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>37</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2410,23 +2410,23 @@
       </c>
       <c r="B19" s="11" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J19))</f>
-        <v>3³ ifadesinin değeri kaçtır?</v>
+        <v>Bir doğal sayının küpünün 5 fazlası 32'dir. Bu sayı kaçtır?</v>
       </c>
       <c r="C19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J19))</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J19))</f>
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J19))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J19))</f>
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="G19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J19))</f>
@@ -2434,11 +2434,11 @@
       </c>
       <c r="H19" s="12" t="str">
         <f aca="false">IF($J19="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J19))</f>
-        <v>Kolay</v>
+        <v>Zor</v>
       </c>
       <c r="J19" s="10" t="n">
         <f aca="false">IF(8&lt;=MIN($B$3,$B$6),MATCH(8,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>3</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2448,23 +2448,23 @@
       </c>
       <c r="B20" s="11" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J20))</f>
-        <v>Bir ayrıtı 7 cm olan küpün yüzey alanı kaç cm²'dir?</v>
+        <v>Bir ayrıtı 10 cm olan küpün yüzey alanı kaç cm²'dir?</v>
       </c>
       <c r="C20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J20))</f>
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="D20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J20))</f>
-        <v>294</v>
+        <v>400</v>
       </c>
       <c r="E20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J20))</f>
-        <v>343</v>
+        <v>600</v>
       </c>
       <c r="F20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J20))</f>
-        <v>196</v>
+        <v>1000</v>
       </c>
       <c r="G20" s="12" t="str">
         <f aca="false">IF($J20="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J20))</f>
@@ -2476,37 +2476,37 @@
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">IF(9&lt;=MIN($B$3,$B$6),MATCH(9,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>191</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="n">
         <f aca="false">IF($J21="","",10)</f>
         <v>10</v>
       </c>
       <c r="B21" s="11" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$D$2:$D$1001,$J21))</f>
-        <v>10³ ifadesinin değeri kaçtır?</v>
+        <v>Bir ayrıtı 8 cm olan küpün hacmi kaç cm³'tür?</v>
       </c>
       <c r="C21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$E$2:$E$1001,$J21))</f>
-        <v>1000</v>
+        <v>64</v>
       </c>
       <c r="D21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$F$2:$F$1001,$J21))</f>
-        <v>100</v>
+        <v>384</v>
       </c>
       <c r="E21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$G$2:$G$1001,$J21))</f>
-        <v>30</v>
+        <v>512</v>
       </c>
       <c r="F21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$H$2:$H$1001,$J21))</f>
-        <v>1010</v>
+        <v>24</v>
       </c>
       <c r="G21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$B$2:$B$1001,$J21))</f>
-        <v>Sayının Küpü</v>
+        <v>Küpün Hacmi</v>
       </c>
       <c r="H21" s="12" t="str">
         <f aca="false">IF($J21="","",INDEX('Soru Havuzu'!$C$2:$C$1001,$J21))</f>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="J21" s="10" t="n">
         <f aca="false">IF(10&lt;=MIN($B$3,$B$6),MATCH(10,'Soru Havuzu'!$L$2:$L$1001,0),"")</f>
-        <v>10</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6063,11 +6063,11 @@
       </c>
       <c r="K2" s="10" t="n">
         <f aca="true">IF($J2=1,RAND(),-1)</f>
-        <v>0.401790495328625</v>
+        <v>0.324194356059361</v>
       </c>
       <c r="L2" s="10" t="n">
         <f aca="false">IF($J2=1,RANK($K2,$K$2:$K$1001),"")</f>
-        <v>134</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6104,11 +6104,11 @@
       </c>
       <c r="K3" s="10" t="n">
         <f aca="true">IF($J3=1,RAND(),-1)</f>
-        <v>0.270641339505107</v>
+        <v>0.60621200332643</v>
       </c>
       <c r="L3" s="10" t="n">
         <f aca="false">IF($J3=1,RANK($K3,$K$2:$K$1001),"")</f>
-        <v>163</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6145,11 +6145,11 @@
       </c>
       <c r="K4" s="10" t="n">
         <f aca="true">IF($J4=1,RAND(),-1)</f>
-        <v>0.965586382232213</v>
+        <v>0.941225340065023</v>
       </c>
       <c r="L4" s="10" t="n">
         <f aca="false">IF($J4=1,RANK($K4,$K$2:$K$1001),"")</f>
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6186,11 +6186,11 @@
       </c>
       <c r="K5" s="10" t="n">
         <f aca="true">IF($J5=1,RAND(),-1)</f>
-        <v>0.195813075787506</v>
+        <v>0.885390369764143</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">IF($J5=1,RANK($K5,$K$2:$K$1001),"")</f>
-        <v>191</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6227,11 +6227,11 @@
       </c>
       <c r="K6" s="10" t="n">
         <f aca="true">IF($J6=1,RAND(),-1)</f>
-        <v>0.982684786987049</v>
+        <v>0.249317177868618</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">IF($J6=1,RANK($K6,$K$2:$K$1001),"")</f>
-        <v>4</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6268,11 +6268,11 @@
       </c>
       <c r="K7" s="10" t="n">
         <f aca="true">IF($J7=1,RAND(),-1)</f>
-        <v>0.17632037147737</v>
+        <v>0.487403232133836</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">IF($J7=1,RANK($K7,$K$2:$K$1001),"")</f>
-        <v>192</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6309,11 +6309,11 @@
       </c>
       <c r="K8" s="10" t="n">
         <f aca="true">IF($J8=1,RAND(),-1)</f>
-        <v>0.452620305531729</v>
+        <v>0.52777662877659</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">IF($J8=1,RANK($K8,$K$2:$K$1001),"")</f>
-        <v>124</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6350,11 +6350,11 @@
       </c>
       <c r="K9" s="10" t="n">
         <f aca="true">IF($J9=1,RAND(),-1)</f>
-        <v>0.12334482841132</v>
+        <v>0.928348992835433</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">IF($J9=1,RANK($K9,$K$2:$K$1001),"")</f>
-        <v>201</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6391,11 +6391,11 @@
       </c>
       <c r="K10" s="10" t="n">
         <f aca="true">IF($J10=1,RAND(),-1)</f>
-        <v>0.76662941253123</v>
+        <v>0.308591638248976</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">IF($J10=1,RANK($K10,$K$2:$K$1001),"")</f>
-        <v>45</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6432,11 +6432,11 @@
       </c>
       <c r="K11" s="10" t="n">
         <f aca="true">IF($J11=1,RAND(),-1)</f>
-        <v>0.948054806682241</v>
+        <v>0.0589177662680296</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">IF($J11=1,RANK($K11,$K$2:$K$1001),"")</f>
-        <v>10</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6473,11 +6473,11 @@
       </c>
       <c r="K12" s="10" t="n">
         <f aca="true">IF($J12=1,RAND(),-1)</f>
-        <v>0.621598539142692</v>
+        <v>0.215484287893834</v>
       </c>
       <c r="L12" s="10" t="n">
         <f aca="false">IF($J12=1,RANK($K12,$K$2:$K$1001),"")</f>
-        <v>89</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6514,11 +6514,11 @@
       </c>
       <c r="K13" s="10" t="n">
         <f aca="true">IF($J13=1,RAND(),-1)</f>
-        <v>0.458327904043481</v>
+        <v>0.87175520068424</v>
       </c>
       <c r="L13" s="10" t="n">
         <f aca="false">IF($J13=1,RANK($K13,$K$2:$K$1001),"")</f>
-        <v>123</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6555,11 +6555,11 @@
       </c>
       <c r="K14" s="10" t="n">
         <f aca="true">IF($J14=1,RAND(),-1)</f>
-        <v>0.44691130729089</v>
+        <v>0.468055484320037</v>
       </c>
       <c r="L14" s="10" t="n">
         <f aca="false">IF($J14=1,RANK($K14,$K$2:$K$1001),"")</f>
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6596,11 +6596,11 @@
       </c>
       <c r="K15" s="10" t="n">
         <f aca="true">IF($J15=1,RAND(),-1)</f>
-        <v>0.648730499163885</v>
+        <v>0.373696132003824</v>
       </c>
       <c r="L15" s="10" t="n">
         <f aca="false">IF($J15=1,RANK($K15,$K$2:$K$1001),"")</f>
-        <v>84</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6637,11 +6637,11 @@
       </c>
       <c r="K16" s="10" t="n">
         <f aca="true">IF($J16=1,RAND(),-1)</f>
-        <v>0.338123648188616</v>
+        <v>0.531740184321222</v>
       </c>
       <c r="L16" s="10" t="n">
         <f aca="false">IF($J16=1,RANK($K16,$K$2:$K$1001),"")</f>
-        <v>149</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6678,11 +6678,11 @@
       </c>
       <c r="K17" s="10" t="n">
         <f aca="true">IF($J17=1,RAND(),-1)</f>
-        <v>0.573864548316189</v>
+        <v>0.495333706820906</v>
       </c>
       <c r="L17" s="10" t="n">
         <f aca="false">IF($J17=1,RANK($K17,$K$2:$K$1001),"")</f>
-        <v>96</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6719,11 +6719,11 @@
       </c>
       <c r="K18" s="10" t="n">
         <f aca="true">IF($J18=1,RAND(),-1)</f>
-        <v>0.0601356146533304</v>
+        <v>0.0689452581166452</v>
       </c>
       <c r="L18" s="10" t="n">
         <f aca="false">IF($J18=1,RANK($K18,$K$2:$K$1001),"")</f>
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="K19" s="10" t="n">
         <f aca="true">IF($J19=1,RAND(),-1)</f>
-        <v>0.904336703453878</v>
+        <v>0.79718541527479</v>
       </c>
       <c r="L19" s="10" t="n">
         <f aca="false">IF($J19=1,RANK($K19,$K$2:$K$1001),"")</f>
-        <v>18</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6801,11 +6801,11 @@
       </c>
       <c r="K20" s="10" t="n">
         <f aca="true">IF($J20=1,RAND(),-1)</f>
-        <v>0.216423731909305</v>
+        <v>0.314442156646051</v>
       </c>
       <c r="L20" s="10" t="n">
         <f aca="false">IF($J20=1,RANK($K20,$K$2:$K$1001),"")</f>
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6842,11 +6842,11 @@
       </c>
       <c r="K21" s="10" t="n">
         <f aca="true">IF($J21=1,RAND(),-1)</f>
-        <v>0.734845784900409</v>
+        <v>0.144332504678708</v>
       </c>
       <c r="L21" s="10" t="n">
         <f aca="false">IF($J21=1,RANK($K21,$K$2:$K$1001),"")</f>
-        <v>59</v>
+        <v>192</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="K22" s="10" t="n">
         <f aca="true">IF($J22=1,RAND(),-1)</f>
-        <v>0.466798374005103</v>
+        <v>0.867779699637747</v>
       </c>
       <c r="L22" s="10" t="n">
         <f aca="false">IF($J22=1,RANK($K22,$K$2:$K$1001),"")</f>
-        <v>119</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6924,11 +6924,11 @@
       </c>
       <c r="K23" s="10" t="n">
         <f aca="true">IF($J23=1,RAND(),-1)</f>
-        <v>0.8615541962897</v>
+        <v>0.820367246021713</v>
       </c>
       <c r="L23" s="10" t="n">
         <f aca="false">IF($J23=1,RANK($K23,$K$2:$K$1001),"")</f>
-        <v>29</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6965,11 +6965,11 @@
       </c>
       <c r="K24" s="10" t="n">
         <f aca="true">IF($J24=1,RAND(),-1)</f>
-        <v>0.791390689534383</v>
+        <v>0.523967620690274</v>
       </c>
       <c r="L24" s="10" t="n">
         <f aca="false">IF($J24=1,RANK($K24,$K$2:$K$1001),"")</f>
-        <v>39</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7006,11 +7006,11 @@
       </c>
       <c r="K25" s="10" t="n">
         <f aca="true">IF($J25=1,RAND(),-1)</f>
-        <v>0.244657422641741</v>
+        <v>0.182497735741151</v>
       </c>
       <c r="L25" s="10" t="n">
         <f aca="false">IF($J25=1,RANK($K25,$K$2:$K$1001),"")</f>
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7047,11 +7047,11 @@
       </c>
       <c r="K26" s="10" t="n">
         <f aca="true">IF($J26=1,RAND(),-1)</f>
-        <v>0.350708021994324</v>
+        <v>0.105069284707777</v>
       </c>
       <c r="L26" s="10" t="n">
         <f aca="false">IF($J26=1,RANK($K26,$K$2:$K$1001),"")</f>
-        <v>145</v>
+        <v>200</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7088,11 +7088,11 @@
       </c>
       <c r="K27" s="10" t="n">
         <f aca="true">IF($J27=1,RAND(),-1)</f>
-        <v>0.840393098282053</v>
+        <v>0.904183459126336</v>
       </c>
       <c r="L27" s="10" t="n">
         <f aca="false">IF($J27=1,RANK($K27,$K$2:$K$1001),"")</f>
-        <v>33</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7129,11 +7129,11 @@
       </c>
       <c r="K28" s="10" t="n">
         <f aca="true">IF($J28=1,RAND(),-1)</f>
-        <v>0.843615942388549</v>
+        <v>0.026560461283536</v>
       </c>
       <c r="L28" s="10" t="n">
         <f aca="false">IF($J28=1,RANK($K28,$K$2:$K$1001),"")</f>
-        <v>32</v>
+        <v>216</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7170,11 +7170,11 @@
       </c>
       <c r="K29" s="10" t="n">
         <f aca="true">IF($J29=1,RAND(),-1)</f>
-        <v>0.751863785052589</v>
+        <v>0.299389777810593</v>
       </c>
       <c r="L29" s="10" t="n">
         <f aca="false">IF($J29=1,RANK($K29,$K$2:$K$1001),"")</f>
-        <v>52</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7211,11 +7211,11 @@
       </c>
       <c r="K30" s="10" t="n">
         <f aca="true">IF($J30=1,RAND(),-1)</f>
-        <v>0.68817368126261</v>
+        <v>0.529543507562507</v>
       </c>
       <c r="L30" s="10" t="n">
         <f aca="false">IF($J30=1,RANK($K30,$K$2:$K$1001),"")</f>
-        <v>69</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7252,11 +7252,11 @@
       </c>
       <c r="K31" s="10" t="n">
         <f aca="true">IF($J31=1,RAND(),-1)</f>
-        <v>0.0227915968839275</v>
+        <v>0.203001067211699</v>
       </c>
       <c r="L31" s="10" t="n">
         <f aca="false">IF($J31=1,RANK($K31,$K$2:$K$1001),"")</f>
-        <v>221</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7293,11 +7293,11 @@
       </c>
       <c r="K32" s="10" t="n">
         <f aca="true">IF($J32=1,RAND(),-1)</f>
-        <v>0.427730869241869</v>
+        <v>0.0176398596386105</v>
       </c>
       <c r="L32" s="10" t="n">
         <f aca="false">IF($J32=1,RANK($K32,$K$2:$K$1001),"")</f>
-        <v>131</v>
+        <v>220</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7334,11 +7334,11 @@
       </c>
       <c r="K33" s="10" t="n">
         <f aca="true">IF($J33=1,RAND(),-1)</f>
-        <v>0.445745721322508</v>
+        <v>0.637330049098196</v>
       </c>
       <c r="L33" s="10" t="n">
         <f aca="false">IF($J33=1,RANK($K33,$K$2:$K$1001),"")</f>
-        <v>128</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7375,11 +7375,11 @@
       </c>
       <c r="K34" s="10" t="n">
         <f aca="true">IF($J34=1,RAND(),-1)</f>
-        <v>0.220301691470674</v>
+        <v>0.979075909884595</v>
       </c>
       <c r="L34" s="10" t="n">
         <f aca="false">IF($J34=1,RANK($K34,$K$2:$K$1001),"")</f>
-        <v>179</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7416,11 +7416,11 @@
       </c>
       <c r="K35" s="10" t="n">
         <f aca="true">IF($J35=1,RAND(),-1)</f>
-        <v>0.682209797115888</v>
+        <v>0.845424163565762</v>
       </c>
       <c r="L35" s="10" t="n">
         <f aca="false">IF($J35=1,RANK($K35,$K$2:$K$1001),"")</f>
-        <v>72</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7457,11 +7457,11 @@
       </c>
       <c r="K36" s="10" t="n">
         <f aca="true">IF($J36=1,RAND(),-1)</f>
-        <v>0.0960798977981393</v>
+        <v>0.502529235315853</v>
       </c>
       <c r="L36" s="10" t="n">
         <f aca="false">IF($J36=1,RANK($K36,$K$2:$K$1001),"")</f>
-        <v>205</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7498,11 +7498,11 @@
       </c>
       <c r="K37" s="10" t="n">
         <f aca="true">IF($J37=1,RAND(),-1)</f>
-        <v>0.692902124286699</v>
+        <v>0.884166118518258</v>
       </c>
       <c r="L37" s="10" t="n">
         <f aca="false">IF($J37=1,RANK($K37,$K$2:$K$1001),"")</f>
-        <v>67</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7539,11 +7539,11 @@
       </c>
       <c r="K38" s="10" t="n">
         <f aca="true">IF($J38=1,RAND(),-1)</f>
-        <v>0.977111994593651</v>
+        <v>0.767105901699038</v>
       </c>
       <c r="L38" s="10" t="n">
         <f aca="false">IF($J38=1,RANK($K38,$K$2:$K$1001),"")</f>
-        <v>7</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7580,11 +7580,11 @@
       </c>
       <c r="K39" s="10" t="n">
         <f aca="true">IF($J39=1,RAND(),-1)</f>
-        <v>0.400035082626107</v>
+        <v>0.885374321115402</v>
       </c>
       <c r="L39" s="10" t="n">
         <f aca="false">IF($J39=1,RANK($K39,$K$2:$K$1001),"")</f>
-        <v>136</v>
+        <v>28</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7621,11 +7621,11 @@
       </c>
       <c r="K40" s="10" t="n">
         <f aca="true">IF($J40=1,RAND(),-1)</f>
-        <v>0.678477002933716</v>
+        <v>0.352808600700951</v>
       </c>
       <c r="L40" s="10" t="n">
         <f aca="false">IF($J40=1,RANK($K40,$K$2:$K$1001),"")</f>
-        <v>74</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7662,11 +7662,11 @@
       </c>
       <c r="K41" s="10" t="n">
         <f aca="true">IF($J41=1,RAND(),-1)</f>
-        <v>0.221261983730159</v>
+        <v>0.421758947797071</v>
       </c>
       <c r="L41" s="10" t="n">
         <f aca="false">IF($J41=1,RANK($K41,$K$2:$K$1001),"")</f>
-        <v>178</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7703,11 +7703,11 @@
       </c>
       <c r="K42" s="10" t="n">
         <f aca="true">IF($J42=1,RAND(),-1)</f>
-        <v>0.762313580187798</v>
+        <v>0.915879240040056</v>
       </c>
       <c r="L42" s="10" t="n">
         <f aca="false">IF($J42=1,RANK($K42,$K$2:$K$1001),"")</f>
-        <v>46</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7744,11 +7744,11 @@
       </c>
       <c r="K43" s="10" t="n">
         <f aca="true">IF($J43=1,RAND(),-1)</f>
-        <v>0.880723488905978</v>
+        <v>0.473621133114158</v>
       </c>
       <c r="L43" s="10" t="n">
         <f aca="false">IF($J43=1,RANK($K43,$K$2:$K$1001),"")</f>
-        <v>24</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7785,11 +7785,11 @@
       </c>
       <c r="K44" s="10" t="n">
         <f aca="true">IF($J44=1,RAND(),-1)</f>
-        <v>0.573442898183365</v>
+        <v>0.0763605765319013</v>
       </c>
       <c r="L44" s="10" t="n">
         <f aca="false">IF($J44=1,RANK($K44,$K$2:$K$1001),"")</f>
-        <v>97</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7826,11 +7826,11 @@
       </c>
       <c r="K45" s="10" t="n">
         <f aca="true">IF($J45=1,RAND(),-1)</f>
-        <v>0.215244272613178</v>
+        <v>0.431460374762144</v>
       </c>
       <c r="L45" s="10" t="n">
         <f aca="false">IF($J45=1,RANK($K45,$K$2:$K$1001),"")</f>
-        <v>181</v>
+        <v>133</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7867,11 +7867,11 @@
       </c>
       <c r="K46" s="10" t="n">
         <f aca="true">IF($J46=1,RAND(),-1)</f>
-        <v>0.362908321866177</v>
+        <v>0.998915487498521</v>
       </c>
       <c r="L46" s="10" t="n">
         <f aca="false">IF($J46=1,RANK($K46,$K$2:$K$1001),"")</f>
-        <v>142</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7908,11 +7908,11 @@
       </c>
       <c r="K47" s="10" t="n">
         <f aca="true">IF($J47=1,RAND(),-1)</f>
-        <v>0.0135532480757304</v>
+        <v>0.524083253209881</v>
       </c>
       <c r="L47" s="10" t="n">
         <f aca="false">IF($J47=1,RANK($K47,$K$2:$K$1001),"")</f>
-        <v>222</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7949,11 +7949,11 @@
       </c>
       <c r="K48" s="10" t="n">
         <f aca="true">IF($J48=1,RAND(),-1)</f>
-        <v>0.0743131790430523</v>
+        <v>0.467901335359731</v>
       </c>
       <c r="L48" s="10" t="n">
         <f aca="false">IF($J48=1,RANK($K48,$K$2:$K$1001),"")</f>
-        <v>211</v>
+        <v>128</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7990,11 +7990,11 @@
       </c>
       <c r="K49" s="10" t="n">
         <f aca="true">IF($J49=1,RAND(),-1)</f>
-        <v>0.738615163116261</v>
+        <v>0.141908538298381</v>
       </c>
       <c r="L49" s="10" t="n">
         <f aca="false">IF($J49=1,RANK($K49,$K$2:$K$1001),"")</f>
-        <v>57</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8031,11 +8031,11 @@
       </c>
       <c r="K50" s="10" t="n">
         <f aca="true">IF($J50=1,RAND(),-1)</f>
-        <v>0.784024237119484</v>
+        <v>0.32581702659774</v>
       </c>
       <c r="L50" s="10" t="n">
         <f aca="false">IF($J50=1,RANK($K50,$K$2:$K$1001),"")</f>
-        <v>40</v>
+        <v>160</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8072,11 +8072,11 @@
       </c>
       <c r="K51" s="10" t="n">
         <f aca="true">IF($J51=1,RAND(),-1)</f>
-        <v>0.747539022888891</v>
+        <v>0.0225837133364474</v>
       </c>
       <c r="L51" s="10" t="n">
         <f aca="false">IF($J51=1,RANK($K51,$K$2:$K$1001),"")</f>
-        <v>54</v>
+        <v>218</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8113,11 +8113,11 @@
       </c>
       <c r="K52" s="10" t="n">
         <f aca="true">IF($J52=1,RAND(),-1)</f>
-        <v>0.209782545801478</v>
+        <v>0.00102019733120313</v>
       </c>
       <c r="L52" s="10" t="n">
         <f aca="false">IF($J52=1,RANK($K52,$K$2:$K$1001),"")</f>
-        <v>183</v>
+        <v>223</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8154,11 +8154,11 @@
       </c>
       <c r="K53" s="10" t="n">
         <f aca="true">IF($J53=1,RAND(),-1)</f>
-        <v>0.696554397787546</v>
+        <v>0.88707257126224</v>
       </c>
       <c r="L53" s="10" t="n">
         <f aca="false">IF($J53=1,RANK($K53,$K$2:$K$1001),"")</f>
-        <v>65</v>
+        <v>26</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8195,11 +8195,11 @@
       </c>
       <c r="K54" s="10" t="n">
         <f aca="true">IF($J54=1,RAND(),-1)</f>
-        <v>0.221279521917633</v>
+        <v>0.454006011351655</v>
       </c>
       <c r="L54" s="10" t="n">
         <f aca="false">IF($J54=1,RANK($K54,$K$2:$K$1001),"")</f>
-        <v>177</v>
+        <v>131</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8236,11 +8236,11 @@
       </c>
       <c r="K55" s="10" t="n">
         <f aca="true">IF($J55=1,RAND(),-1)</f>
-        <v>0.871889297198561</v>
+        <v>0.350962202876998</v>
       </c>
       <c r="L55" s="10" t="n">
         <f aca="false">IF($J55=1,RANK($K55,$K$2:$K$1001),"")</f>
-        <v>26</v>
+        <v>153</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8277,11 +8277,11 @@
       </c>
       <c r="K56" s="10" t="n">
         <f aca="true">IF($J56=1,RAND(),-1)</f>
-        <v>0.4465025555367</v>
+        <v>0.880721568543099</v>
       </c>
       <c r="L56" s="10" t="n">
         <f aca="false">IF($J56=1,RANK($K56,$K$2:$K$1001),"")</f>
-        <v>127</v>
+        <v>31</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8318,11 +8318,11 @@
       </c>
       <c r="K57" s="10" t="n">
         <f aca="true">IF($J57=1,RAND(),-1)</f>
-        <v>0.372086751790402</v>
+        <v>0.180806358888605</v>
       </c>
       <c r="L57" s="10" t="n">
         <f aca="false">IF($J57=1,RANK($K57,$K$2:$K$1001),"")</f>
-        <v>141</v>
+        <v>184</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8359,11 +8359,11 @@
       </c>
       <c r="K58" s="10" t="n">
         <f aca="true">IF($J58=1,RAND(),-1)</f>
-        <v>0.425043563848971</v>
+        <v>0.460445897039425</v>
       </c>
       <c r="L58" s="10" t="n">
         <f aca="false">IF($J58=1,RANK($K58,$K$2:$K$1001),"")</f>
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8400,11 +8400,11 @@
       </c>
       <c r="K59" s="10" t="n">
         <f aca="true">IF($J59=1,RAND(),-1)</f>
-        <v>0.314997672579082</v>
+        <v>0.8306435421273</v>
       </c>
       <c r="L59" s="10" t="n">
         <f aca="false">IF($J59=1,RANK($K59,$K$2:$K$1001),"")</f>
-        <v>155</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8441,11 +8441,11 @@
       </c>
       <c r="K60" s="10" t="n">
         <f aca="true">IF($J60=1,RAND(),-1)</f>
-        <v>0.522303866033181</v>
+        <v>0.315465295669966</v>
       </c>
       <c r="L60" s="10" t="n">
         <f aca="false">IF($J60=1,RANK($K60,$K$2:$K$1001),"")</f>
-        <v>108</v>
+        <v>164</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8482,11 +8482,11 @@
       </c>
       <c r="K61" s="10" t="n">
         <f aca="true">IF($J61=1,RAND(),-1)</f>
-        <v>0.292853094160772</v>
+        <v>0.66952438538844</v>
       </c>
       <c r="L61" s="10" t="n">
         <f aca="false">IF($J61=1,RANK($K61,$K$2:$K$1001),"")</f>
-        <v>160</v>
+        <v>74</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8523,11 +8523,11 @@
       </c>
       <c r="K62" s="10" t="n">
         <f aca="true">IF($J62=1,RAND(),-1)</f>
-        <v>0.058016183756116</v>
+        <v>0.957481947506199</v>
       </c>
       <c r="L62" s="10" t="n">
         <f aca="false">IF($J62=1,RANK($K62,$K$2:$K$1001),"")</f>
-        <v>215</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8564,11 +8564,11 @@
       </c>
       <c r="K63" s="10" t="n">
         <f aca="true">IF($J63=1,RAND(),-1)</f>
-        <v>0.329955147193178</v>
+        <v>0.440769440033902</v>
       </c>
       <c r="L63" s="10" t="n">
         <f aca="false">IF($J63=1,RANK($K63,$K$2:$K$1001),"")</f>
-        <v>152</v>
+        <v>132</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8605,11 +8605,11 @@
       </c>
       <c r="K64" s="10" t="n">
         <f aca="true">IF($J64=1,RAND(),-1)</f>
-        <v>0.643412776415664</v>
+        <v>0.632235517874809</v>
       </c>
       <c r="L64" s="10" t="n">
         <f aca="false">IF($J64=1,RANK($K64,$K$2:$K$1001),"")</f>
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8646,11 +8646,11 @@
       </c>
       <c r="K65" s="10" t="n">
         <f aca="true">IF($J65=1,RAND(),-1)</f>
-        <v>0.922554499432087</v>
+        <v>0.973772376514826</v>
       </c>
       <c r="L65" s="10" t="n">
         <f aca="false">IF($J65=1,RANK($K65,$K$2:$K$1001),"")</f>
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8687,11 +8687,11 @@
       </c>
       <c r="K66" s="10" t="n">
         <f aca="true">IF($J66=1,RAND(),-1)</f>
-        <v>0.751870292434175</v>
+        <v>0.24996767003063</v>
       </c>
       <c r="L66" s="10" t="n">
         <f aca="false">IF($J66=1,RANK($K66,$K$2:$K$1001),"")</f>
-        <v>51</v>
+        <v>171</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8728,11 +8728,11 @@
       </c>
       <c r="K67" s="10" t="n">
         <f aca="true">IF($J67=1,RAND(),-1)</f>
-        <v>0.561625313716552</v>
+        <v>0.148975108053823</v>
       </c>
       <c r="L67" s="10" t="n">
         <f aca="false">IF($J67=1,RANK($K67,$K$2:$K$1001),"")</f>
-        <v>99</v>
+        <v>191</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8769,11 +8769,11 @@
       </c>
       <c r="K68" s="10" t="n">
         <f aca="true">IF($J68=1,RAND(),-1)</f>
-        <v>0.591914204363883</v>
+        <v>0.797368605136827</v>
       </c>
       <c r="L68" s="10" t="n">
         <f aca="false">IF($J68=1,RANK($K68,$K$2:$K$1001),"")</f>
-        <v>94</v>
+        <v>54</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8810,11 +8810,11 @@
       </c>
       <c r="K69" s="10" t="n">
         <f aca="true">IF($J69=1,RAND(),-1)</f>
-        <v>0.884451037768383</v>
+        <v>0.385218870851857</v>
       </c>
       <c r="L69" s="10" t="n">
         <f aca="false">IF($J69=1,RANK($K69,$K$2:$K$1001),"")</f>
-        <v>22</v>
+        <v>146</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8851,11 +8851,11 @@
       </c>
       <c r="K70" s="10" t="n">
         <f aca="true">IF($J70=1,RAND(),-1)</f>
-        <v>0.77351631504857</v>
+        <v>0.880041319290761</v>
       </c>
       <c r="L70" s="10" t="n">
         <f aca="false">IF($J70=1,RANK($K70,$K$2:$K$1001),"")</f>
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8892,11 +8892,11 @@
       </c>
       <c r="K71" s="10" t="n">
         <f aca="true">IF($J71=1,RAND(),-1)</f>
-        <v>0.822324980362926</v>
+        <v>0.924473591044291</v>
       </c>
       <c r="L71" s="10" t="n">
         <f aca="false">IF($J71=1,RANK($K71,$K$2:$K$1001),"")</f>
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="K72" s="10" t="n">
         <f aca="true">IF($J72=1,RAND(),-1)</f>
-        <v>0.321872213271924</v>
+        <v>0.132970919119191</v>
       </c>
       <c r="L72" s="10" t="n">
         <f aca="false">IF($J72=1,RANK($K72,$K$2:$K$1001),"")</f>
-        <v>153</v>
+        <v>195</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8974,11 +8974,11 @@
       </c>
       <c r="K73" s="10" t="n">
         <f aca="true">IF($J73=1,RAND(),-1)</f>
-        <v>0.667784451134759</v>
+        <v>0.791786185527462</v>
       </c>
       <c r="L73" s="10" t="n">
         <f aca="false">IF($J73=1,RANK($K73,$K$2:$K$1001),"")</f>
-        <v>77</v>
+        <v>56</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9015,11 +9015,11 @@
       </c>
       <c r="K74" s="10" t="n">
         <f aca="true">IF($J74=1,RAND(),-1)</f>
-        <v>0.133797529275187</v>
+        <v>0.844025702279627</v>
       </c>
       <c r="L74" s="10" t="n">
         <f aca="false">IF($J74=1,RANK($K74,$K$2:$K$1001),"")</f>
-        <v>199</v>
+        <v>43</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9056,11 +9056,11 @@
       </c>
       <c r="K75" s="10" t="n">
         <f aca="true">IF($J75=1,RAND(),-1)</f>
-        <v>0.254413503080995</v>
+        <v>0.400218103690462</v>
       </c>
       <c r="L75" s="10" t="n">
         <f aca="false">IF($J75=1,RANK($K75,$K$2:$K$1001),"")</f>
-        <v>167</v>
+        <v>140</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9097,11 +9097,11 @@
       </c>
       <c r="K76" s="10" t="n">
         <f aca="true">IF($J76=1,RAND(),-1)</f>
-        <v>0.944840121334961</v>
+        <v>0.323874441275904</v>
       </c>
       <c r="L76" s="10" t="n">
         <f aca="false">IF($J76=1,RANK($K76,$K$2:$K$1001),"")</f>
-        <v>12</v>
+        <v>162</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9138,11 +9138,11 @@
       </c>
       <c r="K77" s="10" t="n">
         <f aca="true">IF($J77=1,RAND(),-1)</f>
-        <v>0.869479177874123</v>
+        <v>0.423150740608448</v>
       </c>
       <c r="L77" s="10" t="n">
         <f aca="false">IF($J77=1,RANK($K77,$K$2:$K$1001),"")</f>
-        <v>28</v>
+        <v>135</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9179,11 +9179,11 @@
       </c>
       <c r="K78" s="10" t="n">
         <f aca="true">IF($J78=1,RAND(),-1)</f>
-        <v>0.657307714572043</v>
+        <v>0.331004765621633</v>
       </c>
       <c r="L78" s="10" t="n">
         <f aca="false">IF($J78=1,RANK($K78,$K$2:$K$1001),"")</f>
-        <v>80</v>
+        <v>159</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9220,11 +9220,11 @@
       </c>
       <c r="K79" s="10" t="n">
         <f aca="true">IF($J79=1,RAND(),-1)</f>
-        <v>0.921501881533406</v>
+        <v>0.0458828659591226</v>
       </c>
       <c r="L79" s="10" t="n">
         <f aca="false">IF($J79=1,RANK($K79,$K$2:$K$1001),"")</f>
-        <v>16</v>
+        <v>214</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9261,11 +9261,11 @@
       </c>
       <c r="K80" s="10" t="n">
         <f aca="true">IF($J80=1,RAND(),-1)</f>
-        <v>0.265009583159018</v>
+        <v>0.0399144058483344</v>
       </c>
       <c r="L80" s="10" t="n">
         <f aca="false">IF($J80=1,RANK($K80,$K$2:$K$1001),"")</f>
-        <v>165</v>
+        <v>215</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9302,11 +9302,11 @@
       </c>
       <c r="K81" s="10" t="n">
         <f aca="true">IF($J81=1,RAND(),-1)</f>
-        <v>0.0952195569671441</v>
+        <v>0.842921902772925</v>
       </c>
       <c r="L81" s="10" t="n">
         <f aca="false">IF($J81=1,RANK($K81,$K$2:$K$1001),"")</f>
-        <v>206</v>
+        <v>44</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9343,11 +9343,11 @@
       </c>
       <c r="K82" s="10" t="n">
         <f aca="true">IF($J82=1,RAND(),-1)</f>
-        <v>0.921345169608819</v>
+        <v>0.660040512072826</v>
       </c>
       <c r="L82" s="10" t="n">
         <f aca="false">IF($J82=1,RANK($K82,$K$2:$K$1001),"")</f>
-        <v>17</v>
+        <v>78</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9384,11 +9384,11 @@
       </c>
       <c r="K83" s="10" t="n">
         <f aca="true">IF($J83=1,RAND(),-1)</f>
-        <v>0.720437804925562</v>
+        <v>0.986702757246564</v>
       </c>
       <c r="L83" s="10" t="n">
         <f aca="false">IF($J83=1,RANK($K83,$K$2:$K$1001),"")</f>
-        <v>61</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9425,11 +9425,11 @@
       </c>
       <c r="K84" s="10" t="n">
         <f aca="true">IF($J84=1,RAND(),-1)</f>
-        <v>0.882019226393073</v>
+        <v>0.508033512596879</v>
       </c>
       <c r="L84" s="10" t="n">
         <f aca="false">IF($J84=1,RANK($K84,$K$2:$K$1001),"")</f>
-        <v>23</v>
+        <v>109</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9466,11 +9466,11 @@
       </c>
       <c r="K85" s="10" t="n">
         <f aca="true">IF($J85=1,RAND(),-1)</f>
-        <v>0.599840158003984</v>
+        <v>0.0814825386460371</v>
       </c>
       <c r="L85" s="10" t="n">
         <f aca="false">IF($J85=1,RANK($K85,$K$2:$K$1001),"")</f>
-        <v>93</v>
+        <v>207</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9507,11 +9507,11 @@
       </c>
       <c r="K86" s="10" t="n">
         <f aca="true">IF($J86=1,RAND(),-1)</f>
-        <v>0.309414765566614</v>
+        <v>0.0974298484359966</v>
       </c>
       <c r="L86" s="10" t="n">
         <f aca="false">IF($J86=1,RANK($K86,$K$2:$K$1001),"")</f>
-        <v>157</v>
+        <v>204</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9548,11 +9548,11 @@
       </c>
       <c r="K87" s="10" t="n">
         <f aca="true">IF($J87=1,RAND(),-1)</f>
-        <v>0.770276488238241</v>
+        <v>0.0853044025055115</v>
       </c>
       <c r="L87" s="10" t="n">
         <f aca="false">IF($J87=1,RANK($K87,$K$2:$K$1001),"")</f>
-        <v>43</v>
+        <v>206</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9589,11 +9589,11 @@
       </c>
       <c r="K88" s="10" t="n">
         <f aca="true">IF($J88=1,RAND(),-1)</f>
-        <v>0.613643854318183</v>
+        <v>0.982066129950845</v>
       </c>
       <c r="L88" s="10" t="n">
         <f aca="false">IF($J88=1,RANK($K88,$K$2:$K$1001),"")</f>
-        <v>91</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9630,11 +9630,11 @@
       </c>
       <c r="K89" s="10" t="n">
         <f aca="true">IF($J89=1,RAND(),-1)</f>
-        <v>0.319035162616265</v>
+        <v>0.60950900105969</v>
       </c>
       <c r="L89" s="10" t="n">
         <f aca="false">IF($J89=1,RANK($K89,$K$2:$K$1001),"")</f>
-        <v>154</v>
+        <v>91</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9671,11 +9671,11 @@
       </c>
       <c r="K90" s="10" t="n">
         <f aca="true">IF($J90=1,RAND(),-1)</f>
-        <v>0.542459441864758</v>
+        <v>0.587291950265124</v>
       </c>
       <c r="L90" s="10" t="n">
         <f aca="false">IF($J90=1,RANK($K90,$K$2:$K$1001),"")</f>
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9712,11 +9712,11 @@
       </c>
       <c r="K91" s="10" t="n">
         <f aca="true">IF($J91=1,RAND(),-1)</f>
-        <v>0.759094058455269</v>
+        <v>0.972837272265946</v>
       </c>
       <c r="L91" s="10" t="n">
         <f aca="false">IF($J91=1,RANK($K91,$K$2:$K$1001),"")</f>
-        <v>47</v>
+        <v>8</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9753,11 +9753,11 @@
       </c>
       <c r="K92" s="10" t="n">
         <f aca="true">IF($J92=1,RAND(),-1)</f>
-        <v>0.479620124590537</v>
+        <v>0.266169234891242</v>
       </c>
       <c r="L92" s="10" t="n">
         <f aca="false">IF($J92=1,RANK($K92,$K$2:$K$1001),"")</f>
-        <v>118</v>
+        <v>170</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9794,11 +9794,11 @@
       </c>
       <c r="K93" s="10" t="n">
         <f aca="true">IF($J93=1,RAND(),-1)</f>
-        <v>0.548137814837727</v>
+        <v>0.718819109572753</v>
       </c>
       <c r="L93" s="10" t="n">
         <f aca="false">IF($J93=1,RANK($K93,$K$2:$K$1001),"")</f>
-        <v>104</v>
+        <v>66</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9835,11 +9835,11 @@
       </c>
       <c r="K94" s="10" t="n">
         <f aca="true">IF($J94=1,RAND(),-1)</f>
-        <v>0.80848002134682</v>
+        <v>0.519725648130786</v>
       </c>
       <c r="L94" s="10" t="n">
         <f aca="false">IF($J94=1,RANK($K94,$K$2:$K$1001),"")</f>
-        <v>38</v>
+        <v>106</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9876,11 +9876,11 @@
       </c>
       <c r="K95" s="10" t="n">
         <f aca="true">IF($J95=1,RAND(),-1)</f>
-        <v>0.635082793882476</v>
+        <v>0.487770288842777</v>
       </c>
       <c r="L95" s="10" t="n">
         <f aca="false">IF($J95=1,RANK($K95,$K$2:$K$1001),"")</f>
-        <v>87</v>
+        <v>118</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9917,11 +9917,11 @@
       </c>
       <c r="K96" s="10" t="n">
         <f aca="true">IF($J96=1,RAND(),-1)</f>
-        <v>0.0423926407650656</v>
+        <v>0.865161138553538</v>
       </c>
       <c r="L96" s="10" t="n">
         <f aca="false">IF($J96=1,RANK($K96,$K$2:$K$1001),"")</f>
-        <v>218</v>
+        <v>38</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9958,11 +9958,11 @@
       </c>
       <c r="K97" s="10" t="n">
         <f aca="true">IF($J97=1,RAND(),-1)</f>
-        <v>0.637608409198012</v>
+        <v>0.394322331263874</v>
       </c>
       <c r="L97" s="10" t="n">
         <f aca="false">IF($J97=1,RANK($K97,$K$2:$K$1001),"")</f>
-        <v>86</v>
+        <v>141</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9999,11 +9999,11 @@
       </c>
       <c r="K98" s="10" t="n">
         <f aca="true">IF($J98=1,RAND(),-1)</f>
-        <v>0.779207849745604</v>
+        <v>0.69299906804051</v>
       </c>
       <c r="L98" s="10" t="n">
         <f aca="false">IF($J98=1,RANK($K98,$K$2:$K$1001),"")</f>
-        <v>41</v>
+        <v>69</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10040,11 +10040,11 @@
       </c>
       <c r="K99" s="10" t="n">
         <f aca="true">IF($J99=1,RAND(),-1)</f>
-        <v>0.50668120328547</v>
+        <v>0.361289084216756</v>
       </c>
       <c r="L99" s="10" t="n">
         <f aca="false">IF($J99=1,RANK($K99,$K$2:$K$1001),"")</f>
-        <v>113</v>
+        <v>150</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10081,11 +10081,11 @@
       </c>
       <c r="K100" s="10" t="n">
         <f aca="true">IF($J100=1,RAND(),-1)</f>
-        <v>0.738550358783783</v>
+        <v>0.857505334891268</v>
       </c>
       <c r="L100" s="10" t="n">
         <f aca="false">IF($J100=1,RANK($K100,$K$2:$K$1001),"")</f>
-        <v>58</v>
+        <v>39</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10122,11 +10122,11 @@
       </c>
       <c r="K101" s="10" t="n">
         <f aca="true">IF($J101=1,RAND(),-1)</f>
-        <v>0.340154285135085</v>
+        <v>0.0085454298272071</v>
       </c>
       <c r="L101" s="10" t="n">
         <f aca="false">IF($J101=1,RANK($K101,$K$2:$K$1001),"")</f>
-        <v>147</v>
+        <v>221</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10163,11 +10163,11 @@
       </c>
       <c r="K102" s="10" t="n">
         <f aca="true">IF($J102=1,RAND(),-1)</f>
-        <v>0.746174210407143</v>
+        <v>0.0500666216787506</v>
       </c>
       <c r="L102" s="10" t="n">
         <f aca="false">IF($J102=1,RANK($K102,$K$2:$K$1001),"")</f>
-        <v>55</v>
+        <v>213</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10204,11 +10204,11 @@
       </c>
       <c r="K103" s="10" t="n">
         <f aca="true">IF($J103=1,RAND(),-1)</f>
-        <v>0.341315955454172</v>
+        <v>0.659693996074889</v>
       </c>
       <c r="L103" s="10" t="n">
         <f aca="false">IF($J103=1,RANK($K103,$K$2:$K$1001),"")</f>
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10245,11 +10245,11 @@
       </c>
       <c r="K104" s="10" t="n">
         <f aca="true">IF($J104=1,RAND(),-1)</f>
-        <v>0.00215534206579871</v>
+        <v>0.0904324555342125</v>
       </c>
       <c r="L104" s="10" t="n">
         <f aca="false">IF($J104=1,RANK($K104,$K$2:$K$1001),"")</f>
-        <v>224</v>
+        <v>205</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10286,11 +10286,11 @@
       </c>
       <c r="K105" s="10" t="n">
         <f aca="true">IF($J105=1,RAND(),-1)</f>
-        <v>0.755592147915079</v>
+        <v>0.385564515276341</v>
       </c>
       <c r="L105" s="10" t="n">
         <f aca="false">IF($J105=1,RANK($K105,$K$2:$K$1001),"")</f>
-        <v>48</v>
+        <v>145</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10327,11 +10327,11 @@
       </c>
       <c r="K106" s="10" t="n">
         <f aca="true">IF($J106=1,RAND(),-1)</f>
-        <v>0.516989573728296</v>
+        <v>0.0203937736530781</v>
       </c>
       <c r="L106" s="10" t="n">
         <f aca="false">IF($J106=1,RANK($K106,$K$2:$K$1001),"")</f>
-        <v>110</v>
+        <v>219</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10368,11 +10368,11 @@
       </c>
       <c r="K107" s="10" t="n">
         <f aca="true">IF($J107=1,RAND(),-1)</f>
-        <v>0.630285688359229</v>
+        <v>0.000511676368642079</v>
       </c>
       <c r="L107" s="10" t="n">
         <f aca="false">IF($J107=1,RANK($K107,$K$2:$K$1001),"")</f>
-        <v>88</v>
+        <v>224</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10409,11 +10409,11 @@
       </c>
       <c r="K108" s="10" t="n">
         <f aca="true">IF($J108=1,RAND(),-1)</f>
-        <v>0.417717872928716</v>
+        <v>0.23428617794462</v>
       </c>
       <c r="L108" s="10" t="n">
         <f aca="false">IF($J108=1,RANK($K108,$K$2:$K$1001),"")</f>
-        <v>133</v>
+        <v>175</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10450,11 +10450,11 @@
       </c>
       <c r="K109" s="10" t="n">
         <f aca="true">IF($J109=1,RAND(),-1)</f>
-        <v>0.927616239372093</v>
+        <v>0.719670427979772</v>
       </c>
       <c r="L109" s="10" t="n">
         <f aca="false">IF($J109=1,RANK($K109,$K$2:$K$1001),"")</f>
-        <v>14</v>
+        <v>65</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10491,11 +10491,11 @@
       </c>
       <c r="K110" s="10" t="n">
         <f aca="true">IF($J110=1,RAND(),-1)</f>
-        <v>0.247443042950957</v>
+        <v>0.668875119288646</v>
       </c>
       <c r="L110" s="10" t="n">
         <f aca="false">IF($J110=1,RANK($K110,$K$2:$K$1001),"")</f>
-        <v>168</v>
+        <v>75</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10532,11 +10532,11 @@
       </c>
       <c r="K111" s="10" t="n">
         <f aca="true">IF($J111=1,RAND(),-1)</f>
-        <v>0.300470771786984</v>
+        <v>0.961011270179639</v>
       </c>
       <c r="L111" s="10" t="n">
         <f aca="false">IF($J111=1,RANK($K111,$K$2:$K$1001),"")</f>
-        <v>159</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10573,11 +10573,11 @@
       </c>
       <c r="K112" s="10" t="n">
         <f aca="true">IF($J112=1,RAND(),-1)</f>
-        <v>0.655680982953881</v>
+        <v>0.791246261977891</v>
       </c>
       <c r="L112" s="10" t="n">
         <f aca="false">IF($J112=1,RANK($K112,$K$2:$K$1001),"")</f>
-        <v>82</v>
+        <v>57</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10614,11 +10614,11 @@
       </c>
       <c r="K113" s="10" t="n">
         <f aca="true">IF($J113=1,RAND(),-1)</f>
-        <v>0.121861610677491</v>
+        <v>0.340597115786885</v>
       </c>
       <c r="L113" s="10" t="n">
         <f aca="false">IF($J113=1,RANK($K113,$K$2:$K$1001),"")</f>
-        <v>203</v>
+        <v>155</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10655,11 +10655,11 @@
       </c>
       <c r="K114" s="10" t="n">
         <f aca="true">IF($J114=1,RAND(),-1)</f>
-        <v>0.196099628974739</v>
+        <v>0.676595018888443</v>
       </c>
       <c r="L114" s="10" t="n">
         <f aca="false">IF($J114=1,RANK($K114,$K$2:$K$1001),"")</f>
-        <v>190</v>
+        <v>72</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10696,11 +10696,11 @@
       </c>
       <c r="K115" s="10" t="n">
         <f aca="true">IF($J115=1,RAND(),-1)</f>
-        <v>0.443359526167945</v>
+        <v>0.123608914800153</v>
       </c>
       <c r="L115" s="10" t="n">
         <f aca="false">IF($J115=1,RANK($K115,$K$2:$K$1001),"")</f>
-        <v>129</v>
+        <v>197</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10737,11 +10737,11 @@
       </c>
       <c r="K116" s="10" t="n">
         <f aca="true">IF($J116=1,RAND(),-1)</f>
-        <v>0.850541606578792</v>
+        <v>0.296385560900438</v>
       </c>
       <c r="L116" s="10" t="n">
         <f aca="false">IF($J116=1,RANK($K116,$K$2:$K$1001),"")</f>
-        <v>30</v>
+        <v>169</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10778,11 +10778,11 @@
       </c>
       <c r="K117" s="10" t="n">
         <f aca="true">IF($J117=1,RAND(),-1)</f>
-        <v>0.48969266027149</v>
+        <v>0.0240653473670062</v>
       </c>
       <c r="L117" s="10" t="n">
         <f aca="false">IF($J117=1,RANK($K117,$K$2:$K$1001),"")</f>
-        <v>116</v>
+        <v>217</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10819,11 +10819,11 @@
       </c>
       <c r="K118" s="10" t="n">
         <f aca="true">IF($J118=1,RAND(),-1)</f>
-        <v>0.447273376993088</v>
+        <v>0.771819116925714</v>
       </c>
       <c r="L118" s="10" t="n">
         <f aca="false">IF($J118=1,RANK($K118,$K$2:$K$1001),"")</f>
-        <v>125</v>
+        <v>60</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10860,11 +10860,11 @@
       </c>
       <c r="K119" s="10" t="n">
         <f aca="true">IF($J119=1,RAND(),-1)</f>
-        <v>0.521175176280773</v>
+        <v>0.42092718711933</v>
       </c>
       <c r="L119" s="10" t="n">
         <f aca="false">IF($J119=1,RANK($K119,$K$2:$K$1001),"")</f>
-        <v>109</v>
+        <v>137</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10901,11 +10901,11 @@
       </c>
       <c r="K120" s="10" t="n">
         <f aca="true">IF($J120=1,RAND(),-1)</f>
-        <v>0.085699202164786</v>
+        <v>0.93689506322256</v>
       </c>
       <c r="L120" s="10" t="n">
         <f aca="false">IF($J120=1,RANK($K120,$K$2:$K$1001),"")</f>
-        <v>209</v>
+        <v>17</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10942,11 +10942,11 @@
       </c>
       <c r="K121" s="10" t="n">
         <f aca="true">IF($J121=1,RAND(),-1)</f>
-        <v>0.682203228816003</v>
+        <v>0.335009094208523</v>
       </c>
       <c r="L121" s="10" t="n">
         <f aca="false">IF($J121=1,RANK($K121,$K$2:$K$1001),"")</f>
-        <v>73</v>
+        <v>158</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10983,11 +10983,11 @@
       </c>
       <c r="K122" s="10" t="n">
         <f aca="true">IF($J122=1,RAND(),-1)</f>
-        <v>0.557647613963379</v>
+        <v>0.94472446819476</v>
       </c>
       <c r="L122" s="10" t="n">
         <f aca="false">IF($J122=1,RANK($K122,$K$2:$K$1001),"")</f>
-        <v>100</v>
+        <v>13</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11024,11 +11024,11 @@
       </c>
       <c r="K123" s="10" t="n">
         <f aca="true">IF($J123=1,RAND(),-1)</f>
-        <v>0.828808031928115</v>
+        <v>0.357631194715776</v>
       </c>
       <c r="L123" s="10" t="n">
         <f aca="false">IF($J123=1,RANK($K123,$K$2:$K$1001),"")</f>
-        <v>34</v>
+        <v>151</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11065,11 +11065,11 @@
       </c>
       <c r="K124" s="10" t="n">
         <f aca="true">IF($J124=1,RAND(),-1)</f>
-        <v>0.87233867851634</v>
+        <v>0.80281967370356</v>
       </c>
       <c r="L124" s="10" t="n">
         <f aca="false">IF($J124=1,RANK($K124,$K$2:$K$1001),"")</f>
-        <v>25</v>
+        <v>51</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11106,11 +11106,11 @@
       </c>
       <c r="K125" s="10" t="n">
         <f aca="true">IF($J125=1,RAND(),-1)</f>
-        <v>0.55539836076465</v>
+        <v>0.871396163152209</v>
       </c>
       <c r="L125" s="10" t="n">
         <f aca="false">IF($J125=1,RANK($K125,$K$2:$K$1001),"")</f>
-        <v>101</v>
+        <v>35</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11147,11 +11147,11 @@
       </c>
       <c r="K126" s="10" t="n">
         <f aca="true">IF($J126=1,RAND(),-1)</f>
-        <v>0.717474308952177</v>
+        <v>0.683756605991947</v>
       </c>
       <c r="L126" s="10" t="n">
         <f aca="false">IF($J126=1,RANK($K126,$K$2:$K$1001),"")</f>
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11188,11 +11188,11 @@
       </c>
       <c r="K127" s="10" t="n">
         <f aca="true">IF($J127=1,RAND(),-1)</f>
-        <v>0.770005274964834</v>
+        <v>0.143060150532722</v>
       </c>
       <c r="L127" s="10" t="n">
         <f aca="false">IF($J127=1,RANK($K127,$K$2:$K$1001),"")</f>
-        <v>44</v>
+        <v>193</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11229,11 +11229,11 @@
       </c>
       <c r="K128" s="10" t="n">
         <f aca="true">IF($J128=1,RAND(),-1)</f>
-        <v>0.693337847553307</v>
+        <v>0.219506479746253</v>
       </c>
       <c r="L128" s="10" t="n">
         <f aca="false">IF($J128=1,RANK($K128,$K$2:$K$1001),"")</f>
-        <v>66</v>
+        <v>177</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11270,11 +11270,11 @@
       </c>
       <c r="K129" s="10" t="n">
         <f aca="true">IF($J129=1,RAND(),-1)</f>
-        <v>0.339734730289051</v>
+        <v>0.210058299074953</v>
       </c>
       <c r="L129" s="10" t="n">
         <f aca="false">IF($J129=1,RANK($K129,$K$2:$K$1001),"")</f>
-        <v>148</v>
+        <v>179</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11311,11 +11311,11 @@
       </c>
       <c r="K130" s="10" t="n">
         <f aca="true">IF($J130=1,RAND(),-1)</f>
-        <v>0.462676854451784</v>
+        <v>0.911021369532592</v>
       </c>
       <c r="L130" s="10" t="n">
         <f aca="false">IF($J130=1,RANK($K130,$K$2:$K$1001),"")</f>
-        <v>121</v>
+        <v>22</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11352,11 +11352,11 @@
       </c>
       <c r="K131" s="10" t="n">
         <f aca="true">IF($J131=1,RAND(),-1)</f>
-        <v>0.0117478145349655</v>
+        <v>0.62920578801608</v>
       </c>
       <c r="L131" s="10" t="n">
         <f aca="false">IF($J131=1,RANK($K131,$K$2:$K$1001),"")</f>
-        <v>223</v>
+        <v>88</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11393,11 +11393,11 @@
       </c>
       <c r="K132" s="10" t="n">
         <f aca="true">IF($J132=1,RAND(),-1)</f>
-        <v>0.104452886900925</v>
+        <v>0.687173232745821</v>
       </c>
       <c r="L132" s="10" t="n">
         <f aca="false">IF($J132=1,RANK($K132,$K$2:$K$1001),"")</f>
-        <v>204</v>
+        <v>70</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11434,11 +11434,11 @@
       </c>
       <c r="K133" s="10" t="n">
         <f aca="true">IF($J133=1,RAND(),-1)</f>
-        <v>0.566823975446791</v>
+        <v>0.871166971319386</v>
       </c>
       <c r="L133" s="10" t="n">
         <f aca="false">IF($J133=1,RANK($K133,$K$2:$K$1001),"")</f>
-        <v>98</v>
+        <v>36</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11475,11 +11475,11 @@
       </c>
       <c r="K134" s="10" t="n">
         <f aca="true">IF($J134=1,RAND(),-1)</f>
-        <v>0.899664568396896</v>
+        <v>0.103830452119329</v>
       </c>
       <c r="L134" s="10" t="n">
         <f aca="false">IF($J134=1,RANK($K134,$K$2:$K$1001),"")</f>
-        <v>21</v>
+        <v>201</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11516,11 +11516,11 @@
       </c>
       <c r="K135" s="10" t="n">
         <f aca="true">IF($J135=1,RAND(),-1)</f>
-        <v>0.703217580624776</v>
+        <v>0.824840709209188</v>
       </c>
       <c r="L135" s="10" t="n">
         <f aca="false">IF($J135=1,RANK($K135,$K$2:$K$1001),"")</f>
-        <v>64</v>
+        <v>48</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11557,11 +11557,11 @@
       </c>
       <c r="K136" s="10" t="n">
         <f aca="true">IF($J136=1,RAND(),-1)</f>
-        <v>0.689125552468828</v>
+        <v>0.231945948178568</v>
       </c>
       <c r="L136" s="10" t="n">
         <f aca="false">IF($J136=1,RANK($K136,$K$2:$K$1001),"")</f>
-        <v>68</v>
+        <v>176</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11598,11 +11598,11 @@
       </c>
       <c r="K137" s="10" t="n">
         <f aca="true">IF($J137=1,RAND(),-1)</f>
-        <v>0.750403063118331</v>
+        <v>0.491211211907866</v>
       </c>
       <c r="L137" s="10" t="n">
         <f aca="false">IF($J137=1,RANK($K137,$K$2:$K$1001),"")</f>
-        <v>53</v>
+        <v>116</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11639,11 +11639,11 @@
       </c>
       <c r="K138" s="10" t="n">
         <f aca="true">IF($J138=1,RAND(),-1)</f>
-        <v>0.395861700449384</v>
+        <v>0.837077514857528</v>
       </c>
       <c r="L138" s="10" t="n">
         <f aca="false">IF($J138=1,RANK($K138,$K$2:$K$1001),"")</f>
-        <v>138</v>
+        <v>45</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11680,11 +11680,11 @@
       </c>
       <c r="K139" s="10" t="n">
         <f aca="true">IF($J139=1,RAND(),-1)</f>
-        <v>0.266617483398485</v>
+        <v>0.673776350438688</v>
       </c>
       <c r="L139" s="10" t="n">
         <f aca="false">IF($J139=1,RANK($K139,$K$2:$K$1001),"")</f>
-        <v>164</v>
+        <v>73</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11721,11 +11721,11 @@
       </c>
       <c r="K140" s="10" t="n">
         <f aca="true">IF($J140=1,RAND(),-1)</f>
-        <v>0.301583796925558</v>
+        <v>0.182254781063211</v>
       </c>
       <c r="L140" s="10" t="n">
         <f aca="false">IF($J140=1,RANK($K140,$K$2:$K$1001),"")</f>
-        <v>158</v>
+        <v>183</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11762,11 +11762,11 @@
       </c>
       <c r="K141" s="10" t="n">
         <f aca="true">IF($J141=1,RAND(),-1)</f>
-        <v>0.0626956173311706</v>
+        <v>0.389493107680685</v>
       </c>
       <c r="L141" s="10" t="n">
         <f aca="false">IF($J141=1,RANK($K141,$K$2:$K$1001),"")</f>
-        <v>213</v>
+        <v>143</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11803,11 +11803,11 @@
       </c>
       <c r="K142" s="10" t="n">
         <f aca="true">IF($J142=1,RAND(),-1)</f>
-        <v>0.231202680749116</v>
+        <v>0.942266334514505</v>
       </c>
       <c r="L142" s="10" t="n">
         <f aca="false">IF($J142=1,RANK($K142,$K$2:$K$1001),"")</f>
-        <v>174</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11844,11 +11844,11 @@
       </c>
       <c r="K143" s="10" t="n">
         <f aca="true">IF($J143=1,RAND(),-1)</f>
-        <v>0.820728171842168</v>
+        <v>0.0999027801806504</v>
       </c>
       <c r="L143" s="10" t="n">
         <f aca="false">IF($J143=1,RANK($K143,$K$2:$K$1001),"")</f>
-        <v>36</v>
+        <v>202</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11885,11 +11885,11 @@
       </c>
       <c r="K144" s="10" t="n">
         <f aca="true">IF($J144=1,RAND(),-1)</f>
-        <v>0.161695879619471</v>
+        <v>0.897547671865621</v>
       </c>
       <c r="L144" s="10" t="n">
         <f aca="false">IF($J144=1,RANK($K144,$K$2:$K$1001),"")</f>
-        <v>195</v>
+        <v>25</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11926,11 +11926,11 @@
       </c>
       <c r="K145" s="10" t="n">
         <f aca="true">IF($J145=1,RAND(),-1)</f>
-        <v>0.23728613606772</v>
+        <v>0.806330663198525</v>
       </c>
       <c r="L145" s="10" t="n">
         <f aca="false">IF($J145=1,RANK($K145,$K$2:$K$1001),"")</f>
-        <v>172</v>
+        <v>50</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11967,11 +11967,11 @@
       </c>
       <c r="K146" s="10" t="n">
         <f aca="true">IF($J146=1,RAND(),-1)</f>
-        <v>0.255834361872587</v>
+        <v>0.778098856076334</v>
       </c>
       <c r="L146" s="10" t="n">
         <f aca="false">IF($J146=1,RANK($K146,$K$2:$K$1001),"")</f>
-        <v>166</v>
+        <v>59</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12008,11 +12008,11 @@
       </c>
       <c r="K147" s="10" t="n">
         <f aca="true">IF($J147=1,RAND(),-1)</f>
-        <v>0.655585730608817</v>
+        <v>0.912635003153463</v>
       </c>
       <c r="L147" s="10" t="n">
         <f aca="false">IF($J147=1,RANK($K147,$K$2:$K$1001),"")</f>
-        <v>83</v>
+        <v>21</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12049,11 +12049,11 @@
       </c>
       <c r="K148" s="10" t="n">
         <f aca="true">IF($J148=1,RAND(),-1)</f>
-        <v>0.382063407839916</v>
+        <v>0.110232691653009</v>
       </c>
       <c r="L148" s="10" t="n">
         <f aca="false">IF($J148=1,RANK($K148,$K$2:$K$1001),"")</f>
-        <v>140</v>
+        <v>199</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12090,11 +12090,11 @@
       </c>
       <c r="K149" s="10" t="n">
         <f aca="true">IF($J149=1,RAND(),-1)</f>
-        <v>0.603051310496443</v>
+        <v>0.584969864151499</v>
       </c>
       <c r="L149" s="10" t="n">
         <f aca="false">IF($J149=1,RANK($K149,$K$2:$K$1001),"")</f>
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12131,11 +12131,11 @@
       </c>
       <c r="K150" s="10" t="n">
         <f aca="true">IF($J150=1,RAND(),-1)</f>
-        <v>0.0338854736977528</v>
+        <v>0.157921774291848</v>
       </c>
       <c r="L150" s="10" t="n">
         <f aca="false">IF($J150=1,RANK($K150,$K$2:$K$1001),"")</f>
-        <v>220</v>
+        <v>189</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12172,11 +12172,11 @@
       </c>
       <c r="K151" s="10" t="n">
         <f aca="true">IF($J151=1,RAND(),-1)</f>
-        <v>0.487151604139895</v>
+        <v>0.619060930429667</v>
       </c>
       <c r="L151" s="10" t="n">
         <f aca="false">IF($J151=1,RANK($K151,$K$2:$K$1001),"")</f>
-        <v>117</v>
+        <v>90</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12213,11 +12213,11 @@
       </c>
       <c r="K152" s="10" t="n">
         <f aca="true">IF($J152=1,RAND(),-1)</f>
-        <v>0.209748709944224</v>
+        <v>0.855990854216188</v>
       </c>
       <c r="L152" s="10" t="n">
         <f aca="false">IF($J152=1,RANK($K152,$K$2:$K$1001),"")</f>
-        <v>184</v>
+        <v>41</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12254,11 +12254,11 @@
       </c>
       <c r="K153" s="10" t="n">
         <f aca="true">IF($J153=1,RAND(),-1)</f>
-        <v>0.549125921689886</v>
+        <v>0.802036002436179</v>
       </c>
       <c r="L153" s="10" t="n">
         <f aca="false">IF($J153=1,RANK($K153,$K$2:$K$1001),"")</f>
-        <v>103</v>
+        <v>53</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12295,11 +12295,11 @@
       </c>
       <c r="K154" s="10" t="n">
         <f aca="true">IF($J154=1,RAND(),-1)</f>
-        <v>0.977769072890851</v>
+        <v>0.424245841497622</v>
       </c>
       <c r="L154" s="10" t="n">
         <f aca="false">IF($J154=1,RANK($K154,$K$2:$K$1001),"")</f>
-        <v>6</v>
+        <v>134</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12336,11 +12336,11 @@
       </c>
       <c r="K155" s="10" t="n">
         <f aca="true">IF($J155=1,RAND(),-1)</f>
-        <v>0.721899558721715</v>
+        <v>0.475351549567344</v>
       </c>
       <c r="L155" s="10" t="n">
         <f aca="false">IF($J155=1,RANK($K155,$K$2:$K$1001),"")</f>
-        <v>60</v>
+        <v>122</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12377,11 +12377,11 @@
       </c>
       <c r="K156" s="10" t="n">
         <f aca="true">IF($J156=1,RAND(),-1)</f>
-        <v>0.508496316922985</v>
+        <v>0.337349371237416</v>
       </c>
       <c r="L156" s="10" t="n">
         <f aca="false">IF($J156=1,RANK($K156,$K$2:$K$1001),"")</f>
-        <v>112</v>
+        <v>156</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12418,11 +12418,11 @@
       </c>
       <c r="K157" s="10" t="n">
         <f aca="true">IF($J157=1,RAND(),-1)</f>
-        <v>0.337179863372609</v>
+        <v>0.164542856925713</v>
       </c>
       <c r="L157" s="10" t="n">
         <f aca="false">IF($J157=1,RANK($K157,$K$2:$K$1001),"")</f>
-        <v>150</v>
+        <v>187</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12459,11 +12459,11 @@
       </c>
       <c r="K158" s="10" t="n">
         <f aca="true">IF($J158=1,RAND(),-1)</f>
-        <v>0.753861264017616</v>
+        <v>0.0993892966982251</v>
       </c>
       <c r="L158" s="10" t="n">
         <f aca="false">IF($J158=1,RANK($K158,$K$2:$K$1001),"")</f>
-        <v>50</v>
+        <v>203</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12500,11 +12500,11 @@
       </c>
       <c r="K159" s="10" t="n">
         <f aca="true">IF($J159=1,RAND(),-1)</f>
-        <v>0.685657388755455</v>
+        <v>0.051935386722993</v>
       </c>
       <c r="L159" s="10" t="n">
         <f aca="false">IF($J159=1,RANK($K159,$K$2:$K$1001),"")</f>
-        <v>71</v>
+        <v>212</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12541,11 +12541,11 @@
       </c>
       <c r="K160" s="10" t="n">
         <f aca="true">IF($J160=1,RAND(),-1)</f>
-        <v>0.163918923809161</v>
+        <v>0.632299723861741</v>
       </c>
       <c r="L160" s="10" t="n">
         <f aca="false">IF($J160=1,RANK($K160,$K$2:$K$1001),"")</f>
-        <v>194</v>
+        <v>86</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12582,11 +12582,11 @@
       </c>
       <c r="K161" s="10" t="n">
         <f aca="true">IF($J161=1,RAND(),-1)</f>
-        <v>0.815767602998773</v>
+        <v>0.488471513279944</v>
       </c>
       <c r="L161" s="10" t="n">
         <f aca="false">IF($J161=1,RANK($K161,$K$2:$K$1001),"")</f>
-        <v>37</v>
+        <v>117</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12623,11 +12623,11 @@
       </c>
       <c r="K162" s="10" t="n">
         <f aca="true">IF($J162=1,RAND(),-1)</f>
-        <v>0.334341538662202</v>
+        <v>0.459280401318719</v>
       </c>
       <c r="L162" s="10" t="n">
         <f aca="false">IF($J162=1,RANK($K162,$K$2:$K$1001),"")</f>
-        <v>151</v>
+        <v>130</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12664,11 +12664,11 @@
       </c>
       <c r="K163" s="10" t="n">
         <f aca="true">IF($J163=1,RAND(),-1)</f>
-        <v>0.134071274788761</v>
+        <v>0.508198060206101</v>
       </c>
       <c r="L163" s="10" t="n">
         <f aca="false">IF($J163=1,RANK($K163,$K$2:$K$1001),"")</f>
-        <v>198</v>
+        <v>108</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12705,11 +12705,11 @@
       </c>
       <c r="K164" s="10" t="n">
         <f aca="true">IF($J164=1,RAND(),-1)</f>
-        <v>0.205390393028098</v>
+        <v>0.65993792795874</v>
       </c>
       <c r="L164" s="10" t="n">
         <f aca="false">IF($J164=1,RANK($K164,$K$2:$K$1001),"")</f>
-        <v>186</v>
+        <v>79</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12746,11 +12746,11 @@
       </c>
       <c r="K165" s="10" t="n">
         <f aca="true">IF($J165=1,RAND(),-1)</f>
-        <v>0.19985362622563</v>
+        <v>0.527668571187509</v>
       </c>
       <c r="L165" s="10" t="n">
         <f aca="false">IF($J165=1,RANK($K165,$K$2:$K$1001),"")</f>
-        <v>189</v>
+        <v>103</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12787,11 +12787,11 @@
       </c>
       <c r="K166" s="10" t="n">
         <f aca="true">IF($J166=1,RAND(),-1)</f>
-        <v>0.353863805768526</v>
+        <v>0.493765718681731</v>
       </c>
       <c r="L166" s="10" t="n">
         <f aca="false">IF($J166=1,RANK($K166,$K$2:$K$1001),"")</f>
-        <v>143</v>
+        <v>115</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12828,11 +12828,11 @@
       </c>
       <c r="K167" s="10" t="n">
         <f aca="true">IF($J167=1,RAND(),-1)</f>
-        <v>0.224897974806035</v>
+        <v>0.536588241775471</v>
       </c>
       <c r="L167" s="10" t="n">
         <f aca="false">IF($J167=1,RANK($K167,$K$2:$K$1001),"")</f>
-        <v>175</v>
+        <v>99</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12869,11 +12869,11 @@
       </c>
       <c r="K168" s="10" t="n">
         <f aca="true">IF($J168=1,RAND(),-1)</f>
-        <v>0.671675376000405</v>
+        <v>0.802350072293827</v>
       </c>
       <c r="L168" s="10" t="n">
         <f aca="false">IF($J168=1,RANK($K168,$K$2:$K$1001),"")</f>
-        <v>76</v>
+        <v>52</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12910,11 +12910,11 @@
       </c>
       <c r="K169" s="10" t="n">
         <f aca="true">IF($J169=1,RAND(),-1)</f>
-        <v>0.242528180185341</v>
+        <v>0.365470227994834</v>
       </c>
       <c r="L169" s="10" t="n">
         <f aca="false">IF($J169=1,RANK($K169,$K$2:$K$1001),"")</f>
-        <v>170</v>
+        <v>149</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12951,11 +12951,11 @@
       </c>
       <c r="K170" s="10" t="n">
         <f aca="true">IF($J170=1,RAND(),-1)</f>
-        <v>0.902060037908911</v>
+        <v>0.487513108726873</v>
       </c>
       <c r="L170" s="10" t="n">
         <f aca="false">IF($J170=1,RANK($K170,$K$2:$K$1001),"")</f>
-        <v>19</v>
+        <v>119</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12992,11 +12992,11 @@
       </c>
       <c r="K171" s="10" t="n">
         <f aca="true">IF($J171=1,RAND(),-1)</f>
-        <v>0.685965510224414</v>
+        <v>0.132738112239013</v>
       </c>
       <c r="L171" s="10" t="n">
         <f aca="false">IF($J171=1,RANK($K171,$K$2:$K$1001),"")</f>
-        <v>70</v>
+        <v>196</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13033,11 +13033,11 @@
       </c>
       <c r="K172" s="10" t="n">
         <f aca="true">IF($J172=1,RAND(),-1)</f>
-        <v>0.947827068218964</v>
+        <v>0.661045610228075</v>
       </c>
       <c r="L172" s="10" t="n">
         <f aca="false">IF($J172=1,RANK($K172,$K$2:$K$1001),"")</f>
-        <v>11</v>
+        <v>77</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13074,11 +13074,11 @@
       </c>
       <c r="K173" s="10" t="n">
         <f aca="true">IF($J173=1,RAND(),-1)</f>
-        <v>0.0512148855371338</v>
+        <v>0.00259121062085419</v>
       </c>
       <c r="L173" s="10" t="n">
         <f aca="false">IF($J173=1,RANK($K173,$K$2:$K$1001),"")</f>
-        <v>216</v>
+        <v>222</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13115,11 +13115,11 @@
       </c>
       <c r="K174" s="10" t="n">
         <f aca="true">IF($J174=1,RAND(),-1)</f>
-        <v>0.98124004370203</v>
+        <v>0.474621708559967</v>
       </c>
       <c r="L174" s="10" t="n">
         <f aca="false">IF($J174=1,RANK($K174,$K$2:$K$1001),"")</f>
-        <v>5</v>
+        <v>123</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13156,11 +13156,11 @@
       </c>
       <c r="K175" s="10" t="n">
         <f aca="true">IF($J175=1,RAND(),-1)</f>
-        <v>0.205374799370152</v>
+        <v>0.202825324495148</v>
       </c>
       <c r="L175" s="10" t="n">
         <f aca="false">IF($J175=1,RANK($K175,$K$2:$K$1001),"")</f>
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13197,11 +13197,11 @@
       </c>
       <c r="K176" s="10" t="n">
         <f aca="true">IF($J176=1,RAND(),-1)</f>
-        <v>0.660739065571654</v>
+        <v>0.34175063927248</v>
       </c>
       <c r="L176" s="10" t="n">
         <f aca="false">IF($J176=1,RANK($K176,$K$2:$K$1001),"")</f>
-        <v>78</v>
+        <v>154</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13238,11 +13238,11 @@
       </c>
       <c r="K177" s="10" t="n">
         <f aca="true">IF($J177=1,RAND(),-1)</f>
-        <v>0.22372964825133</v>
+        <v>0.897897112690067</v>
       </c>
       <c r="L177" s="10" t="n">
         <f aca="false">IF($J177=1,RANK($K177,$K$2:$K$1001),"")</f>
-        <v>176</v>
+        <v>24</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13279,11 +13279,11 @@
       </c>
       <c r="K178" s="10" t="n">
         <f aca="true">IF($J178=1,RAND(),-1)</f>
-        <v>0.205407181625224</v>
+        <v>0.179265847200796</v>
       </c>
       <c r="L178" s="10" t="n">
         <f aca="false">IF($J178=1,RANK($K178,$K$2:$K$1001),"")</f>
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13320,11 +13320,11 @@
       </c>
       <c r="K179" s="10" t="n">
         <f aca="true">IF($J179=1,RAND(),-1)</f>
-        <v>0.619824893006421</v>
+        <v>0.641842943027085</v>
       </c>
       <c r="L179" s="10" t="n">
         <f aca="false">IF($J179=1,RANK($K179,$K$2:$K$1001),"")</f>
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13361,11 +13361,11 @@
       </c>
       <c r="K180" s="10" t="n">
         <f aca="true">IF($J180=1,RAND(),-1)</f>
-        <v>0.234540691598122</v>
+        <v>0.763305544873065</v>
       </c>
       <c r="L180" s="10" t="n">
         <f aca="false">IF($J180=1,RANK($K180,$K$2:$K$1001),"")</f>
-        <v>173</v>
+        <v>63</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13402,11 +13402,11 @@
       </c>
       <c r="K181" s="10" t="n">
         <f aca="true">IF($J181=1,RAND(),-1)</f>
-        <v>0.12417332513389</v>
+        <v>0.234372575814042</v>
       </c>
       <c r="L181" s="10" t="n">
         <f aca="false">IF($J181=1,RANK($K181,$K$2:$K$1001),"")</f>
-        <v>200</v>
+        <v>174</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13443,11 +13443,11 @@
       </c>
       <c r="K182" s="10" t="n">
         <f aca="true">IF($J182=1,RAND(),-1)</f>
-        <v>0.755333735876371</v>
+        <v>0.543922441310942</v>
       </c>
       <c r="L182" s="10" t="n">
         <f aca="false">IF($J182=1,RANK($K182,$K$2:$K$1001),"")</f>
-        <v>49</v>
+        <v>98</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13484,11 +13484,11 @@
       </c>
       <c r="K183" s="10" t="n">
         <f aca="true">IF($J183=1,RAND(),-1)</f>
-        <v>0.400898885594811</v>
+        <v>0.981975943982737</v>
       </c>
       <c r="L183" s="10" t="n">
         <f aca="false">IF($J183=1,RANK($K183,$K$2:$K$1001),"")</f>
-        <v>135</v>
+        <v>5</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13525,11 +13525,11 @@
       </c>
       <c r="K184" s="10" t="n">
         <f aca="true">IF($J184=1,RAND(),-1)</f>
-        <v>0.991426560939617</v>
+        <v>0.709924161053546</v>
       </c>
       <c r="L184" s="10" t="n">
         <f aca="false">IF($J184=1,RANK($K184,$K$2:$K$1001),"")</f>
-        <v>1</v>
+        <v>67</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13566,11 +13566,11 @@
       </c>
       <c r="K185" s="10" t="n">
         <f aca="true">IF($J185=1,RAND(),-1)</f>
-        <v>0.937456787432041</v>
+        <v>0.789632026038344</v>
       </c>
       <c r="L185" s="10" t="n">
         <f aca="false">IF($J185=1,RANK($K185,$K$2:$K$1001),"")</f>
-        <v>13</v>
+        <v>58</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13607,11 +13607,11 @@
       </c>
       <c r="K186" s="10" t="n">
         <f aca="true">IF($J186=1,RAND(),-1)</f>
-        <v>0.0918633295716413</v>
+        <v>0.771200411761574</v>
       </c>
       <c r="L186" s="10" t="n">
         <f aca="false">IF($J186=1,RANK($K186,$K$2:$K$1001),"")</f>
-        <v>208</v>
+        <v>61</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13648,11 +13648,11 @@
       </c>
       <c r="K187" s="10" t="n">
         <f aca="true">IF($J187=1,RAND(),-1)</f>
-        <v>0.0928951235954888</v>
+        <v>0.950702146338996</v>
       </c>
       <c r="L187" s="10" t="n">
         <f aca="false">IF($J187=1,RANK($K187,$K$2:$K$1001),"")</f>
-        <v>207</v>
+        <v>12</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13689,11 +13689,11 @@
       </c>
       <c r="K188" s="10" t="n">
         <f aca="true">IF($J188=1,RAND(),-1)</f>
-        <v>0.287845533092415</v>
+        <v>0.163280166830969</v>
       </c>
       <c r="L188" s="10" t="n">
         <f aca="false">IF($J188=1,RANK($K188,$K$2:$K$1001),"")</f>
-        <v>161</v>
+        <v>188</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13730,11 +13730,11 @@
       </c>
       <c r="K189" s="10" t="n">
         <f aca="true">IF($J189=1,RAND(),-1)</f>
-        <v>0.513632256887471</v>
+        <v>0.392979682347132</v>
       </c>
       <c r="L189" s="10" t="n">
         <f aca="false">IF($J189=1,RANK($K189,$K$2:$K$1001),"")</f>
-        <v>111</v>
+        <v>142</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13771,11 +13771,11 @@
       </c>
       <c r="K190" s="10" t="n">
         <f aca="true">IF($J190=1,RAND(),-1)</f>
-        <v>0.213734625138024</v>
+        <v>0.113574504775628</v>
       </c>
       <c r="L190" s="10" t="n">
         <f aca="false">IF($J190=1,RANK($K190,$K$2:$K$1001),"")</f>
-        <v>182</v>
+        <v>198</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13812,11 +13812,11 @@
       </c>
       <c r="K191" s="10" t="n">
         <f aca="true">IF($J191=1,RAND(),-1)</f>
-        <v>0.549772543356447</v>
+        <v>0.409610157219202</v>
       </c>
       <c r="L191" s="10" t="n">
         <f aca="false">IF($J191=1,RANK($K191,$K$2:$K$1001),"")</f>
-        <v>102</v>
+        <v>138</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13853,11 +13853,11 @@
       </c>
       <c r="K192" s="10" t="n">
         <f aca="true">IF($J192=1,RAND(),-1)</f>
-        <v>0.964740477711216</v>
+        <v>0.0711183634764639</v>
       </c>
       <c r="L192" s="10" t="n">
         <f aca="false">IF($J192=1,RANK($K192,$K$2:$K$1001),"")</f>
-        <v>9</v>
+        <v>209</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13894,11 +13894,11 @@
       </c>
       <c r="K193" s="10" t="n">
         <f aca="true">IF($J193=1,RAND(),-1)</f>
-        <v>0.52863231421442</v>
+        <v>0.486437279335669</v>
       </c>
       <c r="L193" s="10" t="n">
         <f aca="false">IF($J193=1,RANK($K193,$K$2:$K$1001),"")</f>
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13935,11 +13935,11 @@
       </c>
       <c r="K194" s="10" t="n">
         <f aca="true">IF($J194=1,RAND(),-1)</f>
-        <v>0.746030674148794</v>
+        <v>0.380824764511713</v>
       </c>
       <c r="L194" s="10" t="n">
         <f aca="false">IF($J194=1,RANK($K194,$K$2:$K$1001),"")</f>
-        <v>56</v>
+        <v>147</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13976,11 +13976,11 @@
       </c>
       <c r="K195" s="10" t="n">
         <f aca="true">IF($J195=1,RAND(),-1)</f>
-        <v>0.461391732218371</v>
+        <v>0.971292746926386</v>
       </c>
       <c r="L195" s="10" t="n">
         <f aca="false">IF($J195=1,RANK($K195,$K$2:$K$1001),"")</f>
-        <v>122</v>
+        <v>9</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14017,11 +14017,11 @@
       </c>
       <c r="K196" s="10" t="n">
         <f aca="true">IF($J196=1,RAND(),-1)</f>
-        <v>0.200154936373282</v>
+        <v>0.33673214609163</v>
       </c>
       <c r="L196" s="10" t="n">
         <f aca="false">IF($J196=1,RANK($K196,$K$2:$K$1001),"")</f>
-        <v>188</v>
+        <v>157</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14058,11 +14058,11 @@
       </c>
       <c r="K197" s="10" t="n">
         <f aca="true">IF($J197=1,RAND(),-1)</f>
-        <v>0.65645997674559</v>
+        <v>0.309351883826743</v>
       </c>
       <c r="L197" s="10" t="n">
         <f aca="false">IF($J197=1,RANK($K197,$K$2:$K$1001),"")</f>
-        <v>81</v>
+        <v>166</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14099,11 +14099,11 @@
       </c>
       <c r="K198" s="10" t="n">
         <f aca="true">IF($J198=1,RAND(),-1)</f>
-        <v>0.70804585461972</v>
+        <v>0.637756444938491</v>
       </c>
       <c r="L198" s="10" t="n">
         <f aca="false">IF($J198=1,RANK($K198,$K$2:$K$1001),"")</f>
-        <v>63</v>
+        <v>84</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14140,11 +14140,11 @@
       </c>
       <c r="K199" s="10" t="n">
         <f aca="true">IF($J199=1,RAND(),-1)</f>
-        <v>0.39657515641171</v>
+        <v>0.625542526439631</v>
       </c>
       <c r="L199" s="10" t="n">
         <f aca="false">IF($J199=1,RANK($K199,$K$2:$K$1001),"")</f>
-        <v>137</v>
+        <v>89</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14181,11 +14181,11 @@
       </c>
       <c r="K200" s="10" t="n">
         <f aca="true">IF($J200=1,RAND(),-1)</f>
-        <v>0.314898988797767</v>
+        <v>0.407673034730637</v>
       </c>
       <c r="L200" s="10" t="n">
         <f aca="false">IF($J200=1,RANK($K200,$K$2:$K$1001),"")</f>
-        <v>156</v>
+        <v>139</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14222,11 +14222,11 @@
       </c>
       <c r="K201" s="10" t="n">
         <f aca="true">IF($J201=1,RAND(),-1)</f>
-        <v>0.987948584105874</v>
+        <v>0.651276267119202</v>
       </c>
       <c r="L201" s="10" t="n">
         <f aca="false">IF($J201=1,RANK($K201,$K$2:$K$1001),"")</f>
-        <v>3</v>
+        <v>82</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14263,11 +14263,11 @@
       </c>
       <c r="K202" s="10" t="n">
         <f aca="true">IF($J202=1,RAND(),-1)</f>
-        <v>0.492777007837669</v>
+        <v>0.734183348302033</v>
       </c>
       <c r="L202" s="10" t="n">
         <f aca="false">IF($J202=1,RANK($K202,$K$2:$K$1001),"")</f>
-        <v>115</v>
+        <v>64</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14304,11 +14304,11 @@
       </c>
       <c r="K203" s="10" t="n">
         <f aca="true">IF($J203=1,RAND(),-1)</f>
-        <v>0.158827215751489</v>
+        <v>0.503112791192948</v>
       </c>
       <c r="L203" s="10" t="n">
         <f aca="false">IF($J203=1,RANK($K203,$K$2:$K$1001),"")</f>
-        <v>196</v>
+        <v>111</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14345,11 +14345,11 @@
       </c>
       <c r="K204" s="10" t="n">
         <f aca="true">IF($J204=1,RAND(),-1)</f>
-        <v>0.431955979198979</v>
+        <v>0.317399405349905</v>
       </c>
       <c r="L204" s="10" t="n">
         <f aca="false">IF($J204=1,RANK($K204,$K$2:$K$1001),"")</f>
-        <v>130</v>
+        <v>163</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14386,11 +14386,11 @@
       </c>
       <c r="K205" s="10" t="n">
         <f aca="true">IF($J205=1,RAND(),-1)</f>
-        <v>0.0355310865587619</v>
+        <v>0.704061869788255</v>
       </c>
       <c r="L205" s="10" t="n">
         <f aca="false">IF($J205=1,RANK($K205,$K$2:$K$1001),"")</f>
-        <v>219</v>
+        <v>68</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14427,11 +14427,11 @@
       </c>
       <c r="K206" s="10" t="n">
         <f aca="true">IF($J206=1,RAND(),-1)</f>
-        <v>0.165315859747264</v>
+        <v>0.474581002630719</v>
       </c>
       <c r="L206" s="10" t="n">
         <f aca="false">IF($J206=1,RANK($K206,$K$2:$K$1001),"")</f>
-        <v>193</v>
+        <v>124</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14468,11 +14468,11 @@
       </c>
       <c r="K207" s="10" t="n">
         <f aca="true">IF($J207=1,RAND(),-1)</f>
-        <v>0.845115465557651</v>
+        <v>0.249941262886327</v>
       </c>
       <c r="L207" s="10" t="n">
         <f aca="false">IF($J207=1,RANK($K207,$K$2:$K$1001),"")</f>
-        <v>31</v>
+        <v>172</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14509,11 +14509,11 @@
       </c>
       <c r="K208" s="10" t="n">
         <f aca="true">IF($J208=1,RAND(),-1)</f>
-        <v>0.676140089274124</v>
+        <v>0.513507807116659</v>
       </c>
       <c r="L208" s="10" t="n">
         <f aca="false">IF($J208=1,RANK($K208,$K$2:$K$1001),"")</f>
-        <v>75</v>
+        <v>107</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14550,11 +14550,11 @@
       </c>
       <c r="K209" s="10" t="n">
         <f aca="true">IF($J209=1,RAND(),-1)</f>
-        <v>0.241782721484014</v>
+        <v>0.180734135475498</v>
       </c>
       <c r="L209" s="10" t="n">
         <f aca="false">IF($J209=1,RANK($K209,$K$2:$K$1001),"")</f>
-        <v>171</v>
+        <v>185</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14591,11 +14591,11 @@
       </c>
       <c r="K210" s="10" t="n">
         <f aca="true">IF($J210=1,RAND(),-1)</f>
-        <v>0.122971558332874</v>
+        <v>0.387747605850991</v>
       </c>
       <c r="L210" s="10" t="n">
         <f aca="false">IF($J210=1,RANK($K210,$K$2:$K$1001),"")</f>
-        <v>202</v>
+        <v>144</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14632,11 +14632,11 @@
       </c>
       <c r="K211" s="10" t="n">
         <f aca="true">IF($J211=1,RAND(),-1)</f>
-        <v>0.871383154827596</v>
+        <v>0.943572875753399</v>
       </c>
       <c r="L211" s="10" t="n">
         <f aca="false">IF($J211=1,RANK($K211,$K$2:$K$1001),"")</f>
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14673,11 +14673,11 @@
       </c>
       <c r="K212" s="10" t="n">
         <f aca="true">IF($J212=1,RAND(),-1)</f>
-        <v>0.0737808739862672</v>
+        <v>0.576072507629386</v>
       </c>
       <c r="L212" s="10" t="n">
         <f aca="false">IF($J212=1,RANK($K212,$K$2:$K$1001),"")</f>
-        <v>212</v>
+        <v>96</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14714,11 +14714,11 @@
       </c>
       <c r="K213" s="10" t="n">
         <f aca="true">IF($J213=1,RAND(),-1)</f>
-        <v>0.501618801911886</v>
+        <v>0.87439651665626</v>
       </c>
       <c r="L213" s="10" t="n">
         <f aca="false">IF($J213=1,RANK($K213,$K$2:$K$1001),"")</f>
-        <v>114</v>
+        <v>33</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14755,11 +14755,11 @@
       </c>
       <c r="K214" s="10" t="n">
         <f aca="true">IF($J214=1,RAND(),-1)</f>
-        <v>0.6604906671634</v>
+        <v>0.504496277552898</v>
       </c>
       <c r="L214" s="10" t="n">
         <f aca="false">IF($J214=1,RANK($K214,$K$2:$K$1001),"")</f>
-        <v>79</v>
+        <v>110</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14796,11 +14796,11 @@
       </c>
       <c r="K215" s="10" t="n">
         <f aca="true">IF($J215=1,RAND(),-1)</f>
-        <v>0.15704667248935</v>
+        <v>0.6558769985017</v>
       </c>
       <c r="L215" s="10" t="n">
         <f aca="false">IF($J215=1,RANK($K215,$K$2:$K$1001),"")</f>
-        <v>197</v>
+        <v>81</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14837,11 +14837,11 @@
       </c>
       <c r="K216" s="10" t="n">
         <f aca="true">IF($J216=1,RAND(),-1)</f>
-        <v>0.990671621044228</v>
+        <v>0.494016043671386</v>
       </c>
       <c r="L216" s="10" t="n">
         <f aca="false">IF($J216=1,RANK($K216,$K$2:$K$1001),"")</f>
-        <v>2</v>
+        <v>114</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14878,11 +14878,11 @@
       </c>
       <c r="K217" s="10" t="n">
         <f aca="true">IF($J217=1,RAND(),-1)</f>
-        <v>0.353482771407603</v>
+        <v>0.469641892769389</v>
       </c>
       <c r="L217" s="10" t="n">
         <f aca="false">IF($J217=1,RANK($K217,$K$2:$K$1001),"")</f>
-        <v>144</v>
+        <v>126</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14919,11 +14919,11 @@
       </c>
       <c r="K218" s="10" t="n">
         <f aca="true">IF($J218=1,RAND(),-1)</f>
-        <v>0.578435704353801</v>
+        <v>0.856053300105813</v>
       </c>
       <c r="L218" s="10" t="n">
         <f aca="false">IF($J218=1,RANK($K218,$K$2:$K$1001),"")</f>
-        <v>95</v>
+        <v>40</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14960,11 +14960,11 @@
       </c>
       <c r="K219" s="10" t="n">
         <f aca="true">IF($J219=1,RAND(),-1)</f>
-        <v>0.544945531046399</v>
+        <v>0.150727812296675</v>
       </c>
       <c r="L219" s="10" t="n">
         <f aca="false">IF($J219=1,RANK($K219,$K$2:$K$1001),"")</f>
-        <v>105</v>
+        <v>190</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15001,11 +15001,11 @@
       </c>
       <c r="K220" s="10" t="n">
         <f aca="true">IF($J220=1,RAND(),-1)</f>
-        <v>0.049779700825681</v>
+        <v>0.664179764546981</v>
       </c>
       <c r="L220" s="10" t="n">
         <f aca="false">IF($J220=1,RANK($K220,$K$2:$K$1001),"")</f>
-        <v>217</v>
+        <v>76</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15042,11 +15042,11 @@
       </c>
       <c r="K221" s="10" t="n">
         <f aca="true">IF($J221=1,RAND(),-1)</f>
-        <v>0.464718922771775</v>
+        <v>0.826691576040576</v>
       </c>
       <c r="L221" s="10" t="n">
         <f aca="false">IF($J221=1,RANK($K221,$K$2:$K$1001),"")</f>
-        <v>120</v>
+        <v>47</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15083,11 +15083,11 @@
       </c>
       <c r="K222" s="10" t="n">
         <f aca="true">IF($J222=1,RAND(),-1)</f>
-        <v>0.0745229973619508</v>
+        <v>0.56611914748705</v>
       </c>
       <c r="L222" s="10" t="n">
         <f aca="false">IF($J222=1,RANK($K222,$K$2:$K$1001),"")</f>
-        <v>210</v>
+        <v>97</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15124,11 +15124,11 @@
       </c>
       <c r="K223" s="10" t="n">
         <f aca="true">IF($J223=1,RAND(),-1)</f>
-        <v>0.285300327261778</v>
+        <v>0.882391093214056</v>
       </c>
       <c r="L223" s="10" t="n">
         <f aca="false">IF($J223=1,RANK($K223,$K$2:$K$1001),"")</f>
-        <v>162</v>
+        <v>30</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15165,11 +15165,11 @@
       </c>
       <c r="K224" s="10" t="n">
         <f aca="true">IF($J224=1,RAND(),-1)</f>
-        <v>0.900710370681835</v>
+        <v>0.989230485249041</v>
       </c>
       <c r="L224" s="10" t="n">
         <f aca="false">IF($J224=1,RANK($K224,$K$2:$K$1001),"")</f>
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15206,11 +15206,11 @@
       </c>
       <c r="K225" s="10" t="n">
         <f aca="true">IF($J225=1,RAND(),-1)</f>
-        <v>0.394796933386587</v>
+        <v>0.606462043390667</v>
       </c>
       <c r="L225" s="10" t="n">
         <f aca="false">IF($J225=1,RANK($K225,$K$2:$K$1001),"")</f>
-        <v>139</v>
+        <v>92</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26125,11 +26125,11 @@
       </c>
       <c r="B4" s="5" t="str">
         <f aca="false">IF(Test!$J12="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J12))</f>
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="C4" s="12" t="str">
         <f aca="false">IF(B4="","",INDEX(Test!$C12:$F12,MATCH(B4,{"A","B","C","D"},0)))</f>
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26139,11 +26139,11 @@
       </c>
       <c r="B5" s="5" t="str">
         <f aca="false">IF(Test!$J13="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J13))</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="C5" s="12" t="str">
         <f aca="false">IF(B5="","",INDEX(Test!$C13:$F13,MATCH(B5,{"A","B","C","D"},0)))</f>
-        <v>1</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26153,11 +26153,11 @@
       </c>
       <c r="B6" s="5" t="str">
         <f aca="false">IF(Test!$J14="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J14))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="C6" s="12" t="str">
         <f aca="false">IF(B6="","",INDEX(Test!$C14:$F14,MATCH(B6,{"A","B","C","D"},0)))</f>
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26171,7 +26171,7 @@
       </c>
       <c r="C7" s="12" t="str">
         <f aca="false">IF(B7="","",INDEX(Test!$C15:$F15,MATCH(B7,{"A","B","C","D"},0)))</f>
-        <v>125</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26181,11 +26181,11 @@
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">IF(Test!$J16="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J16))</f>
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="C8" s="12" t="str">
         <f aca="false">IF(B8="","",INDEX(Test!$C16:$F16,MATCH(B8,{"A","B","C","D"},0)))</f>
-        <v>3</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26195,11 +26195,11 @@
       </c>
       <c r="B9" s="5" t="str">
         <f aca="false">IF(Test!$J17="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J17))</f>
-        <v>C</v>
+        <v>A</v>
       </c>
       <c r="C9" s="12" t="str">
         <f aca="false">IF(B9="","",INDEX(Test!$C17:$F17,MATCH(B9,{"A","B","C","D"},0)))</f>
-        <v>27 L</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26209,11 +26209,11 @@
       </c>
       <c r="B10" s="5" t="str">
         <f aca="false">IF(Test!$J18="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J18))</f>
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="C10" s="12" t="str">
         <f aca="false">IF(B10="","",INDEX(Test!$C18:$F18,MATCH(B10,{"A","B","C","D"},0)))</f>
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26223,11 +26223,11 @@
       </c>
       <c r="B11" s="5" t="str">
         <f aca="false">IF(Test!$J19="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J19))</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="C11" s="12" t="str">
         <f aca="false">IF(B11="","",INDEX(Test!$C19:$F19,MATCH(B11,{"A","B","C","D"},0)))</f>
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26237,11 +26237,11 @@
       </c>
       <c r="B12" s="5" t="str">
         <f aca="false">IF(Test!$J20="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J20))</f>
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="C12" s="12" t="str">
         <f aca="false">IF(B12="","",INDEX(Test!$C20:$F20,MATCH(B12,{"A","B","C","D"},0)))</f>
-        <v>294</v>
+        <v>600</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26251,11 +26251,11 @@
       </c>
       <c r="B13" s="5" t="str">
         <f aca="false">IF(Test!$J21="","",INDEX('Soru Havuzu'!$I$2:$I$1001,Test!$J21))</f>
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="C13" s="12" t="str">
         <f aca="false">IF(B13="","",INDEX(Test!$C21:$F21,MATCH(B13,{"A","B","C","D"},0)))</f>
-        <v>1000</v>
+        <v>512</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>